<commit_message>
Phase 0 steps 4-8: anonymous population, customer master timelines, attribution ground truth
</commit_message>
<xml_diff>
--- a/File_Manifest.xlsx
+++ b/File_Manifest.xlsx
@@ -435,7 +435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D14"/>
+  <dimension ref="A1:D21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="48" customWidth="1" min="1" max="1"/>
@@ -506,7 +506,7 @@
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-29 20:07 PDT</t>
+          <t>2026-07-29 20:35 PDT</t>
         </is>
       </c>
     </row>
@@ -594,7 +594,7 @@
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>2026-07-29 20:01 PDT</t>
+          <t>2026-07-29 20:12 PDT</t>
         </is>
       </c>
     </row>
@@ -638,7 +638,7 @@
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>2026-07-29 20:07 PDT</t>
+          <t>2026-07-29 20:34 PDT</t>
         </is>
       </c>
     </row>
@@ -748,7 +748,161 @@
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>2026-07-29 20:07 PDT</t>
+          <t>2026-07-29 20:35 PDT</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>generator/sim_utils.py</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>Code</t>
+        </is>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>Shared weighted date/channel sampling helpers</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-29 20:11 PDT</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>generator/build_anonymous_population.py</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>Code</t>
+        </is>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>Phase 0 Step 4: builds the ~2,000-person anonymous ghost population</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-29 20:11 PDT</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>generator/simulate_customers.py</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>Code</t>
+        </is>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>Phase 0 Steps 5-6: per-customer master timeline + attribution ground truth</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-29 20:12 PDT</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>internal/_sim_anonymous_population.csv</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>Internal artifact</t>
+        </is>
+      </c>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>Anonymous visitors who never become tracked customers; source of guest merch orders</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-29 20:11 PDT</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>internal/_sim_customer_timeline.json</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>Internal artifact</t>
+        </is>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>Full nested ground-truth simulation for all 100 customers (signup, trial, subscriptions, orders, churn)</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-29 20:12 PDT</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>internal/_sim_customer_timeline_summary.csv</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>Internal artifact</t>
+        </is>
+      </c>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>Flattened, spreadsheet-readable summary of the customer timeline</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-29 20:12 PDT</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>internal/_sim_attribution_ground_truth.json</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>Internal artifact</t>
+        </is>
+      </c>
+      <c r="C21" s="3" t="inlineStr">
+        <is>
+          <t>True acquisition/reactivation channel per customer, kept separate from intentionally messy shipped UTM data</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-29 20:12 PDT</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Recalibrate retention model: 100 active subscribers, two-segment churn, simulation analysis + charts
</commit_message>
<xml_diff>
--- a/File_Manifest.xlsx
+++ b/File_Manifest.xlsx
@@ -435,7 +435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D21"/>
+  <dimension ref="A1:D25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="48" customWidth="1" min="1" max="1"/>
@@ -506,7 +506,7 @@
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-29 20:35 PDT</t>
+          <t>2026-07-29 21:16 PDT</t>
         </is>
       </c>
     </row>
@@ -594,7 +594,7 @@
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>2026-07-29 20:12 PDT</t>
+          <t>2026-07-29 21:12 PDT</t>
         </is>
       </c>
     </row>
@@ -638,7 +638,7 @@
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>2026-07-29 20:34 PDT</t>
+          <t>2026-07-29 21:15 PDT</t>
         </is>
       </c>
     </row>
@@ -748,7 +748,7 @@
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>2026-07-29 20:35 PDT</t>
+          <t>2026-07-29 21:16 PDT</t>
         </is>
       </c>
     </row>
@@ -814,7 +814,7 @@
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t>2026-07-29 20:12 PDT</t>
+          <t>2026-07-29 21:12 PDT</t>
         </is>
       </c>
     </row>
@@ -836,7 +836,7 @@
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>2026-07-29 20:11 PDT</t>
+          <t>2026-07-29 21:13 PDT</t>
         </is>
       </c>
     </row>
@@ -858,7 +858,7 @@
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>2026-07-29 20:12 PDT</t>
+          <t>2026-07-29 21:12 PDT</t>
         </is>
       </c>
     </row>
@@ -880,7 +880,7 @@
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>2026-07-29 20:12 PDT</t>
+          <t>2026-07-29 21:12 PDT</t>
         </is>
       </c>
     </row>
@@ -902,7 +902,95 @@
       </c>
       <c r="D21" s="2" t="inlineStr">
         <is>
-          <t>2026-07-29 20:12 PDT</t>
+          <t>2026-07-29 21:12 PDT</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>generator/build_simulation_charts.py</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>Code</t>
+        </is>
+      </c>
+      <c r="C22" s="3" t="inlineStr">
+        <is>
+          <t>Builds the funnel + segment breakdown charts for the simulation analysis</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-29 21:14 PDT</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>internal/funnel_chart.png</t>
+        </is>
+      </c>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>Chart</t>
+        </is>
+      </c>
+      <c r="C23" s="3" t="inlineStr">
+        <is>
+          <t>Customer funnel: total -&gt; trial started -&gt; converted -&gt; active today</t>
+        </is>
+      </c>
+      <c r="D23" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-29 21:14 PDT</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>internal/segment_breakdown_chart.png</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>Chart</t>
+        </is>
+      </c>
+      <c r="C24" s="3" t="inlineStr">
+        <is>
+          <t>Part-to-whole breakdown of all customers' current status</t>
+        </is>
+      </c>
+      <c r="D24" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-29 21:14 PDT</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>docs/phase0_simulation_analysis.md</t>
+        </is>
+      </c>
+      <c r="B25" s="2" t="inlineStr">
+        <is>
+          <t>Docs</t>
+        </is>
+      </c>
+      <c r="C25" s="3" t="inlineStr">
+        <is>
+          <t>Summary analysis of the recalibrated Phase 0 simulation results</t>
+        </is>
+      </c>
+      <c r="D25" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-29 21:15 PDT</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
January-cluster win-backs; add email-acquired-subscriber pathway; fix 2 latent edge-case bugs
- Win-back timing now sampled by calendar month only (January-clustered),
  independent of the multi-year growth trend that skewed a first attempt.
- New pathway: course/merch-only customers can be nudged into a trial by a
  targeted email based on their own purchase history (17.5% reach, 47.5%
  trial conversion vs 30% baseline).
- Fixed: engagement tier was keyed off original account_type instead of
  actual conversion/active status.
- Fixed: a signup in the final week of the dataset could be marked
  'converted' with zero subscription intervals; now trial_in_progress.
- Recalibrated scale (1,100->860 customers, 21,800->17,050 anonymous) since
  the new email pathway pushed active subscribers to 128; back to 98.
</commit_message>
<xml_diff>
--- a/File_Manifest.xlsx
+++ b/File_Manifest.xlsx
@@ -506,7 +506,7 @@
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-29 21:16 PDT</t>
+          <t>2026-07-29 21:38 PDT</t>
         </is>
       </c>
     </row>
@@ -572,7 +572,7 @@
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>2026-07-29 19:56 PDT</t>
+          <t>2026-07-29 21:38 PDT</t>
         </is>
       </c>
     </row>
@@ -594,7 +594,7 @@
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>2026-07-29 21:12 PDT</t>
+          <t>2026-07-29 21:34 PDT</t>
         </is>
       </c>
     </row>
@@ -748,7 +748,7 @@
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>2026-07-29 21:16 PDT</t>
+          <t>2026-07-29 21:38 PDT</t>
         </is>
       </c>
     </row>
@@ -770,7 +770,7 @@
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>2026-07-29 20:11 PDT</t>
+          <t>2026-07-29 21:33 PDT</t>
         </is>
       </c>
     </row>
@@ -814,7 +814,7 @@
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t>2026-07-29 21:12 PDT</t>
+          <t>2026-07-29 21:37 PDT</t>
         </is>
       </c>
     </row>
@@ -836,7 +836,7 @@
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>2026-07-29 21:13 PDT</t>
+          <t>2026-07-29 21:35 PDT</t>
         </is>
       </c>
     </row>
@@ -858,7 +858,7 @@
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>2026-07-29 21:12 PDT</t>
+          <t>2026-07-29 21:36 PDT</t>
         </is>
       </c>
     </row>
@@ -880,7 +880,7 @@
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>2026-07-29 21:12 PDT</t>
+          <t>2026-07-29 21:36 PDT</t>
         </is>
       </c>
     </row>
@@ -902,7 +902,7 @@
       </c>
       <c r="D21" s="2" t="inlineStr">
         <is>
-          <t>2026-07-29 21:12 PDT</t>
+          <t>2026-07-29 21:36 PDT</t>
         </is>
       </c>
     </row>
@@ -924,7 +924,7 @@
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>2026-07-29 21:14 PDT</t>
+          <t>2026-07-29 21:35 PDT</t>
         </is>
       </c>
     </row>
@@ -946,7 +946,7 @@
       </c>
       <c r="D23" s="2" t="inlineStr">
         <is>
-          <t>2026-07-29 21:14 PDT</t>
+          <t>2026-07-29 21:36 PDT</t>
         </is>
       </c>
     </row>
@@ -968,7 +968,7 @@
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>2026-07-29 21:14 PDT</t>
+          <t>2026-07-29 21:36 PDT</t>
         </is>
       </c>
     </row>
@@ -990,7 +990,7 @@
       </c>
       <c r="D25" s="2" t="inlineStr">
         <is>
-          <t>2026-07-29 21:15 PDT</t>
+          <t>2026-07-29 21:38 PDT</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Phase 1: build + validate products table (1 of 47 shipped tables)
- Minimal 12-item catalog: 5 courses + 7 merch, one product per existing
  price tier (plus one duplicate at the 4.99 merch tier).
- is_subscription_eligible true only for courses.
- 18-check pandas-based validator (duckdb unavailable in this sandbox):
  structural/referential/temporal/business-rule/distributional, including
  an explicit reconciliation against the subscriber merch discount so
  discounted order prices still resolve to a real catalog product.
</commit_message>
<xml_diff>
--- a/File_Manifest.xlsx
+++ b/File_Manifest.xlsx
@@ -435,7 +435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D25"/>
+  <dimension ref="A1:D28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="48" customWidth="1" min="1" max="1"/>
@@ -638,7 +638,7 @@
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>2026-07-29 21:15 PDT</t>
+          <t>2026-07-29 21:55 PDT</t>
         </is>
       </c>
     </row>
@@ -748,7 +748,7 @@
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>2026-07-29 21:38 PDT</t>
+          <t>2026-07-29 21:55 PDT</t>
         </is>
       </c>
     </row>
@@ -991,6 +991,72 @@
       <c r="D25" s="2" t="inlineStr">
         <is>
           <t>2026-07-29 21:38 PDT</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>generator/build_products.py</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>Code</t>
+        </is>
+      </c>
+      <c r="C26" s="3" t="inlineStr">
+        <is>
+          <t>Phase 1: builds the products table (~12-item course/merch catalog)</t>
+        </is>
+      </c>
+      <c r="D26" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-29 21:55 PDT</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="inlineStr">
+        <is>
+          <t>generator/validate_products.py</t>
+        </is>
+      </c>
+      <c r="B27" s="2" t="inlineStr">
+        <is>
+          <t>Code</t>
+        </is>
+      </c>
+      <c r="C27" s="3" t="inlineStr">
+        <is>
+          <t>Phase 1: 5-layer validation for products (structural/referential/temporal/business-rule/distributional)</t>
+        </is>
+      </c>
+      <c r="D27" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-29 21:55 PDT</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t>data/products.csv</t>
+        </is>
+      </c>
+      <c r="B28" s="2" t="inlineStr">
+        <is>
+          <t>Shipped table</t>
+        </is>
+      </c>
+      <c r="C28" s="3" t="inlineStr">
+        <is>
+          <t>Phase 1: products table (course + merch catalog)</t>
+        </is>
+      </c>
+      <c r="D28" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-29 21:55 PDT</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Phase 1: build + validate product_variants table (2 of 47 shipped tables)
- 21 variants across 12 products: sized apparel gets S/M/L/XL, cap gets One
  Size, everything else gets a single Default/Standard Access variant.
- 18-check validator including the project's first real referential-integrity
  check (product_id FK to products, verified both directions).
</commit_message>
<xml_diff>
--- a/File_Manifest.xlsx
+++ b/File_Manifest.xlsx
@@ -435,7 +435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D28"/>
+  <dimension ref="A1:D31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="48" customWidth="1" min="1" max="1"/>
@@ -506,7 +506,7 @@
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-29 21:38 PDT</t>
+          <t>2026-07-29 21:56 PDT</t>
         </is>
       </c>
     </row>
@@ -638,7 +638,7 @@
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>2026-07-29 21:55 PDT</t>
+          <t>2026-07-29 21:58 PDT</t>
         </is>
       </c>
     </row>
@@ -748,7 +748,7 @@
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>2026-07-29 21:55 PDT</t>
+          <t>2026-07-29 21:58 PDT</t>
         </is>
       </c>
     </row>
@@ -1057,6 +1057,72 @@
       <c r="D28" s="2" t="inlineStr">
         <is>
           <t>2026-07-29 21:55 PDT</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="inlineStr">
+        <is>
+          <t>generator/build_product_variants.py</t>
+        </is>
+      </c>
+      <c r="B29" s="2" t="inlineStr">
+        <is>
+          <t>Code</t>
+        </is>
+      </c>
+      <c r="C29" s="3" t="inlineStr">
+        <is>
+          <t>Phase 1: builds product_variants (sizes for apparel, single variant elsewhere)</t>
+        </is>
+      </c>
+      <c r="D29" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-29 21:57 PDT</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="inlineStr">
+        <is>
+          <t>generator/validate_product_variants.py</t>
+        </is>
+      </c>
+      <c r="B30" s="2" t="inlineStr">
+        <is>
+          <t>Code</t>
+        </is>
+      </c>
+      <c r="C30" s="3" t="inlineStr">
+        <is>
+          <t>Phase 1: 5-layer validation for product_variants, including FK to products</t>
+        </is>
+      </c>
+      <c r="D30" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-29 21:57 PDT</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="inlineStr">
+        <is>
+          <t>data/product_variants.csv</t>
+        </is>
+      </c>
+      <c r="B31" s="2" t="inlineStr">
+        <is>
+          <t>Shipped table</t>
+        </is>
+      </c>
+      <c r="C31" s="3" t="inlineStr">
+        <is>
+          <t>Phase 1: product_variants table (21 variants across 12 products)</t>
+        </is>
+      </c>
+      <c r="D31" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-29 21:57 PDT</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Phase 1: build + validate subscription_plans table (3 of 47 shipped tables)
- 4 plans: Basic/Plus x monthly/annual. Added PLUS_ANNUAL=314.00 to params.py
  at the same discount ratio as BASIC_ANNUAL.
- 19-check validator; flagged that the master timeline only tracks plan tier
  (basic/plus), not billing interval -- Phase 2 will need to assign that
  itself when building real subscription interval rows.
</commit_message>
<xml_diff>
--- a/File_Manifest.xlsx
+++ b/File_Manifest.xlsx
@@ -435,7 +435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D31"/>
+  <dimension ref="A1:D34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="48" customWidth="1" min="1" max="1"/>
@@ -506,7 +506,7 @@
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-29 21:56 PDT</t>
+          <t>2026-07-29 21:58 PDT</t>
         </is>
       </c>
     </row>
@@ -594,7 +594,7 @@
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>2026-07-29 21:34 PDT</t>
+          <t>2026-07-29 21:59 PDT</t>
         </is>
       </c>
     </row>
@@ -638,7 +638,7 @@
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>2026-07-29 21:58 PDT</t>
+          <t>2026-07-29 22:00 PDT</t>
         </is>
       </c>
     </row>
@@ -748,7 +748,7 @@
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>2026-07-29 21:58 PDT</t>
+          <t>2026-07-29 22:00 PDT</t>
         </is>
       </c>
     </row>
@@ -1123,6 +1123,72 @@
       <c r="D31" s="2" t="inlineStr">
         <is>
           <t>2026-07-29 21:57 PDT</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="inlineStr">
+        <is>
+          <t>generator/build_subscription_plans.py</t>
+        </is>
+      </c>
+      <c r="B32" s="2" t="inlineStr">
+        <is>
+          <t>Code</t>
+        </is>
+      </c>
+      <c r="C32" s="3" t="inlineStr">
+        <is>
+          <t>Phase 1: builds subscription_plans (Basic/Plus x monthly/annual)</t>
+        </is>
+      </c>
+      <c r="D32" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-29 21:59 PDT</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="2" t="inlineStr">
+        <is>
+          <t>generator/validate_subscription_plans.py</t>
+        </is>
+      </c>
+      <c r="B33" s="2" t="inlineStr">
+        <is>
+          <t>Code</t>
+        </is>
+      </c>
+      <c r="C33" s="3" t="inlineStr">
+        <is>
+          <t>Phase 1: 5-layer validation for subscription_plans</t>
+        </is>
+      </c>
+      <c r="D33" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-29 22:00 PDT</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="2" t="inlineStr">
+        <is>
+          <t>data/subscription_plans.csv</t>
+        </is>
+      </c>
+      <c r="B34" s="2" t="inlineStr">
+        <is>
+          <t>Shipped table</t>
+        </is>
+      </c>
+      <c r="C34" s="3" t="inlineStr">
+        <is>
+          <t>Phase 1: subscription_plans table (4 plans)</t>
+        </is>
+      </c>
+      <c r="D34" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-29 22:00 PDT</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Phase 1: build + validate customers table (4 of 47 shipped tables)
- 860 rows, one per simulated customer, derived directly from the master
  timeline. Defines customer_id_for() mapping for all later tables to reuse.
- Synthetic names/emails (no faker available), soft-delete PII scrubbing
  (~2% rate) while preserving customer_id/history elsewhere.
- 22-check validator including an exact 1:1 reconciliation against the
  timeline's signup_date and signup_source for all 860 rows (0 mismatches).
</commit_message>
<xml_diff>
--- a/File_Manifest.xlsx
+++ b/File_Manifest.xlsx
@@ -435,7 +435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D34"/>
+  <dimension ref="A1:D37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="48" customWidth="1" min="1" max="1"/>
@@ -506,7 +506,7 @@
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-29 21:58 PDT</t>
+          <t>2026-07-29 22:00 PDT</t>
         </is>
       </c>
     </row>
@@ -594,7 +594,7 @@
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>2026-07-29 21:59 PDT</t>
+          <t>2026-07-29 22:02 PDT</t>
         </is>
       </c>
     </row>
@@ -638,7 +638,7 @@
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>2026-07-29 22:00 PDT</t>
+          <t>2026-07-29 22:02 PDT</t>
         </is>
       </c>
     </row>
@@ -748,7 +748,7 @@
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>2026-07-29 22:00 PDT</t>
+          <t>2026-07-29 22:02 PDT</t>
         </is>
       </c>
     </row>
@@ -1189,6 +1189,72 @@
       <c r="D34" s="2" t="inlineStr">
         <is>
           <t>2026-07-29 22:00 PDT</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="2" t="inlineStr">
+        <is>
+          <t>generator/build_customers.py</t>
+        </is>
+      </c>
+      <c r="B35" s="2" t="inlineStr">
+        <is>
+          <t>Code</t>
+        </is>
+      </c>
+      <c r="C35" s="3" t="inlineStr">
+        <is>
+          <t>Phase 1: builds customers table from the master timeline; defines customer_id mapping</t>
+        </is>
+      </c>
+      <c r="D35" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-29 22:02 PDT</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="2" t="inlineStr">
+        <is>
+          <t>generator/validate_customers.py</t>
+        </is>
+      </c>
+      <c r="B36" s="2" t="inlineStr">
+        <is>
+          <t>Code</t>
+        </is>
+      </c>
+      <c r="C36" s="3" t="inlineStr">
+        <is>
+          <t>Phase 1: 5-layer validation for customers, incl. 1:1 reconciliation vs. the timeline</t>
+        </is>
+      </c>
+      <c r="D36" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-29 22:02 PDT</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="2" t="inlineStr">
+        <is>
+          <t>data/customers.csv</t>
+        </is>
+      </c>
+      <c r="B37" s="2" t="inlineStr">
+        <is>
+          <t>Shipped table</t>
+        </is>
+      </c>
+      <c r="C37" s="3" t="inlineStr">
+        <is>
+          <t>Phase 1: customers table (860 rows, one per simulated customer)</t>
+        </is>
+      </c>
+      <c r="D37" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-29 22:02 PDT</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Fix customers: force email/push opt-in True for reactivation touchpoints
Ben caught that email_opt_in/push_opt_in were assigned independently of the
timeline, so a customer who was reactivated (or, for email, converted via
the merch-to-subscriber trigger) via a channel could end up NOT opted into
it -- an impossible state (can't receive a marketing send you never opted
into). Found 9 real violations for email; push had 0 only by chance this
seed. Fixed by forcing the opt-in True for anyone the timeline shows as
touched by that channel, before any random roll. Added 2 permanent
validator checks so this can't silently regress.
</commit_message>
<xml_diff>
--- a/File_Manifest.xlsx
+++ b/File_Manifest.xlsx
@@ -506,7 +506,7 @@
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-29 22:00 PDT</t>
+          <t>2026-07-29 22:06 PDT</t>
         </is>
       </c>
     </row>
@@ -748,7 +748,7 @@
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>2026-07-29 22:02 PDT</t>
+          <t>2026-07-29 22:06 PDT</t>
         </is>
       </c>
     </row>
@@ -1210,7 +1210,7 @@
       </c>
       <c r="D35" s="2" t="inlineStr">
         <is>
-          <t>2026-07-29 22:02 PDT</t>
+          <t>2026-07-29 22:05 PDT</t>
         </is>
       </c>
     </row>
@@ -1232,7 +1232,7 @@
       </c>
       <c r="D36" s="2" t="inlineStr">
         <is>
-          <t>2026-07-29 22:02 PDT</t>
+          <t>2026-07-29 22:05 PDT</t>
         </is>
       </c>
     </row>
@@ -1254,7 +1254,7 @@
       </c>
       <c r="D37" s="2" t="inlineStr">
         <is>
-          <t>2026-07-29 22:02 PDT</t>
+          <t>2026-07-29 22:05 PDT</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Make all generated customer emails unambiguously fake
Prefixed every email domain with 'fake' (gmail.com -> fakegmail.com, etc.)
so no generated address can be mistaken for a real person's real email.
Added a permanent validator check confirming every domain is either
fake-prefixed or the deleted-account placeholder.
</commit_message>
<xml_diff>
--- a/File_Manifest.xlsx
+++ b/File_Manifest.xlsx
@@ -506,7 +506,7 @@
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-29 22:06 PDT</t>
+          <t>2026-07-29 22:07 PDT</t>
         </is>
       </c>
     </row>
@@ -748,7 +748,7 @@
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>2026-07-29 22:06 PDT</t>
+          <t>2026-07-29 22:07 PDT</t>
         </is>
       </c>
     </row>
@@ -1210,7 +1210,7 @@
       </c>
       <c r="D35" s="2" t="inlineStr">
         <is>
-          <t>2026-07-29 22:05 PDT</t>
+          <t>2026-07-29 22:07 PDT</t>
         </is>
       </c>
     </row>
@@ -1232,7 +1232,7 @@
       </c>
       <c r="D36" s="2" t="inlineStr">
         <is>
-          <t>2026-07-29 22:05 PDT</t>
+          <t>2026-07-29 22:07 PDT</t>
         </is>
       </c>
     </row>
@@ -1254,7 +1254,7 @@
       </c>
       <c r="D37" s="2" t="inlineStr">
         <is>
-          <t>2026-07-29 22:05 PDT</t>
+          <t>2026-07-29 22:07 PDT</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Phase 1: build + validate customer_addresses table (5 of 47 shipped tables)
- Billing address for subscriber-path customers + anyone with an order;
  shipping address additionally for anyone with a merch order. Deleted
  customers get zero address rows (full erasure).
- Addresses made obviously fake via a guaranteed-nonexistent street name
  ('<number> Fake <word> <suffix>'), mirroring the fake-email-domain
  approach, while city/state/zip stay realistic for analytics variety.
- 21-check validator with exact set-equality checks on who needs
  billing/shipping, zero rows for deleted customers, and temporal alignment
  between shipping created_at and first merch order date.
</commit_message>
<xml_diff>
--- a/File_Manifest.xlsx
+++ b/File_Manifest.xlsx
@@ -435,7 +435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D37"/>
+  <dimension ref="A1:D40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="48" customWidth="1" min="1" max="1"/>
@@ -638,7 +638,7 @@
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>2026-07-29 22:02 PDT</t>
+          <t>2026-07-29 22:11 PDT</t>
         </is>
       </c>
     </row>
@@ -748,7 +748,7 @@
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>2026-07-29 22:07 PDT</t>
+          <t>2026-07-29 22:11 PDT</t>
         </is>
       </c>
     </row>
@@ -1255,6 +1255,72 @@
       <c r="D37" s="2" t="inlineStr">
         <is>
           <t>2026-07-29 22:07 PDT</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="2" t="inlineStr">
+        <is>
+          <t>generator/build_customer_addresses.py</t>
+        </is>
+      </c>
+      <c r="B38" s="2" t="inlineStr">
+        <is>
+          <t>Code</t>
+        </is>
+      </c>
+      <c r="C38" s="3" t="inlineStr">
+        <is>
+          <t>Phase 1: builds customer_addresses (billing/shipping, obviously-fake streets)</t>
+        </is>
+      </c>
+      <c r="D38" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-29 22:10 PDT</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="2" t="inlineStr">
+        <is>
+          <t>generator/validate_customer_addresses.py</t>
+        </is>
+      </c>
+      <c r="B39" s="2" t="inlineStr">
+        <is>
+          <t>Code</t>
+        </is>
+      </c>
+      <c r="C39" s="3" t="inlineStr">
+        <is>
+          <t>Phase 1: 5-layer validation for customer_addresses</t>
+        </is>
+      </c>
+      <c r="D39" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-29 22:11 PDT</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="2" t="inlineStr">
+        <is>
+          <t>data/customer_addresses.csv</t>
+        </is>
+      </c>
+      <c r="B40" s="2" t="inlineStr">
+        <is>
+          <t>Shipped table</t>
+        </is>
+      </c>
+      <c r="C40" s="3" t="inlineStr">
+        <is>
+          <t>Phase 1: customer_addresses table (1,431 rows)</t>
+        </is>
+      </c>
+      <c r="D40" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-29 22:10 PDT</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Phase 1: build + validate devices table (6 of 47); fix 2 real date-overflow bugs
- devices.csv: primary device per non-deleted customer (exact
  pre_signup_anonymous_id) + optional 2nd device, plus one device per
  anonymous ghost. Deleted customers get zero devices.
- Validation caught two real bugs, both fixed at the source rather than
  patched around:
  1. build_anonymous_population.py sampled first_seen_date with no
     start/end bounds, letting 47 of 17,050 ghosts land up to 3 days past
     END_DATE. Fixed by passing explicit bounds; regenerated
     _sim_anonymous_population.csv.
  2. devices.py's last-activity calc didn't clip the trial_in_progress
     edge case's trial.end (legitimately past END_DATE) before using it.
- 20-check validator; all pass after both fixes.
</commit_message>
<xml_diff>
--- a/File_Manifest.xlsx
+++ b/File_Manifest.xlsx
@@ -435,7 +435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D40"/>
+  <dimension ref="A1:D43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="48" customWidth="1" min="1" max="1"/>
@@ -506,7 +506,7 @@
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-29 22:07 PDT</t>
+          <t>2026-07-29 22:11 PDT</t>
         </is>
       </c>
     </row>
@@ -594,7 +594,7 @@
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>2026-07-29 22:02 PDT</t>
+          <t>2026-07-29 22:13 PDT</t>
         </is>
       </c>
     </row>
@@ -638,7 +638,7 @@
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>2026-07-29 22:11 PDT</t>
+          <t>2026-07-29 22:16 PDT</t>
         </is>
       </c>
     </row>
@@ -748,7 +748,7 @@
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>2026-07-29 22:11 PDT</t>
+          <t>2026-07-29 22:16 PDT</t>
         </is>
       </c>
     </row>
@@ -792,7 +792,7 @@
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>2026-07-29 20:11 PDT</t>
+          <t>2026-07-29 22:14 PDT</t>
         </is>
       </c>
     </row>
@@ -836,7 +836,7 @@
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>2026-07-29 21:35 PDT</t>
+          <t>2026-07-29 22:15 PDT</t>
         </is>
       </c>
     </row>
@@ -1321,6 +1321,72 @@
       <c r="D40" s="2" t="inlineStr">
         <is>
           <t>2026-07-29 22:10 PDT</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="2" t="inlineStr">
+        <is>
+          <t>generator/build_devices.py</t>
+        </is>
+      </c>
+      <c r="B41" s="2" t="inlineStr">
+        <is>
+          <t>Code</t>
+        </is>
+      </c>
+      <c r="C41" s="3" t="inlineStr">
+        <is>
+          <t>Phase 1: builds devices (customer + anonymous-ghost devices)</t>
+        </is>
+      </c>
+      <c r="D41" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-29 22:14 PDT</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="2" t="inlineStr">
+        <is>
+          <t>generator/validate_devices.py</t>
+        </is>
+      </c>
+      <c r="B42" s="2" t="inlineStr">
+        <is>
+          <t>Code</t>
+        </is>
+      </c>
+      <c r="C42" s="3" t="inlineStr">
+        <is>
+          <t>Phase 1: 5-layer validation for devices</t>
+        </is>
+      </c>
+      <c r="D42" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-29 22:13 PDT</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="2" t="inlineStr">
+        <is>
+          <t>data/devices.csv</t>
+        </is>
+      </c>
+      <c r="B43" s="2" t="inlineStr">
+        <is>
+          <t>Shipped table</t>
+        </is>
+      </c>
+      <c r="C43" s="3" t="inlineStr">
+        <is>
+          <t>Phase 1: devices table (18,042 rows: known-customer + ghost devices)</t>
+        </is>
+      </c>
+      <c r="D43" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-29 22:15 PDT</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Phase 1: build + validate identity_map table (7 of 47 shipped tables)
- 992 rows derived from devices.csv + customers.csv: one signup resolution
  per non-deleted customer (their exact pre_signup_anonymous_id, timestamped
  to account creation) plus one login resolution per 2nd device.
- 17-check validator: exact row-count parity with devices.csv (992=992, no
  orphans either direction), exact anonymous_id match vs the timeline, and
  resolved_at never preceding the device's own first_seen_at.
- One Phase 1 table remains: segments (definitions).
</commit_message>
<xml_diff>
--- a/File_Manifest.xlsx
+++ b/File_Manifest.xlsx
@@ -435,7 +435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D43"/>
+  <dimension ref="A1:D46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="48" customWidth="1" min="1" max="1"/>
@@ -506,7 +506,7 @@
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-29 22:11 PDT</t>
+          <t>2026-07-29 22:17 PDT</t>
         </is>
       </c>
     </row>
@@ -638,7 +638,7 @@
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>2026-07-29 22:16 PDT</t>
+          <t>2026-07-29 22:22 PDT</t>
         </is>
       </c>
     </row>
@@ -748,7 +748,7 @@
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>2026-07-29 22:16 PDT</t>
+          <t>2026-07-29 22:22 PDT</t>
         </is>
       </c>
     </row>
@@ -1387,6 +1387,72 @@
       <c r="D43" s="2" t="inlineStr">
         <is>
           <t>2026-07-29 22:15 PDT</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="2" t="inlineStr">
+        <is>
+          <t>generator/build_identity_map.py</t>
+        </is>
+      </c>
+      <c r="B44" s="2" t="inlineStr">
+        <is>
+          <t>Code</t>
+        </is>
+      </c>
+      <c r="C44" s="3" t="inlineStr">
+        <is>
+          <t>Phase 1: builds identity_map (anonymous_id -&gt; customer_id resolution events)</t>
+        </is>
+      </c>
+      <c r="D44" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-29 22:21 PDT</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="2" t="inlineStr">
+        <is>
+          <t>generator/validate_identity_map.py</t>
+        </is>
+      </c>
+      <c r="B45" s="2" t="inlineStr">
+        <is>
+          <t>Code</t>
+        </is>
+      </c>
+      <c r="C45" s="3" t="inlineStr">
+        <is>
+          <t>Phase 1: 5-layer validation for identity_map</t>
+        </is>
+      </c>
+      <c r="D45" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-29 22:22 PDT</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="2" t="inlineStr">
+        <is>
+          <t>data/identity_map.csv</t>
+        </is>
+      </c>
+      <c r="B46" s="2" t="inlineStr">
+        <is>
+          <t>Shipped table</t>
+        </is>
+      </c>
+      <c r="C46" s="3" t="inlineStr">
+        <is>
+          <t>Phase 1: identity_map table (992 rows) -- last Phase 1 table</t>
+        </is>
+      </c>
+      <c r="D46" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-29 22:21 PDT</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Phase 1 complete: build + validate segments table (8 of 8)
- 10 segment definitions: 7 customer-grain (subscription-lifecycle-based),
  3 anonymous_device-grain ad-platform audiences (Meta/Google/TikTok).
- The Lookalike audience's created_at is dated after a real seed audience
  of >=50 converters exists in the simulation, not day 1, since a
  lookalike algorithm needs real converters to model itself on.
- 14-check validator, all passing.
- Phase 1 (products, product_variants, subscription_plans, customers,
  customer_addresses, devices, identity_map, segments) is now fully built
  and validated -- 8 of 47 shipped tables done.
</commit_message>
<xml_diff>
--- a/File_Manifest.xlsx
+++ b/File_Manifest.xlsx
@@ -435,7 +435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D46"/>
+  <dimension ref="A1:D49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="48" customWidth="1" min="1" max="1"/>
@@ -506,7 +506,7 @@
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-29 22:17 PDT</t>
+          <t>2026-07-29 22:22 PDT</t>
         </is>
       </c>
     </row>
@@ -638,7 +638,7 @@
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>2026-07-29 22:22 PDT</t>
+          <t>2026-07-29 22:33 PDT</t>
         </is>
       </c>
     </row>
@@ -748,7 +748,7 @@
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>2026-07-29 22:22 PDT</t>
+          <t>2026-07-29 22:33 PDT</t>
         </is>
       </c>
     </row>
@@ -1447,12 +1447,78 @@
       </c>
       <c r="C46" s="3" t="inlineStr">
         <is>
-          <t>Phase 1: identity_map table (992 rows) -- last Phase 1 table</t>
+          <t>Phase 1: identity_map table (992 rows)</t>
         </is>
       </c>
       <c r="D46" s="2" t="inlineStr">
         <is>
           <t>2026-07-29 22:21 PDT</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="2" t="inlineStr">
+        <is>
+          <t>generator/build_segments.py</t>
+        </is>
+      </c>
+      <c r="B47" s="2" t="inlineStr">
+        <is>
+          <t>Code</t>
+        </is>
+      </c>
+      <c r="C47" s="3" t="inlineStr">
+        <is>
+          <t>Phase 1: builds segments (10 definitions: 7 customer-grain, 3 anonymous)</t>
+        </is>
+      </c>
+      <c r="D47" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-29 22:32 PDT</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="2" t="inlineStr">
+        <is>
+          <t>generator/validate_segments.py</t>
+        </is>
+      </c>
+      <c r="B48" s="2" t="inlineStr">
+        <is>
+          <t>Code</t>
+        </is>
+      </c>
+      <c r="C48" s="3" t="inlineStr">
+        <is>
+          <t>Phase 1: 5-layer validation for segments</t>
+        </is>
+      </c>
+      <c r="D48" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-29 22:33 PDT</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="2" t="inlineStr">
+        <is>
+          <t>data/segments.csv</t>
+        </is>
+      </c>
+      <c r="B49" s="2" t="inlineStr">
+        <is>
+          <t>Shipped table</t>
+        </is>
+      </c>
+      <c r="C49" s="3" t="inlineStr">
+        <is>
+          <t>Phase 1: segments table (10 rows) -- completes Phase 1 (all 8 tables)</t>
+        </is>
+      </c>
+      <c r="D49" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-29 22:33 PDT</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Fix segments: lapsed-but-still-buying customers didn't fit any segment
Ben caught that 'Lapsed 90+ Days (Quiet)' baked a purchase-activity
condition into a time-based bucket, so a real, explicitly-modeled
population (6 of 76 lapsed subscribers still buying courses/merch) didn't
cleanly belong to any segment. Fixed by making all 3 lapsed time buckets
purely time-based and adding a separate overlapping behavioral segment,
'Lapsed - Still Buying (Courses/Merch)', that can co-occur with any of
them. Added 2 validator checks: confirmed the new segment is non-vacuous
(6 real matches) and guards against reintroducing the same bug.
</commit_message>
<xml_diff>
--- a/File_Manifest.xlsx
+++ b/File_Manifest.xlsx
@@ -506,7 +506,7 @@
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-29 22:22 PDT</t>
+          <t>2026-07-29 22:36 PDT</t>
         </is>
       </c>
     </row>
@@ -748,7 +748,7 @@
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>2026-07-29 22:33 PDT</t>
+          <t>2026-07-29 22:36 PDT</t>
         </is>
       </c>
     </row>
@@ -1474,7 +1474,7 @@
       </c>
       <c r="D47" s="2" t="inlineStr">
         <is>
-          <t>2026-07-29 22:32 PDT</t>
+          <t>2026-07-29 22:36 PDT</t>
         </is>
       </c>
     </row>
@@ -1496,7 +1496,7 @@
       </c>
       <c r="D48" s="2" t="inlineStr">
         <is>
-          <t>2026-07-29 22:33 PDT</t>
+          <t>2026-07-29 22:36 PDT</t>
         </is>
       </c>
     </row>
@@ -1518,7 +1518,7 @@
       </c>
       <c r="D49" s="2" t="inlineStr">
         <is>
-          <t>2026-07-29 22:33 PDT</t>
+          <t>2026-07-29 22:36 PDT</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add 'High Churn Risk' segment: renewal approaching + low engagement
Ben asked for a segment covering active subscribers with an upcoming
renewal decision and low usage. Added as a 9th customer-grain segment,
honestly flagged as only partially computable today: the renewal-timing
half needs Phase 2's subscriptions.billing_interval (not yet built), and
the low-engagement half is proxied by engagement_tier='regular' since
active subscribers can currently only be tiered power/regular (never
casual) -- a real modeling gap surfaced while building this. Gave it its
own source_system ('churn_propensity_model') and grounded its created_at
in the simulation's actual churn history (21 churns by that date).
4 new validator checks; 20/20 pass.
</commit_message>
<xml_diff>
--- a/File_Manifest.xlsx
+++ b/File_Manifest.xlsx
@@ -506,7 +506,7 @@
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-29 22:36 PDT</t>
+          <t>2026-07-29 22:42 PDT</t>
         </is>
       </c>
     </row>
@@ -748,7 +748,7 @@
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>2026-07-29 22:36 PDT</t>
+          <t>2026-07-29 22:42 PDT</t>
         </is>
       </c>
     </row>
@@ -1474,7 +1474,7 @@
       </c>
       <c r="D47" s="2" t="inlineStr">
         <is>
-          <t>2026-07-29 22:36 PDT</t>
+          <t>2026-07-29 22:41 PDT</t>
         </is>
       </c>
     </row>
@@ -1496,7 +1496,7 @@
       </c>
       <c r="D48" s="2" t="inlineStr">
         <is>
-          <t>2026-07-29 22:36 PDT</t>
+          <t>2026-07-29 22:41 PDT</t>
         </is>
       </c>
     </row>
@@ -1518,7 +1518,7 @@
       </c>
       <c r="D49" s="2" t="inlineStr">
         <is>
-          <t>2026-07-29 22:36 PDT</t>
+          <t>2026-07-29 22:41 PDT</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Record cross-phase consistency commitments for Phase 2/5 dependencies
Added a 'Cross-phase consistency commitments' section to
docs/generation_plan.md consolidating two flagged gaps that can't be
resolved until later phases exist: (1) billing_interval/next-renewal-date
needed by 'High Churn Risk', to be built in Phase 2's subscriptions table,
and (2) per Ben's decision, low engagement must be shown directly in real
Phase 5 app/web usage volume, with segment membership (Phase 4) required
to match rather than being computed independently.
</commit_message>
<xml_diff>
--- a/File_Manifest.xlsx
+++ b/File_Manifest.xlsx
@@ -572,7 +572,7 @@
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>2026-07-29 21:38 PDT</t>
+          <t>2026-07-29 22:45 PDT</t>
         </is>
       </c>
     </row>
@@ -748,7 +748,7 @@
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>2026-07-29 22:42 PDT</t>
+          <t>2026-07-29 22:45 PDT</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Replicate anonymous-grain segments across all 6 ad platforms
Website Visitors, Cart Abandoners, and Lookalike now each get one row per
platform (meta, google_search, youtube, dv360, snap, tiktok) instead of
one row total -- 27 total segments (9 customer + 18 anonymous), up from
12. Fixed a Snap UUID generator bug that collapsed small-i ids to
near-duplicate values. Updated validator distributional + completeness
checks accordingly; 23/23 pass.
</commit_message>
<xml_diff>
--- a/File_Manifest.xlsx
+++ b/File_Manifest.xlsx
@@ -506,7 +506,7 @@
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-29 22:42 PDT</t>
+          <t>2026-07-29 22:54 PDT</t>
         </is>
       </c>
     </row>
@@ -638,7 +638,7 @@
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>2026-07-29 22:33 PDT</t>
+          <t>2026-07-29 22:54 PDT</t>
         </is>
       </c>
     </row>
@@ -748,7 +748,7 @@
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>2026-07-29 22:45 PDT</t>
+          <t>2026-07-29 22:54 PDT</t>
         </is>
       </c>
     </row>
@@ -1469,12 +1469,12 @@
       </c>
       <c r="C47" s="3" t="inlineStr">
         <is>
-          <t>Phase 1: builds segments (10 definitions: 7 customer-grain, 3 anonymous)</t>
+          <t>Phase 1: builds segments (27 definitions: 9 customer-grain, 18 anonymous -- 3 audience concepts x 6 ad platforms)</t>
         </is>
       </c>
       <c r="D47" s="2" t="inlineStr">
         <is>
-          <t>2026-07-29 22:41 PDT</t>
+          <t>2026-07-29 22:53 PDT</t>
         </is>
       </c>
     </row>
@@ -1496,7 +1496,7 @@
       </c>
       <c r="D48" s="2" t="inlineStr">
         <is>
-          <t>2026-07-29 22:41 PDT</t>
+          <t>2026-07-29 22:53 PDT</t>
         </is>
       </c>
     </row>
@@ -1513,12 +1513,12 @@
       </c>
       <c r="C49" s="3" t="inlineStr">
         <is>
-          <t>Phase 1: segments table (10 rows) -- completes Phase 1 (all 8 tables)</t>
+          <t>Phase 1: segments table (27 rows) -- completes Phase 1 (all 8 tables)</t>
         </is>
       </c>
       <c r="D49" s="2" t="inlineStr">
         <is>
-          <t>2026-07-29 22:41 PDT</t>
+          <t>2026-07-29 22:54 PDT</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Phase 2: build + validate subscriptions table (1 of 3)
Stripe-shaped subscription objects derived from the master timeline's
trial/interval structure. Resolves the long-flagged billing_interval gap
by assigning billing_interval + computing a real future-dated
current_period_end for every open subscription -- exactly what the
High Churn Risk segment needed. 27/27 validator checks pass; 576
subscription objects reconcile exactly against the timeline, and 98
currently-open subscriptions match the established ground truth.
</commit_message>
<xml_diff>
--- a/File_Manifest.xlsx
+++ b/File_Manifest.xlsx
@@ -435,7 +435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D49"/>
+  <dimension ref="A1:D52"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="48" customWidth="1" min="1" max="1"/>
@@ -506,7 +506,7 @@
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-29 22:54 PDT</t>
+          <t>2026-07-29 23:03 PDT</t>
         </is>
       </c>
     </row>
@@ -572,7 +572,7 @@
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>2026-07-29 22:45 PDT</t>
+          <t>2026-07-29 23:03 PDT</t>
         </is>
       </c>
     </row>
@@ -594,7 +594,7 @@
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>2026-07-29 22:13 PDT</t>
+          <t>2026-07-29 22:59 PDT</t>
         </is>
       </c>
     </row>
@@ -638,7 +638,7 @@
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>2026-07-29 22:54 PDT</t>
+          <t>2026-07-29 23:03 PDT</t>
         </is>
       </c>
     </row>
@@ -748,7 +748,7 @@
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>2026-07-29 22:54 PDT</t>
+          <t>2026-07-29 23:04 PDT</t>
         </is>
       </c>
     </row>
@@ -1474,7 +1474,7 @@
       </c>
       <c r="D47" s="2" t="inlineStr">
         <is>
-          <t>2026-07-29 22:53 PDT</t>
+          <t>2026-07-29 23:03 PDT</t>
         </is>
       </c>
     </row>
@@ -1496,7 +1496,7 @@
       </c>
       <c r="D48" s="2" t="inlineStr">
         <is>
-          <t>2026-07-29 22:53 PDT</t>
+          <t>2026-07-29 23:03 PDT</t>
         </is>
       </c>
     </row>
@@ -1518,7 +1518,73 @@
       </c>
       <c r="D49" s="2" t="inlineStr">
         <is>
-          <t>2026-07-29 22:54 PDT</t>
+          <t>2026-07-29 23:03 PDT</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="2" t="inlineStr">
+        <is>
+          <t>generator/build_subscriptions.py</t>
+        </is>
+      </c>
+      <c r="B50" s="2" t="inlineStr">
+        <is>
+          <t>Code</t>
+        </is>
+      </c>
+      <c r="C50" s="3" t="inlineStr">
+        <is>
+          <t>Phase 2: builds subscriptions (Stripe-shaped subscription objects; assigns billing_interval + next-renewal date, resolving the long-flagged Phase 2 gap)</t>
+        </is>
+      </c>
+      <c r="D50" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-29 23:02 PDT</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="2" t="inlineStr">
+        <is>
+          <t>generator/validate_subscriptions.py</t>
+        </is>
+      </c>
+      <c r="B51" s="2" t="inlineStr">
+        <is>
+          <t>Code</t>
+        </is>
+      </c>
+      <c r="C51" s="3" t="inlineStr">
+        <is>
+          <t>Phase 2: 5-layer validation for subscriptions</t>
+        </is>
+      </c>
+      <c r="D51" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-29 23:02 PDT</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="2" t="inlineStr">
+        <is>
+          <t>data/subscriptions.csv</t>
+        </is>
+      </c>
+      <c r="B52" s="2" t="inlineStr">
+        <is>
+          <t>Shipped table</t>
+        </is>
+      </c>
+      <c r="C52" s="3" t="inlineStr">
+        <is>
+          <t>Phase 2: subscriptions table (576 rows: one Stripe-shaped subscription object per trial-or-interval)</t>
+        </is>
+      </c>
+      <c r="D52" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-29 23:02 PDT</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Phase 2: build + validate subscription_events table (2 of 3)
Event log derived from build_subscription_objects() (single source of
truth shared with subscriptions.py) plus the raw timeline's payment
failure/upgrade/downgrade/resumed events. Adds the 'renewed' event type
(computed from billing-cycle math) and the duplicate-webhook-style
messiness promised in schema_reference.md. Also amends subscriptions.csv
with a past_due_since column so both tables agree on why a subscription
is past_due. 22/22 and 28/28 validator checks pass respectively.
</commit_message>
<xml_diff>
--- a/File_Manifest.xlsx
+++ b/File_Manifest.xlsx
@@ -435,7 +435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D52"/>
+  <dimension ref="A1:D55"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="48" customWidth="1" min="1" max="1"/>
@@ -506,7 +506,7 @@
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-29 23:03 PDT</t>
+          <t>2026-07-30 10:34 PDT</t>
         </is>
       </c>
     </row>
@@ -594,7 +594,7 @@
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>2026-07-29 22:59 PDT</t>
+          <t>2026-07-30 10:31 PDT</t>
         </is>
       </c>
     </row>
@@ -638,7 +638,7 @@
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>2026-07-29 23:03 PDT</t>
+          <t>2026-07-30 10:33 PDT</t>
         </is>
       </c>
     </row>
@@ -748,7 +748,7 @@
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>2026-07-29 23:04 PDT</t>
+          <t>2026-07-30 10:34 PDT</t>
         </is>
       </c>
     </row>
@@ -1540,7 +1540,7 @@
       </c>
       <c r="D50" s="2" t="inlineStr">
         <is>
-          <t>2026-07-29 23:02 PDT</t>
+          <t>2026-07-30 10:29 PDT</t>
         </is>
       </c>
     </row>
@@ -1562,7 +1562,7 @@
       </c>
       <c r="D51" s="2" t="inlineStr">
         <is>
-          <t>2026-07-29 23:02 PDT</t>
+          <t>2026-07-30 10:30 PDT</t>
         </is>
       </c>
     </row>
@@ -1584,7 +1584,73 @@
       </c>
       <c r="D52" s="2" t="inlineStr">
         <is>
-          <t>2026-07-29 23:02 PDT</t>
+          <t>2026-07-30 10:30 PDT</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="2" t="inlineStr">
+        <is>
+          <t>generator/build_subscription_events.py</t>
+        </is>
+      </c>
+      <c r="B53" s="2" t="inlineStr">
+        <is>
+          <t>Code</t>
+        </is>
+      </c>
+      <c r="C53" s="3" t="inlineStr">
+        <is>
+          <t>Phase 2: builds subscription_events (event log behind every subscription: trial_started/converted/expired, renewed, upgraded/downgraded, payment_failed, canceled, resumed)</t>
+        </is>
+      </c>
+      <c r="D53" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-30 10:32 PDT</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="2" t="inlineStr">
+        <is>
+          <t>generator/validate_subscription_events.py</t>
+        </is>
+      </c>
+      <c r="B54" s="2" t="inlineStr">
+        <is>
+          <t>Code</t>
+        </is>
+      </c>
+      <c r="C54" s="3" t="inlineStr">
+        <is>
+          <t>Phase 2: 5-layer validation for subscription_events</t>
+        </is>
+      </c>
+      <c r="D54" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-30 10:33 PDT</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="2" t="inlineStr">
+        <is>
+          <t>data/subscription_events.csv</t>
+        </is>
+      </c>
+      <c r="B55" s="2" t="inlineStr">
+        <is>
+          <t>Shipped table</t>
+        </is>
+      </c>
+      <c r="C55" s="3" t="inlineStr">
+        <is>
+          <t>Phase 2: subscription_events table (2,424 rows, incl. ~3% deliberate duplicate webhook-style rows)</t>
+        </is>
+      </c>
+      <c r="D55" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-30 10:32 PDT</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Phase 2 complete: build + validate invoices table (3 of 3)
One invoice per initial charge + successful renewal, plus uncollectible/
open invoices for genuine payment-failure preconditions. Caught and fixed
two real bugs in the process: a relativedelta month-end chaining drift
that broke invoice period contiguity, and a cross-table logical
contradiction in subscription_events.csv where past_due subscriptions
got both a 'renewed' and a 'payment_failed' event for the same billing
attempt. 24/24 invoice checks pass; subscription_events re-validated at
22/22 after the fix. Phase 2 (subscriptions, subscription_events,
invoices) is now complete.
</commit_message>
<xml_diff>
--- a/File_Manifest.xlsx
+++ b/File_Manifest.xlsx
@@ -435,7 +435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D55"/>
+  <dimension ref="A1:D58"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="48" customWidth="1" min="1" max="1"/>
@@ -506,7 +506,7 @@
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-30 10:34 PDT</t>
+          <t>2026-07-30 11:29 PDT</t>
         </is>
       </c>
     </row>
@@ -638,7 +638,7 @@
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>2026-07-30 10:33 PDT</t>
+          <t>2026-07-30 11:28 PDT</t>
         </is>
       </c>
     </row>
@@ -748,7 +748,7 @@
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>2026-07-30 10:34 PDT</t>
+          <t>2026-07-30 11:29 PDT</t>
         </is>
       </c>
     </row>
@@ -1606,7 +1606,7 @@
       </c>
       <c r="D53" s="2" t="inlineStr">
         <is>
-          <t>2026-07-30 10:32 PDT</t>
+          <t>2026-07-30 11:28 PDT</t>
         </is>
       </c>
     </row>
@@ -1628,7 +1628,7 @@
       </c>
       <c r="D54" s="2" t="inlineStr">
         <is>
-          <t>2026-07-30 10:33 PDT</t>
+          <t>2026-07-30 11:27 PDT</t>
         </is>
       </c>
     </row>
@@ -1645,12 +1645,78 @@
       </c>
       <c r="C55" s="3" t="inlineStr">
         <is>
-          <t>Phase 2: subscription_events table (2,424 rows, incl. ~3% deliberate duplicate webhook-style rows)</t>
+          <t>Phase 2: subscription_events table (2,423 rows, incl. ~3% deliberate duplicate webhook-style rows)</t>
         </is>
       </c>
       <c r="D55" s="2" t="inlineStr">
         <is>
-          <t>2026-07-30 10:32 PDT</t>
+          <t>2026-07-30 11:28 PDT</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="2" t="inlineStr">
+        <is>
+          <t>generator/build_invoices.py</t>
+        </is>
+      </c>
+      <c r="B56" s="2" t="inlineStr">
+        <is>
+          <t>Code</t>
+        </is>
+      </c>
+      <c r="C56" s="3" t="inlineStr">
+        <is>
+          <t>Phase 2: builds invoices (one per initial charge + renewal, plus uncollectible/open for failed payments) -- completes Phase 2 (all 3 tables)</t>
+        </is>
+      </c>
+      <c r="D56" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-30 11:28 PDT</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="2" t="inlineStr">
+        <is>
+          <t>generator/validate_invoices.py</t>
+        </is>
+      </c>
+      <c r="B57" s="2" t="inlineStr">
+        <is>
+          <t>Code</t>
+        </is>
+      </c>
+      <c r="C57" s="3" t="inlineStr">
+        <is>
+          <t>Phase 2: 5-layer validation for invoices</t>
+        </is>
+      </c>
+      <c r="D57" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-30 11:28 PDT</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="2" t="inlineStr">
+        <is>
+          <t>data/invoices.csv</t>
+        </is>
+      </c>
+      <c r="B58" s="2" t="inlineStr">
+        <is>
+          <t>Shipped table</t>
+        </is>
+      </c>
+      <c r="C58" s="3" t="inlineStr">
+        <is>
+          <t>Phase 2: invoices table (1,229 rows) -- completes Phase 2</t>
+        </is>
+      </c>
+      <c r="D58" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-30 11:28 PDT</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Phase 3 begins: build + validate discount_codes table (1 of 5)
Built first within Phase 3 (ahead of schema_reference.md's listing
order) since orders.discount_code_id will need real definitions to
redeem against, and discount_codes has no dependencies of its own. 7
hand-curated codes mixing evergreen and seasonal (January-themed,
consistent with the project's established seasonality). is_active is
derived from valid_until vs END_DATE rather than hand-picked. 19/19
validator checks pass.
</commit_message>
<xml_diff>
--- a/File_Manifest.xlsx
+++ b/File_Manifest.xlsx
@@ -435,7 +435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D58"/>
+  <dimension ref="A1:D61"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="48" customWidth="1" min="1" max="1"/>
@@ -506,7 +506,7 @@
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-30 11:29 PDT</t>
+          <t>2026-07-30 13:06 PDT</t>
         </is>
       </c>
     </row>
@@ -638,7 +638,7 @@
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>2026-07-30 11:28 PDT</t>
+          <t>2026-07-30 13:06 PDT</t>
         </is>
       </c>
     </row>
@@ -748,7 +748,7 @@
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>2026-07-30 11:29 PDT</t>
+          <t>2026-07-30 13:06 PDT</t>
         </is>
       </c>
     </row>
@@ -1717,6 +1717,72 @@
       <c r="D58" s="2" t="inlineStr">
         <is>
           <t>2026-07-30 11:28 PDT</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="2" t="inlineStr">
+        <is>
+          <t>generator/build_discount_codes.py</t>
+        </is>
+      </c>
+      <c r="B59" s="2" t="inlineStr">
+        <is>
+          <t>Code</t>
+        </is>
+      </c>
+      <c r="C59" s="3" t="inlineStr">
+        <is>
+          <t>Phase 3: builds discount_codes (hand-curated list: evergreen + seasonal promo codes) -- built first in Phase 3 since orders needs it</t>
+        </is>
+      </c>
+      <c r="D59" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-30 13:05 PDT</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="2" t="inlineStr">
+        <is>
+          <t>generator/validate_discount_codes.py</t>
+        </is>
+      </c>
+      <c r="B60" s="2" t="inlineStr">
+        <is>
+          <t>Code</t>
+        </is>
+      </c>
+      <c r="C60" s="3" t="inlineStr">
+        <is>
+          <t>Phase 3: 5-layer validation for discount_codes</t>
+        </is>
+      </c>
+      <c r="D60" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-30 13:06 PDT</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="2" t="inlineStr">
+        <is>
+          <t>data/discount_codes.csv</t>
+        </is>
+      </c>
+      <c r="B61" s="2" t="inlineStr">
+        <is>
+          <t>Shipped table</t>
+        </is>
+      </c>
+      <c r="C61" s="3" t="inlineStr">
+        <is>
+          <t>Phase 3: discount_codes table (7 rows)</t>
+        </is>
+      </c>
+      <c r="D61" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-30 13:05 PDT</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Phase 3: build + validate order_line_items (3 of 5)
- One row per order: resolves each order's price tier down to a specific
  product_id + variant_id (orders.csv only carries the amount, not which
  product). quantity always 1, unit_price == line_total == subtotal by
  construction (no multi-item carts in this simulated storefront).
- Ambiguity resolved: the $24.99 merch tier maps to two products (Cap vs
  Water Bottle), split randomly; apparel variants picked with a size skew
  (M/L most common).
- validate_order_line_items.py: 14/14 checks passed on first run, incl.
  per-order sum(line_total) reconciling exactly against orders.csv subtotal.
- 3,650 rows total, matching orders.csv 1:1.
</commit_message>
<xml_diff>
--- a/File_Manifest.xlsx
+++ b/File_Manifest.xlsx
@@ -435,7 +435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D64"/>
+  <dimension ref="A1:D67"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="48" customWidth="1" min="1" max="1"/>
@@ -638,7 +638,7 @@
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>2026-07-30 13:22 PDT</t>
+          <t>2026-07-30 13:42 PDT</t>
         </is>
       </c>
     </row>
@@ -748,7 +748,7 @@
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>2026-07-30 13:23 PDT</t>
+          <t>2026-07-30 13:42 PDT</t>
         </is>
       </c>
     </row>
@@ -1849,6 +1849,72 @@
       <c r="D64" s="2" t="inlineStr">
         <is>
           <t>2026-07-30 13:21 PDT</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="2" t="inlineStr">
+        <is>
+          <t>generator/build_order_line_items.py</t>
+        </is>
+      </c>
+      <c r="B65" s="2" t="inlineStr">
+        <is>
+          <t>Code</t>
+        </is>
+      </c>
+      <c r="C65" s="3" t="inlineStr">
+        <is>
+          <t>Phase 3: builds order_line_items (one row per order -- resolves each order's price tier down to a specific product + variant)</t>
+        </is>
+      </c>
+      <c r="D65" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-30 13:39 PDT</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="2" t="inlineStr">
+        <is>
+          <t>generator/validate_order_line_items.py</t>
+        </is>
+      </c>
+      <c r="B66" s="2" t="inlineStr">
+        <is>
+          <t>Code</t>
+        </is>
+      </c>
+      <c r="C66" s="3" t="inlineStr">
+        <is>
+          <t>Phase 3: 5-layer validation for order_line_items</t>
+        </is>
+      </c>
+      <c r="D66" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-30 13:40 PDT</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="2" t="inlineStr">
+        <is>
+          <t>data/order_line_items.csv</t>
+        </is>
+      </c>
+      <c r="B67" s="2" t="inlineStr">
+        <is>
+          <t>Shipped table</t>
+        </is>
+      </c>
+      <c r="C67" s="3" t="inlineStr">
+        <is>
+          <t>Phase 3: order_line_items table (3,650 rows, one per order)</t>
+        </is>
+      </c>
+      <c r="D67" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-30 13:39 PDT</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Phase 3: build + validate payments (4 of 5)
- One row per Stripe-shaped Charge attempt (not per order): every order
  succeeded eventually, but 7.7% of orders had 1-2 declined-then-retried
  attempts first, modeling realistic checkout messiness. Every order gets
  exactly one succeeded payment by construction.
- validate_payments.py: 16/16 checks passed on first run, incl. exactly-one-
  succeeded-payment-per-order and amount/currency/customer_id reconciliation
  against orders.csv.
- 3,964 rows total (3,650 succeeded + 314 failed attempts).
</commit_message>
<xml_diff>
--- a/File_Manifest.xlsx
+++ b/File_Manifest.xlsx
@@ -435,7 +435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D67"/>
+  <dimension ref="A1:D70"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="48" customWidth="1" min="1" max="1"/>
@@ -506,7 +506,7 @@
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-30 13:22 PDT</t>
+          <t>2026-07-30 13:42 PDT</t>
         </is>
       </c>
     </row>
@@ -594,7 +594,7 @@
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>2026-07-30 13:15 PDT</t>
+          <t>2026-07-30 13:45 PDT</t>
         </is>
       </c>
     </row>
@@ -638,7 +638,7 @@
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>2026-07-30 13:42 PDT</t>
+          <t>2026-07-30 13:46 PDT</t>
         </is>
       </c>
     </row>
@@ -748,7 +748,7 @@
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>2026-07-30 13:42 PDT</t>
+          <t>2026-07-30 13:46 PDT</t>
         </is>
       </c>
     </row>
@@ -1915,6 +1915,72 @@
       <c r="D67" s="2" t="inlineStr">
         <is>
           <t>2026-07-30 13:39 PDT</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="2" t="inlineStr">
+        <is>
+          <t>generator/build_payments.py</t>
+        </is>
+      </c>
+      <c r="B68" s="2" t="inlineStr">
+        <is>
+          <t>Code</t>
+        </is>
+      </c>
+      <c r="C68" s="3" t="inlineStr">
+        <is>
+          <t>Phase 3: builds payments (one Stripe-shaped Charge attempt per row; models realistic declined-then-retried charge attempts)</t>
+        </is>
+      </c>
+      <c r="D68" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-30 13:45 PDT</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="2" t="inlineStr">
+        <is>
+          <t>generator/validate_payments.py</t>
+        </is>
+      </c>
+      <c r="B69" s="2" t="inlineStr">
+        <is>
+          <t>Code</t>
+        </is>
+      </c>
+      <c r="C69" s="3" t="inlineStr">
+        <is>
+          <t>Phase 3: 5-layer validation for payments</t>
+        </is>
+      </c>
+      <c r="D69" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-30 13:46 PDT</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="2" t="inlineStr">
+        <is>
+          <t>data/payments.csv</t>
+        </is>
+      </c>
+      <c r="B70" s="2" t="inlineStr">
+        <is>
+          <t>Shipped table</t>
+        </is>
+      </c>
+      <c r="C70" s="3" t="inlineStr">
+        <is>
+          <t>Phase 3: payments table (3,964 rows: 3,650 succeeded + 314 failed retry attempts)</t>
+        </is>
+      </c>
+      <c r="D70" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-30 13:45 PDT</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Phase 3: build + validate refunds (5 of 5) -- Phase 3 complete
- Refunds reuse payments.csv's succeeded payment per order directly. 4.4%
  of orders refunded (75% full / 25% partial), amount always <= order
  total_amount, refunded_at always after order_date and never past END_DATE.
- Caught and fixed a validator bug (not a data bug): END_DATE boundary check
  compared full timestamps instead of calendar dates, flagging correct
  noon-on-END_DATE refunds as out of window. Fixed to date-granularity
  comparison, matching convention used elsewhere (devices.py).
- validate_refunds.py: 17/17 checks passed after the fix.
- 159 rows total. Completes Phase 3 (discount_codes, orders,
  order_line_items, payments, refunds).
</commit_message>
<xml_diff>
--- a/File_Manifest.xlsx
+++ b/File_Manifest.xlsx
@@ -435,7 +435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D70"/>
+  <dimension ref="A1:D73"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="48" customWidth="1" min="1" max="1"/>
@@ -506,7 +506,7 @@
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-30 13:42 PDT</t>
+          <t>2026-07-30 13:46 PDT</t>
         </is>
       </c>
     </row>
@@ -638,7 +638,7 @@
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>2026-07-30 13:46 PDT</t>
+          <t>2026-07-30 17:51 PDT</t>
         </is>
       </c>
     </row>
@@ -748,7 +748,7 @@
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>2026-07-30 13:46 PDT</t>
+          <t>2026-07-30 17:51 PDT</t>
         </is>
       </c>
     </row>
@@ -1981,6 +1981,72 @@
       <c r="D70" s="2" t="inlineStr">
         <is>
           <t>2026-07-30 13:45 PDT</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="2" t="inlineStr">
+        <is>
+          <t>generator/build_refunds.py</t>
+        </is>
+      </c>
+      <c r="B71" s="2" t="inlineStr">
+        <is>
+          <t>Code</t>
+        </is>
+      </c>
+      <c r="C71" s="3" t="inlineStr">
+        <is>
+          <t>Phase 3: builds refunds (against a small share of orders' succeeded payments) -- completes Phase 3 (all 5 tables)</t>
+        </is>
+      </c>
+      <c r="D71" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-30 17:50 PDT</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="2" t="inlineStr">
+        <is>
+          <t>generator/validate_refunds.py</t>
+        </is>
+      </c>
+      <c r="B72" s="2" t="inlineStr">
+        <is>
+          <t>Code</t>
+        </is>
+      </c>
+      <c r="C72" s="3" t="inlineStr">
+        <is>
+          <t>Phase 3: 5-layer validation for refunds</t>
+        </is>
+      </c>
+      <c r="D72" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-30 17:51 PDT</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="2" t="inlineStr">
+        <is>
+          <t>data/refunds.csv</t>
+        </is>
+      </c>
+      <c r="B73" s="2" t="inlineStr">
+        <is>
+          <t>Shipped table</t>
+        </is>
+      </c>
+      <c r="C73" s="3" t="inlineStr">
+        <is>
+          <t>Phase 3: refunds table (159 rows, 4.4% of orders) -- completes Phase 3</t>
+        </is>
+      </c>
+      <c r="D73" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-30 17:50 PDT</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Phase 5: build + validate web_sessions (1 of 4)
- Marketing-site browsing sessions for known customers (pre-signup +
  signup + reactivation + order-day + engagement_tier-driven filler
  sessions) and anonymous ghosts (reusing _sim_anonymous_population.csv's
  own num_sessions/channel as single source of truth).
- Fixed two real bugs: single-session guest purchasers landing on
  first_seen instead of guest_purchase_date, and a fractional-second
  timestamp formatting bug (plus a latent replace=False crash risk it
  shared a root cause with).
- validate_web_sessions.py: 13/13 checks passed after fixes.
- 30,285 rows total (6,476 identity-resolved + 23,809 anonymous).
</commit_message>
<xml_diff>
--- a/File_Manifest.xlsx
+++ b/File_Manifest.xlsx
@@ -435,7 +435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D76"/>
+  <dimension ref="A1:D79"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="48" customWidth="1" min="1" max="1"/>
@@ -506,7 +506,7 @@
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-30 17:51 PDT</t>
+          <t>2026-08-13 07:02 PDT</t>
         </is>
       </c>
     </row>
@@ -638,7 +638,7 @@
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>2026-08-13 07:02 PDT</t>
+          <t>2026-08-13 07:11 PDT</t>
         </is>
       </c>
     </row>
@@ -748,7 +748,7 @@
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>2026-08-13 07:02 PDT</t>
+          <t>2026-08-13 07:11 PDT</t>
         </is>
       </c>
     </row>
@@ -2113,6 +2113,72 @@
       <c r="D76" s="2" t="inlineStr">
         <is>
           <t>2026-08-13 07:00 PDT</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="2" t="inlineStr">
+        <is>
+          <t>generator/build_web_sessions.py</t>
+        </is>
+      </c>
+      <c r="B77" s="2" t="inlineStr">
+        <is>
+          <t>Code</t>
+        </is>
+      </c>
+      <c r="C77" s="3" t="inlineStr">
+        <is>
+          <t>Phase 5: builds web_sessions (marketing-site browsing; known customers + anonymous ghosts, engagement_tier-driven volume)</t>
+        </is>
+      </c>
+      <c r="D77" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-13 07:11 PDT</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="2" t="inlineStr">
+        <is>
+          <t>generator/validate_web_sessions.py</t>
+        </is>
+      </c>
+      <c r="B78" s="2" t="inlineStr">
+        <is>
+          <t>Code</t>
+        </is>
+      </c>
+      <c r="C78" s="3" t="inlineStr">
+        <is>
+          <t>Phase 5: 5-layer validation for web_sessions</t>
+        </is>
+      </c>
+      <c r="D78" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-13 07:11 PDT</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="2" t="inlineStr">
+        <is>
+          <t>data/web_sessions.csv</t>
+        </is>
+      </c>
+      <c r="B79" s="2" t="inlineStr">
+        <is>
+          <t>Shipped table</t>
+        </is>
+      </c>
+      <c r="C79" s="3" t="inlineStr">
+        <is>
+          <t>Phase 5: web_sessions table (30,285 rows: 6,476 identity-resolved + 23,809 anonymous)</t>
+        </is>
+      </c>
+      <c r="D79" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-13 07:11 PDT</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Phase 5: build + validate web_events (2 of 4)
- Page-level events (page_view/product_view/add_to_cart/begin_checkout/
  purchase/search) per web_sessions.csv row. Every eligible order gets
  exactly one purchase event, linked back through a deterministic queue-
  based pairing that solves two real FK gaps (same-day multi-order
  disambiguation for known customers; guest order<->ghost linkage despite
  276 date+amount collisions across 1,257 guest purchasers).
- Fixed a real reproducibility bug: the timestamp-spacing helper used an
  unseeded np.random.default_rng() instead of the shared seeded rng.
- Fixed a validator calibration issue (not a data bug): cart-abandonment
  distributional band didn't match the build's own configured rate.
- validate_web_events.py: 15/15 checks passed after fixes.
- 117,706 rows total (3,633 purchase events, matching orders.csv minus the
  17 orders belonging to soft-deleted customers).
</commit_message>
<xml_diff>
--- a/File_Manifest.xlsx
+++ b/File_Manifest.xlsx
@@ -435,7 +435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D79"/>
+  <dimension ref="A1:D82"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="48" customWidth="1" min="1" max="1"/>
@@ -506,7 +506,7 @@
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>2026-08-13 07:02 PDT</t>
+          <t>2026-08-13 07:11 PDT</t>
         </is>
       </c>
     </row>
@@ -638,7 +638,7 @@
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>2026-08-13 07:11 PDT</t>
+          <t>2026-08-13 07:21 PDT</t>
         </is>
       </c>
     </row>
@@ -748,7 +748,7 @@
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>2026-08-13 07:11 PDT</t>
+          <t>2026-08-13 07:21 PDT</t>
         </is>
       </c>
     </row>
@@ -2179,6 +2179,72 @@
       <c r="D79" s="2" t="inlineStr">
         <is>
           <t>2026-08-13 07:11 PDT</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="2" t="inlineStr">
+        <is>
+          <t>generator/build_web_events.py</t>
+        </is>
+      </c>
+      <c r="B80" s="2" t="inlineStr">
+        <is>
+          <t>Code</t>
+        </is>
+      </c>
+      <c r="C80" s="3" t="inlineStr">
+        <is>
+          <t>Phase 5: builds web_events (page_view/product_view/add_to_cart/begin_checkout/purchase/search; every order gets exactly one purchase event)</t>
+        </is>
+      </c>
+      <c r="D80" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-13 07:19 PDT</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="2" t="inlineStr">
+        <is>
+          <t>generator/validate_web_events.py</t>
+        </is>
+      </c>
+      <c r="B81" s="2" t="inlineStr">
+        <is>
+          <t>Code</t>
+        </is>
+      </c>
+      <c r="C81" s="3" t="inlineStr">
+        <is>
+          <t>Phase 5: 5-layer validation for web_events</t>
+        </is>
+      </c>
+      <c r="D81" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-13 07:21 PDT</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="2" t="inlineStr">
+        <is>
+          <t>data/web_events.csv</t>
+        </is>
+      </c>
+      <c r="B82" s="2" t="inlineStr">
+        <is>
+          <t>Shipped table</t>
+        </is>
+      </c>
+      <c r="C82" s="3" t="inlineStr">
+        <is>
+          <t>Phase 5: web_events table (117,706 rows)</t>
+        </is>
+      </c>
+      <c r="D82" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-13 07:19 PDT</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Phase 5: build + validate app_sessions (3 of 4)
- In-app fitness usage, driven by two real sources: subscription intervals
  (ongoing usage at an engagement_tier-keyed weekly rate, stopping at
  lapse) and course orders (a 45-day post-purchase access burst). Merch-
  only customers get zero rows. Every session pins to the customer's
  primary device; platform mirrors that device's device_type exactly.
- Fixed a validator calibration issue (not a data bug): required an exact
  customer-coverage match, but 5 casual-tier ~1-month subscribers
  legitimately drew zero sessions from the Poisson process before
  churning. Loosened to a tolerance band.
- validate_app_sessions.py: 12/12 checks passed after the fix.
- 19,610 rows across 496 of 501 eligible customers.
</commit_message>
<xml_diff>
--- a/File_Manifest.xlsx
+++ b/File_Manifest.xlsx
@@ -435,7 +435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D82"/>
+  <dimension ref="A1:D85"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="48" customWidth="1" min="1" max="1"/>
@@ -506,7 +506,7 @@
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>2026-08-13 07:11 PDT</t>
+          <t>2026-08-13 07:21 PDT</t>
         </is>
       </c>
     </row>
@@ -638,7 +638,7 @@
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>2026-08-13 07:21 PDT</t>
+          <t>2026-08-13 07:34 PDT</t>
         </is>
       </c>
     </row>
@@ -748,7 +748,7 @@
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>2026-08-13 07:21 PDT</t>
+          <t>2026-08-13 07:34 PDT</t>
         </is>
       </c>
     </row>
@@ -2245,6 +2245,72 @@
       <c r="D82" s="2" t="inlineStr">
         <is>
           <t>2026-08-13 07:19 PDT</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="2" t="inlineStr">
+        <is>
+          <t>generator/build_app_sessions.py</t>
+        </is>
+      </c>
+      <c r="B83" s="2" t="inlineStr">
+        <is>
+          <t>Code</t>
+        </is>
+      </c>
+      <c r="C83" s="3" t="inlineStr">
+        <is>
+          <t>Phase 5: builds app_sessions (in-app fitness usage, driven by real subscription intervals + course orders, keyed off engagement_tier)</t>
+        </is>
+      </c>
+      <c r="D83" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-13 07:33 PDT</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="2" t="inlineStr">
+        <is>
+          <t>generator/validate_app_sessions.py</t>
+        </is>
+      </c>
+      <c r="B84" s="2" t="inlineStr">
+        <is>
+          <t>Code</t>
+        </is>
+      </c>
+      <c r="C84" s="3" t="inlineStr">
+        <is>
+          <t>Phase 5: 5-layer validation for app_sessions</t>
+        </is>
+      </c>
+      <c r="D84" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-13 07:34 PDT</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="2" t="inlineStr">
+        <is>
+          <t>data/app_sessions.csv</t>
+        </is>
+      </c>
+      <c r="B85" s="2" t="inlineStr">
+        <is>
+          <t>Shipped table</t>
+        </is>
+      </c>
+      <c r="C85" s="3" t="inlineStr">
+        <is>
+          <t>Phase 5: app_sessions table (19,610 rows across 496 customers)</t>
+        </is>
+      </c>
+      <c r="D85" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-13 07:33 PDT</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Phase 5: build + validate app_events (4 of 4) -- Phase 5 complete
- Fitness event vocabulary per app_sessions.csv row: class_started,
  workout_completed/workout_abandoned (exactly one of the two, 85%
  complete), streak_achieved. Streaks are derived from each customer's own
  real consecutive-day session dates in app_sessions.csv, not sprinkled in
  -- independently re-derivable and re-verified exactly in the validator.
- Proactively caught and fixed a fractional-second timestamp bug (same
  class already hit twice this phase) before the first validation run.
- validate_app_events.py: 15/15 checks passed on the first run.
- 39,370 rows total. Completes Phase 5 (web_sessions, web_events,
  app_sessions, app_events).
</commit_message>
<xml_diff>
--- a/File_Manifest.xlsx
+++ b/File_Manifest.xlsx
@@ -435,7 +435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D85"/>
+  <dimension ref="A1:D88"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="48" customWidth="1" min="1" max="1"/>
@@ -506,7 +506,7 @@
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>2026-08-13 07:21 PDT</t>
+          <t>2026-08-13 07:35 PDT</t>
         </is>
       </c>
     </row>
@@ -638,7 +638,7 @@
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>2026-08-13 07:34 PDT</t>
+          <t>2026-08-13 07:44 PDT</t>
         </is>
       </c>
     </row>
@@ -748,7 +748,7 @@
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>2026-08-13 07:34 PDT</t>
+          <t>2026-08-13 07:44 PDT</t>
         </is>
       </c>
     </row>
@@ -2311,6 +2311,72 @@
       <c r="D85" s="2" t="inlineStr">
         <is>
           <t>2026-08-13 07:33 PDT</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="2" t="inlineStr">
+        <is>
+          <t>generator/build_app_events.py</t>
+        </is>
+      </c>
+      <c r="B86" s="2" t="inlineStr">
+        <is>
+          <t>Code</t>
+        </is>
+      </c>
+      <c r="C86" s="3" t="inlineStr">
+        <is>
+          <t>Phase 5: builds app_events (class_started/workout_completed/workout_abandoned/streak_achieved -- streaks derived from real consecutive session dates) -- completes Phase 5</t>
+        </is>
+      </c>
+      <c r="D86" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-13 07:44 PDT</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="2" t="inlineStr">
+        <is>
+          <t>generator/validate_app_events.py</t>
+        </is>
+      </c>
+      <c r="B87" s="2" t="inlineStr">
+        <is>
+          <t>Code</t>
+        </is>
+      </c>
+      <c r="C87" s="3" t="inlineStr">
+        <is>
+          <t>Phase 5: 5-layer validation for app_events</t>
+        </is>
+      </c>
+      <c r="D87" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-13 07:43 PDT</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="2" t="inlineStr">
+        <is>
+          <t>data/app_events.csv</t>
+        </is>
+      </c>
+      <c r="B88" s="2" t="inlineStr">
+        <is>
+          <t>Shipped table</t>
+        </is>
+      </c>
+      <c r="C88" s="3" t="inlineStr">
+        <is>
+          <t>Phase 5: app_events table (39,370 rows) -- completes Phase 5</t>
+        </is>
+      </c>
+      <c r="D88" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-13 07:44 PDT</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Phase 6: build + validate braze_email_campaigns (1 of 4)
- Hand-curated campaign definitions (9 rows: 7 triggered + 2 broadcast),
  built first since braze_email_events needs real campaigns to send
  against. Triggered campaigns each name a trigger_event mapping to a real
  source in an earlier phase's shipped tables; the seasonal broadcast is
  timed to discount_codes.csv's own real promo windows.
- validate_braze_email_campaigns.py: 10/10 checks passed.
</commit_message>
<xml_diff>
--- a/File_Manifest.xlsx
+++ b/File_Manifest.xlsx
@@ -435,7 +435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D88"/>
+  <dimension ref="A1:D91"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="48" customWidth="1" min="1" max="1"/>
@@ -506,7 +506,7 @@
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>2026-08-13 07:35 PDT</t>
+          <t>2026-08-13 07:44 PDT</t>
         </is>
       </c>
     </row>
@@ -638,7 +638,7 @@
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>2026-08-13 07:44 PDT</t>
+          <t>2026-08-13 07:49 PDT</t>
         </is>
       </c>
     </row>
@@ -748,7 +748,7 @@
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>2026-08-13 07:44 PDT</t>
+          <t>2026-08-13 07:49 PDT</t>
         </is>
       </c>
     </row>
@@ -2377,6 +2377,72 @@
       <c r="D88" s="2" t="inlineStr">
         <is>
           <t>2026-08-13 07:44 PDT</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="2" t="inlineStr">
+        <is>
+          <t>generator/build_braze_email_campaigns.py</t>
+        </is>
+      </c>
+      <c r="B89" s="2" t="inlineStr">
+        <is>
+          <t>Code</t>
+        </is>
+      </c>
+      <c r="C89" s="3" t="inlineStr">
+        <is>
+          <t>Phase 6: builds braze_email_campaigns (hand-curated: 7 triggered + 2 broadcast) -- built first, events table needs it</t>
+        </is>
+      </c>
+      <c r="D89" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-13 07:48 PDT</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="2" t="inlineStr">
+        <is>
+          <t>generator/validate_braze_email_campaigns.py</t>
+        </is>
+      </c>
+      <c r="B90" s="2" t="inlineStr">
+        <is>
+          <t>Code</t>
+        </is>
+      </c>
+      <c r="C90" s="3" t="inlineStr">
+        <is>
+          <t>Phase 6: 5-layer validation for braze_email_campaigns</t>
+        </is>
+      </c>
+      <c r="D90" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-13 07:49 PDT</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="2" t="inlineStr">
+        <is>
+          <t>data/braze_email_campaigns.csv</t>
+        </is>
+      </c>
+      <c r="B91" s="2" t="inlineStr">
+        <is>
+          <t>Shipped table</t>
+        </is>
+      </c>
+      <c r="C91" s="3" t="inlineStr">
+        <is>
+          <t>Phase 6: braze_email_campaigns table (9 rows)</t>
+        </is>
+      </c>
+      <c r="D91" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-13 07:48 PDT</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Phase 6: build + validate braze_push_campaigns (3 of 4)
- Hand-curated campaign definitions (7 rows: 5 triggered + 2 broadcast),
  a push-appropriate subset of email's campaigns rather than a blind
  mirror. Order Shipped is deliberately known-customers-only (push has no
  guest-checkout equivalent).
- validate_braze_push_campaigns.py: 11/11 checks passed.
</commit_message>
<xml_diff>
--- a/File_Manifest.xlsx
+++ b/File_Manifest.xlsx
@@ -435,7 +435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D96"/>
+  <dimension ref="A1:D99"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="48" customWidth="1" min="1" max="1"/>
@@ -506,7 +506,7 @@
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>2026-08-13 07:49 PDT</t>
+          <t>2026-08-13 07:58 PDT</t>
         </is>
       </c>
     </row>
@@ -638,7 +638,7 @@
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>2026-08-13 07:57 PDT</t>
+          <t>2026-08-13 08:00 PDT</t>
         </is>
       </c>
     </row>
@@ -748,7 +748,7 @@
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>2026-08-13 07:58 PDT</t>
+          <t>2026-08-13 08:00 PDT</t>
         </is>
       </c>
     </row>
@@ -2553,6 +2553,72 @@
       <c r="D96" s="2" t="inlineStr">
         <is>
           <t>2026-08-13 07:57 PDT</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" s="2" t="inlineStr">
+        <is>
+          <t>generator/build_braze_push_campaigns.py</t>
+        </is>
+      </c>
+      <c r="B97" s="2" t="inlineStr">
+        <is>
+          <t>Code</t>
+        </is>
+      </c>
+      <c r="C97" s="3" t="inlineStr">
+        <is>
+          <t>Phase 6: builds braze_push_campaigns (hand-curated: 5 triggered + 2 broadcast, push-appropriate subset) -- built before events table needs it</t>
+        </is>
+      </c>
+      <c r="D97" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-13 07:59 PDT</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" s="2" t="inlineStr">
+        <is>
+          <t>generator/validate_braze_push_campaigns.py</t>
+        </is>
+      </c>
+      <c r="B98" s="2" t="inlineStr">
+        <is>
+          <t>Code</t>
+        </is>
+      </c>
+      <c r="C98" s="3" t="inlineStr">
+        <is>
+          <t>Phase 6: 5-layer validation for braze_push_campaigns</t>
+        </is>
+      </c>
+      <c r="D98" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-13 08:00 PDT</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" s="2" t="inlineStr">
+        <is>
+          <t>data/braze_push_campaigns.csv</t>
+        </is>
+      </c>
+      <c r="B99" s="2" t="inlineStr">
+        <is>
+          <t>Shipped table</t>
+        </is>
+      </c>
+      <c r="C99" s="3" t="inlineStr">
+        <is>
+          <t>Phase 6: braze_push_campaigns table (7 rows)</t>
+        </is>
+      </c>
+      <c r="D99" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-13 07:59 PDT</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Phase 6 complete: build + validate braze_push_events (4 of 4)
Final Phase 6 table: Send/Open/Click/Bounce/Unsubscribe funnel under the
users.messages.pushnotification.* namespace, gated on push_opt_in as a hard
delivery precondition (unlike email, where a transactional message can
always be attempted). Reuses trial_ending/payment_failed/reactivation/
order_placed populations from braze_email_events.py plus a new
streak_achieved population sourced from app_events.csv. 9,897 rows (7,851
sends), validate_braze_push_events.py 19/19 checks passed on the first run.

Phase 6 (all 4 tables) is now complete. 25 of 47 tables shipped.
</commit_message>
<xml_diff>
--- a/File_Manifest.xlsx
+++ b/File_Manifest.xlsx
@@ -435,7 +435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D99"/>
+  <dimension ref="A1:D102"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="48" customWidth="1" min="1" max="1"/>
@@ -506,7 +506,7 @@
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>2026-08-13 07:58 PDT</t>
+          <t>2026-08-13 08:00 PDT</t>
         </is>
       </c>
     </row>
@@ -638,7 +638,7 @@
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>2026-08-13 08:00 PDT</t>
+          <t>2026-08-13 08:07 PDT</t>
         </is>
       </c>
     </row>
@@ -748,7 +748,7 @@
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>2026-08-13 08:00 PDT</t>
+          <t>2026-08-13 08:07 PDT</t>
         </is>
       </c>
     </row>
@@ -2619,6 +2619,72 @@
       <c r="D99" s="2" t="inlineStr">
         <is>
           <t>2026-08-13 07:59 PDT</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" s="2" t="inlineStr">
+        <is>
+          <t>generator/build_braze_push_events.py</t>
+        </is>
+      </c>
+      <c r="B100" s="2" t="inlineStr">
+        <is>
+          <t>Code</t>
+        </is>
+      </c>
+      <c r="C100" s="3" t="inlineStr">
+        <is>
+          <t>Phase 6: builds braze_push_events (Send/Open/Click/Bounce/Unsubscribe funnel, gated on push_opt_in as a hard delivery precondition) -- completes Phase 6 (all 4 tables)</t>
+        </is>
+      </c>
+      <c r="D100" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-13 08:03 PDT</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" s="2" t="inlineStr">
+        <is>
+          <t>generator/validate_braze_push_events.py</t>
+        </is>
+      </c>
+      <c r="B101" s="2" t="inlineStr">
+        <is>
+          <t>Code</t>
+        </is>
+      </c>
+      <c r="C101" s="3" t="inlineStr">
+        <is>
+          <t>Phase 6: 5-layer validation for braze_push_events</t>
+        </is>
+      </c>
+      <c r="D101" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-13 08:06 PDT</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" s="2" t="inlineStr">
+        <is>
+          <t>data/braze_push_events.csv</t>
+        </is>
+      </c>
+      <c r="B102" s="2" t="inlineStr">
+        <is>
+          <t>Shipped table</t>
+        </is>
+      </c>
+      <c r="C102" s="3" t="inlineStr">
+        <is>
+          <t>Phase 6: braze_push_events table (9,897 rows, 7,851 sends) -- completes Phase 6 (25 of 47 tables shipped; Phase 7 paid media remains)</t>
+        </is>
+      </c>
+      <c r="D102" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-13 08:05 PDT</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Phase 7: build + validate Google Search (2 of 6 paid-media platforms)
google_search_campaigns (5 evergreen objective campaigns, incl. an
always-on brand-term defense campaign rather than a flighted study since
that's realistic for search specifically), google_search_ad_groups (8
rows, RLSA/similar-audience targeting), google_search_keyword_performance_daily
(19,932 rows, the granular ground truth -- no separate keywords dimension
table exists in the schema so keyword rosters are defined in-script),
google_search_performance_daily (8,751 rows, an EXACT aggregation up from
the keyword table, reconciled to the penny).

One calibration adjustment made before shipping, informed by the Meta
over-attribution lesson: conversion rates retuned down ~25% so Google
Search's self-attributed conversions land at 2.42x actual real purchases
instead of an initial 3.13x. 49/49 validation checks passed across all 4
tables.

33 of 47 tables now shipped.
</commit_message>
<xml_diff>
--- a/File_Manifest.xlsx
+++ b/File_Manifest.xlsx
@@ -435,7 +435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D115"/>
+  <dimension ref="A1:D127"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="48" customWidth="1" min="1" max="1"/>
@@ -506,7 +506,7 @@
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>2026-08-13 08:08 PDT</t>
+          <t>2026-08-13 10:59 PDT</t>
         </is>
       </c>
     </row>
@@ -594,7 +594,7 @@
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>2026-08-13 10:57 PDT</t>
+          <t>2026-08-13 12:17 PDT</t>
         </is>
       </c>
     </row>
@@ -638,7 +638,7 @@
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>2026-08-13 10:59 PDT</t>
+          <t>2026-08-13 12:19 PDT</t>
         </is>
       </c>
     </row>
@@ -748,7 +748,7 @@
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>2026-08-13 10:59 PDT</t>
+          <t>2026-08-13 12:19 PDT</t>
         </is>
       </c>
     </row>
@@ -2971,6 +2971,270 @@
       <c r="D115" s="2" t="inlineStr">
         <is>
           <t>2026-08-13 10:57 PDT</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" s="2" t="inlineStr">
+        <is>
+          <t>generator/build_google_search_campaigns.py</t>
+        </is>
+      </c>
+      <c r="B116" s="2" t="inlineStr">
+        <is>
+          <t>Code</t>
+        </is>
+      </c>
+      <c r="C116" s="3" t="inlineStr">
+        <is>
+          <t>Phase 7 (Google Search 1/4): builds google_search_campaigns (5 evergreen objective campaigns, incl. an always-on brand-term defense campaign)</t>
+        </is>
+      </c>
+      <c r="D116" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-13 12:16 PDT</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" s="2" t="inlineStr">
+        <is>
+          <t>generator/validate_google_search_campaigns.py</t>
+        </is>
+      </c>
+      <c r="B117" s="2" t="inlineStr">
+        <is>
+          <t>Code</t>
+        </is>
+      </c>
+      <c r="C117" s="3" t="inlineStr">
+        <is>
+          <t>Phase 7: 5-layer validation for google_search_campaigns</t>
+        </is>
+      </c>
+      <c r="D117" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-13 12:18 PDT</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" s="2" t="inlineStr">
+        <is>
+          <t>data/google_search_campaigns.csv</t>
+        </is>
+      </c>
+      <c r="B118" s="2" t="inlineStr">
+        <is>
+          <t>Shipped table</t>
+        </is>
+      </c>
+      <c r="C118" s="3" t="inlineStr">
+        <is>
+          <t>Phase 7 (Google Search 1/4): google_search_campaigns table (5 rows)</t>
+        </is>
+      </c>
+      <c r="D118" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-13 12:16 PDT</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" s="2" t="inlineStr">
+        <is>
+          <t>generator/build_google_search_ad_groups.py</t>
+        </is>
+      </c>
+      <c r="B119" s="2" t="inlineStr">
+        <is>
+          <t>Code</t>
+        </is>
+      </c>
+      <c r="C119" s="3" t="inlineStr">
+        <is>
+          <t>Phase 7 (Google Search 2/4): builds google_search_ad_groups (targeting_segment_id for RLSA retargeting/similar-audience lookalike only)</t>
+        </is>
+      </c>
+      <c r="D119" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-13 12:16 PDT</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" s="2" t="inlineStr">
+        <is>
+          <t>generator/validate_google_search_ad_groups.py</t>
+        </is>
+      </c>
+      <c r="B120" s="2" t="inlineStr">
+        <is>
+          <t>Code</t>
+        </is>
+      </c>
+      <c r="C120" s="3" t="inlineStr">
+        <is>
+          <t>Phase 7: 5-layer validation for google_search_ad_groups</t>
+        </is>
+      </c>
+      <c r="D120" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-13 12:18 PDT</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" s="2" t="inlineStr">
+        <is>
+          <t>data/google_search_ad_groups.csv</t>
+        </is>
+      </c>
+      <c r="B121" s="2" t="inlineStr">
+        <is>
+          <t>Shipped table</t>
+        </is>
+      </c>
+      <c r="C121" s="3" t="inlineStr">
+        <is>
+          <t>Phase 7 (Google Search 2/4): google_search_ad_groups table (8 rows)</t>
+        </is>
+      </c>
+      <c r="D121" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-13 12:16 PDT</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" s="2" t="inlineStr">
+        <is>
+          <t>generator/build_google_search_keyword_performance_daily.py</t>
+        </is>
+      </c>
+      <c r="B122" s="2" t="inlineStr">
+        <is>
+          <t>Code</t>
+        </is>
+      </c>
+      <c r="C122" s="3" t="inlineStr">
+        <is>
+          <t>Phase 7 (Google Search 4/4 by build order): builds google_search_keyword_performance_daily -- the granular ground truth google_search_performance_daily aggregates from</t>
+        </is>
+      </c>
+      <c r="D122" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-13 12:17 PDT</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" s="2" t="inlineStr">
+        <is>
+          <t>generator/validate_google_search_keyword_performance_daily.py</t>
+        </is>
+      </c>
+      <c r="B123" s="2" t="inlineStr">
+        <is>
+          <t>Code</t>
+        </is>
+      </c>
+      <c r="C123" s="3" t="inlineStr">
+        <is>
+          <t>Phase 7: 5-layer validation for google_search_keyword_performance_daily, incl. weekly-spend-vs-web_sessions correlation check</t>
+        </is>
+      </c>
+      <c r="D123" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-13 12:18 PDT</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" s="2" t="inlineStr">
+        <is>
+          <t>data/google_search_keyword_performance_daily.csv</t>
+        </is>
+      </c>
+      <c r="B124" s="2" t="inlineStr">
+        <is>
+          <t>Shipped table</t>
+        </is>
+      </c>
+      <c r="C124" s="3" t="inlineStr">
+        <is>
+          <t>Phase 7 (Google Search 4/4 by build order): google_search_keyword_performance_daily table (19,932 rows)</t>
+        </is>
+      </c>
+      <c r="D124" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-13 12:17 PDT</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" s="2" t="inlineStr">
+        <is>
+          <t>generator/build_google_search_performance_daily.py</t>
+        </is>
+      </c>
+      <c r="B125" s="2" t="inlineStr">
+        <is>
+          <t>Code</t>
+        </is>
+      </c>
+      <c r="C125" s="3" t="inlineStr">
+        <is>
+          <t>Phase 7 (Google Search 3/4 by schema order): builds google_search_performance_daily, aggregated exactly from keyword_performance_daily.csv up to ad_group/day grain -- completes Google Search (2 of 6 platforms)</t>
+        </is>
+      </c>
+      <c r="D125" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-13 12:17 PDT</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" s="2" t="inlineStr">
+        <is>
+          <t>generator/validate_google_search_performance_daily.py</t>
+        </is>
+      </c>
+      <c r="B126" s="2" t="inlineStr">
+        <is>
+          <t>Code</t>
+        </is>
+      </c>
+      <c r="C126" s="3" t="inlineStr">
+        <is>
+          <t>Phase 7: 5-layer validation for google_search_performance_daily, incl. exact-sum reconciliation against keyword_performance_daily.csv</t>
+        </is>
+      </c>
+      <c r="D126" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-13 12:19 PDT</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" s="2" t="inlineStr">
+        <is>
+          <t>data/google_search_performance_daily.csv</t>
+        </is>
+      </c>
+      <c r="B127" s="2" t="inlineStr">
+        <is>
+          <t>Shipped table</t>
+        </is>
+      </c>
+      <c r="C127" s="3" t="inlineStr">
+        <is>
+          <t>Phase 7 (Google Search 3/4 by schema order): google_search_performance_daily table (8,751 rows) -- completes Google Search</t>
+        </is>
+      </c>
+      <c r="D127" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-13 12:17 PDT</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Phase 7: build + validate DV360 (4 of 6 paid-media platforms)
dv360_insertion_orders (5 evergreen objective IOs), dv360_line_items (6
rows), dv360_performance_daily (25,776 rows) -- the genuinely different-
shaped table schema_reference.md calls out: real-time bidding fragments
each line_item/day into 1-7 (exchange, environment) rows across 5
exchanges and up to 4 environments, with Connected TV inventory reachable
only by the video/brand_lift line item.

No bugs found this round -- spend matched the seasonality-formula
expectation cleanly and self-attributed conversions landed at a lower,
appropriately-realistic ratio (0.38x actual purchases) than search/social
platforms. 40/40 validation checks passed across all 3 tables on the
first run.

39 of 47 tables now shipped.
</commit_message>
<xml_diff>
--- a/File_Manifest.xlsx
+++ b/File_Manifest.xlsx
@@ -435,7 +435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D136"/>
+  <dimension ref="A1:D145"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="48" customWidth="1" min="1" max="1"/>
@@ -506,7 +506,7 @@
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>2026-08-13 12:19 PDT</t>
+          <t>2026-08-13 12:29 PDT</t>
         </is>
       </c>
     </row>
@@ -594,7 +594,7 @@
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>2026-08-13 12:29 PDT</t>
+          <t>2026-08-13 12:32 PDT</t>
         </is>
       </c>
     </row>
@@ -638,7 +638,7 @@
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>2026-08-13 12:29 PDT</t>
+          <t>2026-08-13 12:34 PDT</t>
         </is>
       </c>
     </row>
@@ -748,7 +748,7 @@
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>2026-08-13 12:29 PDT</t>
+          <t>2026-08-13 12:34 PDT</t>
         </is>
       </c>
     </row>
@@ -3433,6 +3433,204 @@
       <c r="D136" s="2" t="inlineStr">
         <is>
           <t>2026-08-13 12:29 PDT</t>
+        </is>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" s="2" t="inlineStr">
+        <is>
+          <t>generator/build_dv360_insertion_orders.py</t>
+        </is>
+      </c>
+      <c r="B137" s="2" t="inlineStr">
+        <is>
+          <t>Code</t>
+        </is>
+      </c>
+      <c r="C137" s="3" t="inlineStr">
+        <is>
+          <t>Phase 7 (DV360 1/3): builds dv360_insertion_orders (5 evergreen objective IOs, incl. a VIEWABLE_CPM awareness IO)</t>
+        </is>
+      </c>
+      <c r="D137" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-13 12:32 PDT</t>
+        </is>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" s="2" t="inlineStr">
+        <is>
+          <t>generator/validate_dv360_insertion_orders.py</t>
+        </is>
+      </c>
+      <c r="B138" s="2" t="inlineStr">
+        <is>
+          <t>Code</t>
+        </is>
+      </c>
+      <c r="C138" s="3" t="inlineStr">
+        <is>
+          <t>Phase 7: 5-layer validation for dv360_insertion_orders</t>
+        </is>
+      </c>
+      <c r="D138" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-13 12:33 PDT</t>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" s="2" t="inlineStr">
+        <is>
+          <t>data/dv360_insertion_orders.csv</t>
+        </is>
+      </c>
+      <c r="B139" s="2" t="inlineStr">
+        <is>
+          <t>Shipped table</t>
+        </is>
+      </c>
+      <c r="C139" s="3" t="inlineStr">
+        <is>
+          <t>Phase 7 (DV360 1/3): dv360_insertion_orders table (5 rows)</t>
+        </is>
+      </c>
+      <c r="D139" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-13 12:32 PDT</t>
+        </is>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" s="2" t="inlineStr">
+        <is>
+          <t>generator/build_dv360_line_items.py</t>
+        </is>
+      </c>
+      <c r="B140" s="2" t="inlineStr">
+        <is>
+          <t>Code</t>
+        </is>
+      </c>
+      <c r="C140" s="3" t="inlineStr">
+        <is>
+          <t>Phase 7 (DV360 2/3): builds dv360_line_items (targeting_segment_id for retargeting/lookalike only; brand_lift IO's line item is VIDEO type)</t>
+        </is>
+      </c>
+      <c r="D140" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-13 12:32 PDT</t>
+        </is>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" s="2" t="inlineStr">
+        <is>
+          <t>generator/validate_dv360_line_items.py</t>
+        </is>
+      </c>
+      <c r="B141" s="2" t="inlineStr">
+        <is>
+          <t>Code</t>
+        </is>
+      </c>
+      <c r="C141" s="3" t="inlineStr">
+        <is>
+          <t>Phase 7: 5-layer validation for dv360_line_items</t>
+        </is>
+      </c>
+      <c r="D141" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-13 12:33 PDT</t>
+        </is>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" s="2" t="inlineStr">
+        <is>
+          <t>data/dv360_line_items.csv</t>
+        </is>
+      </c>
+      <c r="B142" s="2" t="inlineStr">
+        <is>
+          <t>Shipped table</t>
+        </is>
+      </c>
+      <c r="C142" s="3" t="inlineStr">
+        <is>
+          <t>Phase 7 (DV360 2/3): dv360_line_items table (6 rows)</t>
+        </is>
+      </c>
+      <c r="D142" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-13 12:32 PDT</t>
+        </is>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" s="2" t="inlineStr">
+        <is>
+          <t>generator/build_dv360_performance_daily.py</t>
+        </is>
+      </c>
+      <c r="B143" s="2" t="inlineStr">
+        <is>
+          <t>Code</t>
+        </is>
+      </c>
+      <c r="C143" s="3" t="inlineStr">
+        <is>
+          <t>Phase 7 (DV360 3/3): builds dv360_performance_daily -- fragments each line_item/day into several (exchange, environment) rows, DV360's genuinely different real-time-bidding schema shape -- completes DV360 (4 of 6 platforms)</t>
+        </is>
+      </c>
+      <c r="D143" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-13 12:33 PDT</t>
+        </is>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" s="2" t="inlineStr">
+        <is>
+          <t>generator/validate_dv360_performance_daily.py</t>
+        </is>
+      </c>
+      <c r="B144" s="2" t="inlineStr">
+        <is>
+          <t>Code</t>
+        </is>
+      </c>
+      <c r="C144" s="3" t="inlineStr">
+        <is>
+          <t>Phase 7: 5-layer validation for dv360_performance_daily, incl. weekly-spend-vs-web_sessions correlation check and CONNECTED_TV-only-on-video-line-item check</t>
+        </is>
+      </c>
+      <c r="D144" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-13 12:34 PDT</t>
+        </is>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" s="2" t="inlineStr">
+        <is>
+          <t>data/dv360_performance_daily.csv</t>
+        </is>
+      </c>
+      <c r="B145" s="2" t="inlineStr">
+        <is>
+          <t>Shipped table</t>
+        </is>
+      </c>
+      <c r="C145" s="3" t="inlineStr">
+        <is>
+          <t>Phase 7 (DV360 3/3): dv360_performance_daily table (25,776 rows) -- completes DV360</t>
+        </is>
+      </c>
+      <c r="D145" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-13 12:33 PDT</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Phase 7: build + validate Snap (5 of 6 paid-media platforms)
snap_campaigns (7 rows: 4 evergreen + 3 flighted brand_lift, budgets
calibrated up front using the proportion lesson learned from YouTube's
build), snap_ad_squads (8 rows, Snap's real ad-set-level targeting entity),
snap_ads (10 rows, pure creative), snap_stats_daily (7,407 rows, spend in
Snap's micro-currency unit, swipes as the click-equivalent).

No bugs found this round -- spend and conversions landed within expected
ranges on the first build. 47/47 validation checks passed across all 4
tables.

43 of 47 tables now shipped.
</commit_message>
<xml_diff>
--- a/File_Manifest.xlsx
+++ b/File_Manifest.xlsx
@@ -435,7 +435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D145"/>
+  <dimension ref="A1:D157"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="48" customWidth="1" min="1" max="1"/>
@@ -506,7 +506,7 @@
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>2026-08-13 12:29 PDT</t>
+          <t>2026-08-13 12:34 PDT</t>
         </is>
       </c>
     </row>
@@ -594,7 +594,7 @@
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>2026-08-13 12:32 PDT</t>
+          <t>2026-08-13 12:46 PDT</t>
         </is>
       </c>
     </row>
@@ -638,7 +638,7 @@
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>2026-08-13 12:34 PDT</t>
+          <t>2026-08-13 12:48 PDT</t>
         </is>
       </c>
     </row>
@@ -748,7 +748,7 @@
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>2026-08-13 12:34 PDT</t>
+          <t>2026-08-13 12:48 PDT</t>
         </is>
       </c>
     </row>
@@ -3631,6 +3631,270 @@
       <c r="D145" s="2" t="inlineStr">
         <is>
           <t>2026-08-13 12:33 PDT</t>
+        </is>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" s="2" t="inlineStr">
+        <is>
+          <t>generator/build_snap_campaigns.py</t>
+        </is>
+      </c>
+      <c r="B146" s="2" t="inlineStr">
+        <is>
+          <t>Code</t>
+        </is>
+      </c>
+      <c r="C146" s="3" t="inlineStr">
+        <is>
+          <t>Phase 7 (Snap 1/4): builds snap_campaigns (4 evergreen objective campaigns + 3 flighted brand_lift campaigns, flight budgets calibrated to avoid YouTube's earlier scale bug)</t>
+        </is>
+      </c>
+      <c r="D146" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-13 12:46 PDT</t>
+        </is>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" s="2" t="inlineStr">
+        <is>
+          <t>generator/validate_snap_campaigns.py</t>
+        </is>
+      </c>
+      <c r="B147" s="2" t="inlineStr">
+        <is>
+          <t>Code</t>
+        </is>
+      </c>
+      <c r="C147" s="3" t="inlineStr">
+        <is>
+          <t>Phase 7: 5-layer validation for snap_campaigns</t>
+        </is>
+      </c>
+      <c r="D147" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-13 12:47 PDT</t>
+        </is>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" s="2" t="inlineStr">
+        <is>
+          <t>data/snap_campaigns.csv</t>
+        </is>
+      </c>
+      <c r="B148" s="2" t="inlineStr">
+        <is>
+          <t>Shipped table</t>
+        </is>
+      </c>
+      <c r="C148" s="3" t="inlineStr">
+        <is>
+          <t>Phase 7 (Snap 1/4): snap_campaigns table (7 rows)</t>
+        </is>
+      </c>
+      <c r="D148" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-13 12:46 PDT</t>
+        </is>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" s="2" t="inlineStr">
+        <is>
+          <t>generator/build_snap_ad_squads.py</t>
+        </is>
+      </c>
+      <c r="B149" s="2" t="inlineStr">
+        <is>
+          <t>Code</t>
+        </is>
+      </c>
+      <c r="C149" s="3" t="inlineStr">
+        <is>
+          <t>Phase 7 (Snap 2/4): builds snap_ad_squads (Snap's own real ad-set-level targeting entity, unlike Meta -- targeting_segment_id for retargeting/lookalike only)</t>
+        </is>
+      </c>
+      <c r="D149" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-13 12:46 PDT</t>
+        </is>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" s="2" t="inlineStr">
+        <is>
+          <t>generator/validate_snap_ad_squads.py</t>
+        </is>
+      </c>
+      <c r="B150" s="2" t="inlineStr">
+        <is>
+          <t>Code</t>
+        </is>
+      </c>
+      <c r="C150" s="3" t="inlineStr">
+        <is>
+          <t>Phase 7: 5-layer validation for snap_ad_squads</t>
+        </is>
+      </c>
+      <c r="D150" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-13 12:48 PDT</t>
+        </is>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" s="2" t="inlineStr">
+        <is>
+          <t>data/snap_ad_squads.csv</t>
+        </is>
+      </c>
+      <c r="B151" s="2" t="inlineStr">
+        <is>
+          <t>Shipped table</t>
+        </is>
+      </c>
+      <c r="C151" s="3" t="inlineStr">
+        <is>
+          <t>Phase 7 (Snap 2/4): snap_ad_squads table (8 rows)</t>
+        </is>
+      </c>
+      <c r="D151" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-13 12:46 PDT</t>
+        </is>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" s="2" t="inlineStr">
+        <is>
+          <t>generator/build_snap_ads.py</t>
+        </is>
+      </c>
+      <c r="B152" s="2" t="inlineStr">
+        <is>
+          <t>Code</t>
+        </is>
+      </c>
+      <c r="C152" s="3" t="inlineStr">
+        <is>
+          <t>Phase 7 (Snap 3/4): builds snap_ads (creative-level entity, no targeting -- that lives on the ad squad)</t>
+        </is>
+      </c>
+      <c r="D152" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-13 12:47 PDT</t>
+        </is>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" s="2" t="inlineStr">
+        <is>
+          <t>generator/validate_snap_ads.py</t>
+        </is>
+      </c>
+      <c r="B153" s="2" t="inlineStr">
+        <is>
+          <t>Code</t>
+        </is>
+      </c>
+      <c r="C153" s="3" t="inlineStr">
+        <is>
+          <t>Phase 7: 5-layer validation for snap_ads</t>
+        </is>
+      </c>
+      <c r="D153" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-13 12:48 PDT</t>
+        </is>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" s="2" t="inlineStr">
+        <is>
+          <t>data/snap_ads.csv</t>
+        </is>
+      </c>
+      <c r="B154" s="2" t="inlineStr">
+        <is>
+          <t>Shipped table</t>
+        </is>
+      </c>
+      <c r="C154" s="3" t="inlineStr">
+        <is>
+          <t>Phase 7 (Snap 3/4): snap_ads table (10 rows)</t>
+        </is>
+      </c>
+      <c r="D154" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-13 12:47 PDT</t>
+        </is>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" s="2" t="inlineStr">
+        <is>
+          <t>generator/build_snap_stats_daily.py</t>
+        </is>
+      </c>
+      <c r="B155" s="2" t="inlineStr">
+        <is>
+          <t>Code</t>
+        </is>
+      </c>
+      <c r="C155" s="3" t="inlineStr">
+        <is>
+          <t>Phase 7 (Snap 4/4): builds snap_stats_daily (spend in Snap's own micro-currency unit, swipes as the click-equivalent) -- completes Snap (5 of 6 platforms)</t>
+        </is>
+      </c>
+      <c r="D155" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-13 12:47 PDT</t>
+        </is>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" s="2" t="inlineStr">
+        <is>
+          <t>generator/validate_snap_stats_daily.py</t>
+        </is>
+      </c>
+      <c r="B156" s="2" t="inlineStr">
+        <is>
+          <t>Code</t>
+        </is>
+      </c>
+      <c r="C156" s="3" t="inlineStr">
+        <is>
+          <t>Phase 7: 5-layer validation for snap_stats_daily, incl. weekly-spend-vs-web_sessions correlation check</t>
+        </is>
+      </c>
+      <c r="D156" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-13 12:48 PDT</t>
+        </is>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" s="2" t="inlineStr">
+        <is>
+          <t>data/snap_stats_daily.csv</t>
+        </is>
+      </c>
+      <c r="B157" s="2" t="inlineStr">
+        <is>
+          <t>Shipped table</t>
+        </is>
+      </c>
+      <c r="C157" s="3" t="inlineStr">
+        <is>
+          <t>Phase 7 (Snap 4/4): snap_stats_daily table (7,407 rows) -- completes Snap</t>
+        </is>
+      </c>
+      <c r="D157" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-13 12:47 PDT</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Phase 7 complete: build + validate TikTok (6 of 6) -- PROJECT COMPLETE (47/47 tables)
tiktok_campaigns (7 rows: 4 evergreen + 3 flighted brand_lift), tiktok_adgroups
(8 rows, TikTok's own real ad-set-level targeting entity), tiktok_ads (10 rows,
pure creative), tiktok_reports_daily (7,416 rows, TikTok's always-video ad
format). No bugs found -- calibration-up-front discipline from the YouTube fix
held. 46/46 validation checks passed across all 4 tables.

This completes Phase 7 (all 22 paid-media tables across Meta, Google Search,
YouTube, DV360, Snap, TikTok) and the entire 47-table Kinetic dataset.

Ran a final full-suite validation across all 47 tables' validators in one
pass: all 47 pass, 720 checks total, zero failures -- confirms the Phase 0
shared master-timeline design held its promise across the whole project,
with no cross-table impossible scenarios anywhere in the dataset.
</commit_message>
<xml_diff>
--- a/File_Manifest.xlsx
+++ b/File_Manifest.xlsx
@@ -435,7 +435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D157"/>
+  <dimension ref="A1:D169"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="48" customWidth="1" min="1" max="1"/>
@@ -506,7 +506,7 @@
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>2026-08-13 12:34 PDT</t>
+          <t>2026-08-13 12:49 PDT</t>
         </is>
       </c>
     </row>
@@ -638,7 +638,7 @@
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>2026-08-13 12:48 PDT</t>
+          <t>2026-08-13 14:38 PDT</t>
         </is>
       </c>
     </row>
@@ -748,7 +748,7 @@
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>2026-08-13 12:48 PDT</t>
+          <t>2026-08-13 14:38 PDT</t>
         </is>
       </c>
     </row>
@@ -3895,6 +3895,270 @@
       <c r="D157" s="2" t="inlineStr">
         <is>
           <t>2026-08-13 12:47 PDT</t>
+        </is>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" s="2" t="inlineStr">
+        <is>
+          <t>generator/build_tiktok_campaigns.py</t>
+        </is>
+      </c>
+      <c r="B158" s="2" t="inlineStr">
+        <is>
+          <t>Code</t>
+        </is>
+      </c>
+      <c r="C158" s="3" t="inlineStr">
+        <is>
+          <t>Phase 7 (TikTok 1/4): builds tiktok_campaigns (4 evergreen objective campaigns + 3 flighted brand_lift campaigns)</t>
+        </is>
+      </c>
+      <c r="D158" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-13 14:34 PDT</t>
+        </is>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" s="2" t="inlineStr">
+        <is>
+          <t>generator/validate_tiktok_campaigns.py</t>
+        </is>
+      </c>
+      <c r="B159" s="2" t="inlineStr">
+        <is>
+          <t>Code</t>
+        </is>
+      </c>
+      <c r="C159" s="3" t="inlineStr">
+        <is>
+          <t>Phase 7: 5-layer validation for tiktok_campaigns</t>
+        </is>
+      </c>
+      <c r="D159" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-13 14:36 PDT</t>
+        </is>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" s="2" t="inlineStr">
+        <is>
+          <t>data/tiktok_campaigns.csv</t>
+        </is>
+      </c>
+      <c r="B160" s="2" t="inlineStr">
+        <is>
+          <t>Shipped table</t>
+        </is>
+      </c>
+      <c r="C160" s="3" t="inlineStr">
+        <is>
+          <t>Phase 7 (TikTok 1/4): tiktok_campaigns table (7 rows)</t>
+        </is>
+      </c>
+      <c r="D160" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-13 14:34 PDT</t>
+        </is>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" s="2" t="inlineStr">
+        <is>
+          <t>generator/build_tiktok_adgroups.py</t>
+        </is>
+      </c>
+      <c r="B161" s="2" t="inlineStr">
+        <is>
+          <t>Code</t>
+        </is>
+      </c>
+      <c r="C161" s="3" t="inlineStr">
+        <is>
+          <t>Phase 7 (TikTok 2/4): builds tiktok_adgroups (TikTok's own real ad-set-level targeting entity -- targeting_segment_id for retargeting/lookalike only)</t>
+        </is>
+      </c>
+      <c r="D161" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-13 14:34 PDT</t>
+        </is>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" s="2" t="inlineStr">
+        <is>
+          <t>generator/validate_tiktok_adgroups.py</t>
+        </is>
+      </c>
+      <c r="B162" s="2" t="inlineStr">
+        <is>
+          <t>Code</t>
+        </is>
+      </c>
+      <c r="C162" s="3" t="inlineStr">
+        <is>
+          <t>Phase 7: 5-layer validation for tiktok_adgroups</t>
+        </is>
+      </c>
+      <c r="D162" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-13 14:36 PDT</t>
+        </is>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" s="2" t="inlineStr">
+        <is>
+          <t>data/tiktok_adgroups.csv</t>
+        </is>
+      </c>
+      <c r="B163" s="2" t="inlineStr">
+        <is>
+          <t>Shipped table</t>
+        </is>
+      </c>
+      <c r="C163" s="3" t="inlineStr">
+        <is>
+          <t>Phase 7 (TikTok 2/4): tiktok_adgroups table (8 rows)</t>
+        </is>
+      </c>
+      <c r="D163" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-13 14:34 PDT</t>
+        </is>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" s="2" t="inlineStr">
+        <is>
+          <t>generator/build_tiktok_ads.py</t>
+        </is>
+      </c>
+      <c r="B164" s="2" t="inlineStr">
+        <is>
+          <t>Code</t>
+        </is>
+      </c>
+      <c r="C164" s="3" t="inlineStr">
+        <is>
+          <t>Phase 7 (TikTok 3/4): builds tiktok_ads (creative-level entity, no targeting -- that lives on the ad group)</t>
+        </is>
+      </c>
+      <c r="D164" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-13 14:35 PDT</t>
+        </is>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" s="2" t="inlineStr">
+        <is>
+          <t>generator/validate_tiktok_ads.py</t>
+        </is>
+      </c>
+      <c r="B165" s="2" t="inlineStr">
+        <is>
+          <t>Code</t>
+        </is>
+      </c>
+      <c r="C165" s="3" t="inlineStr">
+        <is>
+          <t>Phase 7: 5-layer validation for tiktok_ads</t>
+        </is>
+      </c>
+      <c r="D165" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-13 14:36 PDT</t>
+        </is>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" s="2" t="inlineStr">
+        <is>
+          <t>data/tiktok_ads.csv</t>
+        </is>
+      </c>
+      <c r="B166" s="2" t="inlineStr">
+        <is>
+          <t>Shipped table</t>
+        </is>
+      </c>
+      <c r="C166" s="3" t="inlineStr">
+        <is>
+          <t>Phase 7 (TikTok 3/4): tiktok_ads table (10 rows)</t>
+        </is>
+      </c>
+      <c r="D166" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-13 14:35 PDT</t>
+        </is>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" s="2" t="inlineStr">
+        <is>
+          <t>generator/build_tiktok_reports_daily.py</t>
+        </is>
+      </c>
+      <c r="B167" s="2" t="inlineStr">
+        <is>
+          <t>Code</t>
+        </is>
+      </c>
+      <c r="C167" s="3" t="inlineStr">
+        <is>
+          <t>Phase 7 (TikTok 4/4): builds tiktok_reports_daily (spend/impressions/video_views, TikTok's always-video ad format) -- completes TikTok (6 of 6 platforms) AND all 47 tables</t>
+        </is>
+      </c>
+      <c r="D167" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-13 14:35 PDT</t>
+        </is>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" s="2" t="inlineStr">
+        <is>
+          <t>generator/validate_tiktok_reports_daily.py</t>
+        </is>
+      </c>
+      <c r="B168" s="2" t="inlineStr">
+        <is>
+          <t>Code</t>
+        </is>
+      </c>
+      <c r="C168" s="3" t="inlineStr">
+        <is>
+          <t>Phase 7: 5-layer validation for tiktok_reports_daily, incl. weekly-spend-vs-web_sessions correlation check</t>
+        </is>
+      </c>
+      <c r="D168" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-13 14:36 PDT</t>
+        </is>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" s="2" t="inlineStr">
+        <is>
+          <t>data/tiktok_reports_daily.csv</t>
+        </is>
+      </c>
+      <c r="B169" s="2" t="inlineStr">
+        <is>
+          <t>Shipped table</t>
+        </is>
+      </c>
+      <c r="C169" s="3" t="inlineStr">
+        <is>
+          <t>Phase 7 (TikTok 4/4): tiktok_reports_daily table (7,416 rows) -- completes TikTok, Phase 7, and the full 47-table dataset</t>
+        </is>
+      </c>
+      <c r="D169" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-13 14:35 PDT</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Cross-dataset alignment audit (7 checks) + fix merch_to_sub_trigger midnight-send bug
Adds generator/audit_cross_dataset_alignment.py, a post-completion audit
checking aggregate signals across all 47 tables against the shared
seasonality calendar/channel-mix schedule (correlation/growth/volatility
based, distinct from the per-table validators).

6 of 7 checks passed clean. Check 6 (day-of-week/hour-of-day) caught a
real bug: all 38 merch_to_sub_trigger Braze email sends landed at exactly
midnight because that trigger type never called the randomized
business-hours send-time helper every other trigger type uses. Fixed in
build_braze_email_events.py and rebuilt data/braze_email_events.csv
(re-validated 13/13). Checks 3 and 5 surfaced genuine, documented
non-bug characteristics (asymmetric BFCM promo coverage across years;
renewal invoice volatility not lower than fresh-start volatility).

Full write-up in docs/cross_dataset_alignment_audit.md. Manifest and
changelog updated to match.
</commit_message>
<xml_diff>
--- a/File_Manifest.xlsx
+++ b/File_Manifest.xlsx
@@ -435,7 +435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D169"/>
+  <dimension ref="A1:D171"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="48" customWidth="1" min="1" max="1"/>
@@ -506,7 +506,7 @@
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>2026-08-13 12:49 PDT</t>
+          <t>2026-08-13 15:13 PDT</t>
         </is>
       </c>
     </row>
@@ -638,7 +638,7 @@
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>2026-08-13 14:38 PDT</t>
+          <t>2026-08-13 15:15 PDT</t>
         </is>
       </c>
     </row>
@@ -748,7 +748,7 @@
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>2026-08-13 14:38 PDT</t>
+          <t>2026-08-13 15:15 PDT</t>
         </is>
       </c>
     </row>
@@ -2508,7 +2508,7 @@
       </c>
       <c r="D94" s="2" t="inlineStr">
         <is>
-          <t>2026-08-13 07:55 PDT</t>
+          <t>2026-08-13 15:11 PDT</t>
         </is>
       </c>
     </row>
@@ -2547,12 +2547,12 @@
       </c>
       <c r="C96" s="3" t="inlineStr">
         <is>
-          <t>Phase 6: braze_email_events table (26,328 rows, 18,187 sends)</t>
+          <t>Phase 6: braze_email_events table (26,335 rows, 18,187 sends) -- updated 2026-08-13 by the cross-dataset audit's Check 6 fix (merch_to_sub_trigger send time-of-day)</t>
         </is>
       </c>
       <c r="D96" s="2" t="inlineStr">
         <is>
-          <t>2026-08-13 07:57 PDT</t>
+          <t>2026-08-13 15:11 PDT</t>
         </is>
       </c>
     </row>
@@ -4159,6 +4159,50 @@
       <c r="D169" s="2" t="inlineStr">
         <is>
           <t>2026-08-13 14:35 PDT</t>
+        </is>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" s="2" t="inlineStr">
+        <is>
+          <t>generator/audit_cross_dataset_alignment.py</t>
+        </is>
+      </c>
+      <c r="B170" s="2" t="inlineStr">
+        <is>
+          <t>Code</t>
+        </is>
+      </c>
+      <c r="C170" s="3" t="inlineStr">
+        <is>
+          <t>Post-completion cross-dataset alignment audit -- NOT a shipped-table script. 7 checks: aggregate spend vs. demand, channel mix vs. schedule, calendar-event alignment, long-run growth trend, renewal/lag structure, day-of-week/hour-of-day, timezone/precision sweep. Found and fixed a real bug (Check 6 -- merch_to_sub_trigger Braze sends all landing at exactly midnight); Checks 3 and 5 surfaced genuine, documented (non-bug) characteristics.</t>
+        </is>
+      </c>
+      <c r="D170" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-13 15:12 PDT</t>
+        </is>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" s="2" t="inlineStr">
+        <is>
+          <t>docs/cross_dataset_alignment_audit.md</t>
+        </is>
+      </c>
+      <c r="B171" s="2" t="inlineStr">
+        <is>
+          <t>Docs</t>
+        </is>
+      </c>
+      <c r="C171" s="3" t="inlineStr">
+        <is>
+          <t>Write-up of the 7-check cross-dataset alignment audit's results, including the merch_to_sub_trigger bug fix and the two documented (non-bug) findings from Checks 3 and 5</t>
+        </is>
+      </c>
+      <c r="D171" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-13 15:14 PDT</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add MotherDuck loader script for warehouse migration stage
New warehouse/load_to_motherduck.py loads all 47 CSVs into a free
MotherDuck database, one table per CSV, with per-table row-count
verification. Designed to run on the user's own machine -- confirmed
the Cowork cloud sandbox's network allowlist blocks both pypi.org and
motherduck.com directly, so this can't be executed in-session.

Manifest and changelog updated to match.
</commit_message>
<xml_diff>
--- a/File_Manifest.xlsx
+++ b/File_Manifest.xlsx
@@ -435,7 +435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D171"/>
+  <dimension ref="A1:D172"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="48" customWidth="1" min="1" max="1"/>
@@ -638,7 +638,7 @@
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>2026-08-13 15:15 PDT</t>
+          <t>2026-08-13 15:37 PDT</t>
         </is>
       </c>
     </row>
@@ -748,7 +748,7 @@
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>2026-08-13 15:15 PDT</t>
+          <t>2026-08-13 15:37 PDT</t>
         </is>
       </c>
     </row>
@@ -4203,6 +4203,28 @@
       <c r="D171" s="2" t="inlineStr">
         <is>
           <t>2026-08-13 15:14 PDT</t>
+        </is>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" s="2" t="inlineStr">
+        <is>
+          <t>warehouse/load_to_motherduck.py</t>
+        </is>
+      </c>
+      <c r="B172" s="2" t="inlineStr">
+        <is>
+          <t>Code</t>
+        </is>
+      </c>
+      <c r="C172" s="3" t="inlineStr">
+        <is>
+          <t>Post-dataset-completion tooling -- loads all 47 CSVs into a free MotherDuck (hosted DuckDB) database, one table per CSV, with a row-count verification per table. Run on the user's own machine, not inside the Cowork cloud sandbox (MotherDuck needs outbound internet the sandbox doesn't have).</t>
+        </is>
+      </c>
+      <c r="D172" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-13 15:37 PDT</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Document MotherDuck token handling decision in changelog/manifest
Records that the user's token was deliberately kept out of git/iCloud
sync (see prior commit for the .gitignore + loader script changes) --
no secret values in this commit, just documentation of the choice.
</commit_message>
<xml_diff>
--- a/File_Manifest.xlsx
+++ b/File_Manifest.xlsx
@@ -506,7 +506,7 @@
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>2026-08-13 15:13 PDT</t>
+          <t>2026-08-13 15:37 PDT</t>
         </is>
       </c>
     </row>
@@ -638,7 +638,7 @@
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>2026-08-13 15:37 PDT</t>
+          <t>2026-08-13 15:45 PDT</t>
         </is>
       </c>
     </row>
@@ -726,7 +726,7 @@
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>2026-07-29 20:06 PDT</t>
+          <t>2026-08-13 15:44 PDT</t>
         </is>
       </c>
     </row>
@@ -748,7 +748,7 @@
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>2026-08-13 15:37 PDT</t>
+          <t>2026-08-13 15:45 PDT</t>
         </is>
       </c>
     </row>
@@ -4219,12 +4219,12 @@
       </c>
       <c r="C172" s="3" t="inlineStr">
         <is>
-          <t>Post-dataset-completion tooling -- loads all 47 CSVs into a free MotherDuck (hosted DuckDB) database, one table per CSV, with a row-count verification per table. Run on the user's own machine, not inside the Cowork cloud sandbox (MotherDuck needs outbound internet the sandbox doesn't have).</t>
+          <t>Post-dataset-completion tooling -- loads all 47 CSVs into a free MotherDuck (hosted DuckDB) database, one table per CSV, with a row-count verification per table. Run on the user's own machine, not inside the Cowork cloud sandbox (MotherDuck needs outbound internet the sandbox doesn't have). Reads its motherduck_token from either a shell env var or an optional warehouse/.env file (gitignored -- NOT tracked or synced by this manifest, since it holds a live credential).</t>
         </is>
       </c>
       <c r="D172" s="2" t="inlineStr">
         <is>
-          <t>2026-08-13 15:37 PDT</t>
+          <t>2026-08-13 15:45 PDT</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Fix load_to_motherduck.py: create the database before attaching to it
md:<name> attaches to an existing MotherDuck database rather than
creating one, so a first-ever run against a brand new database name
failed. Now connects bare, runs CREATE DATABASE IF NOT EXISTS + USE,
then proceeds with the per-CSV table loads as before.
</commit_message>
<xml_diff>
--- a/File_Manifest.xlsx
+++ b/File_Manifest.xlsx
@@ -506,7 +506,7 @@
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>2026-08-13 15:37 PDT</t>
+          <t>2026-08-13 15:56 PDT</t>
         </is>
       </c>
     </row>
@@ -748,7 +748,7 @@
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>2026-08-13 15:45 PDT</t>
+          <t>2026-08-13 15:56 PDT</t>
         </is>
       </c>
     </row>
@@ -4224,7 +4224,7 @@
       </c>
       <c r="D172" s="2" t="inlineStr">
         <is>
-          <t>2026-08-13 15:45 PDT</t>
+          <t>2026-08-13 15:56 PDT</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add first analysis queries + confirm MotherDuck load succeeded
6 starter SQL queries (paid media spend, attributed revenue by paid/
owned channel, active subscribers, non-subscription revenue, churn
rate, top products by year) against the kinetic MotherDuck database.
Logic validated against source CSVs in pandas since this sandbox can't
reach motherduck.com directly to run the SQL itself.

Also records the user's successful first end-to-end load (47/47 tables,
exact row-count match) confirming the earlier database-creation fix.
</commit_message>
<xml_diff>
--- a/File_Manifest.xlsx
+++ b/File_Manifest.xlsx
@@ -435,7 +435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D172"/>
+  <dimension ref="A1:D173"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="48" customWidth="1" min="1" max="1"/>
@@ -506,7 +506,7 @@
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>2026-08-13 15:56 PDT</t>
+          <t>2026-08-14 10:16 PDT</t>
         </is>
       </c>
     </row>
@@ -638,7 +638,7 @@
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>2026-08-13 15:45 PDT</t>
+          <t>2026-08-14 10:16 PDT</t>
         </is>
       </c>
     </row>
@@ -748,7 +748,7 @@
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>2026-08-13 15:56 PDT</t>
+          <t>2026-08-14 10:17 PDT</t>
         </is>
       </c>
     </row>
@@ -4219,12 +4219,34 @@
       </c>
       <c r="C172" s="3" t="inlineStr">
         <is>
-          <t>Post-dataset-completion tooling -- loads all 47 CSVs into a free MotherDuck (hosted DuckDB) database, one table per CSV, with a row-count verification per table. Run on the user's own machine, not inside the Cowork cloud sandbox (MotherDuck needs outbound internet the sandbox doesn't have). Reads its motherduck_token from either a shell env var or an optional warehouse/.env file (gitignored -- NOT tracked or synced by this manifest, since it holds a live credential).</t>
+          <t>Post-dataset-completion tooling -- loads all 47 CSVs into a free MotherDuck (hosted DuckDB) database, one table per CSV, with a row-count verification per table. Run on the user's own machine, not inside the Cowork cloud sandbox (MotherDuck needs outbound internet the sandbox doesn't have). Reads its motherduck_token from either a shell env var or an optional warehouse/.env file (gitignored -- NOT tracked or synced by this manifest, since it holds a live credential). Confirmed working end-to-end against the user's own MotherDuck account (47/47 tables, exact row-count match).</t>
         </is>
       </c>
       <c r="D172" s="2" t="inlineStr">
         <is>
           <t>2026-08-13 15:56 PDT</t>
+        </is>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" s="2" t="inlineStr">
+        <is>
+          <t>warehouse/analysis_queries.sql</t>
+        </is>
+      </c>
+      <c r="B173" s="2" t="inlineStr">
+        <is>
+          <t>Code</t>
+        </is>
+      </c>
+      <c r="C173" s="3" t="inlineStr">
+        <is>
+          <t>6 starter SQL queries against the kinetic MotherDuck database: monthly paid media spend by partner, directly attributed revenue by paid/owned channel, active subscribers by month, non-subscription revenue by month, monthly churn rate, top 5 grossing products per year. Heavily commented to explain modeling choices (e.g. the paid/owned attribution methodology split between storefront orders and subscription invoices).</t>
+        </is>
+      </c>
+      <c r="D173" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-14 10:16 PDT</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add first MotherDuck query visualization (paid media spend by partner)
Interactive HTML chart built from the user's actual Query 1 output,
following the dataviz skill's full procedure (form, validated
categorical palette, hover/crosshair, dark mode, table view fallback).
Rendered headlessly and screenshotted before delivery.
</commit_message>
<xml_diff>
--- a/File_Manifest.xlsx
+++ b/File_Manifest.xlsx
@@ -435,7 +435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D173"/>
+  <dimension ref="A1:D174"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="48" customWidth="1" min="1" max="1"/>
@@ -638,7 +638,7 @@
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>2026-08-14 10:16 PDT</t>
+          <t>2026-08-14 10:56 PDT</t>
         </is>
       </c>
     </row>
@@ -748,7 +748,7 @@
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>2026-08-14 10:17 PDT</t>
+          <t>2026-08-14 10:56 PDT</t>
         </is>
       </c>
     </row>
@@ -4247,6 +4247,28 @@
       <c r="D173" s="2" t="inlineStr">
         <is>
           <t>2026-08-14 10:16 PDT</t>
+        </is>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" s="2" t="inlineStr">
+        <is>
+          <t>warehouse/query1_paid_media_spend.html</t>
+        </is>
+      </c>
+      <c r="B174" s="2" t="inlineStr">
+        <is>
+          <t>Deliverable</t>
+        </is>
+      </c>
+      <c r="C174" s="3" t="inlineStr">
+        <is>
+          <t>One-off interactive chart visualizing Query 1's actual output (pasted by the user from their own MotherDuck run): monthly paid media spend by partner, Aug 2023-Jul 2026. Multi-line chart with hover tooltip, legend isolate-toggle, dark mode, and a table view -- built per the dataviz skill (validated categorical palette, accessible contrast handling).</t>
+        </is>
+      </c>
+      <c r="D174" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-14 10:55 PDT</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Log MotherDuck Dive dashboard: covers all 6 analysis queries live
</commit_message>
<xml_diff>
--- a/File_Manifest.xlsx
+++ b/File_Manifest.xlsx
@@ -435,7 +435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D174"/>
+  <dimension ref="A1:D175"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="48" customWidth="1" min="1" max="1"/>
@@ -506,7 +506,7 @@
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>2026-08-14 10:16 PDT</t>
+          <t>2026-08-14 13:42 PDT</t>
         </is>
       </c>
     </row>
@@ -638,7 +638,7 @@
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>2026-08-14 10:56 PDT</t>
+          <t>2026-08-14 13:42 PDT</t>
         </is>
       </c>
     </row>
@@ -748,7 +748,7 @@
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>2026-08-14 10:56 PDT</t>
+          <t>2026-08-14 13:42 PDT</t>
         </is>
       </c>
     </row>
@@ -4269,6 +4269,28 @@
       <c r="D174" s="2" t="inlineStr">
         <is>
           <t>2026-08-14 10:55 PDT</t>
+        </is>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175" s="2" t="inlineStr">
+        <is>
+          <t>warehouse/kinetic_dive.tsx</t>
+        </is>
+      </c>
+      <c r="B175" s="2" t="inlineStr">
+        <is>
+          <t>Deliverable</t>
+        </is>
+      </c>
+      <c r="C175" s="3" t="inlineStr">
+        <is>
+          <t>Source for the 'Kinetic -- Marketing &amp; Revenue Overview' MotherDuck Dive -- a live, hosted interactive dashboard (React/Recharts) covering all 6 requested queries (spend by partner, attributed revenue by channel, active subscribers, non-subscription revenue, churn rate, top products by year) plus a KPI row. Re-runs the real SQL against the live kinetic database on every open, unlike the earlier static HTML chart. Saved to MotherDuck via the MCP tools; this file is the local source-of-truth copy for sync/history. Live at https://app.motherduck.com/dives/kinetic-marketing-revenue-overview-58909b4e-d301-4794-bb59-ce46f9dc73a6 (dive_id 58909b4e-d301-4794-bb59-ce46f9dc73a6).</t>
+        </is>
+      </c>
+      <c r="D175" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-14 13:42 PDT</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add 8 persona-specific user stories (CEO/CMO/CFO/PMM) to the MotherDuck Dive, v2
</commit_message>
<xml_diff>
--- a/File_Manifest.xlsx
+++ b/File_Manifest.xlsx
@@ -506,7 +506,7 @@
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>2026-08-14 13:42 PDT</t>
+          <t>2026-08-14 14:17 PDT</t>
         </is>
       </c>
     </row>
@@ -638,7 +638,7 @@
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>2026-08-14 13:42 PDT</t>
+          <t>2026-08-14 14:16 PDT</t>
         </is>
       </c>
     </row>
@@ -748,7 +748,7 @@
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>2026-08-14 13:42 PDT</t>
+          <t>2026-08-14 14:17 PDT</t>
         </is>
       </c>
     </row>
@@ -4285,12 +4285,12 @@
       </c>
       <c r="C175" s="3" t="inlineStr">
         <is>
-          <t>Source for the 'Kinetic -- Marketing &amp; Revenue Overview' MotherDuck Dive -- a live, hosted interactive dashboard (React/Recharts) covering all 6 requested queries (spend by partner, attributed revenue by channel, active subscribers, non-subscription revenue, churn rate, top products by year) plus a KPI row. Re-runs the real SQL against the live kinetic database on every open, unlike the earlier static HTML chart. Saved to MotherDuck via the MCP tools; this file is the local source-of-truth copy for sync/history. Live at https://app.motherduck.com/dives/kinetic-marketing-revenue-overview-58909b4e-d301-4794-bb59-ce46f9dc73a6 (dive_id 58909b4e-d301-4794-bb59-ce46f9dc73a6).</t>
+          <t>Source for the 'Kinetic -- Marketing &amp; Revenue Overview' MotherDuck Dive -- a live, hosted interactive dashboard (React/Recharts), now organized as 5 tabs. Overview tab: the original 6 starter queries + KPI row. CEO tab: revenue growth/net-new-vs-churned subscribers/CAC payback, revenue mix (subscription vs. course vs. merch). CMO tab: acquisition funnel by channel (sessions -&gt; trial starts -&gt; conversions), retention/app engagement by acquisition channel. CFO tab: CAC and LTV:CAC by acquisition cohort, discount code cost + failed-payment recovery rate + a documented net-margin proxy (no COGS data exists for a true gross margin). Performance Marketing tab: campaign-level spend and platform-self-reported efficiency across all 38 real campaigns (sorted worst-CAC-first), CTR/CVR by platform and ad format. Each new section documents its modeling limits explicitly (e.g. platform-reported vs. site-attributed conversions have no shared join key in this dataset). Re-runs live SQL against the kinetic database on every open. Saved to MotherDuck via the MCP tools; this file is the local source-of-truth copy for sync/history. Live at https://app.motherduck.com/dives/kinetic-marketing-revenue-overview-58909b4e-d301-4794-bb59-ce46f9dc73a6 (dive_id 58909b4e-d301-4794-bb59-ce46f9dc73a6, version 2).</t>
         </is>
       </c>
       <c r="D175" s="2" t="inlineStr">
         <is>
-          <t>2026-08-14 13:42 PDT</t>
+          <t>2026-08-14 14:13 PDT</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
dbt Phase 3: storefront revenue staging + mart
- Staging models for orders, order_line_items, payments, refunds,
  discount_codes.
- New intermediate model int_orders_refunded (succeeded-refund totals per
  order only).
- New mart mart_storefront_revenue_monthly: gross/net revenue, AOV,
  guest-checkout share, discount-usage share, refund rate by month.
  Validated against a hand-run equivalent query on the live kinetic
  database before writing any dbt SQL.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014EdkVLDs4dt6TCgduxMMyp
</commit_message>
<xml_diff>
--- a/File_Manifest.xlsx
+++ b/File_Manifest.xlsx
@@ -435,7 +435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D191"/>
+  <dimension ref="A1:D199"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="48" customWidth="1" min="1" max="1"/>
@@ -638,7 +638,7 @@
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28 14:49 PDT</t>
+          <t>2026-09-28 14:53 PDT</t>
         </is>
       </c>
     </row>
@@ -748,7 +748,7 @@
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28 14:49 PDT</t>
+          <t>2026-09-28 14:53 PDT</t>
         </is>
       </c>
     </row>
@@ -4400,7 +4400,7 @@
       </c>
       <c r="D180" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28 14:48 PDT</t>
+          <t>2026-09-28 14:53 PDT</t>
         </is>
       </c>
     </row>
@@ -4554,7 +4554,7 @@
       </c>
       <c r="D187" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28 14:48 PDT</t>
+          <t>2026-09-28 14:53 PDT</t>
         </is>
       </c>
     </row>
@@ -4598,7 +4598,7 @@
       </c>
       <c r="D189" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28 14:48 PDT</t>
+          <t>2026-09-28 14:53 PDT</t>
         </is>
       </c>
     </row>
@@ -4642,7 +4642,183 @@
       </c>
       <c r="D191" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28 14:48 PDT</t>
+          <t>2026-09-28 14:53 PDT</t>
+        </is>
+      </c>
+    </row>
+    <row r="192">
+      <c r="A192" s="2" t="inlineStr">
+        <is>
+          <t>dbt/README.md</t>
+        </is>
+      </c>
+      <c r="B192" s="2" t="inlineStr">
+        <is>
+          <t>Docs</t>
+        </is>
+      </c>
+      <c r="C192" s="3" t="inlineStr">
+        <is>
+          <t>Updated: what's built so far now includes the Phase 3 storefront staging models + mart_storefront_revenue_monthly</t>
+        </is>
+      </c>
+      <c r="D192" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-28 14:53 PDT</t>
+        </is>
+      </c>
+    </row>
+    <row r="193">
+      <c r="A193" s="2" t="inlineStr">
+        <is>
+          <t>dbt/models/staging/kinetic/stg_kinetic__orders.sql</t>
+        </is>
+      </c>
+      <c r="B193" s="2" t="inlineStr">
+        <is>
+          <t>Code</t>
+        </is>
+      </c>
+      <c r="C193" s="3" t="inlineStr">
+        <is>
+          <t>Staging model: 1:1 pass-through of orders, plus is_guest_order/has_discount convenience booleans</t>
+        </is>
+      </c>
+      <c r="D193" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-28 14:53 PDT</t>
+        </is>
+      </c>
+    </row>
+    <row r="194">
+      <c r="A194" s="2" t="inlineStr">
+        <is>
+          <t>dbt/models/staging/kinetic/stg_kinetic__order_line_items.sql</t>
+        </is>
+      </c>
+      <c r="B194" s="2" t="inlineStr">
+        <is>
+          <t>Code</t>
+        </is>
+      </c>
+      <c r="C194" s="3" t="inlineStr">
+        <is>
+          <t>Staging model: 1:1 pass-through of order_line_items</t>
+        </is>
+      </c>
+      <c r="D194" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-28 14:53 PDT</t>
+        </is>
+      </c>
+    </row>
+    <row r="195">
+      <c r="A195" s="2" t="inlineStr">
+        <is>
+          <t>dbt/models/staging/kinetic/stg_kinetic__payments.sql</t>
+        </is>
+      </c>
+      <c r="B195" s="2" t="inlineStr">
+        <is>
+          <t>Code</t>
+        </is>
+      </c>
+      <c r="C195" s="3" t="inlineStr">
+        <is>
+          <t>Staging model: 1:1 pass-through of payments</t>
+        </is>
+      </c>
+      <c r="D195" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-28 14:53 PDT</t>
+        </is>
+      </c>
+    </row>
+    <row r="196">
+      <c r="A196" s="2" t="inlineStr">
+        <is>
+          <t>dbt/models/staging/kinetic/stg_kinetic__refunds.sql</t>
+        </is>
+      </c>
+      <c r="B196" s="2" t="inlineStr">
+        <is>
+          <t>Code</t>
+        </is>
+      </c>
+      <c r="C196" s="3" t="inlineStr">
+        <is>
+          <t>Staging model: 1:1 pass-through of refunds</t>
+        </is>
+      </c>
+      <c r="D196" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-28 14:53 PDT</t>
+        </is>
+      </c>
+    </row>
+    <row r="197">
+      <c r="A197" s="2" t="inlineStr">
+        <is>
+          <t>dbt/models/staging/kinetic/stg_kinetic__discount_codes.sql</t>
+        </is>
+      </c>
+      <c r="B197" s="2" t="inlineStr">
+        <is>
+          <t>Code</t>
+        </is>
+      </c>
+      <c r="C197" s="3" t="inlineStr">
+        <is>
+          <t>Staging model: 1:1 pass-through of discount_codes</t>
+        </is>
+      </c>
+      <c r="D197" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-28 14:53 PDT</t>
+        </is>
+      </c>
+    </row>
+    <row r="198">
+      <c r="A198" s="2" t="inlineStr">
+        <is>
+          <t>dbt/models/intermediate/int_orders_refunded.sql</t>
+        </is>
+      </c>
+      <c r="B198" s="2" t="inlineStr">
+        <is>
+          <t>Code</t>
+        </is>
+      </c>
+      <c r="C198" s="3" t="inlineStr">
+        <is>
+          <t>Intermediate model: per-order total of succeeded refunds only (failed/pending refunds don't reduce reported revenue)</t>
+        </is>
+      </c>
+      <c r="D198" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-28 14:53 PDT</t>
+        </is>
+      </c>
+    </row>
+    <row r="199">
+      <c r="A199" s="2" t="inlineStr">
+        <is>
+          <t>dbt/models/marts/mart_storefront_revenue_monthly.sql</t>
+        </is>
+      </c>
+      <c r="B199" s="2" t="inlineStr">
+        <is>
+          <t>Code</t>
+        </is>
+      </c>
+      <c r="C199" s="3" t="inlineStr">
+        <is>
+          <t>Second canonical metric mart: non-subscription (course+merch) gross/net revenue, AOV, guest-checkout share, discount-usage share, refund rate by month -- validated against a hand-run equivalent query on the live database (2026-07: 246 orders, $13,843.71 gross revenue, $56.28 AOV)</t>
+        </is>
+      </c>
+      <c r="D199" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-28 14:53 PDT</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
dbt Phase 2 sub-batch 1: Customer 360 staging models
Staging models + tests for customer_addresses, devices, identity_map,
segments, customer_segment_membership, subscription_events (16 of 47 raw
tables now staged). Every PK/FK test was hand-verified against the live
kinetic database first, since dbt test can't run yet.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014EdkVLDs4dt6TCgduxMMyp
</commit_message>
<xml_diff>
--- a/File_Manifest.xlsx
+++ b/File_Manifest.xlsx
@@ -435,7 +435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D199"/>
+  <dimension ref="A1:D206"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="48" customWidth="1" min="1" max="1"/>
@@ -506,7 +506,7 @@
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28 14:47 PDT</t>
+          <t>2026-09-29 10:27 PDT</t>
         </is>
       </c>
     </row>
@@ -638,7 +638,7 @@
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28 14:53 PDT</t>
+          <t>2026-09-29 10:27 PDT</t>
         </is>
       </c>
     </row>
@@ -748,7 +748,7 @@
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28 14:53 PDT</t>
+          <t>2026-09-29 10:27 PDT</t>
         </is>
       </c>
     </row>
@@ -4400,7 +4400,7 @@
       </c>
       <c r="D180" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28 14:53 PDT</t>
+          <t>2026-09-29 10:27 PDT</t>
         </is>
       </c>
     </row>
@@ -4554,7 +4554,7 @@
       </c>
       <c r="D187" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28 14:53 PDT</t>
+          <t>2026-09-29 10:26 PDT</t>
         </is>
       </c>
     </row>
@@ -4664,7 +4664,7 @@
       </c>
       <c r="D192" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28 14:53 PDT</t>
+          <t>2026-09-29 10:27 PDT</t>
         </is>
       </c>
     </row>
@@ -4819,6 +4819,160 @@
       <c r="D199" s="2" t="inlineStr">
         <is>
           <t>2026-09-28 14:53 PDT</t>
+        </is>
+      </c>
+    </row>
+    <row r="200">
+      <c r="A200" s="2" t="inlineStr">
+        <is>
+          <t>dbt/models/staging/kinetic/stg_kinetic__customer_addresses.sql</t>
+        </is>
+      </c>
+      <c r="B200" s="2" t="inlineStr">
+        <is>
+          <t>Code</t>
+        </is>
+      </c>
+      <c r="C200" s="3" t="inlineStr">
+        <is>
+          <t>Phase 2 staging (Customer 360): 1:1 pass-through of customer_addresses</t>
+        </is>
+      </c>
+      <c r="D200" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-29 10:26 PDT</t>
+        </is>
+      </c>
+    </row>
+    <row r="201">
+      <c r="A201" s="2" t="inlineStr">
+        <is>
+          <t>dbt/models/staging/kinetic/stg_kinetic__devices.sql</t>
+        </is>
+      </c>
+      <c r="B201" s="2" t="inlineStr">
+        <is>
+          <t>Code</t>
+        </is>
+      </c>
+      <c r="C201" s="3" t="inlineStr">
+        <is>
+          <t>Phase 2 staging (Customer 360): 1:1 pass-through of devices, plus is_anonymous_device flag (customer_id null for ~94% of devices by design)</t>
+        </is>
+      </c>
+      <c r="D201" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-29 10:26 PDT</t>
+        </is>
+      </c>
+    </row>
+    <row r="202">
+      <c r="A202" s="2" t="inlineStr">
+        <is>
+          <t>dbt/models/staging/kinetic/stg_kinetic__identity_map.sql</t>
+        </is>
+      </c>
+      <c r="B202" s="2" t="inlineStr">
+        <is>
+          <t>Code</t>
+        </is>
+      </c>
+      <c r="C202" s="3" t="inlineStr">
+        <is>
+          <t>Phase 2 staging (Customer 360): 1:1 pass-through of identity_map</t>
+        </is>
+      </c>
+      <c r="D202" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-29 10:26 PDT</t>
+        </is>
+      </c>
+    </row>
+    <row r="203">
+      <c r="A203" s="2" t="inlineStr">
+        <is>
+          <t>dbt/models/staging/kinetic/stg_kinetic__segments.sql</t>
+        </is>
+      </c>
+      <c r="B203" s="2" t="inlineStr">
+        <is>
+          <t>Code</t>
+        </is>
+      </c>
+      <c r="C203" s="3" t="inlineStr">
+        <is>
+          <t>Phase 2 staging (Customer 360): 1:1 pass-through of segments</t>
+        </is>
+      </c>
+      <c r="D203" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-29 10:26 PDT</t>
+        </is>
+      </c>
+    </row>
+    <row r="204">
+      <c r="A204" s="2" t="inlineStr">
+        <is>
+          <t>dbt/models/staging/kinetic/stg_kinetic__customer_segment_membership.sql</t>
+        </is>
+      </c>
+      <c r="B204" s="2" t="inlineStr">
+        <is>
+          <t>Code</t>
+        </is>
+      </c>
+      <c r="C204" s="3" t="inlineStr">
+        <is>
+          <t>Phase 2 staging (Customer 360): 1:1 pass-through of customer_segment_membership, plus is_current_member flag</t>
+        </is>
+      </c>
+      <c r="D204" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-29 10:26 PDT</t>
+        </is>
+      </c>
+    </row>
+    <row r="205">
+      <c r="A205" s="2" t="inlineStr">
+        <is>
+          <t>dbt/models/staging/kinetic/stg_kinetic__subscription_events.sql</t>
+        </is>
+      </c>
+      <c r="B205" s="2" t="inlineStr">
+        <is>
+          <t>Code</t>
+        </is>
+      </c>
+      <c r="C205" s="3" t="inlineStr">
+        <is>
+          <t>Phase 2 staging (Customer 360): 1:1 pass-through of subscription_events; old_plan/new_plan renamed to old_plan_id/new_plan_id</t>
+        </is>
+      </c>
+      <c r="D205" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-29 10:26 PDT</t>
+        </is>
+      </c>
+    </row>
+    <row r="206">
+      <c r="A206" s="2" t="inlineStr">
+        <is>
+          <t>dbt/models/staging/kinetic/_kinetic__staging.yml</t>
+        </is>
+      </c>
+      <c r="B206" s="2" t="inlineStr">
+        <is>
+          <t>Code</t>
+        </is>
+      </c>
+      <c r="C206" s="3" t="inlineStr">
+        <is>
+          <t>Updated: tests for the 6 Customer 360 staging models (PK not_null/unique, FK relationships) -- all hand-verified against live data first</t>
+        </is>
+      </c>
+      <c r="D206" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-29 10:26 PDT</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
dbt Phase 2 sub-batch 2: web/app engagement staging models
Staging models + tests for web_sessions, web_events, app_sessions,
app_events (20 of 47 raw tables now staged). Every PK/FK test was
hand-verified against the live kinetic database first.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014EdkVLDs4dt6TCgduxMMyp
</commit_message>
<xml_diff>
--- a/File_Manifest.xlsx
+++ b/File_Manifest.xlsx
@@ -435,7 +435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D206"/>
+  <dimension ref="A1:D211"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="48" customWidth="1" min="1" max="1"/>
@@ -506,7 +506,7 @@
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 10:27 PDT</t>
+          <t>2026-09-29 12:58 PDT</t>
         </is>
       </c>
     </row>
@@ -638,7 +638,7 @@
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 10:27 PDT</t>
+          <t>2026-09-29 12:58 PDT</t>
         </is>
       </c>
     </row>
@@ -748,7 +748,7 @@
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 10:27 PDT</t>
+          <t>2026-09-29 12:58 PDT</t>
         </is>
       </c>
     </row>
@@ -4400,7 +4400,7 @@
       </c>
       <c r="D180" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 10:27 PDT</t>
+          <t>2026-09-29 12:58 PDT</t>
         </is>
       </c>
     </row>
@@ -4554,7 +4554,7 @@
       </c>
       <c r="D187" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 10:26 PDT</t>
+          <t>2026-09-29 12:58 PDT</t>
         </is>
       </c>
     </row>
@@ -4664,7 +4664,7 @@
       </c>
       <c r="D192" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 10:27 PDT</t>
+          <t>2026-09-29 12:58 PDT</t>
         </is>
       </c>
     </row>
@@ -4972,7 +4972,117 @@
       </c>
       <c r="D206" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 10:26 PDT</t>
+          <t>2026-09-29 12:58 PDT</t>
+        </is>
+      </c>
+    </row>
+    <row r="207">
+      <c r="A207" s="2" t="inlineStr">
+        <is>
+          <t>dbt/models/staging/kinetic/stg_kinetic__web_sessions.sql</t>
+        </is>
+      </c>
+      <c r="B207" s="2" t="inlineStr">
+        <is>
+          <t>Code</t>
+        </is>
+      </c>
+      <c r="C207" s="3" t="inlineStr">
+        <is>
+          <t>Phase 2 staging (web/app engagement): 1:1 pass-through of web_sessions, plus is_known_customer flag (customer_id null for ~79% of sessions by design)</t>
+        </is>
+      </c>
+      <c r="D207" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-29 12:58 PDT</t>
+        </is>
+      </c>
+    </row>
+    <row r="208">
+      <c r="A208" s="2" t="inlineStr">
+        <is>
+          <t>dbt/models/staging/kinetic/stg_kinetic__web_events.sql</t>
+        </is>
+      </c>
+      <c r="B208" s="2" t="inlineStr">
+        <is>
+          <t>Code</t>
+        </is>
+      </c>
+      <c r="C208" s="3" t="inlineStr">
+        <is>
+          <t>Phase 2 staging (web/app engagement): 1:1 pass-through of web_events</t>
+        </is>
+      </c>
+      <c r="D208" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-29 12:58 PDT</t>
+        </is>
+      </c>
+    </row>
+    <row r="209">
+      <c r="A209" s="2" t="inlineStr">
+        <is>
+          <t>dbt/models/staging/kinetic/stg_kinetic__app_sessions.sql</t>
+        </is>
+      </c>
+      <c r="B209" s="2" t="inlineStr">
+        <is>
+          <t>Code</t>
+        </is>
+      </c>
+      <c r="C209" s="3" t="inlineStr">
+        <is>
+          <t>Phase 2 staging (web/app engagement): 1:1 pass-through of app_sessions</t>
+        </is>
+      </c>
+      <c r="D209" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-29 12:58 PDT</t>
+        </is>
+      </c>
+    </row>
+    <row r="210">
+      <c r="A210" s="2" t="inlineStr">
+        <is>
+          <t>dbt/models/staging/kinetic/stg_kinetic__app_events.sql</t>
+        </is>
+      </c>
+      <c r="B210" s="2" t="inlineStr">
+        <is>
+          <t>Code</t>
+        </is>
+      </c>
+      <c r="C210" s="3" t="inlineStr">
+        <is>
+          <t>Phase 2 staging (web/app engagement): 1:1 pass-through of app_events</t>
+        </is>
+      </c>
+      <c r="D210" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-29 12:58 PDT</t>
+        </is>
+      </c>
+    </row>
+    <row r="211">
+      <c r="A211" s="2" t="inlineStr">
+        <is>
+          <t>dbt/models/staging/kinetic/_kinetic__staging.yml</t>
+        </is>
+      </c>
+      <c r="B211" s="2" t="inlineStr">
+        <is>
+          <t>Code</t>
+        </is>
+      </c>
+      <c r="C211" s="3" t="inlineStr">
+        <is>
+          <t>Updated: tests for the 4 web/app engagement staging models -- all hand-verified against live data first</t>
+        </is>
+      </c>
+      <c r="D211" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-29 12:58 PDT</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
dbt Phase 2 sub-batch 3: email/push (Braze) staging models
Staging models + tests for the 4 Braze tables (24 of 47 raw tables now
staged). external_user_id renamed to customer_id; short event_name added
next to Braze's raw event_type. Every test hand-verified against the live
kinetic database first.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014EdkVLDs4dt6TCgduxMMyp
</commit_message>
<xml_diff>
--- a/File_Manifest.xlsx
+++ b/File_Manifest.xlsx
@@ -435,7 +435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D211"/>
+  <dimension ref="A1:D216"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="48" customWidth="1" min="1" max="1"/>
@@ -506,7 +506,7 @@
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 12:58 PDT</t>
+          <t>2026-09-29 13:00 PDT</t>
         </is>
       </c>
     </row>
@@ -638,7 +638,7 @@
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 12:58 PDT</t>
+          <t>2026-09-29 13:00 PDT</t>
         </is>
       </c>
     </row>
@@ -748,7 +748,7 @@
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 12:58 PDT</t>
+          <t>2026-09-29 13:00 PDT</t>
         </is>
       </c>
     </row>
@@ -4400,7 +4400,7 @@
       </c>
       <c r="D180" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 12:58 PDT</t>
+          <t>2026-09-29 13:00 PDT</t>
         </is>
       </c>
     </row>
@@ -4554,7 +4554,7 @@
       </c>
       <c r="D187" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 12:58 PDT</t>
+          <t>2026-09-29 12:59 PDT</t>
         </is>
       </c>
     </row>
@@ -4664,7 +4664,7 @@
       </c>
       <c r="D192" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 12:58 PDT</t>
+          <t>2026-09-29 13:00 PDT</t>
         </is>
       </c>
     </row>
@@ -4972,7 +4972,7 @@
       </c>
       <c r="D206" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 12:58 PDT</t>
+          <t>2026-09-29 12:59 PDT</t>
         </is>
       </c>
     </row>
@@ -5082,7 +5082,117 @@
       </c>
       <c r="D211" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 12:58 PDT</t>
+          <t>2026-09-29 12:59 PDT</t>
+        </is>
+      </c>
+    </row>
+    <row r="212">
+      <c r="A212" s="2" t="inlineStr">
+        <is>
+          <t>dbt/models/staging/kinetic/stg_kinetic__braze_email_campaigns.sql</t>
+        </is>
+      </c>
+      <c r="B212" s="2" t="inlineStr">
+        <is>
+          <t>Code</t>
+        </is>
+      </c>
+      <c r="C212" s="3" t="inlineStr">
+        <is>
+          <t>Phase 2 staging (email/push): 1:1 pass-through of braze_email_campaigns</t>
+        </is>
+      </c>
+      <c r="D212" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-29 12:59 PDT</t>
+        </is>
+      </c>
+    </row>
+    <row r="213">
+      <c r="A213" s="2" t="inlineStr">
+        <is>
+          <t>dbt/models/staging/kinetic/stg_kinetic__braze_push_campaigns.sql</t>
+        </is>
+      </c>
+      <c r="B213" s="2" t="inlineStr">
+        <is>
+          <t>Code</t>
+        </is>
+      </c>
+      <c r="C213" s="3" t="inlineStr">
+        <is>
+          <t>Phase 2 staging (email/push): 1:1 pass-through of braze_push_campaigns</t>
+        </is>
+      </c>
+      <c r="D213" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-29 12:59 PDT</t>
+        </is>
+      </c>
+    </row>
+    <row r="214">
+      <c r="A214" s="2" t="inlineStr">
+        <is>
+          <t>dbt/models/staging/kinetic/stg_kinetic__braze_email_events.sql</t>
+        </is>
+      </c>
+      <c r="B214" s="2" t="inlineStr">
+        <is>
+          <t>Code</t>
+        </is>
+      </c>
+      <c r="C214" s="3" t="inlineStr">
+        <is>
+          <t>Phase 2 staging (email/push): braze_email_events with external_user_id renamed to customer_id and a short event_name (send/open/click/bounce/unsubscribe) alongside Braze's raw event_type</t>
+        </is>
+      </c>
+      <c r="D214" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-29 12:59 PDT</t>
+        </is>
+      </c>
+    </row>
+    <row r="215">
+      <c r="A215" s="2" t="inlineStr">
+        <is>
+          <t>dbt/models/staging/kinetic/stg_kinetic__braze_push_events.sql</t>
+        </is>
+      </c>
+      <c r="B215" s="2" t="inlineStr">
+        <is>
+          <t>Code</t>
+        </is>
+      </c>
+      <c r="C215" s="3" t="inlineStr">
+        <is>
+          <t>Phase 2 staging (email/push): braze_push_events with external_user_id renamed to customer_id and a short event_name alongside Braze's raw event_type</t>
+        </is>
+      </c>
+      <c r="D215" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-29 12:59 PDT</t>
+        </is>
+      </c>
+    </row>
+    <row r="216">
+      <c r="A216" s="2" t="inlineStr">
+        <is>
+          <t>dbt/models/staging/kinetic/_kinetic__staging.yml</t>
+        </is>
+      </c>
+      <c r="B216" s="2" t="inlineStr">
+        <is>
+          <t>Code</t>
+        </is>
+      </c>
+      <c r="C216" s="3" t="inlineStr">
+        <is>
+          <t>Updated: tests for the 4 Braze staging models, incl. accepted_values on event_name -- all hand-verified against live data first</t>
+        </is>
+      </c>
+      <c r="D216" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-29 12:59 PDT</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
dbt Phase 2 sub-batch 4: Meta staging models
Staging models + tests for the 4 Meta tables (28 of 47 raw tables now
staged). Budgets converted from cents to dollars, units in column names,
ctr renamed ctr_fraction, combined keys for the two daily tables. Every
test hand-verified against the live kinetic database first.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014EdkVLDs4dt6TCgduxMMyp
</commit_message>
<xml_diff>
--- a/File_Manifest.xlsx
+++ b/File_Manifest.xlsx
@@ -435,7 +435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D216"/>
+  <dimension ref="A1:D221"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="48" customWidth="1" min="1" max="1"/>
@@ -506,7 +506,7 @@
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 13:00 PDT</t>
+          <t>2026-09-29 13:03 PDT</t>
         </is>
       </c>
     </row>
@@ -638,7 +638,7 @@
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 13:00 PDT</t>
+          <t>2026-09-29 13:03 PDT</t>
         </is>
       </c>
     </row>
@@ -748,7 +748,7 @@
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 13:00 PDT</t>
+          <t>2026-09-29 13:03 PDT</t>
         </is>
       </c>
     </row>
@@ -4400,7 +4400,7 @@
       </c>
       <c r="D180" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 13:00 PDT</t>
+          <t>2026-09-29 13:03 PDT</t>
         </is>
       </c>
     </row>
@@ -4554,7 +4554,7 @@
       </c>
       <c r="D187" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 12:59 PDT</t>
+          <t>2026-09-29 13:02 PDT</t>
         </is>
       </c>
     </row>
@@ -4664,7 +4664,7 @@
       </c>
       <c r="D192" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 13:00 PDT</t>
+          <t>2026-09-29 13:03 PDT</t>
         </is>
       </c>
     </row>
@@ -4972,7 +4972,7 @@
       </c>
       <c r="D206" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 12:59 PDT</t>
+          <t>2026-09-29 13:02 PDT</t>
         </is>
       </c>
     </row>
@@ -5082,7 +5082,7 @@
       </c>
       <c r="D211" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 12:59 PDT</t>
+          <t>2026-09-29 13:02 PDT</t>
         </is>
       </c>
     </row>
@@ -5192,7 +5192,117 @@
       </c>
       <c r="D216" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 12:59 PDT</t>
+          <t>2026-09-29 13:02 PDT</t>
+        </is>
+      </c>
+    </row>
+    <row r="217">
+      <c r="A217" s="2" t="inlineStr">
+        <is>
+          <t>dbt/models/staging/kinetic/stg_kinetic__meta_campaigns.sql</t>
+        </is>
+      </c>
+      <c r="B217" s="2" t="inlineStr">
+        <is>
+          <t>Code</t>
+        </is>
+      </c>
+      <c r="C217" s="3" t="inlineStr">
+        <is>
+          <t>Phase 2 staging (paid media: Meta): meta_campaigns with budgets in both raw cents and dollars (Meta API stores budgets in cents)</t>
+        </is>
+      </c>
+      <c r="D217" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-29 13:02 PDT</t>
+        </is>
+      </c>
+    </row>
+    <row r="218">
+      <c r="A218" s="2" t="inlineStr">
+        <is>
+          <t>dbt/models/staging/kinetic/stg_kinetic__meta_ads.sql</t>
+        </is>
+      </c>
+      <c r="B218" s="2" t="inlineStr">
+        <is>
+          <t>Code</t>
+        </is>
+      </c>
+      <c r="C218" s="3" t="inlineStr">
+        <is>
+          <t>Phase 2 staging (paid media: Meta): 1:1 pass-through of meta_ads</t>
+        </is>
+      </c>
+      <c r="D218" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-29 13:02 PDT</t>
+        </is>
+      </c>
+    </row>
+    <row r="219">
+      <c r="A219" s="2" t="inlineStr">
+        <is>
+          <t>dbt/models/staging/kinetic/stg_kinetic__meta_ad_insights_daily.sql</t>
+        </is>
+      </c>
+      <c r="B219" s="2" t="inlineStr">
+        <is>
+          <t>Code</t>
+        </is>
+      </c>
+      <c r="C219" s="3" t="inlineStr">
+        <is>
+          <t>Phase 2 staging (paid media: Meta): meta_ad_insights_daily with a combined ad_day_id key, unit-suffixed columns (spend_usd, cpm_usd, cpc_usd) and ctr renamed ctr_fraction (0.017 = 1.7%)</t>
+        </is>
+      </c>
+      <c r="D219" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-29 13:02 PDT</t>
+        </is>
+      </c>
+    </row>
+    <row r="220">
+      <c r="A220" s="2" t="inlineStr">
+        <is>
+          <t>dbt/models/staging/kinetic/stg_kinetic__meta_ad_actions_daily.sql</t>
+        </is>
+      </c>
+      <c r="B220" s="2" t="inlineStr">
+        <is>
+          <t>Code</t>
+        </is>
+      </c>
+      <c r="C220" s="3" t="inlineStr">
+        <is>
+          <t>Phase 2 staging (paid media: Meta): meta_ad_actions_daily with a combined ad_day_action_id key; value renamed action_count</t>
+        </is>
+      </c>
+      <c r="D220" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-29 13:02 PDT</t>
+        </is>
+      </c>
+    </row>
+    <row r="221">
+      <c r="A221" s="2" t="inlineStr">
+        <is>
+          <t>dbt/models/staging/kinetic/_kinetic__staging.yml</t>
+        </is>
+      </c>
+      <c r="B221" s="2" t="inlineStr">
+        <is>
+          <t>Code</t>
+        </is>
+      </c>
+      <c r="C221" s="3" t="inlineStr">
+        <is>
+          <t>Updated: tests for the 4 Meta staging models, incl. uniqueness of the combined daily keys -- all hand-verified against live data first</t>
+        </is>
+      </c>
+      <c r="D221" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-29 13:02 PDT</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
dbt Phase 2 sub-batch 5: Google Search staging models
Staging models + tests for the 4 Google Search tables (32 of 47 raw
tables now staged). customer_id renamed google_ads_account_id (it's the
ad account, not a Kinetic customer); micros converted to dollars; empty
text-typed columns cast back; keyword and ad-group tables documented as
the same spend at two levels of detail. Every test hand-verified against
the live kinetic database first.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014EdkVLDs4dt6TCgduxMMyp
</commit_message>
<xml_diff>
--- a/File_Manifest.xlsx
+++ b/File_Manifest.xlsx
@@ -435,7 +435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D221"/>
+  <dimension ref="A1:D226"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="48" customWidth="1" min="1" max="1"/>
@@ -506,7 +506,7 @@
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 13:03 PDT</t>
+          <t>2026-09-29 13:13 PDT</t>
         </is>
       </c>
     </row>
@@ -638,7 +638,7 @@
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 13:03 PDT</t>
+          <t>2026-09-29 13:13 PDT</t>
         </is>
       </c>
     </row>
@@ -748,7 +748,7 @@
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 13:03 PDT</t>
+          <t>2026-09-29 13:13 PDT</t>
         </is>
       </c>
     </row>
@@ -4400,7 +4400,7 @@
       </c>
       <c r="D180" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 13:03 PDT</t>
+          <t>2026-09-29 13:13 PDT</t>
         </is>
       </c>
     </row>
@@ -4554,7 +4554,7 @@
       </c>
       <c r="D187" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 13:02 PDT</t>
+          <t>2026-09-29 13:13 PDT</t>
         </is>
       </c>
     </row>
@@ -4664,7 +4664,7 @@
       </c>
       <c r="D192" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 13:03 PDT</t>
+          <t>2026-09-29 13:13 PDT</t>
         </is>
       </c>
     </row>
@@ -4972,7 +4972,7 @@
       </c>
       <c r="D206" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 13:02 PDT</t>
+          <t>2026-09-29 13:13 PDT</t>
         </is>
       </c>
     </row>
@@ -5082,7 +5082,7 @@
       </c>
       <c r="D211" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 13:02 PDT</t>
+          <t>2026-09-29 13:13 PDT</t>
         </is>
       </c>
     </row>
@@ -5192,7 +5192,7 @@
       </c>
       <c r="D216" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 13:02 PDT</t>
+          <t>2026-09-29 13:13 PDT</t>
         </is>
       </c>
     </row>
@@ -5302,7 +5302,117 @@
       </c>
       <c r="D221" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 13:02 PDT</t>
+          <t>2026-09-29 13:13 PDT</t>
+        </is>
+      </c>
+    </row>
+    <row r="222">
+      <c r="A222" s="2" t="inlineStr">
+        <is>
+          <t>dbt/models/staging/kinetic/stg_kinetic__google_search_campaigns.sql</t>
+        </is>
+      </c>
+      <c r="B222" s="2" t="inlineStr">
+        <is>
+          <t>Code</t>
+        </is>
+      </c>
+      <c r="C222" s="3" t="inlineStr">
+        <is>
+          <t>Phase 2 staging (paid media: Google Search): campaigns with the raw customer_id renamed google_ads_account_id (it's the Google Ads account number, not a Kinetic customer), daily budget in micros and dollars, end_date cast back to a date</t>
+        </is>
+      </c>
+      <c r="D222" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-29 13:13 PDT</t>
+        </is>
+      </c>
+    </row>
+    <row r="223">
+      <c r="A223" s="2" t="inlineStr">
+        <is>
+          <t>dbt/models/staging/kinetic/stg_kinetic__google_search_ad_groups.sql</t>
+        </is>
+      </c>
+      <c r="B223" s="2" t="inlineStr">
+        <is>
+          <t>Code</t>
+        </is>
+      </c>
+      <c r="C223" s="3" t="inlineStr">
+        <is>
+          <t>Phase 2 staging (paid media: Google Search): ad groups; cpc_bid_micros cast back to a number (always empty -- automated bidding)</t>
+        </is>
+      </c>
+      <c r="D223" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-29 13:13 PDT</t>
+        </is>
+      </c>
+    </row>
+    <row r="224">
+      <c r="A224" s="2" t="inlineStr">
+        <is>
+          <t>dbt/models/staging/kinetic/stg_kinetic__google_search_performance_daily.sql</t>
+        </is>
+      </c>
+      <c r="B224" s="2" t="inlineStr">
+        <is>
+          <t>Code</t>
+        </is>
+      </c>
+      <c r="C224" s="3" t="inlineStr">
+        <is>
+          <t>Phase 2 staging (paid media: Google Search): ad-group-day performance with combined ad_group_day_id key, cost converted from micros to dollars, ctr_fraction. The keyword table rolled up -- never add the two together</t>
+        </is>
+      </c>
+      <c r="D224" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-29 13:13 PDT</t>
+        </is>
+      </c>
+    </row>
+    <row r="225">
+      <c r="A225" s="2" t="inlineStr">
+        <is>
+          <t>dbt/models/staging/kinetic/stg_kinetic__google_search_keyword_performance_daily.sql</t>
+        </is>
+      </c>
+      <c r="B225" s="2" t="inlineStr">
+        <is>
+          <t>Code</t>
+        </is>
+      </c>
+      <c r="C225" s="3" t="inlineStr">
+        <is>
+          <t>Phase 2 staging (paid media: Google Search): keyword-day performance with combined keyword_day_id key, cost converted from micros to dollars, ctr_fraction</t>
+        </is>
+      </c>
+      <c r="D225" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-29 13:13 PDT</t>
+        </is>
+      </c>
+    </row>
+    <row r="226">
+      <c r="A226" s="2" t="inlineStr">
+        <is>
+          <t>dbt/models/staging/kinetic/_kinetic__staging.yml</t>
+        </is>
+      </c>
+      <c r="B226" s="2" t="inlineStr">
+        <is>
+          <t>Code</t>
+        </is>
+      </c>
+      <c r="C226" s="3" t="inlineStr">
+        <is>
+          <t>Updated: tests for the 4 Google Search staging models -- all hand-verified against live data first</t>
+        </is>
+      </c>
+      <c r="D226" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-29 13:13 PDT</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
dbt Phase 2 sub-batch 6: YouTube staging models
Staging models + tests for the 3 YouTube tables (35 of 47 raw tables now
staged). customer_id renamed google_ads_account_id; micros converted to
dollars; view rate labeled as a fraction. Every test hand-verified against
the live kinetic database first.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014EdkVLDs4dt6TCgduxMMyp
</commit_message>
<xml_diff>
--- a/File_Manifest.xlsx
+++ b/File_Manifest.xlsx
@@ -435,7 +435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D226"/>
+  <dimension ref="A1:D230"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="48" customWidth="1" min="1" max="1"/>
@@ -506,7 +506,7 @@
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 13:13 PDT</t>
+          <t>2026-09-29 13:15 PDT</t>
         </is>
       </c>
     </row>
@@ -638,7 +638,7 @@
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 13:13 PDT</t>
+          <t>2026-09-29 13:15 PDT</t>
         </is>
       </c>
     </row>
@@ -748,7 +748,7 @@
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 13:13 PDT</t>
+          <t>2026-09-29 13:15 PDT</t>
         </is>
       </c>
     </row>
@@ -4400,7 +4400,7 @@
       </c>
       <c r="D180" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 13:13 PDT</t>
+          <t>2026-09-29 13:15 PDT</t>
         </is>
       </c>
     </row>
@@ -4554,7 +4554,7 @@
       </c>
       <c r="D187" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 13:13 PDT</t>
+          <t>2026-09-29 13:14 PDT</t>
         </is>
       </c>
     </row>
@@ -4664,7 +4664,7 @@
       </c>
       <c r="D192" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 13:13 PDT</t>
+          <t>2026-09-29 13:15 PDT</t>
         </is>
       </c>
     </row>
@@ -4972,7 +4972,7 @@
       </c>
       <c r="D206" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 13:13 PDT</t>
+          <t>2026-09-29 13:14 PDT</t>
         </is>
       </c>
     </row>
@@ -5082,7 +5082,7 @@
       </c>
       <c r="D211" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 13:13 PDT</t>
+          <t>2026-09-29 13:14 PDT</t>
         </is>
       </c>
     </row>
@@ -5192,7 +5192,7 @@
       </c>
       <c r="D216" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 13:13 PDT</t>
+          <t>2026-09-29 13:14 PDT</t>
         </is>
       </c>
     </row>
@@ -5302,7 +5302,7 @@
       </c>
       <c r="D221" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 13:13 PDT</t>
+          <t>2026-09-29 13:14 PDT</t>
         </is>
       </c>
     </row>
@@ -5412,7 +5412,95 @@
       </c>
       <c r="D226" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 13:13 PDT</t>
+          <t>2026-09-29 13:14 PDT</t>
+        </is>
+      </c>
+    </row>
+    <row r="227">
+      <c r="A227" s="2" t="inlineStr">
+        <is>
+          <t>dbt/models/staging/kinetic/stg_kinetic__youtube_campaigns.sql</t>
+        </is>
+      </c>
+      <c r="B227" s="2" t="inlineStr">
+        <is>
+          <t>Code</t>
+        </is>
+      </c>
+      <c r="C227" s="3" t="inlineStr">
+        <is>
+          <t>Phase 2 staging (paid media: YouTube): campaigns with customer_id renamed google_ads_account_id (the ad account, not a Kinetic customer), budgets in micros and dollars</t>
+        </is>
+      </c>
+      <c r="D227" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-29 13:14 PDT</t>
+        </is>
+      </c>
+    </row>
+    <row r="228">
+      <c r="A228" s="2" t="inlineStr">
+        <is>
+          <t>dbt/models/staging/kinetic/stg_kinetic__youtube_ad_groups.sql</t>
+        </is>
+      </c>
+      <c r="B228" s="2" t="inlineStr">
+        <is>
+          <t>Code</t>
+        </is>
+      </c>
+      <c r="C228" s="3" t="inlineStr">
+        <is>
+          <t>Phase 2 staging (paid media: YouTube): 1:1 pass-through of youtube_ad_groups</t>
+        </is>
+      </c>
+      <c r="D228" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-29 13:14 PDT</t>
+        </is>
+      </c>
+    </row>
+    <row r="229">
+      <c r="A229" s="2" t="inlineStr">
+        <is>
+          <t>dbt/models/staging/kinetic/stg_kinetic__youtube_performance_daily.sql</t>
+        </is>
+      </c>
+      <c r="B229" s="2" t="inlineStr">
+        <is>
+          <t>Code</t>
+        </is>
+      </c>
+      <c r="C229" s="3" t="inlineStr">
+        <is>
+          <t>Phase 2 staging (paid media: YouTube): ad-group-day performance with combined ad_group_day_id key, cost and cost-per-view converted from micros to dollars, video_view_rate_fraction</t>
+        </is>
+      </c>
+      <c r="D229" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-29 13:14 PDT</t>
+        </is>
+      </c>
+    </row>
+    <row r="230">
+      <c r="A230" s="2" t="inlineStr">
+        <is>
+          <t>dbt/models/staging/kinetic/_kinetic__staging.yml</t>
+        </is>
+      </c>
+      <c r="B230" s="2" t="inlineStr">
+        <is>
+          <t>Code</t>
+        </is>
+      </c>
+      <c r="C230" s="3" t="inlineStr">
+        <is>
+          <t>Updated: tests for the 3 YouTube staging models -- all hand-verified against live data first</t>
+        </is>
+      </c>
+      <c r="D230" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-29 13:14 PDT</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
dbt Phase 2 sub-batch 7: DV360 staging models; flag budget-vs-spend issue
Staging models + tests for the 3 DV360 tables (38 of 47 raw tables now
staged). Monthly budget named as such; combined key for the
line-item x day x exchange x environment grain. Found and documented that
stored budgets are flat while spend grows past them on Meta, Google
Search, YouTube and DV360 (fix pending decision); corrected an earlier
CHANGELOG claim about Meta budgets.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014EdkVLDs4dt6TCgduxMMyp
</commit_message>
<xml_diff>
--- a/File_Manifest.xlsx
+++ b/File_Manifest.xlsx
@@ -435,7 +435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D230"/>
+  <dimension ref="A1:D234"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="48" customWidth="1" min="1" max="1"/>
@@ -506,7 +506,7 @@
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 13:15 PDT</t>
+          <t>2026-09-29 13:19 PDT</t>
         </is>
       </c>
     </row>
@@ -638,7 +638,7 @@
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 13:15 PDT</t>
+          <t>2026-09-29 13:19 PDT</t>
         </is>
       </c>
     </row>
@@ -748,7 +748,7 @@
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 13:15 PDT</t>
+          <t>2026-09-29 13:19 PDT</t>
         </is>
       </c>
     </row>
@@ -4400,7 +4400,7 @@
       </c>
       <c r="D180" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 13:15 PDT</t>
+          <t>2026-09-29 13:19 PDT</t>
         </is>
       </c>
     </row>
@@ -4554,7 +4554,7 @@
       </c>
       <c r="D187" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 13:14 PDT</t>
+          <t>2026-09-29 13:19 PDT</t>
         </is>
       </c>
     </row>
@@ -4664,7 +4664,7 @@
       </c>
       <c r="D192" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 13:15 PDT</t>
+          <t>2026-09-29 13:19 PDT</t>
         </is>
       </c>
     </row>
@@ -4972,7 +4972,7 @@
       </c>
       <c r="D206" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 13:14 PDT</t>
+          <t>2026-09-29 13:19 PDT</t>
         </is>
       </c>
     </row>
@@ -5082,7 +5082,7 @@
       </c>
       <c r="D211" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 13:14 PDT</t>
+          <t>2026-09-29 13:19 PDT</t>
         </is>
       </c>
     </row>
@@ -5192,7 +5192,7 @@
       </c>
       <c r="D216" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 13:14 PDT</t>
+          <t>2026-09-29 13:19 PDT</t>
         </is>
       </c>
     </row>
@@ -5302,7 +5302,7 @@
       </c>
       <c r="D221" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 13:14 PDT</t>
+          <t>2026-09-29 13:19 PDT</t>
         </is>
       </c>
     </row>
@@ -5412,7 +5412,7 @@
       </c>
       <c r="D226" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 13:14 PDT</t>
+          <t>2026-09-29 13:19 PDT</t>
         </is>
       </c>
     </row>
@@ -5500,7 +5500,95 @@
       </c>
       <c r="D230" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 13:14 PDT</t>
+          <t>2026-09-29 13:19 PDT</t>
+        </is>
+      </c>
+    </row>
+    <row r="231">
+      <c r="A231" s="2" t="inlineStr">
+        <is>
+          <t>dbt/models/staging/kinetic/stg_kinetic__dv360_insertion_orders.sql</t>
+        </is>
+      </c>
+      <c r="B231" s="2" t="inlineStr">
+        <is>
+          <t>Code</t>
+        </is>
+      </c>
+      <c r="C231" s="3" t="inlineStr">
+        <is>
+          <t>Phase 2 staging (paid media: DV360): insertion orders with budget_micros named monthly_budget_* (it's a monthly budget), end_date cast back to a date; flags the flat-budget-vs-growing-spend known issue</t>
+        </is>
+      </c>
+      <c r="D231" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-29 13:19 PDT</t>
+        </is>
+      </c>
+    </row>
+    <row r="232">
+      <c r="A232" s="2" t="inlineStr">
+        <is>
+          <t>dbt/models/staging/kinetic/stg_kinetic__dv360_line_items.sql</t>
+        </is>
+      </c>
+      <c r="B232" s="2" t="inlineStr">
+        <is>
+          <t>Code</t>
+        </is>
+      </c>
+      <c r="C232" s="3" t="inlineStr">
+        <is>
+          <t>Phase 2 staging (paid media: DV360): 1:1 pass-through of dv360_line_items</t>
+        </is>
+      </c>
+      <c r="D232" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-29 13:19 PDT</t>
+        </is>
+      </c>
+    </row>
+    <row r="233">
+      <c r="A233" s="2" t="inlineStr">
+        <is>
+          <t>dbt/models/staging/kinetic/stg_kinetic__dv360_performance_daily.sql</t>
+        </is>
+      </c>
+      <c r="B233" s="2" t="inlineStr">
+        <is>
+          <t>Code</t>
+        </is>
+      </c>
+      <c r="C233" s="3" t="inlineStr">
+        <is>
+          <t>Phase 2 staging (paid media: DV360): line-item x day x exchange x environment performance with combined line_item_day_slice_id key, micros converted to dollars, ctr_fraction</t>
+        </is>
+      </c>
+      <c r="D233" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-29 13:19 PDT</t>
+        </is>
+      </c>
+    </row>
+    <row r="234">
+      <c r="A234" s="2" t="inlineStr">
+        <is>
+          <t>dbt/models/staging/kinetic/_kinetic__staging.yml</t>
+        </is>
+      </c>
+      <c r="B234" s="2" t="inlineStr">
+        <is>
+          <t>Code</t>
+        </is>
+      </c>
+      <c r="C234" s="3" t="inlineStr">
+        <is>
+          <t>Updated: tests for the 3 DV360 staging models, incl. accepted_values on exchange and environment -- all hand-verified against live data first</t>
+        </is>
+      </c>
+      <c r="D234" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-29 13:19 PDT</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Fix ad budgets: store each campaign's current budget
Evergreen budgets on all 6 platforms were flat launch-era figures while
spend grew 2.4x, so later months spent up to ~20x the stored budget.
params.py now sets each evergreen budget to its current value, sized from
realized spend; only the 6 campaign tables' budget columns changed, spend
untouched. Adds audit Check 8 (spend vs budget, all campaigns) -- now 0
violations for always-on campaigns. MotherDuck updated to match.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014EdkVLDs4dt6TCgduxMMyp
</commit_message>
<xml_diff>
--- a/File_Manifest.xlsx
+++ b/File_Manifest.xlsx
@@ -435,7 +435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D234"/>
+  <dimension ref="A1:D243"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="48" customWidth="1" min="1" max="1"/>
@@ -506,7 +506,7 @@
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 13:19 PDT</t>
+          <t>2026-09-29 13:27 PDT</t>
         </is>
       </c>
     </row>
@@ -594,7 +594,7 @@
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28 14:09 PDT</t>
+          <t>2026-09-29 13:23 PDT</t>
         </is>
       </c>
     </row>
@@ -638,7 +638,7 @@
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 13:19 PDT</t>
+          <t>2026-09-29 13:27 PDT</t>
         </is>
       </c>
     </row>
@@ -748,7 +748,7 @@
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 13:19 PDT</t>
+          <t>2026-09-29 13:28 PDT</t>
         </is>
       </c>
     </row>
@@ -2772,7 +2772,7 @@
       </c>
       <c r="D106" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28 14:09 PDT</t>
+          <t>2026-09-29 13:24 PDT</t>
         </is>
       </c>
     </row>
@@ -3036,7 +3036,7 @@
       </c>
       <c r="D118" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28 14:09 PDT</t>
+          <t>2026-09-29 13:24 PDT</t>
         </is>
       </c>
     </row>
@@ -3300,7 +3300,7 @@
       </c>
       <c r="D130" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28 14:09 PDT</t>
+          <t>2026-09-29 13:24 PDT</t>
         </is>
       </c>
     </row>
@@ -3498,7 +3498,7 @@
       </c>
       <c r="D139" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28 14:09 PDT</t>
+          <t>2026-09-29 13:24 PDT</t>
         </is>
       </c>
     </row>
@@ -3696,7 +3696,7 @@
       </c>
       <c r="D148" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28 14:09 PDT</t>
+          <t>2026-09-29 13:24 PDT</t>
         </is>
       </c>
     </row>
@@ -3960,7 +3960,7 @@
       </c>
       <c r="D160" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28 14:09 PDT</t>
+          <t>2026-09-29 13:24 PDT</t>
         </is>
       </c>
     </row>
@@ -4180,7 +4180,7 @@
       </c>
       <c r="D170" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28 14:09 PDT</t>
+          <t>2026-09-29 13:24 PDT</t>
         </is>
       </c>
     </row>
@@ -4554,7 +4554,7 @@
       </c>
       <c r="D187" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 13:19 PDT</t>
+          <t>2026-09-29 13:27 PDT</t>
         </is>
       </c>
     </row>
@@ -4972,7 +4972,7 @@
       </c>
       <c r="D206" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 13:19 PDT</t>
+          <t>2026-09-29 13:27 PDT</t>
         </is>
       </c>
     </row>
@@ -5082,7 +5082,7 @@
       </c>
       <c r="D211" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 13:19 PDT</t>
+          <t>2026-09-29 13:27 PDT</t>
         </is>
       </c>
     </row>
@@ -5192,7 +5192,7 @@
       </c>
       <c r="D216" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 13:19 PDT</t>
+          <t>2026-09-29 13:27 PDT</t>
         </is>
       </c>
     </row>
@@ -5302,7 +5302,7 @@
       </c>
       <c r="D221" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 13:19 PDT</t>
+          <t>2026-09-29 13:27 PDT</t>
         </is>
       </c>
     </row>
@@ -5412,7 +5412,7 @@
       </c>
       <c r="D226" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 13:19 PDT</t>
+          <t>2026-09-29 13:27 PDT</t>
         </is>
       </c>
     </row>
@@ -5500,7 +5500,7 @@
       </c>
       <c r="D230" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 13:19 PDT</t>
+          <t>2026-09-29 13:27 PDT</t>
         </is>
       </c>
     </row>
@@ -5522,7 +5522,7 @@
       </c>
       <c r="D231" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 13:19 PDT</t>
+          <t>2026-09-29 13:27 PDT</t>
         </is>
       </c>
     </row>
@@ -5588,7 +5588,205 @@
       </c>
       <c r="D234" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 13:19 PDT</t>
+          <t>2026-09-29 13:27 PDT</t>
+        </is>
+      </c>
+    </row>
+    <row r="235">
+      <c r="A235" s="2" t="inlineStr">
+        <is>
+          <t>generator/params.py</t>
+        </is>
+      </c>
+      <c r="B235" s="2" t="inlineStr">
+        <is>
+          <t>Code</t>
+        </is>
+      </c>
+      <c r="C235" s="3" t="inlineStr">
+        <is>
+          <t>Updated 2026-09-29: every evergreen ad budget on all 6 platforms is now the campaign's CURRENT budget, sized from realized spend (weekly average &lt;= budget, no day &gt; 1.75x; DV360 monthly &gt;= highest month). The old flat 'typical day' budgets let later months spend up to ~20x the stored budget</t>
+        </is>
+      </c>
+      <c r="D235" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-29 13:23 PDT</t>
+        </is>
+      </c>
+    </row>
+    <row r="236">
+      <c r="A236" s="2" t="inlineStr">
+        <is>
+          <t>data/meta_campaigns.csv</t>
+        </is>
+      </c>
+      <c r="B236" s="2" t="inlineStr">
+        <is>
+          <t>Shipped table</t>
+        </is>
+      </c>
+      <c r="C236" s="3" t="inlineStr">
+        <is>
+          <t>Regenerated 2026-09-29: evergreen daily_budget values updated to current budgets (only that column, only the 4 evergreen rows changed)</t>
+        </is>
+      </c>
+      <c r="D236" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-29 13:24 PDT</t>
+        </is>
+      </c>
+    </row>
+    <row r="237">
+      <c r="A237" s="2" t="inlineStr">
+        <is>
+          <t>data/google_search_campaigns.csv</t>
+        </is>
+      </c>
+      <c r="B237" s="2" t="inlineStr">
+        <is>
+          <t>Shipped table</t>
+        </is>
+      </c>
+      <c r="C237" s="3" t="inlineStr">
+        <is>
+          <t>Regenerated 2026-09-29: campaign_budget_micros updated to current budgets (only that column changed)</t>
+        </is>
+      </c>
+      <c r="D237" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-29 13:24 PDT</t>
+        </is>
+      </c>
+    </row>
+    <row r="238">
+      <c r="A238" s="2" t="inlineStr">
+        <is>
+          <t>data/youtube_campaigns.csv</t>
+        </is>
+      </c>
+      <c r="B238" s="2" t="inlineStr">
+        <is>
+          <t>Shipped table</t>
+        </is>
+      </c>
+      <c r="C238" s="3" t="inlineStr">
+        <is>
+          <t>Regenerated 2026-09-29: evergreen campaign_budget_micros updated to current budgets (only that column, only the 4 evergreen rows changed)</t>
+        </is>
+      </c>
+      <c r="D238" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-29 13:24 PDT</t>
+        </is>
+      </c>
+    </row>
+    <row r="239">
+      <c r="A239" s="2" t="inlineStr">
+        <is>
+          <t>data/dv360_insertion_orders.csv</t>
+        </is>
+      </c>
+      <c r="B239" s="2" t="inlineStr">
+        <is>
+          <t>Shipped table</t>
+        </is>
+      </c>
+      <c r="C239" s="3" t="inlineStr">
+        <is>
+          <t>Regenerated 2026-09-29: monthly budget_micros updated to current budgets (only that column changed)</t>
+        </is>
+      </c>
+      <c r="D239" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-29 13:24 PDT</t>
+        </is>
+      </c>
+    </row>
+    <row r="240">
+      <c r="A240" s="2" t="inlineStr">
+        <is>
+          <t>data/snap_campaigns.csv</t>
+        </is>
+      </c>
+      <c r="B240" s="2" t="inlineStr">
+        <is>
+          <t>Shipped table</t>
+        </is>
+      </c>
+      <c r="C240" s="3" t="inlineStr">
+        <is>
+          <t>Regenerated 2026-09-29: evergreen daily_budget_micro updated to current budgets (only that column, only the 4 evergreen rows changed)</t>
+        </is>
+      </c>
+      <c r="D240" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-29 13:24 PDT</t>
+        </is>
+      </c>
+    </row>
+    <row r="241">
+      <c r="A241" s="2" t="inlineStr">
+        <is>
+          <t>data/tiktok_campaigns.csv</t>
+        </is>
+      </c>
+      <c r="B241" s="2" t="inlineStr">
+        <is>
+          <t>Shipped table</t>
+        </is>
+      </c>
+      <c r="C241" s="3" t="inlineStr">
+        <is>
+          <t>Regenerated 2026-09-29: BUDGET_MODE_DAY budget_micro updated to current budgets (only that column, only the 4 evergreen rows changed)</t>
+        </is>
+      </c>
+      <c r="D241" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-29 13:24 PDT</t>
+        </is>
+      </c>
+    </row>
+    <row r="242">
+      <c r="A242" s="2" t="inlineStr">
+        <is>
+          <t>generator/audit_cross_dataset_alignment.py</t>
+        </is>
+      </c>
+      <c r="B242" s="2" t="inlineStr">
+        <is>
+          <t>Code</t>
+        </is>
+      </c>
+      <c r="C242" s="3" t="inlineStr">
+        <is>
+          <t>Updated 2026-09-29: new Check 8 -- spend vs stored budget for every campaign on all 6 platforms (weekly/daily limits for daily budgets, monthly for DV360, total for holiday flights)</t>
+        </is>
+      </c>
+      <c r="D242" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-29 13:24 PDT</t>
+        </is>
+      </c>
+    </row>
+    <row r="243">
+      <c r="A243" s="2" t="inlineStr">
+        <is>
+          <t>dbt/models/staging/kinetic/stg_kinetic__dv360_insertion_orders.sql</t>
+        </is>
+      </c>
+      <c r="B243" s="2" t="inlineStr">
+        <is>
+          <t>Code</t>
+        </is>
+      </c>
+      <c r="C243" s="3" t="inlineStr">
+        <is>
+          <t>Updated: budget known-issue note replaced -- budgets are now current budgets</t>
+        </is>
+      </c>
+      <c r="D243" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-29 13:27 PDT</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Cap holiday brand-lift flights at their lifetime budget
6 of 12 flights overshot their lifetime budgets by 0.7-6.4% ($430) from
unbounded daily random variation. New cap_flight_at_budget() rescales an
overshooting flight's days to spend exactly its budget, replaying the same
random rates so no other row changes. Rebuilt the Meta/Snap/TikTok/YouTube
spend tables (+ Meta actions); only the 5 affected flights changed.
Check 8 tightened to require flights <= budget; passes. MotherDuck updated
and verified against the CSVs.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014EdkVLDs4dt6TCgduxMMyp
</commit_message>
<xml_diff>
--- a/File_Manifest.xlsx
+++ b/File_Manifest.xlsx
@@ -435,7 +435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D243"/>
+  <dimension ref="A1:D254"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="48" customWidth="1" min="1" max="1"/>
@@ -506,7 +506,7 @@
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 13:27 PDT</t>
+          <t>2026-09-29 13:54 PDT</t>
         </is>
       </c>
     </row>
@@ -638,7 +638,7 @@
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 13:27 PDT</t>
+          <t>2026-09-29 13:54 PDT</t>
         </is>
       </c>
     </row>
@@ -748,7 +748,7 @@
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 13:28 PDT</t>
+          <t>2026-09-29 13:54 PDT</t>
         </is>
       </c>
     </row>
@@ -2706,7 +2706,7 @@
       </c>
       <c r="D103" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28 14:09 PDT</t>
+          <t>2026-09-29 13:29 PDT</t>
         </is>
       </c>
     </row>
@@ -2860,7 +2860,7 @@
       </c>
       <c r="D110" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28 14:09 PDT</t>
+          <t>2026-09-29 13:29 PDT</t>
         </is>
       </c>
     </row>
@@ -2904,7 +2904,7 @@
       </c>
       <c r="D112" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28 14:09 PDT</t>
+          <t>2026-09-29 13:29 PDT</t>
         </is>
       </c>
     </row>
@@ -2970,7 +2970,7 @@
       </c>
       <c r="D115" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28 14:09 PDT</t>
+          <t>2026-09-29 13:29 PDT</t>
         </is>
       </c>
     </row>
@@ -3388,7 +3388,7 @@
       </c>
       <c r="D134" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28 14:09 PDT</t>
+          <t>2026-09-29 13:29 PDT</t>
         </is>
       </c>
     </row>
@@ -3432,7 +3432,7 @@
       </c>
       <c r="D136" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28 14:09 PDT</t>
+          <t>2026-09-29 13:29 PDT</t>
         </is>
       </c>
     </row>
@@ -3850,7 +3850,7 @@
       </c>
       <c r="D155" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28 14:09 PDT</t>
+          <t>2026-09-29 13:29 PDT</t>
         </is>
       </c>
     </row>
@@ -3894,7 +3894,7 @@
       </c>
       <c r="D157" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28 14:09 PDT</t>
+          <t>2026-09-29 13:29 PDT</t>
         </is>
       </c>
     </row>
@@ -4114,7 +4114,7 @@
       </c>
       <c r="D167" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28 14:09 PDT</t>
+          <t>2026-09-29 13:29 PDT</t>
         </is>
       </c>
     </row>
@@ -4158,7 +4158,7 @@
       </c>
       <c r="D169" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28 14:09 PDT</t>
+          <t>2026-09-29 13:29 PDT</t>
         </is>
       </c>
     </row>
@@ -4180,7 +4180,7 @@
       </c>
       <c r="D170" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 13:24 PDT</t>
+          <t>2026-09-29 13:30 PDT</t>
         </is>
       </c>
     </row>
@@ -4202,7 +4202,7 @@
       </c>
       <c r="D171" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28 14:47 PDT</t>
+          <t>2026-09-29 13:54 PDT</t>
         </is>
       </c>
     </row>
@@ -4334,7 +4334,7 @@
       </c>
       <c r="D177" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28 14:47 PDT</t>
+          <t>2026-09-29 13:54 PDT</t>
         </is>
       </c>
     </row>
@@ -5764,7 +5764,7 @@
       </c>
       <c r="D242" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 13:24 PDT</t>
+          <t>2026-09-29 13:30 PDT</t>
         </is>
       </c>
     </row>
@@ -5787,6 +5787,248 @@
       <c r="D243" s="2" t="inlineStr">
         <is>
           <t>2026-09-29 13:27 PDT</t>
+        </is>
+      </c>
+    </row>
+    <row r="244">
+      <c r="A244" s="2" t="inlineStr">
+        <is>
+          <t>generator/paid_media_common.py</t>
+        </is>
+      </c>
+      <c r="B244" s="2" t="inlineStr">
+        <is>
+          <t>Code</t>
+        </is>
+      </c>
+      <c r="C244" s="3" t="inlineStr">
+        <is>
+          <t>Updated 2026-09-29: new cap_flight_at_budget() -- rescales a holiday flight's days so it never spends past its lifetime budget, replaying the same random rates so every other row is unchanged</t>
+        </is>
+      </c>
+      <c r="D244" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-29 13:29 PDT</t>
+        </is>
+      </c>
+    </row>
+    <row r="245">
+      <c r="A245" s="2" t="inlineStr">
+        <is>
+          <t>generator/build_meta_ad_insights_daily.py</t>
+        </is>
+      </c>
+      <c r="B245" s="2" t="inlineStr">
+        <is>
+          <t>Code</t>
+        </is>
+      </c>
+      <c r="C245" s="3" t="inlineStr">
+        <is>
+          <t>Updated 2026-09-29: holiday flights capped at their lifetime budget via cap_flight_at_budget()</t>
+        </is>
+      </c>
+      <c r="D245" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-29 13:29 PDT</t>
+        </is>
+      </c>
+    </row>
+    <row r="246">
+      <c r="A246" s="2" t="inlineStr">
+        <is>
+          <t>generator/build_snap_stats_daily.py</t>
+        </is>
+      </c>
+      <c r="B246" s="2" t="inlineStr">
+        <is>
+          <t>Code</t>
+        </is>
+      </c>
+      <c r="C246" s="3" t="inlineStr">
+        <is>
+          <t>Updated 2026-09-29: holiday flights capped at their lifetime budget via cap_flight_at_budget()</t>
+        </is>
+      </c>
+      <c r="D246" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-29 13:29 PDT</t>
+        </is>
+      </c>
+    </row>
+    <row r="247">
+      <c r="A247" s="2" t="inlineStr">
+        <is>
+          <t>generator/build_tiktok_reports_daily.py</t>
+        </is>
+      </c>
+      <c r="B247" s="2" t="inlineStr">
+        <is>
+          <t>Code</t>
+        </is>
+      </c>
+      <c r="C247" s="3" t="inlineStr">
+        <is>
+          <t>Updated 2026-09-29: holiday flights capped at their lifetime budget via cap_flight_at_budget()</t>
+        </is>
+      </c>
+      <c r="D247" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-29 13:29 PDT</t>
+        </is>
+      </c>
+    </row>
+    <row r="248">
+      <c r="A248" s="2" t="inlineStr">
+        <is>
+          <t>generator/build_youtube_performance_daily.py</t>
+        </is>
+      </c>
+      <c r="B248" s="2" t="inlineStr">
+        <is>
+          <t>Code</t>
+        </is>
+      </c>
+      <c r="C248" s="3" t="inlineStr">
+        <is>
+          <t>Updated 2026-09-29: holiday flights capped at their lifetime budget via cap_flight_at_budget() (no-op today -- all YouTube flights were already under budget)</t>
+        </is>
+      </c>
+      <c r="D248" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-29 13:29 PDT</t>
+        </is>
+      </c>
+    </row>
+    <row r="249">
+      <c r="A249" s="2" t="inlineStr">
+        <is>
+          <t>data/meta_ad_insights_daily.csv</t>
+        </is>
+      </c>
+      <c r="B249" s="2" t="inlineStr">
+        <is>
+          <t>Shipped table</t>
+        </is>
+      </c>
+      <c r="C249" s="3" t="inlineStr">
+        <is>
+          <t>Regenerated 2026-09-29: the 2023 and 2024 holiday flights (38 rows) trimmed to spend exactly their lifetime budget; every other row identical</t>
+        </is>
+      </c>
+      <c r="D249" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-29 13:29 PDT</t>
+        </is>
+      </c>
+    </row>
+    <row r="250">
+      <c r="A250" s="2" t="inlineStr">
+        <is>
+          <t>data/meta_ad_actions_daily.csv</t>
+        </is>
+      </c>
+      <c r="B250" s="2" t="inlineStr">
+        <is>
+          <t>Shipped table</t>
+        </is>
+      </c>
+      <c r="C250" s="3" t="inlineStr">
+        <is>
+          <t>Regenerated 2026-09-29: re-derived from the trimmed insights rows -- only the 2023/2024 holiday flights' action rows changed (one initiate_checkout row on 2024-11-15 dropped to zero and is no longer emitted)</t>
+        </is>
+      </c>
+      <c r="D250" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-29 13:29 PDT</t>
+        </is>
+      </c>
+    </row>
+    <row r="251">
+      <c r="A251" s="2" t="inlineStr">
+        <is>
+          <t>data/snap_stats_daily.csv</t>
+        </is>
+      </c>
+      <c r="B251" s="2" t="inlineStr">
+        <is>
+          <t>Shipped table</t>
+        </is>
+      </c>
+      <c r="C251" s="3" t="inlineStr">
+        <is>
+          <t>Regenerated 2026-09-29: the 2024 holiday flight (19 rows) trimmed to spend exactly its lifetime budget; every other row identical</t>
+        </is>
+      </c>
+      <c r="D251" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-29 13:29 PDT</t>
+        </is>
+      </c>
+    </row>
+    <row r="252">
+      <c r="A252" s="2" t="inlineStr">
+        <is>
+          <t>data/tiktok_reports_daily.csv</t>
+        </is>
+      </c>
+      <c r="B252" s="2" t="inlineStr">
+        <is>
+          <t>Shipped table</t>
+        </is>
+      </c>
+      <c r="C252" s="3" t="inlineStr">
+        <is>
+          <t>Regenerated 2026-09-29: the 2023/2024/2025 holiday flights (56 rows) trimmed to spend exactly their lifetime budgets; every other row identical</t>
+        </is>
+      </c>
+      <c r="D252" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-29 13:29 PDT</t>
+        </is>
+      </c>
+    </row>
+    <row r="253">
+      <c r="A253" s="2" t="inlineStr">
+        <is>
+          <t>docs/cross_dataset_alignment_audit.md</t>
+        </is>
+      </c>
+      <c r="B253" s="2" t="inlineStr">
+        <is>
+          <t>Docs</t>
+        </is>
+      </c>
+      <c r="C253" s="3" t="inlineStr">
+        <is>
+          <t>Updated 2026-09-29: added Check 8 (spend vs stored budget) with both fixes and results</t>
+        </is>
+      </c>
+      <c r="D253" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-29 13:54 PDT</t>
+        </is>
+      </c>
+    </row>
+    <row r="254">
+      <c r="A254" s="2" t="inlineStr">
+        <is>
+          <t>generator/audit_cross_dataset_alignment.py</t>
+        </is>
+      </c>
+      <c r="B254" s="2" t="inlineStr">
+        <is>
+          <t>Code</t>
+        </is>
+      </c>
+      <c r="C254" s="3" t="inlineStr">
+        <is>
+          <t>Updated 2026-09-29: Check 8's flight limit tightened from 1.05x to 1.0x now that flights are capped</t>
+        </is>
+      </c>
+      <c r="D254" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-29 13:30 PDT</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
dbt Phase 2 sub-batch 8: Snap staging models
Staging models + tests for the 4 Snap tables (42 of 47 raw tables now
staged). Micros converted to dollars, ad account renamed, Snap terms
(ad squad, swipes) documented. Every test hand-verified against the live
kinetic database first.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014EdkVLDs4dt6TCgduxMMyp
</commit_message>
<xml_diff>
--- a/File_Manifest.xlsx
+++ b/File_Manifest.xlsx
@@ -435,7 +435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D254"/>
+  <dimension ref="A1:D259"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="48" customWidth="1" min="1" max="1"/>
@@ -506,7 +506,7 @@
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 13:54 PDT</t>
+          <t>2026-09-29 15:53 PDT</t>
         </is>
       </c>
     </row>
@@ -638,7 +638,7 @@
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 13:54 PDT</t>
+          <t>2026-09-29 15:53 PDT</t>
         </is>
       </c>
     </row>
@@ -748,7 +748,7 @@
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 13:54 PDT</t>
+          <t>2026-09-29 15:53 PDT</t>
         </is>
       </c>
     </row>
@@ -4400,7 +4400,7 @@
       </c>
       <c r="D180" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 13:19 PDT</t>
+          <t>2026-09-29 15:53 PDT</t>
         </is>
       </c>
     </row>
@@ -4554,7 +4554,7 @@
       </c>
       <c r="D187" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 13:27 PDT</t>
+          <t>2026-09-29 15:53 PDT</t>
         </is>
       </c>
     </row>
@@ -4664,7 +4664,7 @@
       </c>
       <c r="D192" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 13:19 PDT</t>
+          <t>2026-09-29 15:53 PDT</t>
         </is>
       </c>
     </row>
@@ -4972,7 +4972,7 @@
       </c>
       <c r="D206" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 13:27 PDT</t>
+          <t>2026-09-29 15:53 PDT</t>
         </is>
       </c>
     </row>
@@ -5082,7 +5082,7 @@
       </c>
       <c r="D211" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 13:27 PDT</t>
+          <t>2026-09-29 15:53 PDT</t>
         </is>
       </c>
     </row>
@@ -5192,7 +5192,7 @@
       </c>
       <c r="D216" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 13:27 PDT</t>
+          <t>2026-09-29 15:53 PDT</t>
         </is>
       </c>
     </row>
@@ -5302,7 +5302,7 @@
       </c>
       <c r="D221" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 13:27 PDT</t>
+          <t>2026-09-29 15:53 PDT</t>
         </is>
       </c>
     </row>
@@ -5412,7 +5412,7 @@
       </c>
       <c r="D226" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 13:27 PDT</t>
+          <t>2026-09-29 15:53 PDT</t>
         </is>
       </c>
     </row>
@@ -5500,7 +5500,7 @@
       </c>
       <c r="D230" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 13:27 PDT</t>
+          <t>2026-09-29 15:53 PDT</t>
         </is>
       </c>
     </row>
@@ -5588,7 +5588,7 @@
       </c>
       <c r="D234" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 13:27 PDT</t>
+          <t>2026-09-29 15:53 PDT</t>
         </is>
       </c>
     </row>
@@ -6029,6 +6029,116 @@
       <c r="D254" s="2" t="inlineStr">
         <is>
           <t>2026-09-29 13:30 PDT</t>
+        </is>
+      </c>
+    </row>
+    <row r="255">
+      <c r="A255" s="2" t="inlineStr">
+        <is>
+          <t>dbt/models/staging/kinetic/stg_kinetic__snap_campaigns.sql</t>
+        </is>
+      </c>
+      <c r="B255" s="2" t="inlineStr">
+        <is>
+          <t>Code</t>
+        </is>
+      </c>
+      <c r="C255" s="3" t="inlineStr">
+        <is>
+          <t>Phase 2 staging (paid media: Snap): campaigns with ad_account_id renamed snap_ad_account_id, current budgets in micros and dollars</t>
+        </is>
+      </c>
+      <c r="D255" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-29 15:53 PDT</t>
+        </is>
+      </c>
+    </row>
+    <row r="256">
+      <c r="A256" s="2" t="inlineStr">
+        <is>
+          <t>dbt/models/staging/kinetic/stg_kinetic__snap_ad_squads.sql</t>
+        </is>
+      </c>
+      <c r="B256" s="2" t="inlineStr">
+        <is>
+          <t>Code</t>
+        </is>
+      </c>
+      <c r="C256" s="3" t="inlineStr">
+        <is>
+          <t>Phase 2 staging (paid media: Snap): 1:1 pass-through of snap_ad_squads (Snap's ad set / ad group level)</t>
+        </is>
+      </c>
+      <c r="D256" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-29 15:53 PDT</t>
+        </is>
+      </c>
+    </row>
+    <row r="257">
+      <c r="A257" s="2" t="inlineStr">
+        <is>
+          <t>dbt/models/staging/kinetic/stg_kinetic__snap_ads.sql</t>
+        </is>
+      </c>
+      <c r="B257" s="2" t="inlineStr">
+        <is>
+          <t>Code</t>
+        </is>
+      </c>
+      <c r="C257" s="3" t="inlineStr">
+        <is>
+          <t>Phase 2 staging (paid media: Snap): 1:1 pass-through of snap_ads</t>
+        </is>
+      </c>
+      <c r="D257" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-29 15:53 PDT</t>
+        </is>
+      </c>
+    </row>
+    <row r="258">
+      <c r="A258" s="2" t="inlineStr">
+        <is>
+          <t>dbt/models/staging/kinetic/stg_kinetic__snap_stats_daily.sql</t>
+        </is>
+      </c>
+      <c r="B258" s="2" t="inlineStr">
+        <is>
+          <t>Code</t>
+        </is>
+      </c>
+      <c r="C258" s="3" t="inlineStr">
+        <is>
+          <t>Phase 2 staging (paid media: Snap): ad-day stats with combined ad_day_id key, spend in micros and dollars; documents swipes as Snap's clicks</t>
+        </is>
+      </c>
+      <c r="D258" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-29 15:53 PDT</t>
+        </is>
+      </c>
+    </row>
+    <row r="259">
+      <c r="A259" s="2" t="inlineStr">
+        <is>
+          <t>dbt/models/staging/kinetic/_kinetic__staging.yml</t>
+        </is>
+      </c>
+      <c r="B259" s="2" t="inlineStr">
+        <is>
+          <t>Code</t>
+        </is>
+      </c>
+      <c r="C259" s="3" t="inlineStr">
+        <is>
+          <t>Updated: tests for the 4 Snap staging models -- all hand-verified against live data first</t>
+        </is>
+      </c>
+      <c r="D259" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-29 15:53 PDT</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
dbt Phase 2 sub-batch 9: TikTok staging models
Staging models + tests for the 4 TikTok tables (46 of 47 raw tables now
staged; all 6 ad platforms done). Single budget split into daily/lifetime
columns to match the other platforms; micros converted to dollars. Every
test hand-verified against the live kinetic database first.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014EdkVLDs4dt6TCgduxMMyp
</commit_message>
<xml_diff>
--- a/File_Manifest.xlsx
+++ b/File_Manifest.xlsx
@@ -435,7 +435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D259"/>
+  <dimension ref="A1:D264"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="48" customWidth="1" min="1" max="1"/>
@@ -506,7 +506,7 @@
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 15:53 PDT</t>
+          <t>2026-09-29 15:57 PDT</t>
         </is>
       </c>
     </row>
@@ -638,7 +638,7 @@
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 15:53 PDT</t>
+          <t>2026-09-29 15:57 PDT</t>
         </is>
       </c>
     </row>
@@ -748,7 +748,7 @@
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 15:53 PDT</t>
+          <t>2026-09-29 15:57 PDT</t>
         </is>
       </c>
     </row>
@@ -4400,7 +4400,7 @@
       </c>
       <c r="D180" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 15:53 PDT</t>
+          <t>2026-09-29 15:57 PDT</t>
         </is>
       </c>
     </row>
@@ -4554,7 +4554,7 @@
       </c>
       <c r="D187" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 15:53 PDT</t>
+          <t>2026-09-29 15:57 PDT</t>
         </is>
       </c>
     </row>
@@ -4664,7 +4664,7 @@
       </c>
       <c r="D192" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 15:53 PDT</t>
+          <t>2026-09-29 15:57 PDT</t>
         </is>
       </c>
     </row>
@@ -4972,7 +4972,7 @@
       </c>
       <c r="D206" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 15:53 PDT</t>
+          <t>2026-09-29 15:57 PDT</t>
         </is>
       </c>
     </row>
@@ -5082,7 +5082,7 @@
       </c>
       <c r="D211" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 15:53 PDT</t>
+          <t>2026-09-29 15:57 PDT</t>
         </is>
       </c>
     </row>
@@ -5192,7 +5192,7 @@
       </c>
       <c r="D216" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 15:53 PDT</t>
+          <t>2026-09-29 15:57 PDT</t>
         </is>
       </c>
     </row>
@@ -5302,7 +5302,7 @@
       </c>
       <c r="D221" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 15:53 PDT</t>
+          <t>2026-09-29 15:57 PDT</t>
         </is>
       </c>
     </row>
@@ -5412,7 +5412,7 @@
       </c>
       <c r="D226" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 15:53 PDT</t>
+          <t>2026-09-29 15:57 PDT</t>
         </is>
       </c>
     </row>
@@ -5500,7 +5500,7 @@
       </c>
       <c r="D230" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 15:53 PDT</t>
+          <t>2026-09-29 15:57 PDT</t>
         </is>
       </c>
     </row>
@@ -5588,7 +5588,7 @@
       </c>
       <c r="D234" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 15:53 PDT</t>
+          <t>2026-09-29 15:57 PDT</t>
         </is>
       </c>
     </row>
@@ -6138,7 +6138,117 @@
       </c>
       <c r="D259" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 15:53 PDT</t>
+          <t>2026-09-29 15:57 PDT</t>
+        </is>
+      </c>
+    </row>
+    <row r="260">
+      <c r="A260" s="2" t="inlineStr">
+        <is>
+          <t>dbt/models/staging/kinetic/stg_kinetic__tiktok_campaigns.sql</t>
+        </is>
+      </c>
+      <c r="B260" s="2" t="inlineStr">
+        <is>
+          <t>Code</t>
+        </is>
+      </c>
+      <c r="C260" s="3" t="inlineStr">
+        <is>
+          <t>Phase 2 staging (paid media: TikTok): campaigns with the single budget split into daily_budget_usd / lifetime_budget_usd by budget_mode (matching the other platforms), advertiser_id renamed tiktok_advertiser_id</t>
+        </is>
+      </c>
+      <c r="D260" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-29 15:57 PDT</t>
+        </is>
+      </c>
+    </row>
+    <row r="261">
+      <c r="A261" s="2" t="inlineStr">
+        <is>
+          <t>dbt/models/staging/kinetic/stg_kinetic__tiktok_adgroups.sql</t>
+        </is>
+      </c>
+      <c r="B261" s="2" t="inlineStr">
+        <is>
+          <t>Code</t>
+        </is>
+      </c>
+      <c r="C261" s="3" t="inlineStr">
+        <is>
+          <t>Phase 2 staging (paid media: TikTok): 1:1 pass-through of tiktok_adgroups</t>
+        </is>
+      </c>
+      <c r="D261" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-29 15:57 PDT</t>
+        </is>
+      </c>
+    </row>
+    <row r="262">
+      <c r="A262" s="2" t="inlineStr">
+        <is>
+          <t>dbt/models/staging/kinetic/stg_kinetic__tiktok_ads.sql</t>
+        </is>
+      </c>
+      <c r="B262" s="2" t="inlineStr">
+        <is>
+          <t>Code</t>
+        </is>
+      </c>
+      <c r="C262" s="3" t="inlineStr">
+        <is>
+          <t>Phase 2 staging (paid media: TikTok): 1:1 pass-through of tiktok_ads</t>
+        </is>
+      </c>
+      <c r="D262" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-29 15:57 PDT</t>
+        </is>
+      </c>
+    </row>
+    <row r="263">
+      <c r="A263" s="2" t="inlineStr">
+        <is>
+          <t>dbt/models/staging/kinetic/stg_kinetic__tiktok_reports_daily.sql</t>
+        </is>
+      </c>
+      <c r="B263" s="2" t="inlineStr">
+        <is>
+          <t>Code</t>
+        </is>
+      </c>
+      <c r="C263" s="3" t="inlineStr">
+        <is>
+          <t>Phase 2 staging (paid media: TikTok): ad-day reports with combined ad_day_id key, spend and CPM in micros and dollars, ctr_fraction</t>
+        </is>
+      </c>
+      <c r="D263" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-29 15:57 PDT</t>
+        </is>
+      </c>
+    </row>
+    <row r="264">
+      <c r="A264" s="2" t="inlineStr">
+        <is>
+          <t>dbt/models/staging/kinetic/_kinetic__staging.yml</t>
+        </is>
+      </c>
+      <c r="B264" s="2" t="inlineStr">
+        <is>
+          <t>Code</t>
+        </is>
+      </c>
+      <c r="C264" s="3" t="inlineStr">
+        <is>
+          <t>Updated: tests for the 4 TikTok staging models -- all hand-verified against live data first</t>
+        </is>
+      </c>
+      <c r="D264" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-29 15:57 PDT</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Phase 2: stage product_variants (47 of 47); Phase 2 complete
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014EdkVLDs4dt6TCgduxMMyp
</commit_message>
<xml_diff>
--- a/File_Manifest.xlsx
+++ b/File_Manifest.xlsx
@@ -435,7 +435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D264"/>
+  <dimension ref="A1:D265"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="48" customWidth="1" min="1" max="1"/>
@@ -506,7 +506,7 @@
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 15:57 PDT</t>
+          <t>2026-09-29 16:09 PDT</t>
         </is>
       </c>
     </row>
@@ -638,7 +638,7 @@
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 15:57 PDT</t>
+          <t>2026-09-29 16:09 PDT</t>
         </is>
       </c>
     </row>
@@ -748,7 +748,7 @@
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 15:57 PDT</t>
+          <t>2026-09-29 16:09 PDT</t>
         </is>
       </c>
     </row>
@@ -4400,7 +4400,7 @@
       </c>
       <c r="D180" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 15:57 PDT</t>
+          <t>2026-09-29 16:09 PDT</t>
         </is>
       </c>
     </row>
@@ -4554,7 +4554,7 @@
       </c>
       <c r="D187" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 15:57 PDT</t>
+          <t>2026-09-29 16:08 PDT</t>
         </is>
       </c>
     </row>
@@ -4664,7 +4664,7 @@
       </c>
       <c r="D192" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 15:57 PDT</t>
+          <t>2026-09-29 16:09 PDT</t>
         </is>
       </c>
     </row>
@@ -4972,7 +4972,7 @@
       </c>
       <c r="D206" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 15:57 PDT</t>
+          <t>2026-09-29 16:08 PDT</t>
         </is>
       </c>
     </row>
@@ -5082,7 +5082,7 @@
       </c>
       <c r="D211" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 15:57 PDT</t>
+          <t>2026-09-29 16:08 PDT</t>
         </is>
       </c>
     </row>
@@ -5192,7 +5192,7 @@
       </c>
       <c r="D216" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 15:57 PDT</t>
+          <t>2026-09-29 16:08 PDT</t>
         </is>
       </c>
     </row>
@@ -5302,7 +5302,7 @@
       </c>
       <c r="D221" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 15:57 PDT</t>
+          <t>2026-09-29 16:08 PDT</t>
         </is>
       </c>
     </row>
@@ -5412,7 +5412,7 @@
       </c>
       <c r="D226" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 15:57 PDT</t>
+          <t>2026-09-29 16:08 PDT</t>
         </is>
       </c>
     </row>
@@ -5500,7 +5500,7 @@
       </c>
       <c r="D230" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 15:57 PDT</t>
+          <t>2026-09-29 16:08 PDT</t>
         </is>
       </c>
     </row>
@@ -5588,7 +5588,7 @@
       </c>
       <c r="D234" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 15:57 PDT</t>
+          <t>2026-09-29 16:08 PDT</t>
         </is>
       </c>
     </row>
@@ -6138,7 +6138,7 @@
       </c>
       <c r="D259" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 15:57 PDT</t>
+          <t>2026-09-29 16:08 PDT</t>
         </is>
       </c>
     </row>
@@ -6233,22 +6233,44 @@
     <row r="264">
       <c r="A264" s="2" t="inlineStr">
         <is>
+          <t>dbt/models/staging/kinetic/stg_kinetic__product_variants.sql</t>
+        </is>
+      </c>
+      <c r="B264" s="2" t="inlineStr">
+        <is>
+          <t>Code</t>
+        </is>
+      </c>
+      <c r="C264" s="3" t="inlineStr">
+        <is>
+          <t>Phase 2 staging (final table, 47 of 47): product variants with variant_option, price_adjustment_usd</t>
+        </is>
+      </c>
+      <c r="D264" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-29 16:08 PDT</t>
+        </is>
+      </c>
+    </row>
+    <row r="265">
+      <c r="A265" s="2" t="inlineStr">
+        <is>
           <t>dbt/models/staging/kinetic/_kinetic__staging.yml</t>
         </is>
       </c>
-      <c r="B264" s="2" t="inlineStr">
-        <is>
-          <t>Code</t>
-        </is>
-      </c>
-      <c r="C264" s="3" t="inlineStr">
+      <c r="B265" s="2" t="inlineStr">
+        <is>
+          <t>Code</t>
+        </is>
+      </c>
+      <c r="C265" s="3" t="inlineStr">
         <is>
           <t>Updated: tests for the 4 TikTok staging models -- all hand-verified against live data first</t>
         </is>
       </c>
-      <c r="D264" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-29 15:57 PDT</t>
+      <c r="D265" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-29 16:08 PDT</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add HANDOFF.md for new project/chat
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014EdkVLDs4dt6TCgduxMMyp
</commit_message>
<xml_diff>
--- a/File_Manifest.xlsx
+++ b/File_Manifest.xlsx
@@ -435,7 +435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D265"/>
+  <dimension ref="A1:D266"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="48" customWidth="1" min="1" max="1"/>
@@ -506,7 +506,7 @@
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 16:09 PDT</t>
+          <t>2026-09-29 16:18 PDT</t>
         </is>
       </c>
     </row>
@@ -638,7 +638,7 @@
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 16:09 PDT</t>
+          <t>2026-09-29 16:18 PDT</t>
         </is>
       </c>
     </row>
@@ -748,7 +748,7 @@
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 16:09 PDT</t>
+          <t>2026-09-29 16:18 PDT</t>
         </is>
       </c>
     </row>
@@ -6255,20 +6255,42 @@
     <row r="265">
       <c r="A265" s="2" t="inlineStr">
         <is>
+          <t>HANDOFF.md</t>
+        </is>
+      </c>
+      <c r="B265" s="2" t="inlineStr">
+        <is>
+          <t>Doc</t>
+        </is>
+      </c>
+      <c r="C265" s="3" t="inlineStr">
+        <is>
+          <t>Handoff note for starting a new chat/project: status, open decisions, prior decisions, pitfalls</t>
+        </is>
+      </c>
+      <c r="D265" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-29 16:18 PDT</t>
+        </is>
+      </c>
+    </row>
+    <row r="266">
+      <c r="A266" s="2" t="inlineStr">
+        <is>
           <t>dbt/models/staging/kinetic/_kinetic__staging.yml</t>
         </is>
       </c>
-      <c r="B265" s="2" t="inlineStr">
-        <is>
-          <t>Code</t>
-        </is>
-      </c>
-      <c r="C265" s="3" t="inlineStr">
+      <c r="B266" s="2" t="inlineStr">
+        <is>
+          <t>Code</t>
+        </is>
+      </c>
+      <c r="C266" s="3" t="inlineStr">
         <is>
           <t>Updated: tests for the 4 TikTok staging models -- all hand-verified against live data first</t>
         </is>
       </c>
-      <c r="D265" s="2" t="inlineStr">
+      <c r="D266" s="2" t="inlineStr">
         <is>
           <t>2026-09-29 16:08 PDT</t>
         </is>

</xml_diff>

<commit_message>
Work from the Data-to-Agents Playbook: HANDOFF rule, changelog, manifest
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011iLTiTsTyvHcVHREQNUg8N
</commit_message>
<xml_diff>
--- a/File_Manifest.xlsx
+++ b/File_Manifest.xlsx
@@ -506,7 +506,7 @@
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 16:18 PDT</t>
+          <t>2026-09-29 16:33 PDT</t>
         </is>
       </c>
     </row>
@@ -748,7 +748,7 @@
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 16:18 PDT</t>
+          <t>2026-09-29 16:33 PDT</t>
         </is>
       </c>
     </row>
@@ -6270,7 +6270,7 @@
       </c>
       <c r="D265" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 16:18 PDT</t>
+          <t>2026-09-29 16:33 PDT</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Phase 3: add int_customer_identity (email match + session back-fill)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011iLTiTsTyvHcVHREQNUg8N
</commit_message>
<xml_diff>
--- a/File_Manifest.xlsx
+++ b/File_Manifest.xlsx
@@ -435,7 +435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D266"/>
+  <dimension ref="A1:D267"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="48" customWidth="1" min="1" max="1"/>
@@ -506,7 +506,7 @@
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 16:33 PDT</t>
+          <t>2026-09-29 16:39 PDT</t>
         </is>
       </c>
     </row>
@@ -638,7 +638,7 @@
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 16:18 PDT</t>
+          <t>2026-09-29 16:39 PDT</t>
         </is>
       </c>
     </row>
@@ -748,7 +748,7 @@
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 16:33 PDT</t>
+          <t>2026-09-29 16:39 PDT</t>
         </is>
       </c>
     </row>
@@ -4400,7 +4400,7 @@
       </c>
       <c r="D180" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 16:09 PDT</t>
+          <t>2026-09-29 16:39 PDT</t>
         </is>
       </c>
     </row>
@@ -4593,12 +4593,12 @@
       </c>
       <c r="C189" s="3" t="inlineStr">
         <is>
-          <t>Tests for int_subscription_paid_periods</t>
+          <t>Descriptions and tests for all intermediate models</t>
         </is>
       </c>
       <c r="D189" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28 14:53 PDT</t>
+          <t>2026-09-29 16:39 PDT</t>
         </is>
       </c>
     </row>
@@ -4664,7 +4664,7 @@
       </c>
       <c r="D192" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 16:09 PDT</t>
+          <t>2026-09-29 16:39 PDT</t>
         </is>
       </c>
     </row>
@@ -4803,7 +4803,7 @@
     <row r="199">
       <c r="A199" s="2" t="inlineStr">
         <is>
-          <t>dbt/models/marts/mart_storefront_revenue_monthly.sql</t>
+          <t>dbt/models/intermediate/int_customer_identity.sql</t>
         </is>
       </c>
       <c r="B199" s="2" t="inlineStr">
@@ -4813,19 +4813,19 @@
       </c>
       <c r="C199" s="3" t="inlineStr">
         <is>
-          <t>Second canonical metric mart: non-subscription (course+merch) gross/net revenue, AOV, guest-checkout share, discount-usage share, refund rate by month -- validated against a hand-run equivalent query on the live database (2026-07: 246 orders, $13,843.71 gross revenue, $56.28 AOV)</t>
+          <t>Intermediate model: lookup from every web anonymous_id and account email to its customer (guest emails matched by email; anonymous sessions back-filled; deleted accounts excluded)</t>
         </is>
       </c>
       <c r="D199" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28 14:53 PDT</t>
+          <t>2026-09-29 16:39 PDT</t>
         </is>
       </c>
     </row>
     <row r="200">
       <c r="A200" s="2" t="inlineStr">
         <is>
-          <t>dbt/models/staging/kinetic/stg_kinetic__customer_addresses.sql</t>
+          <t>dbt/models/marts/mart_storefront_revenue_monthly.sql</t>
         </is>
       </c>
       <c r="B200" s="2" t="inlineStr">
@@ -4835,19 +4835,19 @@
       </c>
       <c r="C200" s="3" t="inlineStr">
         <is>
-          <t>Phase 2 staging (Customer 360): 1:1 pass-through of customer_addresses</t>
+          <t>Second canonical metric mart: non-subscription (course+merch) gross/net revenue, AOV, guest-checkout share, discount-usage share, refund rate by month -- validated against a hand-run equivalent query on the live database (2026-07: 246 orders, $13,843.71 gross revenue, $56.28 AOV)</t>
         </is>
       </c>
       <c r="D200" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 10:26 PDT</t>
+          <t>2026-09-28 14:53 PDT</t>
         </is>
       </c>
     </row>
     <row r="201">
       <c r="A201" s="2" t="inlineStr">
         <is>
-          <t>dbt/models/staging/kinetic/stg_kinetic__devices.sql</t>
+          <t>dbt/models/staging/kinetic/stg_kinetic__customer_addresses.sql</t>
         </is>
       </c>
       <c r="B201" s="2" t="inlineStr">
@@ -4857,7 +4857,7 @@
       </c>
       <c r="C201" s="3" t="inlineStr">
         <is>
-          <t>Phase 2 staging (Customer 360): 1:1 pass-through of devices, plus is_anonymous_device flag (customer_id null for ~94% of devices by design)</t>
+          <t>Phase 2 staging (Customer 360): 1:1 pass-through of customer_addresses</t>
         </is>
       </c>
       <c r="D201" s="2" t="inlineStr">
@@ -4869,7 +4869,7 @@
     <row r="202">
       <c r="A202" s="2" t="inlineStr">
         <is>
-          <t>dbt/models/staging/kinetic/stg_kinetic__identity_map.sql</t>
+          <t>dbt/models/staging/kinetic/stg_kinetic__devices.sql</t>
         </is>
       </c>
       <c r="B202" s="2" t="inlineStr">
@@ -4879,7 +4879,7 @@
       </c>
       <c r="C202" s="3" t="inlineStr">
         <is>
-          <t>Phase 2 staging (Customer 360): 1:1 pass-through of identity_map</t>
+          <t>Phase 2 staging (Customer 360): 1:1 pass-through of devices, plus is_anonymous_device flag (customer_id null for ~94% of devices by design)</t>
         </is>
       </c>
       <c r="D202" s="2" t="inlineStr">
@@ -4891,7 +4891,7 @@
     <row r="203">
       <c r="A203" s="2" t="inlineStr">
         <is>
-          <t>dbt/models/staging/kinetic/stg_kinetic__segments.sql</t>
+          <t>dbt/models/staging/kinetic/stg_kinetic__identity_map.sql</t>
         </is>
       </c>
       <c r="B203" s="2" t="inlineStr">
@@ -4901,7 +4901,7 @@
       </c>
       <c r="C203" s="3" t="inlineStr">
         <is>
-          <t>Phase 2 staging (Customer 360): 1:1 pass-through of segments</t>
+          <t>Phase 2 staging (Customer 360): 1:1 pass-through of identity_map</t>
         </is>
       </c>
       <c r="D203" s="2" t="inlineStr">
@@ -4913,7 +4913,7 @@
     <row r="204">
       <c r="A204" s="2" t="inlineStr">
         <is>
-          <t>dbt/models/staging/kinetic/stg_kinetic__customer_segment_membership.sql</t>
+          <t>dbt/models/staging/kinetic/stg_kinetic__segments.sql</t>
         </is>
       </c>
       <c r="B204" s="2" t="inlineStr">
@@ -4923,7 +4923,7 @@
       </c>
       <c r="C204" s="3" t="inlineStr">
         <is>
-          <t>Phase 2 staging (Customer 360): 1:1 pass-through of customer_segment_membership, plus is_current_member flag</t>
+          <t>Phase 2 staging (Customer 360): 1:1 pass-through of segments</t>
         </is>
       </c>
       <c r="D204" s="2" t="inlineStr">
@@ -4935,7 +4935,7 @@
     <row r="205">
       <c r="A205" s="2" t="inlineStr">
         <is>
-          <t>dbt/models/staging/kinetic/stg_kinetic__subscription_events.sql</t>
+          <t>dbt/models/staging/kinetic/stg_kinetic__customer_segment_membership.sql</t>
         </is>
       </c>
       <c r="B205" s="2" t="inlineStr">
@@ -4945,7 +4945,7 @@
       </c>
       <c r="C205" s="3" t="inlineStr">
         <is>
-          <t>Phase 2 staging (Customer 360): 1:1 pass-through of subscription_events; old_plan/new_plan renamed to old_plan_id/new_plan_id</t>
+          <t>Phase 2 staging (Customer 360): 1:1 pass-through of customer_segment_membership, plus is_current_member flag</t>
         </is>
       </c>
       <c r="D205" s="2" t="inlineStr">
@@ -4957,7 +4957,7 @@
     <row r="206">
       <c r="A206" s="2" t="inlineStr">
         <is>
-          <t>dbt/models/staging/kinetic/_kinetic__staging.yml</t>
+          <t>dbt/models/staging/kinetic/stg_kinetic__subscription_events.sql</t>
         </is>
       </c>
       <c r="B206" s="2" t="inlineStr">
@@ -4967,19 +4967,19 @@
       </c>
       <c r="C206" s="3" t="inlineStr">
         <is>
-          <t>Updated: tests for the 6 Customer 360 staging models (PK not_null/unique, FK relationships) -- all hand-verified against live data first</t>
+          <t>Phase 2 staging (Customer 360): 1:1 pass-through of subscription_events; old_plan/new_plan renamed to old_plan_id/new_plan_id</t>
         </is>
       </c>
       <c r="D206" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 16:08 PDT</t>
+          <t>2026-09-29 10:26 PDT</t>
         </is>
       </c>
     </row>
     <row r="207">
       <c r="A207" s="2" t="inlineStr">
         <is>
-          <t>dbt/models/staging/kinetic/stg_kinetic__web_sessions.sql</t>
+          <t>dbt/models/staging/kinetic/_kinetic__staging.yml</t>
         </is>
       </c>
       <c r="B207" s="2" t="inlineStr">
@@ -4989,19 +4989,19 @@
       </c>
       <c r="C207" s="3" t="inlineStr">
         <is>
-          <t>Phase 2 staging (web/app engagement): 1:1 pass-through of web_sessions, plus is_known_customer flag (customer_id null for ~79% of sessions by design)</t>
+          <t>Updated: tests for the 6 Customer 360 staging models (PK not_null/unique, FK relationships) -- all hand-verified against live data first</t>
         </is>
       </c>
       <c r="D207" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 12:58 PDT</t>
+          <t>2026-09-29 16:08 PDT</t>
         </is>
       </c>
     </row>
     <row r="208">
       <c r="A208" s="2" t="inlineStr">
         <is>
-          <t>dbt/models/staging/kinetic/stg_kinetic__web_events.sql</t>
+          <t>dbt/models/staging/kinetic/stg_kinetic__web_sessions.sql</t>
         </is>
       </c>
       <c r="B208" s="2" t="inlineStr">
@@ -5011,7 +5011,7 @@
       </c>
       <c r="C208" s="3" t="inlineStr">
         <is>
-          <t>Phase 2 staging (web/app engagement): 1:1 pass-through of web_events</t>
+          <t>Phase 2 staging (web/app engagement): 1:1 pass-through of web_sessions, plus is_known_customer flag (customer_id null for ~79% of sessions by design)</t>
         </is>
       </c>
       <c r="D208" s="2" t="inlineStr">
@@ -5023,7 +5023,7 @@
     <row r="209">
       <c r="A209" s="2" t="inlineStr">
         <is>
-          <t>dbt/models/staging/kinetic/stg_kinetic__app_sessions.sql</t>
+          <t>dbt/models/staging/kinetic/stg_kinetic__web_events.sql</t>
         </is>
       </c>
       <c r="B209" s="2" t="inlineStr">
@@ -5033,7 +5033,7 @@
       </c>
       <c r="C209" s="3" t="inlineStr">
         <is>
-          <t>Phase 2 staging (web/app engagement): 1:1 pass-through of app_sessions</t>
+          <t>Phase 2 staging (web/app engagement): 1:1 pass-through of web_events</t>
         </is>
       </c>
       <c r="D209" s="2" t="inlineStr">
@@ -5045,7 +5045,7 @@
     <row r="210">
       <c r="A210" s="2" t="inlineStr">
         <is>
-          <t>dbt/models/staging/kinetic/stg_kinetic__app_events.sql</t>
+          <t>dbt/models/staging/kinetic/stg_kinetic__app_sessions.sql</t>
         </is>
       </c>
       <c r="B210" s="2" t="inlineStr">
@@ -5055,7 +5055,7 @@
       </c>
       <c r="C210" s="3" t="inlineStr">
         <is>
-          <t>Phase 2 staging (web/app engagement): 1:1 pass-through of app_events</t>
+          <t>Phase 2 staging (web/app engagement): 1:1 pass-through of app_sessions</t>
         </is>
       </c>
       <c r="D210" s="2" t="inlineStr">
@@ -5067,7 +5067,7 @@
     <row r="211">
       <c r="A211" s="2" t="inlineStr">
         <is>
-          <t>dbt/models/staging/kinetic/_kinetic__staging.yml</t>
+          <t>dbt/models/staging/kinetic/stg_kinetic__app_events.sql</t>
         </is>
       </c>
       <c r="B211" s="2" t="inlineStr">
@@ -5077,19 +5077,19 @@
       </c>
       <c r="C211" s="3" t="inlineStr">
         <is>
-          <t>Updated: tests for the 4 web/app engagement staging models -- all hand-verified against live data first</t>
+          <t>Phase 2 staging (web/app engagement): 1:1 pass-through of app_events</t>
         </is>
       </c>
       <c r="D211" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 16:08 PDT</t>
+          <t>2026-09-29 12:58 PDT</t>
         </is>
       </c>
     </row>
     <row r="212">
       <c r="A212" s="2" t="inlineStr">
         <is>
-          <t>dbt/models/staging/kinetic/stg_kinetic__braze_email_campaigns.sql</t>
+          <t>dbt/models/staging/kinetic/_kinetic__staging.yml</t>
         </is>
       </c>
       <c r="B212" s="2" t="inlineStr">
@@ -5099,19 +5099,19 @@
       </c>
       <c r="C212" s="3" t="inlineStr">
         <is>
-          <t>Phase 2 staging (email/push): 1:1 pass-through of braze_email_campaigns</t>
+          <t>Updated: tests for the 4 web/app engagement staging models -- all hand-verified against live data first</t>
         </is>
       </c>
       <c r="D212" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 12:59 PDT</t>
+          <t>2026-09-29 16:08 PDT</t>
         </is>
       </c>
     </row>
     <row r="213">
       <c r="A213" s="2" t="inlineStr">
         <is>
-          <t>dbt/models/staging/kinetic/stg_kinetic__braze_push_campaigns.sql</t>
+          <t>dbt/models/staging/kinetic/stg_kinetic__braze_email_campaigns.sql</t>
         </is>
       </c>
       <c r="B213" s="2" t="inlineStr">
@@ -5121,7 +5121,7 @@
       </c>
       <c r="C213" s="3" t="inlineStr">
         <is>
-          <t>Phase 2 staging (email/push): 1:1 pass-through of braze_push_campaigns</t>
+          <t>Phase 2 staging (email/push): 1:1 pass-through of braze_email_campaigns</t>
         </is>
       </c>
       <c r="D213" s="2" t="inlineStr">
@@ -5133,7 +5133,7 @@
     <row r="214">
       <c r="A214" s="2" t="inlineStr">
         <is>
-          <t>dbt/models/staging/kinetic/stg_kinetic__braze_email_events.sql</t>
+          <t>dbt/models/staging/kinetic/stg_kinetic__braze_push_campaigns.sql</t>
         </is>
       </c>
       <c r="B214" s="2" t="inlineStr">
@@ -5143,7 +5143,7 @@
       </c>
       <c r="C214" s="3" t="inlineStr">
         <is>
-          <t>Phase 2 staging (email/push): braze_email_events with external_user_id renamed to customer_id and a short event_name (send/open/click/bounce/unsubscribe) alongside Braze's raw event_type</t>
+          <t>Phase 2 staging (email/push): 1:1 pass-through of braze_push_campaigns</t>
         </is>
       </c>
       <c r="D214" s="2" t="inlineStr">
@@ -5155,7 +5155,7 @@
     <row r="215">
       <c r="A215" s="2" t="inlineStr">
         <is>
-          <t>dbt/models/staging/kinetic/stg_kinetic__braze_push_events.sql</t>
+          <t>dbt/models/staging/kinetic/stg_kinetic__braze_email_events.sql</t>
         </is>
       </c>
       <c r="B215" s="2" t="inlineStr">
@@ -5165,7 +5165,7 @@
       </c>
       <c r="C215" s="3" t="inlineStr">
         <is>
-          <t>Phase 2 staging (email/push): braze_push_events with external_user_id renamed to customer_id and a short event_name alongside Braze's raw event_type</t>
+          <t>Phase 2 staging (email/push): braze_email_events with external_user_id renamed to customer_id and a short event_name (send/open/click/bounce/unsubscribe) alongside Braze's raw event_type</t>
         </is>
       </c>
       <c r="D215" s="2" t="inlineStr">
@@ -5177,7 +5177,7 @@
     <row r="216">
       <c r="A216" s="2" t="inlineStr">
         <is>
-          <t>dbt/models/staging/kinetic/_kinetic__staging.yml</t>
+          <t>dbt/models/staging/kinetic/stg_kinetic__braze_push_events.sql</t>
         </is>
       </c>
       <c r="B216" s="2" t="inlineStr">
@@ -5187,19 +5187,19 @@
       </c>
       <c r="C216" s="3" t="inlineStr">
         <is>
-          <t>Updated: tests for the 4 Braze staging models, incl. accepted_values on event_name -- all hand-verified against live data first</t>
+          <t>Phase 2 staging (email/push): braze_push_events with external_user_id renamed to customer_id and a short event_name alongside Braze's raw event_type</t>
         </is>
       </c>
       <c r="D216" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 16:08 PDT</t>
+          <t>2026-09-29 12:59 PDT</t>
         </is>
       </c>
     </row>
     <row r="217">
       <c r="A217" s="2" t="inlineStr">
         <is>
-          <t>dbt/models/staging/kinetic/stg_kinetic__meta_campaigns.sql</t>
+          <t>dbt/models/staging/kinetic/_kinetic__staging.yml</t>
         </is>
       </c>
       <c r="B217" s="2" t="inlineStr">
@@ -5209,19 +5209,19 @@
       </c>
       <c r="C217" s="3" t="inlineStr">
         <is>
-          <t>Phase 2 staging (paid media: Meta): meta_campaigns with budgets in both raw cents and dollars (Meta API stores budgets in cents)</t>
+          <t>Updated: tests for the 4 Braze staging models, incl. accepted_values on event_name -- all hand-verified against live data first</t>
         </is>
       </c>
       <c r="D217" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 13:02 PDT</t>
+          <t>2026-09-29 16:08 PDT</t>
         </is>
       </c>
     </row>
     <row r="218">
       <c r="A218" s="2" t="inlineStr">
         <is>
-          <t>dbt/models/staging/kinetic/stg_kinetic__meta_ads.sql</t>
+          <t>dbt/models/staging/kinetic/stg_kinetic__meta_campaigns.sql</t>
         </is>
       </c>
       <c r="B218" s="2" t="inlineStr">
@@ -5231,7 +5231,7 @@
       </c>
       <c r="C218" s="3" t="inlineStr">
         <is>
-          <t>Phase 2 staging (paid media: Meta): 1:1 pass-through of meta_ads</t>
+          <t>Phase 2 staging (paid media: Meta): meta_campaigns with budgets in both raw cents and dollars (Meta API stores budgets in cents)</t>
         </is>
       </c>
       <c r="D218" s="2" t="inlineStr">
@@ -5243,7 +5243,7 @@
     <row r="219">
       <c r="A219" s="2" t="inlineStr">
         <is>
-          <t>dbt/models/staging/kinetic/stg_kinetic__meta_ad_insights_daily.sql</t>
+          <t>dbt/models/staging/kinetic/stg_kinetic__meta_ads.sql</t>
         </is>
       </c>
       <c r="B219" s="2" t="inlineStr">
@@ -5253,7 +5253,7 @@
       </c>
       <c r="C219" s="3" t="inlineStr">
         <is>
-          <t>Phase 2 staging (paid media: Meta): meta_ad_insights_daily with a combined ad_day_id key, unit-suffixed columns (spend_usd, cpm_usd, cpc_usd) and ctr renamed ctr_fraction (0.017 = 1.7%)</t>
+          <t>Phase 2 staging (paid media: Meta): 1:1 pass-through of meta_ads</t>
         </is>
       </c>
       <c r="D219" s="2" t="inlineStr">
@@ -5265,7 +5265,7 @@
     <row r="220">
       <c r="A220" s="2" t="inlineStr">
         <is>
-          <t>dbt/models/staging/kinetic/stg_kinetic__meta_ad_actions_daily.sql</t>
+          <t>dbt/models/staging/kinetic/stg_kinetic__meta_ad_insights_daily.sql</t>
         </is>
       </c>
       <c r="B220" s="2" t="inlineStr">
@@ -5275,7 +5275,7 @@
       </c>
       <c r="C220" s="3" t="inlineStr">
         <is>
-          <t>Phase 2 staging (paid media: Meta): meta_ad_actions_daily with a combined ad_day_action_id key; value renamed action_count</t>
+          <t>Phase 2 staging (paid media: Meta): meta_ad_insights_daily with a combined ad_day_id key, unit-suffixed columns (spend_usd, cpm_usd, cpc_usd) and ctr renamed ctr_fraction (0.017 = 1.7%)</t>
         </is>
       </c>
       <c r="D220" s="2" t="inlineStr">
@@ -5287,7 +5287,7 @@
     <row r="221">
       <c r="A221" s="2" t="inlineStr">
         <is>
-          <t>dbt/models/staging/kinetic/_kinetic__staging.yml</t>
+          <t>dbt/models/staging/kinetic/stg_kinetic__meta_ad_actions_daily.sql</t>
         </is>
       </c>
       <c r="B221" s="2" t="inlineStr">
@@ -5297,19 +5297,19 @@
       </c>
       <c r="C221" s="3" t="inlineStr">
         <is>
-          <t>Updated: tests for the 4 Meta staging models, incl. uniqueness of the combined daily keys -- all hand-verified against live data first</t>
+          <t>Phase 2 staging (paid media: Meta): meta_ad_actions_daily with a combined ad_day_action_id key; value renamed action_count</t>
         </is>
       </c>
       <c r="D221" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 16:08 PDT</t>
+          <t>2026-09-29 13:02 PDT</t>
         </is>
       </c>
     </row>
     <row r="222">
       <c r="A222" s="2" t="inlineStr">
         <is>
-          <t>dbt/models/staging/kinetic/stg_kinetic__google_search_campaigns.sql</t>
+          <t>dbt/models/staging/kinetic/_kinetic__staging.yml</t>
         </is>
       </c>
       <c r="B222" s="2" t="inlineStr">
@@ -5319,19 +5319,19 @@
       </c>
       <c r="C222" s="3" t="inlineStr">
         <is>
-          <t>Phase 2 staging (paid media: Google Search): campaigns with the raw customer_id renamed google_ads_account_id (it's the Google Ads account number, not a Kinetic customer), daily budget in micros and dollars, end_date cast back to a date</t>
+          <t>Updated: tests for the 4 Meta staging models, incl. uniqueness of the combined daily keys -- all hand-verified against live data first</t>
         </is>
       </c>
       <c r="D222" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 13:13 PDT</t>
+          <t>2026-09-29 16:08 PDT</t>
         </is>
       </c>
     </row>
     <row r="223">
       <c r="A223" s="2" t="inlineStr">
         <is>
-          <t>dbt/models/staging/kinetic/stg_kinetic__google_search_ad_groups.sql</t>
+          <t>dbt/models/staging/kinetic/stg_kinetic__google_search_campaigns.sql</t>
         </is>
       </c>
       <c r="B223" s="2" t="inlineStr">
@@ -5341,7 +5341,7 @@
       </c>
       <c r="C223" s="3" t="inlineStr">
         <is>
-          <t>Phase 2 staging (paid media: Google Search): ad groups; cpc_bid_micros cast back to a number (always empty -- automated bidding)</t>
+          <t>Phase 2 staging (paid media: Google Search): campaigns with the raw customer_id renamed google_ads_account_id (it's the Google Ads account number, not a Kinetic customer), daily budget in micros and dollars, end_date cast back to a date</t>
         </is>
       </c>
       <c r="D223" s="2" t="inlineStr">
@@ -5353,7 +5353,7 @@
     <row r="224">
       <c r="A224" s="2" t="inlineStr">
         <is>
-          <t>dbt/models/staging/kinetic/stg_kinetic__google_search_performance_daily.sql</t>
+          <t>dbt/models/staging/kinetic/stg_kinetic__google_search_ad_groups.sql</t>
         </is>
       </c>
       <c r="B224" s="2" t="inlineStr">
@@ -5363,7 +5363,7 @@
       </c>
       <c r="C224" s="3" t="inlineStr">
         <is>
-          <t>Phase 2 staging (paid media: Google Search): ad-group-day performance with combined ad_group_day_id key, cost converted from micros to dollars, ctr_fraction. The keyword table rolled up -- never add the two together</t>
+          <t>Phase 2 staging (paid media: Google Search): ad groups; cpc_bid_micros cast back to a number (always empty -- automated bidding)</t>
         </is>
       </c>
       <c r="D224" s="2" t="inlineStr">
@@ -5375,7 +5375,7 @@
     <row r="225">
       <c r="A225" s="2" t="inlineStr">
         <is>
-          <t>dbt/models/staging/kinetic/stg_kinetic__google_search_keyword_performance_daily.sql</t>
+          <t>dbt/models/staging/kinetic/stg_kinetic__google_search_performance_daily.sql</t>
         </is>
       </c>
       <c r="B225" s="2" t="inlineStr">
@@ -5385,7 +5385,7 @@
       </c>
       <c r="C225" s="3" t="inlineStr">
         <is>
-          <t>Phase 2 staging (paid media: Google Search): keyword-day performance with combined keyword_day_id key, cost converted from micros to dollars, ctr_fraction</t>
+          <t>Phase 2 staging (paid media: Google Search): ad-group-day performance with combined ad_group_day_id key, cost converted from micros to dollars, ctr_fraction. The keyword table rolled up -- never add the two together</t>
         </is>
       </c>
       <c r="D225" s="2" t="inlineStr">
@@ -5397,7 +5397,7 @@
     <row r="226">
       <c r="A226" s="2" t="inlineStr">
         <is>
-          <t>dbt/models/staging/kinetic/_kinetic__staging.yml</t>
+          <t>dbt/models/staging/kinetic/stg_kinetic__google_search_keyword_performance_daily.sql</t>
         </is>
       </c>
       <c r="B226" s="2" t="inlineStr">
@@ -5407,19 +5407,19 @@
       </c>
       <c r="C226" s="3" t="inlineStr">
         <is>
-          <t>Updated: tests for the 4 Google Search staging models -- all hand-verified against live data first</t>
+          <t>Phase 2 staging (paid media: Google Search): keyword-day performance with combined keyword_day_id key, cost converted from micros to dollars, ctr_fraction</t>
         </is>
       </c>
       <c r="D226" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 16:08 PDT</t>
+          <t>2026-09-29 13:13 PDT</t>
         </is>
       </c>
     </row>
     <row r="227">
       <c r="A227" s="2" t="inlineStr">
         <is>
-          <t>dbt/models/staging/kinetic/stg_kinetic__youtube_campaigns.sql</t>
+          <t>dbt/models/staging/kinetic/_kinetic__staging.yml</t>
         </is>
       </c>
       <c r="B227" s="2" t="inlineStr">
@@ -5429,19 +5429,19 @@
       </c>
       <c r="C227" s="3" t="inlineStr">
         <is>
-          <t>Phase 2 staging (paid media: YouTube): campaigns with customer_id renamed google_ads_account_id (the ad account, not a Kinetic customer), budgets in micros and dollars</t>
+          <t>Updated: tests for the 4 Google Search staging models -- all hand-verified against live data first</t>
         </is>
       </c>
       <c r="D227" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 13:14 PDT</t>
+          <t>2026-09-29 16:08 PDT</t>
         </is>
       </c>
     </row>
     <row r="228">
       <c r="A228" s="2" t="inlineStr">
         <is>
-          <t>dbt/models/staging/kinetic/stg_kinetic__youtube_ad_groups.sql</t>
+          <t>dbt/models/staging/kinetic/stg_kinetic__youtube_campaigns.sql</t>
         </is>
       </c>
       <c r="B228" s="2" t="inlineStr">
@@ -5451,7 +5451,7 @@
       </c>
       <c r="C228" s="3" t="inlineStr">
         <is>
-          <t>Phase 2 staging (paid media: YouTube): 1:1 pass-through of youtube_ad_groups</t>
+          <t>Phase 2 staging (paid media: YouTube): campaigns with customer_id renamed google_ads_account_id (the ad account, not a Kinetic customer), budgets in micros and dollars</t>
         </is>
       </c>
       <c r="D228" s="2" t="inlineStr">
@@ -5463,7 +5463,7 @@
     <row r="229">
       <c r="A229" s="2" t="inlineStr">
         <is>
-          <t>dbt/models/staging/kinetic/stg_kinetic__youtube_performance_daily.sql</t>
+          <t>dbt/models/staging/kinetic/stg_kinetic__youtube_ad_groups.sql</t>
         </is>
       </c>
       <c r="B229" s="2" t="inlineStr">
@@ -5473,7 +5473,7 @@
       </c>
       <c r="C229" s="3" t="inlineStr">
         <is>
-          <t>Phase 2 staging (paid media: YouTube): ad-group-day performance with combined ad_group_day_id key, cost and cost-per-view converted from micros to dollars, video_view_rate_fraction</t>
+          <t>Phase 2 staging (paid media: YouTube): 1:1 pass-through of youtube_ad_groups</t>
         </is>
       </c>
       <c r="D229" s="2" t="inlineStr">
@@ -5485,7 +5485,7 @@
     <row r="230">
       <c r="A230" s="2" t="inlineStr">
         <is>
-          <t>dbt/models/staging/kinetic/_kinetic__staging.yml</t>
+          <t>dbt/models/staging/kinetic/stg_kinetic__youtube_performance_daily.sql</t>
         </is>
       </c>
       <c r="B230" s="2" t="inlineStr">
@@ -5495,19 +5495,19 @@
       </c>
       <c r="C230" s="3" t="inlineStr">
         <is>
-          <t>Updated: tests for the 3 YouTube staging models -- all hand-verified against live data first</t>
+          <t>Phase 2 staging (paid media: YouTube): ad-group-day performance with combined ad_group_day_id key, cost and cost-per-view converted from micros to dollars, video_view_rate_fraction</t>
         </is>
       </c>
       <c r="D230" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 16:08 PDT</t>
+          <t>2026-09-29 13:14 PDT</t>
         </is>
       </c>
     </row>
     <row r="231">
       <c r="A231" s="2" t="inlineStr">
         <is>
-          <t>dbt/models/staging/kinetic/stg_kinetic__dv360_insertion_orders.sql</t>
+          <t>dbt/models/staging/kinetic/_kinetic__staging.yml</t>
         </is>
       </c>
       <c r="B231" s="2" t="inlineStr">
@@ -5517,19 +5517,19 @@
       </c>
       <c r="C231" s="3" t="inlineStr">
         <is>
-          <t>Phase 2 staging (paid media: DV360): insertion orders with budget_micros named monthly_budget_* (it's a monthly budget), end_date cast back to a date; flags the flat-budget-vs-growing-spend known issue</t>
+          <t>Updated: tests for the 3 YouTube staging models -- all hand-verified against live data first</t>
         </is>
       </c>
       <c r="D231" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 13:27 PDT</t>
+          <t>2026-09-29 16:08 PDT</t>
         </is>
       </c>
     </row>
     <row r="232">
       <c r="A232" s="2" t="inlineStr">
         <is>
-          <t>dbt/models/staging/kinetic/stg_kinetic__dv360_line_items.sql</t>
+          <t>dbt/models/staging/kinetic/stg_kinetic__dv360_insertion_orders.sql</t>
         </is>
       </c>
       <c r="B232" s="2" t="inlineStr">
@@ -5539,19 +5539,19 @@
       </c>
       <c r="C232" s="3" t="inlineStr">
         <is>
-          <t>Phase 2 staging (paid media: DV360): 1:1 pass-through of dv360_line_items</t>
+          <t>Phase 2 staging (paid media: DV360): insertion orders with budget_micros named monthly_budget_* (it's a monthly budget), end_date cast back to a date; flags the flat-budget-vs-growing-spend known issue</t>
         </is>
       </c>
       <c r="D232" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 13:19 PDT</t>
+          <t>2026-09-29 13:27 PDT</t>
         </is>
       </c>
     </row>
     <row r="233">
       <c r="A233" s="2" t="inlineStr">
         <is>
-          <t>dbt/models/staging/kinetic/stg_kinetic__dv360_performance_daily.sql</t>
+          <t>dbt/models/staging/kinetic/stg_kinetic__dv360_line_items.sql</t>
         </is>
       </c>
       <c r="B233" s="2" t="inlineStr">
@@ -5561,7 +5561,7 @@
       </c>
       <c r="C233" s="3" t="inlineStr">
         <is>
-          <t>Phase 2 staging (paid media: DV360): line-item x day x exchange x environment performance with combined line_item_day_slice_id key, micros converted to dollars, ctr_fraction</t>
+          <t>Phase 2 staging (paid media: DV360): 1:1 pass-through of dv360_line_items</t>
         </is>
       </c>
       <c r="D233" s="2" t="inlineStr">
@@ -5573,7 +5573,7 @@
     <row r="234">
       <c r="A234" s="2" t="inlineStr">
         <is>
-          <t>dbt/models/staging/kinetic/_kinetic__staging.yml</t>
+          <t>dbt/models/staging/kinetic/stg_kinetic__dv360_performance_daily.sql</t>
         </is>
       </c>
       <c r="B234" s="2" t="inlineStr">
@@ -5583,19 +5583,19 @@
       </c>
       <c r="C234" s="3" t="inlineStr">
         <is>
-          <t>Updated: tests for the 3 DV360 staging models, incl. accepted_values on exchange and environment -- all hand-verified against live data first</t>
+          <t>Phase 2 staging (paid media: DV360): line-item x day x exchange x environment performance with combined line_item_day_slice_id key, micros converted to dollars, ctr_fraction</t>
         </is>
       </c>
       <c r="D234" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 16:08 PDT</t>
+          <t>2026-09-29 13:19 PDT</t>
         </is>
       </c>
     </row>
     <row r="235">
       <c r="A235" s="2" t="inlineStr">
         <is>
-          <t>generator/params.py</t>
+          <t>dbt/models/staging/kinetic/_kinetic__staging.yml</t>
         </is>
       </c>
       <c r="B235" s="2" t="inlineStr">
@@ -5605,41 +5605,41 @@
       </c>
       <c r="C235" s="3" t="inlineStr">
         <is>
-          <t>Updated 2026-09-29: every evergreen ad budget on all 6 platforms is now the campaign's CURRENT budget, sized from realized spend (weekly average &lt;= budget, no day &gt; 1.75x; DV360 monthly &gt;= highest month). The old flat 'typical day' budgets let later months spend up to ~20x the stored budget</t>
+          <t>Updated: tests for the 3 DV360 staging models, incl. accepted_values on exchange and environment -- all hand-verified against live data first</t>
         </is>
       </c>
       <c r="D235" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 13:23 PDT</t>
+          <t>2026-09-29 16:08 PDT</t>
         </is>
       </c>
     </row>
     <row r="236">
       <c r="A236" s="2" t="inlineStr">
         <is>
-          <t>data/meta_campaigns.csv</t>
+          <t>generator/params.py</t>
         </is>
       </c>
       <c r="B236" s="2" t="inlineStr">
         <is>
-          <t>Shipped table</t>
+          <t>Code</t>
         </is>
       </c>
       <c r="C236" s="3" t="inlineStr">
         <is>
-          <t>Regenerated 2026-09-29: evergreen daily_budget values updated to current budgets (only that column, only the 4 evergreen rows changed)</t>
+          <t>Updated 2026-09-29: every evergreen ad budget on all 6 platforms is now the campaign's CURRENT budget, sized from realized spend (weekly average &lt;= budget, no day &gt; 1.75x; DV360 monthly &gt;= highest month). The old flat 'typical day' budgets let later months spend up to ~20x the stored budget</t>
         </is>
       </c>
       <c r="D236" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 13:24 PDT</t>
+          <t>2026-09-29 13:23 PDT</t>
         </is>
       </c>
     </row>
     <row r="237">
       <c r="A237" s="2" t="inlineStr">
         <is>
-          <t>data/google_search_campaigns.csv</t>
+          <t>data/meta_campaigns.csv</t>
         </is>
       </c>
       <c r="B237" s="2" t="inlineStr">
@@ -5649,7 +5649,7 @@
       </c>
       <c r="C237" s="3" t="inlineStr">
         <is>
-          <t>Regenerated 2026-09-29: campaign_budget_micros updated to current budgets (only that column changed)</t>
+          <t>Regenerated 2026-09-29: evergreen daily_budget values updated to current budgets (only that column, only the 4 evergreen rows changed)</t>
         </is>
       </c>
       <c r="D237" s="2" t="inlineStr">
@@ -5661,7 +5661,7 @@
     <row r="238">
       <c r="A238" s="2" t="inlineStr">
         <is>
-          <t>data/youtube_campaigns.csv</t>
+          <t>data/google_search_campaigns.csv</t>
         </is>
       </c>
       <c r="B238" s="2" t="inlineStr">
@@ -5671,7 +5671,7 @@
       </c>
       <c r="C238" s="3" t="inlineStr">
         <is>
-          <t>Regenerated 2026-09-29: evergreen campaign_budget_micros updated to current budgets (only that column, only the 4 evergreen rows changed)</t>
+          <t>Regenerated 2026-09-29: campaign_budget_micros updated to current budgets (only that column changed)</t>
         </is>
       </c>
       <c r="D238" s="2" t="inlineStr">
@@ -5683,7 +5683,7 @@
     <row r="239">
       <c r="A239" s="2" t="inlineStr">
         <is>
-          <t>data/dv360_insertion_orders.csv</t>
+          <t>data/youtube_campaigns.csv</t>
         </is>
       </c>
       <c r="B239" s="2" t="inlineStr">
@@ -5693,7 +5693,7 @@
       </c>
       <c r="C239" s="3" t="inlineStr">
         <is>
-          <t>Regenerated 2026-09-29: monthly budget_micros updated to current budgets (only that column changed)</t>
+          <t>Regenerated 2026-09-29: evergreen campaign_budget_micros updated to current budgets (only that column, only the 4 evergreen rows changed)</t>
         </is>
       </c>
       <c r="D239" s="2" t="inlineStr">
@@ -5705,7 +5705,7 @@
     <row r="240">
       <c r="A240" s="2" t="inlineStr">
         <is>
-          <t>data/snap_campaigns.csv</t>
+          <t>data/dv360_insertion_orders.csv</t>
         </is>
       </c>
       <c r="B240" s="2" t="inlineStr">
@@ -5715,7 +5715,7 @@
       </c>
       <c r="C240" s="3" t="inlineStr">
         <is>
-          <t>Regenerated 2026-09-29: evergreen daily_budget_micro updated to current budgets (only that column, only the 4 evergreen rows changed)</t>
+          <t>Regenerated 2026-09-29: monthly budget_micros updated to current budgets (only that column changed)</t>
         </is>
       </c>
       <c r="D240" s="2" t="inlineStr">
@@ -5727,7 +5727,7 @@
     <row r="241">
       <c r="A241" s="2" t="inlineStr">
         <is>
-          <t>data/tiktok_campaigns.csv</t>
+          <t>data/snap_campaigns.csv</t>
         </is>
       </c>
       <c r="B241" s="2" t="inlineStr">
@@ -5737,7 +5737,7 @@
       </c>
       <c r="C241" s="3" t="inlineStr">
         <is>
-          <t>Regenerated 2026-09-29: BUDGET_MODE_DAY budget_micro updated to current budgets (only that column, only the 4 evergreen rows changed)</t>
+          <t>Regenerated 2026-09-29: evergreen daily_budget_micro updated to current budgets (only that column, only the 4 evergreen rows changed)</t>
         </is>
       </c>
       <c r="D241" s="2" t="inlineStr">
@@ -5749,29 +5749,29 @@
     <row r="242">
       <c r="A242" s="2" t="inlineStr">
         <is>
-          <t>generator/audit_cross_dataset_alignment.py</t>
+          <t>data/tiktok_campaigns.csv</t>
         </is>
       </c>
       <c r="B242" s="2" t="inlineStr">
         <is>
-          <t>Code</t>
+          <t>Shipped table</t>
         </is>
       </c>
       <c r="C242" s="3" t="inlineStr">
         <is>
-          <t>Updated 2026-09-29: new Check 8 -- spend vs stored budget for every campaign on all 6 platforms (weekly/daily limits for daily budgets, monthly for DV360, total for holiday flights)</t>
+          <t>Regenerated 2026-09-29: BUDGET_MODE_DAY budget_micro updated to current budgets (only that column, only the 4 evergreen rows changed)</t>
         </is>
       </c>
       <c r="D242" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 13:30 PDT</t>
+          <t>2026-09-29 13:24 PDT</t>
         </is>
       </c>
     </row>
     <row r="243">
       <c r="A243" s="2" t="inlineStr">
         <is>
-          <t>dbt/models/staging/kinetic/stg_kinetic__dv360_insertion_orders.sql</t>
+          <t>generator/audit_cross_dataset_alignment.py</t>
         </is>
       </c>
       <c r="B243" s="2" t="inlineStr">
@@ -5781,19 +5781,19 @@
       </c>
       <c r="C243" s="3" t="inlineStr">
         <is>
-          <t>Updated: budget known-issue note replaced -- budgets are now current budgets</t>
+          <t>Updated 2026-09-29: new Check 8 -- spend vs stored budget for every campaign on all 6 platforms (weekly/daily limits for daily budgets, monthly for DV360, total for holiday flights)</t>
         </is>
       </c>
       <c r="D243" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 13:27 PDT</t>
+          <t>2026-09-29 13:30 PDT</t>
         </is>
       </c>
     </row>
     <row r="244">
       <c r="A244" s="2" t="inlineStr">
         <is>
-          <t>generator/paid_media_common.py</t>
+          <t>dbt/models/staging/kinetic/stg_kinetic__dv360_insertion_orders.sql</t>
         </is>
       </c>
       <c r="B244" s="2" t="inlineStr">
@@ -5803,19 +5803,19 @@
       </c>
       <c r="C244" s="3" t="inlineStr">
         <is>
-          <t>Updated 2026-09-29: new cap_flight_at_budget() -- rescales a holiday flight's days so it never spends past its lifetime budget, replaying the same random rates so every other row is unchanged</t>
+          <t>Updated: budget known-issue note replaced -- budgets are now current budgets</t>
         </is>
       </c>
       <c r="D244" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 13:29 PDT</t>
+          <t>2026-09-29 13:27 PDT</t>
         </is>
       </c>
     </row>
     <row r="245">
       <c r="A245" s="2" t="inlineStr">
         <is>
-          <t>generator/build_meta_ad_insights_daily.py</t>
+          <t>generator/paid_media_common.py</t>
         </is>
       </c>
       <c r="B245" s="2" t="inlineStr">
@@ -5825,7 +5825,7 @@
       </c>
       <c r="C245" s="3" t="inlineStr">
         <is>
-          <t>Updated 2026-09-29: holiday flights capped at their lifetime budget via cap_flight_at_budget()</t>
+          <t>Updated 2026-09-29: new cap_flight_at_budget() -- rescales a holiday flight's days so it never spends past its lifetime budget, replaying the same random rates so every other row is unchanged</t>
         </is>
       </c>
       <c r="D245" s="2" t="inlineStr">
@@ -5837,7 +5837,7 @@
     <row r="246">
       <c r="A246" s="2" t="inlineStr">
         <is>
-          <t>generator/build_snap_stats_daily.py</t>
+          <t>generator/build_meta_ad_insights_daily.py</t>
         </is>
       </c>
       <c r="B246" s="2" t="inlineStr">
@@ -5859,7 +5859,7 @@
     <row r="247">
       <c r="A247" s="2" t="inlineStr">
         <is>
-          <t>generator/build_tiktok_reports_daily.py</t>
+          <t>generator/build_snap_stats_daily.py</t>
         </is>
       </c>
       <c r="B247" s="2" t="inlineStr">
@@ -5881,7 +5881,7 @@
     <row r="248">
       <c r="A248" s="2" t="inlineStr">
         <is>
-          <t>generator/build_youtube_performance_daily.py</t>
+          <t>generator/build_tiktok_reports_daily.py</t>
         </is>
       </c>
       <c r="B248" s="2" t="inlineStr">
@@ -5891,7 +5891,7 @@
       </c>
       <c r="C248" s="3" t="inlineStr">
         <is>
-          <t>Updated 2026-09-29: holiday flights capped at their lifetime budget via cap_flight_at_budget() (no-op today -- all YouTube flights were already under budget)</t>
+          <t>Updated 2026-09-29: holiday flights capped at their lifetime budget via cap_flight_at_budget()</t>
         </is>
       </c>
       <c r="D248" s="2" t="inlineStr">
@@ -5903,17 +5903,17 @@
     <row r="249">
       <c r="A249" s="2" t="inlineStr">
         <is>
-          <t>data/meta_ad_insights_daily.csv</t>
+          <t>generator/build_youtube_performance_daily.py</t>
         </is>
       </c>
       <c r="B249" s="2" t="inlineStr">
         <is>
-          <t>Shipped table</t>
+          <t>Code</t>
         </is>
       </c>
       <c r="C249" s="3" t="inlineStr">
         <is>
-          <t>Regenerated 2026-09-29: the 2023 and 2024 holiday flights (38 rows) trimmed to spend exactly their lifetime budget; every other row identical</t>
+          <t>Updated 2026-09-29: holiday flights capped at their lifetime budget via cap_flight_at_budget() (no-op today -- all YouTube flights were already under budget)</t>
         </is>
       </c>
       <c r="D249" s="2" t="inlineStr">
@@ -5925,7 +5925,7 @@
     <row r="250">
       <c r="A250" s="2" t="inlineStr">
         <is>
-          <t>data/meta_ad_actions_daily.csv</t>
+          <t>data/meta_ad_insights_daily.csv</t>
         </is>
       </c>
       <c r="B250" s="2" t="inlineStr">
@@ -5935,7 +5935,7 @@
       </c>
       <c r="C250" s="3" t="inlineStr">
         <is>
-          <t>Regenerated 2026-09-29: re-derived from the trimmed insights rows -- only the 2023/2024 holiday flights' action rows changed (one initiate_checkout row on 2024-11-15 dropped to zero and is no longer emitted)</t>
+          <t>Regenerated 2026-09-29: the 2023 and 2024 holiday flights (38 rows) trimmed to spend exactly their lifetime budget; every other row identical</t>
         </is>
       </c>
       <c r="D250" s="2" t="inlineStr">
@@ -5947,7 +5947,7 @@
     <row r="251">
       <c r="A251" s="2" t="inlineStr">
         <is>
-          <t>data/snap_stats_daily.csv</t>
+          <t>data/meta_ad_actions_daily.csv</t>
         </is>
       </c>
       <c r="B251" s="2" t="inlineStr">
@@ -5957,7 +5957,7 @@
       </c>
       <c r="C251" s="3" t="inlineStr">
         <is>
-          <t>Regenerated 2026-09-29: the 2024 holiday flight (19 rows) trimmed to spend exactly its lifetime budget; every other row identical</t>
+          <t>Regenerated 2026-09-29: re-derived from the trimmed insights rows -- only the 2023/2024 holiday flights' action rows changed (one initiate_checkout row on 2024-11-15 dropped to zero and is no longer emitted)</t>
         </is>
       </c>
       <c r="D251" s="2" t="inlineStr">
@@ -5969,7 +5969,7 @@
     <row r="252">
       <c r="A252" s="2" t="inlineStr">
         <is>
-          <t>data/tiktok_reports_daily.csv</t>
+          <t>data/snap_stats_daily.csv</t>
         </is>
       </c>
       <c r="B252" s="2" t="inlineStr">
@@ -5979,7 +5979,7 @@
       </c>
       <c r="C252" s="3" t="inlineStr">
         <is>
-          <t>Regenerated 2026-09-29: the 2023/2024/2025 holiday flights (56 rows) trimmed to spend exactly their lifetime budgets; every other row identical</t>
+          <t>Regenerated 2026-09-29: the 2024 holiday flight (19 rows) trimmed to spend exactly its lifetime budget; every other row identical</t>
         </is>
       </c>
       <c r="D252" s="2" t="inlineStr">
@@ -5991,51 +5991,51 @@
     <row r="253">
       <c r="A253" s="2" t="inlineStr">
         <is>
-          <t>docs/cross_dataset_alignment_audit.md</t>
+          <t>data/tiktok_reports_daily.csv</t>
         </is>
       </c>
       <c r="B253" s="2" t="inlineStr">
         <is>
-          <t>Docs</t>
+          <t>Shipped table</t>
         </is>
       </c>
       <c r="C253" s="3" t="inlineStr">
         <is>
-          <t>Updated 2026-09-29: added Check 8 (spend vs stored budget) with both fixes and results</t>
+          <t>Regenerated 2026-09-29: the 2023/2024/2025 holiday flights (56 rows) trimmed to spend exactly their lifetime budgets; every other row identical</t>
         </is>
       </c>
       <c r="D253" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 13:54 PDT</t>
+          <t>2026-09-29 13:29 PDT</t>
         </is>
       </c>
     </row>
     <row r="254">
       <c r="A254" s="2" t="inlineStr">
         <is>
-          <t>generator/audit_cross_dataset_alignment.py</t>
+          <t>docs/cross_dataset_alignment_audit.md</t>
         </is>
       </c>
       <c r="B254" s="2" t="inlineStr">
         <is>
-          <t>Code</t>
+          <t>Docs</t>
         </is>
       </c>
       <c r="C254" s="3" t="inlineStr">
         <is>
-          <t>Updated 2026-09-29: Check 8's flight limit tightened from 1.05x to 1.0x now that flights are capped</t>
+          <t>Updated 2026-09-29: added Check 8 (spend vs stored budget) with both fixes and results</t>
         </is>
       </c>
       <c r="D254" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 13:30 PDT</t>
+          <t>2026-09-29 13:54 PDT</t>
         </is>
       </c>
     </row>
     <row r="255">
       <c r="A255" s="2" t="inlineStr">
         <is>
-          <t>dbt/models/staging/kinetic/stg_kinetic__snap_campaigns.sql</t>
+          <t>generator/audit_cross_dataset_alignment.py</t>
         </is>
       </c>
       <c r="B255" s="2" t="inlineStr">
@@ -6045,19 +6045,19 @@
       </c>
       <c r="C255" s="3" t="inlineStr">
         <is>
-          <t>Phase 2 staging (paid media: Snap): campaigns with ad_account_id renamed snap_ad_account_id, current budgets in micros and dollars</t>
+          <t>Updated 2026-09-29: Check 8's flight limit tightened from 1.05x to 1.0x now that flights are capped</t>
         </is>
       </c>
       <c r="D255" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 15:53 PDT</t>
+          <t>2026-09-29 13:30 PDT</t>
         </is>
       </c>
     </row>
     <row r="256">
       <c r="A256" s="2" t="inlineStr">
         <is>
-          <t>dbt/models/staging/kinetic/stg_kinetic__snap_ad_squads.sql</t>
+          <t>dbt/models/staging/kinetic/stg_kinetic__snap_campaigns.sql</t>
         </is>
       </c>
       <c r="B256" s="2" t="inlineStr">
@@ -6067,7 +6067,7 @@
       </c>
       <c r="C256" s="3" t="inlineStr">
         <is>
-          <t>Phase 2 staging (paid media: Snap): 1:1 pass-through of snap_ad_squads (Snap's ad set / ad group level)</t>
+          <t>Phase 2 staging (paid media: Snap): campaigns with ad_account_id renamed snap_ad_account_id, current budgets in micros and dollars</t>
         </is>
       </c>
       <c r="D256" s="2" t="inlineStr">
@@ -6079,7 +6079,7 @@
     <row r="257">
       <c r="A257" s="2" t="inlineStr">
         <is>
-          <t>dbt/models/staging/kinetic/stg_kinetic__snap_ads.sql</t>
+          <t>dbt/models/staging/kinetic/stg_kinetic__snap_ad_squads.sql</t>
         </is>
       </c>
       <c r="B257" s="2" t="inlineStr">
@@ -6089,7 +6089,7 @@
       </c>
       <c r="C257" s="3" t="inlineStr">
         <is>
-          <t>Phase 2 staging (paid media: Snap): 1:1 pass-through of snap_ads</t>
+          <t>Phase 2 staging (paid media: Snap): 1:1 pass-through of snap_ad_squads (Snap's ad set / ad group level)</t>
         </is>
       </c>
       <c r="D257" s="2" t="inlineStr">
@@ -6101,7 +6101,7 @@
     <row r="258">
       <c r="A258" s="2" t="inlineStr">
         <is>
-          <t>dbt/models/staging/kinetic/stg_kinetic__snap_stats_daily.sql</t>
+          <t>dbt/models/staging/kinetic/stg_kinetic__snap_ads.sql</t>
         </is>
       </c>
       <c r="B258" s="2" t="inlineStr">
@@ -6111,7 +6111,7 @@
       </c>
       <c r="C258" s="3" t="inlineStr">
         <is>
-          <t>Phase 2 staging (paid media: Snap): ad-day stats with combined ad_day_id key, spend in micros and dollars; documents swipes as Snap's clicks</t>
+          <t>Phase 2 staging (paid media: Snap): 1:1 pass-through of snap_ads</t>
         </is>
       </c>
       <c r="D258" s="2" t="inlineStr">
@@ -6123,7 +6123,7 @@
     <row r="259">
       <c r="A259" s="2" t="inlineStr">
         <is>
-          <t>dbt/models/staging/kinetic/_kinetic__staging.yml</t>
+          <t>dbt/models/staging/kinetic/stg_kinetic__snap_stats_daily.sql</t>
         </is>
       </c>
       <c r="B259" s="2" t="inlineStr">
@@ -6133,19 +6133,19 @@
       </c>
       <c r="C259" s="3" t="inlineStr">
         <is>
-          <t>Updated: tests for the 4 Snap staging models -- all hand-verified against live data first</t>
+          <t>Phase 2 staging (paid media: Snap): ad-day stats with combined ad_day_id key, spend in micros and dollars; documents swipes as Snap's clicks</t>
         </is>
       </c>
       <c r="D259" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 16:08 PDT</t>
+          <t>2026-09-29 15:53 PDT</t>
         </is>
       </c>
     </row>
     <row r="260">
       <c r="A260" s="2" t="inlineStr">
         <is>
-          <t>dbt/models/staging/kinetic/stg_kinetic__tiktok_campaigns.sql</t>
+          <t>dbt/models/staging/kinetic/_kinetic__staging.yml</t>
         </is>
       </c>
       <c r="B260" s="2" t="inlineStr">
@@ -6155,19 +6155,19 @@
       </c>
       <c r="C260" s="3" t="inlineStr">
         <is>
-          <t>Phase 2 staging (paid media: TikTok): campaigns with the single budget split into daily_budget_usd / lifetime_budget_usd by budget_mode (matching the other platforms), advertiser_id renamed tiktok_advertiser_id</t>
+          <t>Updated: tests for the 4 Snap staging models -- all hand-verified against live data first</t>
         </is>
       </c>
       <c r="D260" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 15:57 PDT</t>
+          <t>2026-09-29 16:08 PDT</t>
         </is>
       </c>
     </row>
     <row r="261">
       <c r="A261" s="2" t="inlineStr">
         <is>
-          <t>dbt/models/staging/kinetic/stg_kinetic__tiktok_adgroups.sql</t>
+          <t>dbt/models/staging/kinetic/stg_kinetic__tiktok_campaigns.sql</t>
         </is>
       </c>
       <c r="B261" s="2" t="inlineStr">
@@ -6177,7 +6177,7 @@
       </c>
       <c r="C261" s="3" t="inlineStr">
         <is>
-          <t>Phase 2 staging (paid media: TikTok): 1:1 pass-through of tiktok_adgroups</t>
+          <t>Phase 2 staging (paid media: TikTok): campaigns with the single budget split into daily_budget_usd / lifetime_budget_usd by budget_mode (matching the other platforms), advertiser_id renamed tiktok_advertiser_id</t>
         </is>
       </c>
       <c r="D261" s="2" t="inlineStr">
@@ -6189,7 +6189,7 @@
     <row r="262">
       <c r="A262" s="2" t="inlineStr">
         <is>
-          <t>dbt/models/staging/kinetic/stg_kinetic__tiktok_ads.sql</t>
+          <t>dbt/models/staging/kinetic/stg_kinetic__tiktok_adgroups.sql</t>
         </is>
       </c>
       <c r="B262" s="2" t="inlineStr">
@@ -6199,7 +6199,7 @@
       </c>
       <c r="C262" s="3" t="inlineStr">
         <is>
-          <t>Phase 2 staging (paid media: TikTok): 1:1 pass-through of tiktok_ads</t>
+          <t>Phase 2 staging (paid media: TikTok): 1:1 pass-through of tiktok_adgroups</t>
         </is>
       </c>
       <c r="D262" s="2" t="inlineStr">
@@ -6211,7 +6211,7 @@
     <row r="263">
       <c r="A263" s="2" t="inlineStr">
         <is>
-          <t>dbt/models/staging/kinetic/stg_kinetic__tiktok_reports_daily.sql</t>
+          <t>dbt/models/staging/kinetic/stg_kinetic__tiktok_ads.sql</t>
         </is>
       </c>
       <c r="B263" s="2" t="inlineStr">
@@ -6221,7 +6221,7 @@
       </c>
       <c r="C263" s="3" t="inlineStr">
         <is>
-          <t>Phase 2 staging (paid media: TikTok): ad-day reports with combined ad_day_id key, spend and CPM in micros and dollars, ctr_fraction</t>
+          <t>Phase 2 staging (paid media: TikTok): 1:1 pass-through of tiktok_ads</t>
         </is>
       </c>
       <c r="D263" s="2" t="inlineStr">
@@ -6233,7 +6233,7 @@
     <row r="264">
       <c r="A264" s="2" t="inlineStr">
         <is>
-          <t>dbt/models/staging/kinetic/stg_kinetic__product_variants.sql</t>
+          <t>dbt/models/staging/kinetic/stg_kinetic__tiktok_reports_daily.sql</t>
         </is>
       </c>
       <c r="B264" s="2" t="inlineStr">
@@ -6243,54 +6243,76 @@
       </c>
       <c r="C264" s="3" t="inlineStr">
         <is>
-          <t>Phase 2 staging (final table, 47 of 47): product variants with variant_option, price_adjustment_usd</t>
+          <t>Phase 2 staging (paid media: TikTok): ad-day reports with combined ad_day_id key, spend and CPM in micros and dollars, ctr_fraction</t>
         </is>
       </c>
       <c r="D264" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 16:08 PDT</t>
+          <t>2026-09-29 15:57 PDT</t>
         </is>
       </c>
     </row>
     <row r="265">
       <c r="A265" s="2" t="inlineStr">
         <is>
-          <t>HANDOFF.md</t>
+          <t>dbt/models/staging/kinetic/stg_kinetic__product_variants.sql</t>
         </is>
       </c>
       <c r="B265" s="2" t="inlineStr">
         <is>
-          <t>Doc</t>
+          <t>Code</t>
         </is>
       </c>
       <c r="C265" s="3" t="inlineStr">
         <is>
-          <t>Handoff note for starting a new chat/project: status, open decisions, prior decisions, pitfalls</t>
+          <t>Phase 2 staging (final table, 47 of 47): product variants with variant_option, price_adjustment_usd</t>
         </is>
       </c>
       <c r="D265" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 16:33 PDT</t>
+          <t>2026-09-29 16:08 PDT</t>
         </is>
       </c>
     </row>
     <row r="266">
       <c r="A266" s="2" t="inlineStr">
         <is>
+          <t>HANDOFF.md</t>
+        </is>
+      </c>
+      <c r="B266" s="2" t="inlineStr">
+        <is>
+          <t>Doc</t>
+        </is>
+      </c>
+      <c r="C266" s="3" t="inlineStr">
+        <is>
+          <t>Handoff note for starting a new chat/project: status, open decisions, prior decisions, pitfalls</t>
+        </is>
+      </c>
+      <c r="D266" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-29 16:39 PDT</t>
+        </is>
+      </c>
+    </row>
+    <row r="267">
+      <c r="A267" s="2" t="inlineStr">
+        <is>
           <t>dbt/models/staging/kinetic/_kinetic__staging.yml</t>
         </is>
       </c>
-      <c r="B266" s="2" t="inlineStr">
-        <is>
-          <t>Code</t>
-        </is>
-      </c>
-      <c r="C266" s="3" t="inlineStr">
+      <c r="B267" s="2" t="inlineStr">
+        <is>
+          <t>Code</t>
+        </is>
+      </c>
+      <c r="C267" s="3" t="inlineStr">
         <is>
           <t>Updated: tests for the 4 TikTok staging models -- all hand-verified against live data first</t>
         </is>
       </c>
-      <c r="D266" s="2" t="inlineStr">
+      <c r="D267" s="2" t="inlineStr">
         <is>
           <t>2026-09-29 16:08 PDT</t>
         </is>

</xml_diff>

<commit_message>
dbt setup: in-project profile (schema dbt_dev), venv install steps, gitignore
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011iLTiTsTyvHcVHREQNUg8N
</commit_message>
<xml_diff>
--- a/File_Manifest.xlsx
+++ b/File_Manifest.xlsx
@@ -435,7 +435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D267"/>
+  <dimension ref="A1:D268"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="48" customWidth="1" min="1" max="1"/>
@@ -506,7 +506,7 @@
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 16:39 PDT</t>
+          <t>2026-09-29 16:43 PDT</t>
         </is>
       </c>
     </row>
@@ -638,7 +638,7 @@
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 16:39 PDT</t>
+          <t>2026-09-29 16:43 PDT</t>
         </is>
       </c>
     </row>
@@ -726,7 +726,7 @@
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28 14:09 PDT</t>
+          <t>2026-09-29 16:43 PDT</t>
         </is>
       </c>
     </row>
@@ -748,7 +748,7 @@
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 16:39 PDT</t>
+          <t>2026-09-29 16:43 PDT</t>
         </is>
       </c>
     </row>
@@ -4363,73 +4363,73 @@
     <row r="179">
       <c r="A179" s="2" t="inlineStr">
         <is>
-          <t>dbt/.gitignore</t>
+          <t>dbt/profiles.yml</t>
         </is>
       </c>
       <c r="B179" s="2" t="inlineStr">
         <is>
-          <t>Repo config</t>
+          <t>Code</t>
         </is>
       </c>
       <c r="C179" s="3" t="inlineStr">
         <is>
-          <t>Excludes dbt's target/, dbt_packages/, logs/ from git</t>
+          <t>dbt connection profile (MotherDuck md:kinetic, schema dbt_dev); no secrets</t>
         </is>
       </c>
       <c r="D179" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28 14:48 PDT</t>
+          <t>2026-09-29 16:43 PDT</t>
         </is>
       </c>
     </row>
     <row r="180">
       <c r="A180" s="2" t="inlineStr">
         <is>
-          <t>dbt/README.md</t>
+          <t>dbt/.gitignore</t>
         </is>
       </c>
       <c r="B180" s="2" t="inlineStr">
         <is>
-          <t>Docs</t>
+          <t>Repo config</t>
         </is>
       </c>
       <c r="C180" s="3" t="inlineStr">
         <is>
-          <t>How to install dbt-core + dbt-duckdb and run this project locally against MotherDuck (neither of Claude's environments can reach motherduck.com directly, so dbt run/test must be executed on the user's own machine)</t>
+          <t>Excludes dbt's target/, dbt_packages/, logs/ from git</t>
         </is>
       </c>
       <c r="D180" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 16:39 PDT</t>
+          <t>2026-09-28 14:48 PDT</t>
         </is>
       </c>
     </row>
     <row r="181">
       <c r="A181" s="2" t="inlineStr">
         <is>
-          <t>dbt/models/staging/kinetic/_kinetic__sources.yml</t>
+          <t>dbt/README.md</t>
         </is>
       </c>
       <c r="B181" s="2" t="inlineStr">
         <is>
-          <t>Code</t>
+          <t>Docs</t>
         </is>
       </c>
       <c r="C181" s="3" t="inlineStr">
         <is>
-          <t>Declares all 47 raw kinetic tables as dbt sources, so every staging model references source() rather than a hardcoded table name</t>
+          <t>How to install dbt-core + dbt-duckdb and run this project locally against MotherDuck (neither of Claude's environments can reach motherduck.com directly, so dbt run/test must be executed on the user's own machine)</t>
         </is>
       </c>
       <c r="D181" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28 14:48 PDT</t>
+          <t>2026-09-29 16:43 PDT</t>
         </is>
       </c>
     </row>
     <row r="182">
       <c r="A182" s="2" t="inlineStr">
         <is>
-          <t>dbt/models/staging/kinetic/stg_kinetic__customers.sql</t>
+          <t>dbt/models/staging/kinetic/_kinetic__sources.yml</t>
         </is>
       </c>
       <c r="B182" s="2" t="inlineStr">
@@ -4439,7 +4439,7 @@
       </c>
       <c r="C182" s="3" t="inlineStr">
         <is>
-          <t>Staging model: 1:1 pass-through of customers with light renaming</t>
+          <t>Declares all 47 raw kinetic tables as dbt sources, so every staging model references source() rather than a hardcoded table name</t>
         </is>
       </c>
       <c r="D182" s="2" t="inlineStr">
@@ -4451,7 +4451,7 @@
     <row r="183">
       <c r="A183" s="2" t="inlineStr">
         <is>
-          <t>dbt/models/staging/kinetic/stg_kinetic__subscription_plans.sql</t>
+          <t>dbt/models/staging/kinetic/stg_kinetic__customers.sql</t>
         </is>
       </c>
       <c r="B183" s="2" t="inlineStr">
@@ -4461,7 +4461,7 @@
       </c>
       <c r="C183" s="3" t="inlineStr">
         <is>
-          <t>Staging model: 1:1 pass-through of subscription_plans</t>
+          <t>Staging model: 1:1 pass-through of customers with light renaming</t>
         </is>
       </c>
       <c r="D183" s="2" t="inlineStr">
@@ -4473,7 +4473,7 @@
     <row r="184">
       <c r="A184" s="2" t="inlineStr">
         <is>
-          <t>dbt/models/staging/kinetic/stg_kinetic__subscriptions.sql</t>
+          <t>dbt/models/staging/kinetic/stg_kinetic__subscription_plans.sql</t>
         </is>
       </c>
       <c r="B184" s="2" t="inlineStr">
@@ -4483,7 +4483,7 @@
       </c>
       <c r="C184" s="3" t="inlineStr">
         <is>
-          <t>Staging model: 1:1 pass-through of subscriptions</t>
+          <t>Staging model: 1:1 pass-through of subscription_plans</t>
         </is>
       </c>
       <c r="D184" s="2" t="inlineStr">
@@ -4495,7 +4495,7 @@
     <row r="185">
       <c r="A185" s="2" t="inlineStr">
         <is>
-          <t>dbt/models/staging/kinetic/stg_kinetic__invoices.sql</t>
+          <t>dbt/models/staging/kinetic/stg_kinetic__subscriptions.sql</t>
         </is>
       </c>
       <c r="B185" s="2" t="inlineStr">
@@ -4505,7 +4505,7 @@
       </c>
       <c r="C185" s="3" t="inlineStr">
         <is>
-          <t>Staging model: 1:1 pass-through of invoices</t>
+          <t>Staging model: 1:1 pass-through of subscriptions</t>
         </is>
       </c>
       <c r="D185" s="2" t="inlineStr">
@@ -4517,7 +4517,7 @@
     <row r="186">
       <c r="A186" s="2" t="inlineStr">
         <is>
-          <t>dbt/models/staging/kinetic/stg_kinetic__products.sql</t>
+          <t>dbt/models/staging/kinetic/stg_kinetic__invoices.sql</t>
         </is>
       </c>
       <c r="B186" s="2" t="inlineStr">
@@ -4527,7 +4527,7 @@
       </c>
       <c r="C186" s="3" t="inlineStr">
         <is>
-          <t>Staging model: 1:1 pass-through of products</t>
+          <t>Staging model: 1:1 pass-through of invoices</t>
         </is>
       </c>
       <c r="D186" s="2" t="inlineStr">
@@ -4539,7 +4539,7 @@
     <row r="187">
       <c r="A187" s="2" t="inlineStr">
         <is>
-          <t>dbt/models/staging/kinetic/_kinetic__staging.yml</t>
+          <t>dbt/models/staging/kinetic/stg_kinetic__products.sql</t>
         </is>
       </c>
       <c r="B187" s="2" t="inlineStr">
@@ -4549,19 +4549,19 @@
       </c>
       <c r="C187" s="3" t="inlineStr">
         <is>
-          <t>not_null/unique/relationships tests for the Phase 1/2 staging models</t>
+          <t>Staging model: 1:1 pass-through of products</t>
         </is>
       </c>
       <c r="D187" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 16:08 PDT</t>
+          <t>2026-09-28 14:48 PDT</t>
         </is>
       </c>
     </row>
     <row r="188">
       <c r="A188" s="2" t="inlineStr">
         <is>
-          <t>dbt/models/intermediate/int_subscription_paid_periods.sql</t>
+          <t>dbt/models/staging/kinetic/_kinetic__staging.yml</t>
         </is>
       </c>
       <c r="B188" s="2" t="inlineStr">
@@ -4571,19 +4571,19 @@
       </c>
       <c r="C188" s="3" t="inlineStr">
         <is>
-          <t>Intermediate model: resolves each subscription's true paid-start date (trial-vs-paid logic), defined once so every downstream mart agrees</t>
+          <t>not_null/unique/relationships tests for the Phase 1/2 staging models</t>
         </is>
       </c>
       <c r="D188" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28 14:48 PDT</t>
+          <t>2026-09-29 16:08 PDT</t>
         </is>
       </c>
     </row>
     <row r="189">
       <c r="A189" s="2" t="inlineStr">
         <is>
-          <t>dbt/models/intermediate/_intermediate.yml</t>
+          <t>dbt/models/intermediate/int_subscription_paid_periods.sql</t>
         </is>
       </c>
       <c r="B189" s="2" t="inlineStr">
@@ -4593,19 +4593,19 @@
       </c>
       <c r="C189" s="3" t="inlineStr">
         <is>
-          <t>Descriptions and tests for all intermediate models</t>
+          <t>Intermediate model: resolves each subscription's true paid-start date (trial-vs-paid logic), defined once so every downstream mart agrees</t>
         </is>
       </c>
       <c r="D189" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 16:39 PDT</t>
+          <t>2026-09-28 14:48 PDT</t>
         </is>
       </c>
     </row>
     <row r="190">
       <c r="A190" s="2" t="inlineStr">
         <is>
-          <t>dbt/models/marts/mart_mrr_monthly.sql</t>
+          <t>dbt/models/intermediate/_intermediate.yml</t>
         </is>
       </c>
       <c r="B190" s="2" t="inlineStr">
@@ -4615,19 +4615,19 @@
       </c>
       <c r="C190" s="3" t="inlineStr">
         <is>
-          <t>First canonical metric mart: active subscribers + MRR/ARR by month, validated against a hand-run equivalent query on the live database (2026-07: 90 active subscribers, ~$2,133 MRR)</t>
+          <t>Descriptions and tests for all intermediate models</t>
         </is>
       </c>
       <c r="D190" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28 14:48 PDT</t>
+          <t>2026-09-29 16:39 PDT</t>
         </is>
       </c>
     </row>
     <row r="191">
       <c r="A191" s="2" t="inlineStr">
         <is>
-          <t>dbt/models/marts/_marts.yml</t>
+          <t>dbt/models/marts/mart_mrr_monthly.sql</t>
         </is>
       </c>
       <c r="B191" s="2" t="inlineStr">
@@ -4637,63 +4637,63 @@
       </c>
       <c r="C191" s="3" t="inlineStr">
         <is>
-          <t>Tests for mart_mrr_monthly</t>
+          <t>First canonical metric mart: active subscribers + MRR/ARR by month, validated against a hand-run equivalent query on the live database (2026-07: 90 active subscribers, ~$2,133 MRR)</t>
         </is>
       </c>
       <c r="D191" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28 14:53 PDT</t>
+          <t>2026-09-28 14:48 PDT</t>
         </is>
       </c>
     </row>
     <row r="192">
       <c r="A192" s="2" t="inlineStr">
         <is>
-          <t>dbt/README.md</t>
+          <t>dbt/models/marts/_marts.yml</t>
         </is>
       </c>
       <c r="B192" s="2" t="inlineStr">
         <is>
-          <t>Docs</t>
+          <t>Code</t>
         </is>
       </c>
       <c r="C192" s="3" t="inlineStr">
         <is>
-          <t>Updated: what's built so far now includes the Phase 3 storefront staging models + mart_storefront_revenue_monthly</t>
+          <t>Tests for mart_mrr_monthly</t>
         </is>
       </c>
       <c r="D192" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 16:39 PDT</t>
+          <t>2026-09-28 14:53 PDT</t>
         </is>
       </c>
     </row>
     <row r="193">
       <c r="A193" s="2" t="inlineStr">
         <is>
-          <t>dbt/models/staging/kinetic/stg_kinetic__orders.sql</t>
+          <t>dbt/README.md</t>
         </is>
       </c>
       <c r="B193" s="2" t="inlineStr">
         <is>
-          <t>Code</t>
+          <t>Docs</t>
         </is>
       </c>
       <c r="C193" s="3" t="inlineStr">
         <is>
-          <t>Staging model: 1:1 pass-through of orders, plus is_guest_order/has_discount convenience booleans</t>
+          <t>Updated: what's built so far now includes the Phase 3 storefront staging models + mart_storefront_revenue_monthly</t>
         </is>
       </c>
       <c r="D193" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28 14:53 PDT</t>
+          <t>2026-09-29 16:43 PDT</t>
         </is>
       </c>
     </row>
     <row r="194">
       <c r="A194" s="2" t="inlineStr">
         <is>
-          <t>dbt/models/staging/kinetic/stg_kinetic__order_line_items.sql</t>
+          <t>dbt/models/staging/kinetic/stg_kinetic__orders.sql</t>
         </is>
       </c>
       <c r="B194" s="2" t="inlineStr">
@@ -4703,7 +4703,7 @@
       </c>
       <c r="C194" s="3" t="inlineStr">
         <is>
-          <t>Staging model: 1:1 pass-through of order_line_items</t>
+          <t>Staging model: 1:1 pass-through of orders, plus is_guest_order/has_discount convenience booleans</t>
         </is>
       </c>
       <c r="D194" s="2" t="inlineStr">
@@ -4715,7 +4715,7 @@
     <row r="195">
       <c r="A195" s="2" t="inlineStr">
         <is>
-          <t>dbt/models/staging/kinetic/stg_kinetic__payments.sql</t>
+          <t>dbt/models/staging/kinetic/stg_kinetic__order_line_items.sql</t>
         </is>
       </c>
       <c r="B195" s="2" t="inlineStr">
@@ -4725,7 +4725,7 @@
       </c>
       <c r="C195" s="3" t="inlineStr">
         <is>
-          <t>Staging model: 1:1 pass-through of payments</t>
+          <t>Staging model: 1:1 pass-through of order_line_items</t>
         </is>
       </c>
       <c r="D195" s="2" t="inlineStr">
@@ -4737,7 +4737,7 @@
     <row r="196">
       <c r="A196" s="2" t="inlineStr">
         <is>
-          <t>dbt/models/staging/kinetic/stg_kinetic__refunds.sql</t>
+          <t>dbt/models/staging/kinetic/stg_kinetic__payments.sql</t>
         </is>
       </c>
       <c r="B196" s="2" t="inlineStr">
@@ -4747,7 +4747,7 @@
       </c>
       <c r="C196" s="3" t="inlineStr">
         <is>
-          <t>Staging model: 1:1 pass-through of refunds</t>
+          <t>Staging model: 1:1 pass-through of payments</t>
         </is>
       </c>
       <c r="D196" s="2" t="inlineStr">
@@ -4759,7 +4759,7 @@
     <row r="197">
       <c r="A197" s="2" t="inlineStr">
         <is>
-          <t>dbt/models/staging/kinetic/stg_kinetic__discount_codes.sql</t>
+          <t>dbt/models/staging/kinetic/stg_kinetic__refunds.sql</t>
         </is>
       </c>
       <c r="B197" s="2" t="inlineStr">
@@ -4769,7 +4769,7 @@
       </c>
       <c r="C197" s="3" t="inlineStr">
         <is>
-          <t>Staging model: 1:1 pass-through of discount_codes</t>
+          <t>Staging model: 1:1 pass-through of refunds</t>
         </is>
       </c>
       <c r="D197" s="2" t="inlineStr">
@@ -4781,7 +4781,7 @@
     <row r="198">
       <c r="A198" s="2" t="inlineStr">
         <is>
-          <t>dbt/models/intermediate/int_orders_refunded.sql</t>
+          <t>dbt/models/staging/kinetic/stg_kinetic__discount_codes.sql</t>
         </is>
       </c>
       <c r="B198" s="2" t="inlineStr">
@@ -4791,7 +4791,7 @@
       </c>
       <c r="C198" s="3" t="inlineStr">
         <is>
-          <t>Intermediate model: per-order total of succeeded refunds only (failed/pending refunds don't reduce reported revenue)</t>
+          <t>Staging model: 1:1 pass-through of discount_codes</t>
         </is>
       </c>
       <c r="D198" s="2" t="inlineStr">
@@ -4803,7 +4803,7 @@
     <row r="199">
       <c r="A199" s="2" t="inlineStr">
         <is>
-          <t>dbt/models/intermediate/int_customer_identity.sql</t>
+          <t>dbt/models/intermediate/int_orders_refunded.sql</t>
         </is>
       </c>
       <c r="B199" s="2" t="inlineStr">
@@ -4813,19 +4813,19 @@
       </c>
       <c r="C199" s="3" t="inlineStr">
         <is>
-          <t>Intermediate model: lookup from every web anonymous_id and account email to its customer (guest emails matched by email; anonymous sessions back-filled; deleted accounts excluded)</t>
+          <t>Intermediate model: per-order total of succeeded refunds only (failed/pending refunds don't reduce reported revenue)</t>
         </is>
       </c>
       <c r="D199" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 16:39 PDT</t>
+          <t>2026-09-28 14:53 PDT</t>
         </is>
       </c>
     </row>
     <row r="200">
       <c r="A200" s="2" t="inlineStr">
         <is>
-          <t>dbt/models/marts/mart_storefront_revenue_monthly.sql</t>
+          <t>dbt/models/intermediate/int_customer_identity.sql</t>
         </is>
       </c>
       <c r="B200" s="2" t="inlineStr">
@@ -4835,19 +4835,19 @@
       </c>
       <c r="C200" s="3" t="inlineStr">
         <is>
-          <t>Second canonical metric mart: non-subscription (course+merch) gross/net revenue, AOV, guest-checkout share, discount-usage share, refund rate by month -- validated against a hand-run equivalent query on the live database (2026-07: 246 orders, $13,843.71 gross revenue, $56.28 AOV)</t>
+          <t>Intermediate model: lookup from every web anonymous_id and account email to its customer (guest emails matched by email; anonymous sessions back-filled; deleted accounts excluded)</t>
         </is>
       </c>
       <c r="D200" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28 14:53 PDT</t>
+          <t>2026-09-29 16:39 PDT</t>
         </is>
       </c>
     </row>
     <row r="201">
       <c r="A201" s="2" t="inlineStr">
         <is>
-          <t>dbt/models/staging/kinetic/stg_kinetic__customer_addresses.sql</t>
+          <t>dbt/models/marts/mart_storefront_revenue_monthly.sql</t>
         </is>
       </c>
       <c r="B201" s="2" t="inlineStr">
@@ -4857,19 +4857,19 @@
       </c>
       <c r="C201" s="3" t="inlineStr">
         <is>
-          <t>Phase 2 staging (Customer 360): 1:1 pass-through of customer_addresses</t>
+          <t>Second canonical metric mart: non-subscription (course+merch) gross/net revenue, AOV, guest-checkout share, discount-usage share, refund rate by month -- validated against a hand-run equivalent query on the live database (2026-07: 246 orders, $13,843.71 gross revenue, $56.28 AOV)</t>
         </is>
       </c>
       <c r="D201" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 10:26 PDT</t>
+          <t>2026-09-28 14:53 PDT</t>
         </is>
       </c>
     </row>
     <row r="202">
       <c r="A202" s="2" t="inlineStr">
         <is>
-          <t>dbt/models/staging/kinetic/stg_kinetic__devices.sql</t>
+          <t>dbt/models/staging/kinetic/stg_kinetic__customer_addresses.sql</t>
         </is>
       </c>
       <c r="B202" s="2" t="inlineStr">
@@ -4879,7 +4879,7 @@
       </c>
       <c r="C202" s="3" t="inlineStr">
         <is>
-          <t>Phase 2 staging (Customer 360): 1:1 pass-through of devices, plus is_anonymous_device flag (customer_id null for ~94% of devices by design)</t>
+          <t>Phase 2 staging (Customer 360): 1:1 pass-through of customer_addresses</t>
         </is>
       </c>
       <c r="D202" s="2" t="inlineStr">
@@ -4891,7 +4891,7 @@
     <row r="203">
       <c r="A203" s="2" t="inlineStr">
         <is>
-          <t>dbt/models/staging/kinetic/stg_kinetic__identity_map.sql</t>
+          <t>dbt/models/staging/kinetic/stg_kinetic__devices.sql</t>
         </is>
       </c>
       <c r="B203" s="2" t="inlineStr">
@@ -4901,7 +4901,7 @@
       </c>
       <c r="C203" s="3" t="inlineStr">
         <is>
-          <t>Phase 2 staging (Customer 360): 1:1 pass-through of identity_map</t>
+          <t>Phase 2 staging (Customer 360): 1:1 pass-through of devices, plus is_anonymous_device flag (customer_id null for ~94% of devices by design)</t>
         </is>
       </c>
       <c r="D203" s="2" t="inlineStr">
@@ -4913,7 +4913,7 @@
     <row r="204">
       <c r="A204" s="2" t="inlineStr">
         <is>
-          <t>dbt/models/staging/kinetic/stg_kinetic__segments.sql</t>
+          <t>dbt/models/staging/kinetic/stg_kinetic__identity_map.sql</t>
         </is>
       </c>
       <c r="B204" s="2" t="inlineStr">
@@ -4923,7 +4923,7 @@
       </c>
       <c r="C204" s="3" t="inlineStr">
         <is>
-          <t>Phase 2 staging (Customer 360): 1:1 pass-through of segments</t>
+          <t>Phase 2 staging (Customer 360): 1:1 pass-through of identity_map</t>
         </is>
       </c>
       <c r="D204" s="2" t="inlineStr">
@@ -4935,7 +4935,7 @@
     <row r="205">
       <c r="A205" s="2" t="inlineStr">
         <is>
-          <t>dbt/models/staging/kinetic/stg_kinetic__customer_segment_membership.sql</t>
+          <t>dbt/models/staging/kinetic/stg_kinetic__segments.sql</t>
         </is>
       </c>
       <c r="B205" s="2" t="inlineStr">
@@ -4945,7 +4945,7 @@
       </c>
       <c r="C205" s="3" t="inlineStr">
         <is>
-          <t>Phase 2 staging (Customer 360): 1:1 pass-through of customer_segment_membership, plus is_current_member flag</t>
+          <t>Phase 2 staging (Customer 360): 1:1 pass-through of segments</t>
         </is>
       </c>
       <c r="D205" s="2" t="inlineStr">
@@ -4957,7 +4957,7 @@
     <row r="206">
       <c r="A206" s="2" t="inlineStr">
         <is>
-          <t>dbt/models/staging/kinetic/stg_kinetic__subscription_events.sql</t>
+          <t>dbt/models/staging/kinetic/stg_kinetic__customer_segment_membership.sql</t>
         </is>
       </c>
       <c r="B206" s="2" t="inlineStr">
@@ -4967,7 +4967,7 @@
       </c>
       <c r="C206" s="3" t="inlineStr">
         <is>
-          <t>Phase 2 staging (Customer 360): 1:1 pass-through of subscription_events; old_plan/new_plan renamed to old_plan_id/new_plan_id</t>
+          <t>Phase 2 staging (Customer 360): 1:1 pass-through of customer_segment_membership, plus is_current_member flag</t>
         </is>
       </c>
       <c r="D206" s="2" t="inlineStr">
@@ -4979,7 +4979,7 @@
     <row r="207">
       <c r="A207" s="2" t="inlineStr">
         <is>
-          <t>dbt/models/staging/kinetic/_kinetic__staging.yml</t>
+          <t>dbt/models/staging/kinetic/stg_kinetic__subscription_events.sql</t>
         </is>
       </c>
       <c r="B207" s="2" t="inlineStr">
@@ -4989,19 +4989,19 @@
       </c>
       <c r="C207" s="3" t="inlineStr">
         <is>
-          <t>Updated: tests for the 6 Customer 360 staging models (PK not_null/unique, FK relationships) -- all hand-verified against live data first</t>
+          <t>Phase 2 staging (Customer 360): 1:1 pass-through of subscription_events; old_plan/new_plan renamed to old_plan_id/new_plan_id</t>
         </is>
       </c>
       <c r="D207" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 16:08 PDT</t>
+          <t>2026-09-29 10:26 PDT</t>
         </is>
       </c>
     </row>
     <row r="208">
       <c r="A208" s="2" t="inlineStr">
         <is>
-          <t>dbt/models/staging/kinetic/stg_kinetic__web_sessions.sql</t>
+          <t>dbt/models/staging/kinetic/_kinetic__staging.yml</t>
         </is>
       </c>
       <c r="B208" s="2" t="inlineStr">
@@ -5011,19 +5011,19 @@
       </c>
       <c r="C208" s="3" t="inlineStr">
         <is>
-          <t>Phase 2 staging (web/app engagement): 1:1 pass-through of web_sessions, plus is_known_customer flag (customer_id null for ~79% of sessions by design)</t>
+          <t>Updated: tests for the 6 Customer 360 staging models (PK not_null/unique, FK relationships) -- all hand-verified against live data first</t>
         </is>
       </c>
       <c r="D208" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 12:58 PDT</t>
+          <t>2026-09-29 16:08 PDT</t>
         </is>
       </c>
     </row>
     <row r="209">
       <c r="A209" s="2" t="inlineStr">
         <is>
-          <t>dbt/models/staging/kinetic/stg_kinetic__web_events.sql</t>
+          <t>dbt/models/staging/kinetic/stg_kinetic__web_sessions.sql</t>
         </is>
       </c>
       <c r="B209" s="2" t="inlineStr">
@@ -5033,7 +5033,7 @@
       </c>
       <c r="C209" s="3" t="inlineStr">
         <is>
-          <t>Phase 2 staging (web/app engagement): 1:1 pass-through of web_events</t>
+          <t>Phase 2 staging (web/app engagement): 1:1 pass-through of web_sessions, plus is_known_customer flag (customer_id null for ~79% of sessions by design)</t>
         </is>
       </c>
       <c r="D209" s="2" t="inlineStr">
@@ -5045,7 +5045,7 @@
     <row r="210">
       <c r="A210" s="2" t="inlineStr">
         <is>
-          <t>dbt/models/staging/kinetic/stg_kinetic__app_sessions.sql</t>
+          <t>dbt/models/staging/kinetic/stg_kinetic__web_events.sql</t>
         </is>
       </c>
       <c r="B210" s="2" t="inlineStr">
@@ -5055,7 +5055,7 @@
       </c>
       <c r="C210" s="3" t="inlineStr">
         <is>
-          <t>Phase 2 staging (web/app engagement): 1:1 pass-through of app_sessions</t>
+          <t>Phase 2 staging (web/app engagement): 1:1 pass-through of web_events</t>
         </is>
       </c>
       <c r="D210" s="2" t="inlineStr">
@@ -5067,7 +5067,7 @@
     <row r="211">
       <c r="A211" s="2" t="inlineStr">
         <is>
-          <t>dbt/models/staging/kinetic/stg_kinetic__app_events.sql</t>
+          <t>dbt/models/staging/kinetic/stg_kinetic__app_sessions.sql</t>
         </is>
       </c>
       <c r="B211" s="2" t="inlineStr">
@@ -5077,7 +5077,7 @@
       </c>
       <c r="C211" s="3" t="inlineStr">
         <is>
-          <t>Phase 2 staging (web/app engagement): 1:1 pass-through of app_events</t>
+          <t>Phase 2 staging (web/app engagement): 1:1 pass-through of app_sessions</t>
         </is>
       </c>
       <c r="D211" s="2" t="inlineStr">
@@ -5089,7 +5089,7 @@
     <row r="212">
       <c r="A212" s="2" t="inlineStr">
         <is>
-          <t>dbt/models/staging/kinetic/_kinetic__staging.yml</t>
+          <t>dbt/models/staging/kinetic/stg_kinetic__app_events.sql</t>
         </is>
       </c>
       <c r="B212" s="2" t="inlineStr">
@@ -5099,19 +5099,19 @@
       </c>
       <c r="C212" s="3" t="inlineStr">
         <is>
-          <t>Updated: tests for the 4 web/app engagement staging models -- all hand-verified against live data first</t>
+          <t>Phase 2 staging (web/app engagement): 1:1 pass-through of app_events</t>
         </is>
       </c>
       <c r="D212" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 16:08 PDT</t>
+          <t>2026-09-29 12:58 PDT</t>
         </is>
       </c>
     </row>
     <row r="213">
       <c r="A213" s="2" t="inlineStr">
         <is>
-          <t>dbt/models/staging/kinetic/stg_kinetic__braze_email_campaigns.sql</t>
+          <t>dbt/models/staging/kinetic/_kinetic__staging.yml</t>
         </is>
       </c>
       <c r="B213" s="2" t="inlineStr">
@@ -5121,19 +5121,19 @@
       </c>
       <c r="C213" s="3" t="inlineStr">
         <is>
-          <t>Phase 2 staging (email/push): 1:1 pass-through of braze_email_campaigns</t>
+          <t>Updated: tests for the 4 web/app engagement staging models -- all hand-verified against live data first</t>
         </is>
       </c>
       <c r="D213" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 12:59 PDT</t>
+          <t>2026-09-29 16:08 PDT</t>
         </is>
       </c>
     </row>
     <row r="214">
       <c r="A214" s="2" t="inlineStr">
         <is>
-          <t>dbt/models/staging/kinetic/stg_kinetic__braze_push_campaigns.sql</t>
+          <t>dbt/models/staging/kinetic/stg_kinetic__braze_email_campaigns.sql</t>
         </is>
       </c>
       <c r="B214" s="2" t="inlineStr">
@@ -5143,7 +5143,7 @@
       </c>
       <c r="C214" s="3" t="inlineStr">
         <is>
-          <t>Phase 2 staging (email/push): 1:1 pass-through of braze_push_campaigns</t>
+          <t>Phase 2 staging (email/push): 1:1 pass-through of braze_email_campaigns</t>
         </is>
       </c>
       <c r="D214" s="2" t="inlineStr">
@@ -5155,7 +5155,7 @@
     <row r="215">
       <c r="A215" s="2" t="inlineStr">
         <is>
-          <t>dbt/models/staging/kinetic/stg_kinetic__braze_email_events.sql</t>
+          <t>dbt/models/staging/kinetic/stg_kinetic__braze_push_campaigns.sql</t>
         </is>
       </c>
       <c r="B215" s="2" t="inlineStr">
@@ -5165,7 +5165,7 @@
       </c>
       <c r="C215" s="3" t="inlineStr">
         <is>
-          <t>Phase 2 staging (email/push): braze_email_events with external_user_id renamed to customer_id and a short event_name (send/open/click/bounce/unsubscribe) alongside Braze's raw event_type</t>
+          <t>Phase 2 staging (email/push): 1:1 pass-through of braze_push_campaigns</t>
         </is>
       </c>
       <c r="D215" s="2" t="inlineStr">
@@ -5177,7 +5177,7 @@
     <row r="216">
       <c r="A216" s="2" t="inlineStr">
         <is>
-          <t>dbt/models/staging/kinetic/stg_kinetic__braze_push_events.sql</t>
+          <t>dbt/models/staging/kinetic/stg_kinetic__braze_email_events.sql</t>
         </is>
       </c>
       <c r="B216" s="2" t="inlineStr">
@@ -5187,7 +5187,7 @@
       </c>
       <c r="C216" s="3" t="inlineStr">
         <is>
-          <t>Phase 2 staging (email/push): braze_push_events with external_user_id renamed to customer_id and a short event_name alongside Braze's raw event_type</t>
+          <t>Phase 2 staging (email/push): braze_email_events with external_user_id renamed to customer_id and a short event_name (send/open/click/bounce/unsubscribe) alongside Braze's raw event_type</t>
         </is>
       </c>
       <c r="D216" s="2" t="inlineStr">
@@ -5199,7 +5199,7 @@
     <row r="217">
       <c r="A217" s="2" t="inlineStr">
         <is>
-          <t>dbt/models/staging/kinetic/_kinetic__staging.yml</t>
+          <t>dbt/models/staging/kinetic/stg_kinetic__braze_push_events.sql</t>
         </is>
       </c>
       <c r="B217" s="2" t="inlineStr">
@@ -5209,19 +5209,19 @@
       </c>
       <c r="C217" s="3" t="inlineStr">
         <is>
-          <t>Updated: tests for the 4 Braze staging models, incl. accepted_values on event_name -- all hand-verified against live data first</t>
+          <t>Phase 2 staging (email/push): braze_push_events with external_user_id renamed to customer_id and a short event_name alongside Braze's raw event_type</t>
         </is>
       </c>
       <c r="D217" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 16:08 PDT</t>
+          <t>2026-09-29 12:59 PDT</t>
         </is>
       </c>
     </row>
     <row r="218">
       <c r="A218" s="2" t="inlineStr">
         <is>
-          <t>dbt/models/staging/kinetic/stg_kinetic__meta_campaigns.sql</t>
+          <t>dbt/models/staging/kinetic/_kinetic__staging.yml</t>
         </is>
       </c>
       <c r="B218" s="2" t="inlineStr">
@@ -5231,19 +5231,19 @@
       </c>
       <c r="C218" s="3" t="inlineStr">
         <is>
-          <t>Phase 2 staging (paid media: Meta): meta_campaigns with budgets in both raw cents and dollars (Meta API stores budgets in cents)</t>
+          <t>Updated: tests for the 4 Braze staging models, incl. accepted_values on event_name -- all hand-verified against live data first</t>
         </is>
       </c>
       <c r="D218" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 13:02 PDT</t>
+          <t>2026-09-29 16:08 PDT</t>
         </is>
       </c>
     </row>
     <row r="219">
       <c r="A219" s="2" t="inlineStr">
         <is>
-          <t>dbt/models/staging/kinetic/stg_kinetic__meta_ads.sql</t>
+          <t>dbt/models/staging/kinetic/stg_kinetic__meta_campaigns.sql</t>
         </is>
       </c>
       <c r="B219" s="2" t="inlineStr">
@@ -5253,7 +5253,7 @@
       </c>
       <c r="C219" s="3" t="inlineStr">
         <is>
-          <t>Phase 2 staging (paid media: Meta): 1:1 pass-through of meta_ads</t>
+          <t>Phase 2 staging (paid media: Meta): meta_campaigns with budgets in both raw cents and dollars (Meta API stores budgets in cents)</t>
         </is>
       </c>
       <c r="D219" s="2" t="inlineStr">
@@ -5265,7 +5265,7 @@
     <row r="220">
       <c r="A220" s="2" t="inlineStr">
         <is>
-          <t>dbt/models/staging/kinetic/stg_kinetic__meta_ad_insights_daily.sql</t>
+          <t>dbt/models/staging/kinetic/stg_kinetic__meta_ads.sql</t>
         </is>
       </c>
       <c r="B220" s="2" t="inlineStr">
@@ -5275,7 +5275,7 @@
       </c>
       <c r="C220" s="3" t="inlineStr">
         <is>
-          <t>Phase 2 staging (paid media: Meta): meta_ad_insights_daily with a combined ad_day_id key, unit-suffixed columns (spend_usd, cpm_usd, cpc_usd) and ctr renamed ctr_fraction (0.017 = 1.7%)</t>
+          <t>Phase 2 staging (paid media: Meta): 1:1 pass-through of meta_ads</t>
         </is>
       </c>
       <c r="D220" s="2" t="inlineStr">
@@ -5287,7 +5287,7 @@
     <row r="221">
       <c r="A221" s="2" t="inlineStr">
         <is>
-          <t>dbt/models/staging/kinetic/stg_kinetic__meta_ad_actions_daily.sql</t>
+          <t>dbt/models/staging/kinetic/stg_kinetic__meta_ad_insights_daily.sql</t>
         </is>
       </c>
       <c r="B221" s="2" t="inlineStr">
@@ -5297,7 +5297,7 @@
       </c>
       <c r="C221" s="3" t="inlineStr">
         <is>
-          <t>Phase 2 staging (paid media: Meta): meta_ad_actions_daily with a combined ad_day_action_id key; value renamed action_count</t>
+          <t>Phase 2 staging (paid media: Meta): meta_ad_insights_daily with a combined ad_day_id key, unit-suffixed columns (spend_usd, cpm_usd, cpc_usd) and ctr renamed ctr_fraction (0.017 = 1.7%)</t>
         </is>
       </c>
       <c r="D221" s="2" t="inlineStr">
@@ -5309,7 +5309,7 @@
     <row r="222">
       <c r="A222" s="2" t="inlineStr">
         <is>
-          <t>dbt/models/staging/kinetic/_kinetic__staging.yml</t>
+          <t>dbt/models/staging/kinetic/stg_kinetic__meta_ad_actions_daily.sql</t>
         </is>
       </c>
       <c r="B222" s="2" t="inlineStr">
@@ -5319,19 +5319,19 @@
       </c>
       <c r="C222" s="3" t="inlineStr">
         <is>
-          <t>Updated: tests for the 4 Meta staging models, incl. uniqueness of the combined daily keys -- all hand-verified against live data first</t>
+          <t>Phase 2 staging (paid media: Meta): meta_ad_actions_daily with a combined ad_day_action_id key; value renamed action_count</t>
         </is>
       </c>
       <c r="D222" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 16:08 PDT</t>
+          <t>2026-09-29 13:02 PDT</t>
         </is>
       </c>
     </row>
     <row r="223">
       <c r="A223" s="2" t="inlineStr">
         <is>
-          <t>dbt/models/staging/kinetic/stg_kinetic__google_search_campaigns.sql</t>
+          <t>dbt/models/staging/kinetic/_kinetic__staging.yml</t>
         </is>
       </c>
       <c r="B223" s="2" t="inlineStr">
@@ -5341,19 +5341,19 @@
       </c>
       <c r="C223" s="3" t="inlineStr">
         <is>
-          <t>Phase 2 staging (paid media: Google Search): campaigns with the raw customer_id renamed google_ads_account_id (it's the Google Ads account number, not a Kinetic customer), daily budget in micros and dollars, end_date cast back to a date</t>
+          <t>Updated: tests for the 4 Meta staging models, incl. uniqueness of the combined daily keys -- all hand-verified against live data first</t>
         </is>
       </c>
       <c r="D223" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 13:13 PDT</t>
+          <t>2026-09-29 16:08 PDT</t>
         </is>
       </c>
     </row>
     <row r="224">
       <c r="A224" s="2" t="inlineStr">
         <is>
-          <t>dbt/models/staging/kinetic/stg_kinetic__google_search_ad_groups.sql</t>
+          <t>dbt/models/staging/kinetic/stg_kinetic__google_search_campaigns.sql</t>
         </is>
       </c>
       <c r="B224" s="2" t="inlineStr">
@@ -5363,7 +5363,7 @@
       </c>
       <c r="C224" s="3" t="inlineStr">
         <is>
-          <t>Phase 2 staging (paid media: Google Search): ad groups; cpc_bid_micros cast back to a number (always empty -- automated bidding)</t>
+          <t>Phase 2 staging (paid media: Google Search): campaigns with the raw customer_id renamed google_ads_account_id (it's the Google Ads account number, not a Kinetic customer), daily budget in micros and dollars, end_date cast back to a date</t>
         </is>
       </c>
       <c r="D224" s="2" t="inlineStr">
@@ -5375,7 +5375,7 @@
     <row r="225">
       <c r="A225" s="2" t="inlineStr">
         <is>
-          <t>dbt/models/staging/kinetic/stg_kinetic__google_search_performance_daily.sql</t>
+          <t>dbt/models/staging/kinetic/stg_kinetic__google_search_ad_groups.sql</t>
         </is>
       </c>
       <c r="B225" s="2" t="inlineStr">
@@ -5385,7 +5385,7 @@
       </c>
       <c r="C225" s="3" t="inlineStr">
         <is>
-          <t>Phase 2 staging (paid media: Google Search): ad-group-day performance with combined ad_group_day_id key, cost converted from micros to dollars, ctr_fraction. The keyword table rolled up -- never add the two together</t>
+          <t>Phase 2 staging (paid media: Google Search): ad groups; cpc_bid_micros cast back to a number (always empty -- automated bidding)</t>
         </is>
       </c>
       <c r="D225" s="2" t="inlineStr">
@@ -5397,7 +5397,7 @@
     <row r="226">
       <c r="A226" s="2" t="inlineStr">
         <is>
-          <t>dbt/models/staging/kinetic/stg_kinetic__google_search_keyword_performance_daily.sql</t>
+          <t>dbt/models/staging/kinetic/stg_kinetic__google_search_performance_daily.sql</t>
         </is>
       </c>
       <c r="B226" s="2" t="inlineStr">
@@ -5407,7 +5407,7 @@
       </c>
       <c r="C226" s="3" t="inlineStr">
         <is>
-          <t>Phase 2 staging (paid media: Google Search): keyword-day performance with combined keyword_day_id key, cost converted from micros to dollars, ctr_fraction</t>
+          <t>Phase 2 staging (paid media: Google Search): ad-group-day performance with combined ad_group_day_id key, cost converted from micros to dollars, ctr_fraction. The keyword table rolled up -- never add the two together</t>
         </is>
       </c>
       <c r="D226" s="2" t="inlineStr">
@@ -5419,7 +5419,7 @@
     <row r="227">
       <c r="A227" s="2" t="inlineStr">
         <is>
-          <t>dbt/models/staging/kinetic/_kinetic__staging.yml</t>
+          <t>dbt/models/staging/kinetic/stg_kinetic__google_search_keyword_performance_daily.sql</t>
         </is>
       </c>
       <c r="B227" s="2" t="inlineStr">
@@ -5429,19 +5429,19 @@
       </c>
       <c r="C227" s="3" t="inlineStr">
         <is>
-          <t>Updated: tests for the 4 Google Search staging models -- all hand-verified against live data first</t>
+          <t>Phase 2 staging (paid media: Google Search): keyword-day performance with combined keyword_day_id key, cost converted from micros to dollars, ctr_fraction</t>
         </is>
       </c>
       <c r="D227" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 16:08 PDT</t>
+          <t>2026-09-29 13:13 PDT</t>
         </is>
       </c>
     </row>
     <row r="228">
       <c r="A228" s="2" t="inlineStr">
         <is>
-          <t>dbt/models/staging/kinetic/stg_kinetic__youtube_campaigns.sql</t>
+          <t>dbt/models/staging/kinetic/_kinetic__staging.yml</t>
         </is>
       </c>
       <c r="B228" s="2" t="inlineStr">
@@ -5451,19 +5451,19 @@
       </c>
       <c r="C228" s="3" t="inlineStr">
         <is>
-          <t>Phase 2 staging (paid media: YouTube): campaigns with customer_id renamed google_ads_account_id (the ad account, not a Kinetic customer), budgets in micros and dollars</t>
+          <t>Updated: tests for the 4 Google Search staging models -- all hand-verified against live data first</t>
         </is>
       </c>
       <c r="D228" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 13:14 PDT</t>
+          <t>2026-09-29 16:08 PDT</t>
         </is>
       </c>
     </row>
     <row r="229">
       <c r="A229" s="2" t="inlineStr">
         <is>
-          <t>dbt/models/staging/kinetic/stg_kinetic__youtube_ad_groups.sql</t>
+          <t>dbt/models/staging/kinetic/stg_kinetic__youtube_campaigns.sql</t>
         </is>
       </c>
       <c r="B229" s="2" t="inlineStr">
@@ -5473,7 +5473,7 @@
       </c>
       <c r="C229" s="3" t="inlineStr">
         <is>
-          <t>Phase 2 staging (paid media: YouTube): 1:1 pass-through of youtube_ad_groups</t>
+          <t>Phase 2 staging (paid media: YouTube): campaigns with customer_id renamed google_ads_account_id (the ad account, not a Kinetic customer), budgets in micros and dollars</t>
         </is>
       </c>
       <c r="D229" s="2" t="inlineStr">
@@ -5485,7 +5485,7 @@
     <row r="230">
       <c r="A230" s="2" t="inlineStr">
         <is>
-          <t>dbt/models/staging/kinetic/stg_kinetic__youtube_performance_daily.sql</t>
+          <t>dbt/models/staging/kinetic/stg_kinetic__youtube_ad_groups.sql</t>
         </is>
       </c>
       <c r="B230" s="2" t="inlineStr">
@@ -5495,7 +5495,7 @@
       </c>
       <c r="C230" s="3" t="inlineStr">
         <is>
-          <t>Phase 2 staging (paid media: YouTube): ad-group-day performance with combined ad_group_day_id key, cost and cost-per-view converted from micros to dollars, video_view_rate_fraction</t>
+          <t>Phase 2 staging (paid media: YouTube): 1:1 pass-through of youtube_ad_groups</t>
         </is>
       </c>
       <c r="D230" s="2" t="inlineStr">
@@ -5507,7 +5507,7 @@
     <row r="231">
       <c r="A231" s="2" t="inlineStr">
         <is>
-          <t>dbt/models/staging/kinetic/_kinetic__staging.yml</t>
+          <t>dbt/models/staging/kinetic/stg_kinetic__youtube_performance_daily.sql</t>
         </is>
       </c>
       <c r="B231" s="2" t="inlineStr">
@@ -5517,19 +5517,19 @@
       </c>
       <c r="C231" s="3" t="inlineStr">
         <is>
-          <t>Updated: tests for the 3 YouTube staging models -- all hand-verified against live data first</t>
+          <t>Phase 2 staging (paid media: YouTube): ad-group-day performance with combined ad_group_day_id key, cost and cost-per-view converted from micros to dollars, video_view_rate_fraction</t>
         </is>
       </c>
       <c r="D231" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 16:08 PDT</t>
+          <t>2026-09-29 13:14 PDT</t>
         </is>
       </c>
     </row>
     <row r="232">
       <c r="A232" s="2" t="inlineStr">
         <is>
-          <t>dbt/models/staging/kinetic/stg_kinetic__dv360_insertion_orders.sql</t>
+          <t>dbt/models/staging/kinetic/_kinetic__staging.yml</t>
         </is>
       </c>
       <c r="B232" s="2" t="inlineStr">
@@ -5539,19 +5539,19 @@
       </c>
       <c r="C232" s="3" t="inlineStr">
         <is>
-          <t>Phase 2 staging (paid media: DV360): insertion orders with budget_micros named monthly_budget_* (it's a monthly budget), end_date cast back to a date; flags the flat-budget-vs-growing-spend known issue</t>
+          <t>Updated: tests for the 3 YouTube staging models -- all hand-verified against live data first</t>
         </is>
       </c>
       <c r="D232" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 13:27 PDT</t>
+          <t>2026-09-29 16:08 PDT</t>
         </is>
       </c>
     </row>
     <row r="233">
       <c r="A233" s="2" t="inlineStr">
         <is>
-          <t>dbt/models/staging/kinetic/stg_kinetic__dv360_line_items.sql</t>
+          <t>dbt/models/staging/kinetic/stg_kinetic__dv360_insertion_orders.sql</t>
         </is>
       </c>
       <c r="B233" s="2" t="inlineStr">
@@ -5561,19 +5561,19 @@
       </c>
       <c r="C233" s="3" t="inlineStr">
         <is>
-          <t>Phase 2 staging (paid media: DV360): 1:1 pass-through of dv360_line_items</t>
+          <t>Phase 2 staging (paid media: DV360): insertion orders with budget_micros named monthly_budget_* (it's a monthly budget), end_date cast back to a date; flags the flat-budget-vs-growing-spend known issue</t>
         </is>
       </c>
       <c r="D233" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 13:19 PDT</t>
+          <t>2026-09-29 13:27 PDT</t>
         </is>
       </c>
     </row>
     <row r="234">
       <c r="A234" s="2" t="inlineStr">
         <is>
-          <t>dbt/models/staging/kinetic/stg_kinetic__dv360_performance_daily.sql</t>
+          <t>dbt/models/staging/kinetic/stg_kinetic__dv360_line_items.sql</t>
         </is>
       </c>
       <c r="B234" s="2" t="inlineStr">
@@ -5583,7 +5583,7 @@
       </c>
       <c r="C234" s="3" t="inlineStr">
         <is>
-          <t>Phase 2 staging (paid media: DV360): line-item x day x exchange x environment performance with combined line_item_day_slice_id key, micros converted to dollars, ctr_fraction</t>
+          <t>Phase 2 staging (paid media: DV360): 1:1 pass-through of dv360_line_items</t>
         </is>
       </c>
       <c r="D234" s="2" t="inlineStr">
@@ -5595,7 +5595,7 @@
     <row r="235">
       <c r="A235" s="2" t="inlineStr">
         <is>
-          <t>dbt/models/staging/kinetic/_kinetic__staging.yml</t>
+          <t>dbt/models/staging/kinetic/stg_kinetic__dv360_performance_daily.sql</t>
         </is>
       </c>
       <c r="B235" s="2" t="inlineStr">
@@ -5605,19 +5605,19 @@
       </c>
       <c r="C235" s="3" t="inlineStr">
         <is>
-          <t>Updated: tests for the 3 DV360 staging models, incl. accepted_values on exchange and environment -- all hand-verified against live data first</t>
+          <t>Phase 2 staging (paid media: DV360): line-item x day x exchange x environment performance with combined line_item_day_slice_id key, micros converted to dollars, ctr_fraction</t>
         </is>
       </c>
       <c r="D235" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 16:08 PDT</t>
+          <t>2026-09-29 13:19 PDT</t>
         </is>
       </c>
     </row>
     <row r="236">
       <c r="A236" s="2" t="inlineStr">
         <is>
-          <t>generator/params.py</t>
+          <t>dbt/models/staging/kinetic/_kinetic__staging.yml</t>
         </is>
       </c>
       <c r="B236" s="2" t="inlineStr">
@@ -5627,41 +5627,41 @@
       </c>
       <c r="C236" s="3" t="inlineStr">
         <is>
-          <t>Updated 2026-09-29: every evergreen ad budget on all 6 platforms is now the campaign's CURRENT budget, sized from realized spend (weekly average &lt;= budget, no day &gt; 1.75x; DV360 monthly &gt;= highest month). The old flat 'typical day' budgets let later months spend up to ~20x the stored budget</t>
+          <t>Updated: tests for the 3 DV360 staging models, incl. accepted_values on exchange and environment -- all hand-verified against live data first</t>
         </is>
       </c>
       <c r="D236" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 13:23 PDT</t>
+          <t>2026-09-29 16:08 PDT</t>
         </is>
       </c>
     </row>
     <row r="237">
       <c r="A237" s="2" t="inlineStr">
         <is>
-          <t>data/meta_campaigns.csv</t>
+          <t>generator/params.py</t>
         </is>
       </c>
       <c r="B237" s="2" t="inlineStr">
         <is>
-          <t>Shipped table</t>
+          <t>Code</t>
         </is>
       </c>
       <c r="C237" s="3" t="inlineStr">
         <is>
-          <t>Regenerated 2026-09-29: evergreen daily_budget values updated to current budgets (only that column, only the 4 evergreen rows changed)</t>
+          <t>Updated 2026-09-29: every evergreen ad budget on all 6 platforms is now the campaign's CURRENT budget, sized from realized spend (weekly average &lt;= budget, no day &gt; 1.75x; DV360 monthly &gt;= highest month). The old flat 'typical day' budgets let later months spend up to ~20x the stored budget</t>
         </is>
       </c>
       <c r="D237" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 13:24 PDT</t>
+          <t>2026-09-29 13:23 PDT</t>
         </is>
       </c>
     </row>
     <row r="238">
       <c r="A238" s="2" t="inlineStr">
         <is>
-          <t>data/google_search_campaigns.csv</t>
+          <t>data/meta_campaigns.csv</t>
         </is>
       </c>
       <c r="B238" s="2" t="inlineStr">
@@ -5671,7 +5671,7 @@
       </c>
       <c r="C238" s="3" t="inlineStr">
         <is>
-          <t>Regenerated 2026-09-29: campaign_budget_micros updated to current budgets (only that column changed)</t>
+          <t>Regenerated 2026-09-29: evergreen daily_budget values updated to current budgets (only that column, only the 4 evergreen rows changed)</t>
         </is>
       </c>
       <c r="D238" s="2" t="inlineStr">
@@ -5683,7 +5683,7 @@
     <row r="239">
       <c r="A239" s="2" t="inlineStr">
         <is>
-          <t>data/youtube_campaigns.csv</t>
+          <t>data/google_search_campaigns.csv</t>
         </is>
       </c>
       <c r="B239" s="2" t="inlineStr">
@@ -5693,7 +5693,7 @@
       </c>
       <c r="C239" s="3" t="inlineStr">
         <is>
-          <t>Regenerated 2026-09-29: evergreen campaign_budget_micros updated to current budgets (only that column, only the 4 evergreen rows changed)</t>
+          <t>Regenerated 2026-09-29: campaign_budget_micros updated to current budgets (only that column changed)</t>
         </is>
       </c>
       <c r="D239" s="2" t="inlineStr">
@@ -5705,7 +5705,7 @@
     <row r="240">
       <c r="A240" s="2" t="inlineStr">
         <is>
-          <t>data/dv360_insertion_orders.csv</t>
+          <t>data/youtube_campaigns.csv</t>
         </is>
       </c>
       <c r="B240" s="2" t="inlineStr">
@@ -5715,7 +5715,7 @@
       </c>
       <c r="C240" s="3" t="inlineStr">
         <is>
-          <t>Regenerated 2026-09-29: monthly budget_micros updated to current budgets (only that column changed)</t>
+          <t>Regenerated 2026-09-29: evergreen campaign_budget_micros updated to current budgets (only that column, only the 4 evergreen rows changed)</t>
         </is>
       </c>
       <c r="D240" s="2" t="inlineStr">
@@ -5727,7 +5727,7 @@
     <row r="241">
       <c r="A241" s="2" t="inlineStr">
         <is>
-          <t>data/snap_campaigns.csv</t>
+          <t>data/dv360_insertion_orders.csv</t>
         </is>
       </c>
       <c r="B241" s="2" t="inlineStr">
@@ -5737,7 +5737,7 @@
       </c>
       <c r="C241" s="3" t="inlineStr">
         <is>
-          <t>Regenerated 2026-09-29: evergreen daily_budget_micro updated to current budgets (only that column, only the 4 evergreen rows changed)</t>
+          <t>Regenerated 2026-09-29: monthly budget_micros updated to current budgets (only that column changed)</t>
         </is>
       </c>
       <c r="D241" s="2" t="inlineStr">
@@ -5749,7 +5749,7 @@
     <row r="242">
       <c r="A242" s="2" t="inlineStr">
         <is>
-          <t>data/tiktok_campaigns.csv</t>
+          <t>data/snap_campaigns.csv</t>
         </is>
       </c>
       <c r="B242" s="2" t="inlineStr">
@@ -5759,7 +5759,7 @@
       </c>
       <c r="C242" s="3" t="inlineStr">
         <is>
-          <t>Regenerated 2026-09-29: BUDGET_MODE_DAY budget_micro updated to current budgets (only that column, only the 4 evergreen rows changed)</t>
+          <t>Regenerated 2026-09-29: evergreen daily_budget_micro updated to current budgets (only that column, only the 4 evergreen rows changed)</t>
         </is>
       </c>
       <c r="D242" s="2" t="inlineStr">
@@ -5771,29 +5771,29 @@
     <row r="243">
       <c r="A243" s="2" t="inlineStr">
         <is>
-          <t>generator/audit_cross_dataset_alignment.py</t>
+          <t>data/tiktok_campaigns.csv</t>
         </is>
       </c>
       <c r="B243" s="2" t="inlineStr">
         <is>
-          <t>Code</t>
+          <t>Shipped table</t>
         </is>
       </c>
       <c r="C243" s="3" t="inlineStr">
         <is>
-          <t>Updated 2026-09-29: new Check 8 -- spend vs stored budget for every campaign on all 6 platforms (weekly/daily limits for daily budgets, monthly for DV360, total for holiday flights)</t>
+          <t>Regenerated 2026-09-29: BUDGET_MODE_DAY budget_micro updated to current budgets (only that column, only the 4 evergreen rows changed)</t>
         </is>
       </c>
       <c r="D243" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 13:30 PDT</t>
+          <t>2026-09-29 13:24 PDT</t>
         </is>
       </c>
     </row>
     <row r="244">
       <c r="A244" s="2" t="inlineStr">
         <is>
-          <t>dbt/models/staging/kinetic/stg_kinetic__dv360_insertion_orders.sql</t>
+          <t>generator/audit_cross_dataset_alignment.py</t>
         </is>
       </c>
       <c r="B244" s="2" t="inlineStr">
@@ -5803,19 +5803,19 @@
       </c>
       <c r="C244" s="3" t="inlineStr">
         <is>
-          <t>Updated: budget known-issue note replaced -- budgets are now current budgets</t>
+          <t>Updated 2026-09-29: new Check 8 -- spend vs stored budget for every campaign on all 6 platforms (weekly/daily limits for daily budgets, monthly for DV360, total for holiday flights)</t>
         </is>
       </c>
       <c r="D244" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 13:27 PDT</t>
+          <t>2026-09-29 13:30 PDT</t>
         </is>
       </c>
     </row>
     <row r="245">
       <c r="A245" s="2" t="inlineStr">
         <is>
-          <t>generator/paid_media_common.py</t>
+          <t>dbt/models/staging/kinetic/stg_kinetic__dv360_insertion_orders.sql</t>
         </is>
       </c>
       <c r="B245" s="2" t="inlineStr">
@@ -5825,19 +5825,19 @@
       </c>
       <c r="C245" s="3" t="inlineStr">
         <is>
-          <t>Updated 2026-09-29: new cap_flight_at_budget() -- rescales a holiday flight's days so it never spends past its lifetime budget, replaying the same random rates so every other row is unchanged</t>
+          <t>Updated: budget known-issue note replaced -- budgets are now current budgets</t>
         </is>
       </c>
       <c r="D245" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 13:29 PDT</t>
+          <t>2026-09-29 13:27 PDT</t>
         </is>
       </c>
     </row>
     <row r="246">
       <c r="A246" s="2" t="inlineStr">
         <is>
-          <t>generator/build_meta_ad_insights_daily.py</t>
+          <t>generator/paid_media_common.py</t>
         </is>
       </c>
       <c r="B246" s="2" t="inlineStr">
@@ -5847,7 +5847,7 @@
       </c>
       <c r="C246" s="3" t="inlineStr">
         <is>
-          <t>Updated 2026-09-29: holiday flights capped at their lifetime budget via cap_flight_at_budget()</t>
+          <t>Updated 2026-09-29: new cap_flight_at_budget() -- rescales a holiday flight's days so it never spends past its lifetime budget, replaying the same random rates so every other row is unchanged</t>
         </is>
       </c>
       <c r="D246" s="2" t="inlineStr">
@@ -5859,7 +5859,7 @@
     <row r="247">
       <c r="A247" s="2" t="inlineStr">
         <is>
-          <t>generator/build_snap_stats_daily.py</t>
+          <t>generator/build_meta_ad_insights_daily.py</t>
         </is>
       </c>
       <c r="B247" s="2" t="inlineStr">
@@ -5881,7 +5881,7 @@
     <row r="248">
       <c r="A248" s="2" t="inlineStr">
         <is>
-          <t>generator/build_tiktok_reports_daily.py</t>
+          <t>generator/build_snap_stats_daily.py</t>
         </is>
       </c>
       <c r="B248" s="2" t="inlineStr">
@@ -5903,7 +5903,7 @@
     <row r="249">
       <c r="A249" s="2" t="inlineStr">
         <is>
-          <t>generator/build_youtube_performance_daily.py</t>
+          <t>generator/build_tiktok_reports_daily.py</t>
         </is>
       </c>
       <c r="B249" s="2" t="inlineStr">
@@ -5913,7 +5913,7 @@
       </c>
       <c r="C249" s="3" t="inlineStr">
         <is>
-          <t>Updated 2026-09-29: holiday flights capped at their lifetime budget via cap_flight_at_budget() (no-op today -- all YouTube flights were already under budget)</t>
+          <t>Updated 2026-09-29: holiday flights capped at their lifetime budget via cap_flight_at_budget()</t>
         </is>
       </c>
       <c r="D249" s="2" t="inlineStr">
@@ -5925,17 +5925,17 @@
     <row r="250">
       <c r="A250" s="2" t="inlineStr">
         <is>
-          <t>data/meta_ad_insights_daily.csv</t>
+          <t>generator/build_youtube_performance_daily.py</t>
         </is>
       </c>
       <c r="B250" s="2" t="inlineStr">
         <is>
-          <t>Shipped table</t>
+          <t>Code</t>
         </is>
       </c>
       <c r="C250" s="3" t="inlineStr">
         <is>
-          <t>Regenerated 2026-09-29: the 2023 and 2024 holiday flights (38 rows) trimmed to spend exactly their lifetime budget; every other row identical</t>
+          <t>Updated 2026-09-29: holiday flights capped at their lifetime budget via cap_flight_at_budget() (no-op today -- all YouTube flights were already under budget)</t>
         </is>
       </c>
       <c r="D250" s="2" t="inlineStr">
@@ -5947,7 +5947,7 @@
     <row r="251">
       <c r="A251" s="2" t="inlineStr">
         <is>
-          <t>data/meta_ad_actions_daily.csv</t>
+          <t>data/meta_ad_insights_daily.csv</t>
         </is>
       </c>
       <c r="B251" s="2" t="inlineStr">
@@ -5957,7 +5957,7 @@
       </c>
       <c r="C251" s="3" t="inlineStr">
         <is>
-          <t>Regenerated 2026-09-29: re-derived from the trimmed insights rows -- only the 2023/2024 holiday flights' action rows changed (one initiate_checkout row on 2024-11-15 dropped to zero and is no longer emitted)</t>
+          <t>Regenerated 2026-09-29: the 2023 and 2024 holiday flights (38 rows) trimmed to spend exactly their lifetime budget; every other row identical</t>
         </is>
       </c>
       <c r="D251" s="2" t="inlineStr">
@@ -5969,7 +5969,7 @@
     <row r="252">
       <c r="A252" s="2" t="inlineStr">
         <is>
-          <t>data/snap_stats_daily.csv</t>
+          <t>data/meta_ad_actions_daily.csv</t>
         </is>
       </c>
       <c r="B252" s="2" t="inlineStr">
@@ -5979,7 +5979,7 @@
       </c>
       <c r="C252" s="3" t="inlineStr">
         <is>
-          <t>Regenerated 2026-09-29: the 2024 holiday flight (19 rows) trimmed to spend exactly its lifetime budget; every other row identical</t>
+          <t>Regenerated 2026-09-29: re-derived from the trimmed insights rows -- only the 2023/2024 holiday flights' action rows changed (one initiate_checkout row on 2024-11-15 dropped to zero and is no longer emitted)</t>
         </is>
       </c>
       <c r="D252" s="2" t="inlineStr">
@@ -5991,7 +5991,7 @@
     <row r="253">
       <c r="A253" s="2" t="inlineStr">
         <is>
-          <t>data/tiktok_reports_daily.csv</t>
+          <t>data/snap_stats_daily.csv</t>
         </is>
       </c>
       <c r="B253" s="2" t="inlineStr">
@@ -6001,7 +6001,7 @@
       </c>
       <c r="C253" s="3" t="inlineStr">
         <is>
-          <t>Regenerated 2026-09-29: the 2023/2024/2025 holiday flights (56 rows) trimmed to spend exactly their lifetime budgets; every other row identical</t>
+          <t>Regenerated 2026-09-29: the 2024 holiday flight (19 rows) trimmed to spend exactly its lifetime budget; every other row identical</t>
         </is>
       </c>
       <c r="D253" s="2" t="inlineStr">
@@ -6013,51 +6013,51 @@
     <row r="254">
       <c r="A254" s="2" t="inlineStr">
         <is>
-          <t>docs/cross_dataset_alignment_audit.md</t>
+          <t>data/tiktok_reports_daily.csv</t>
         </is>
       </c>
       <c r="B254" s="2" t="inlineStr">
         <is>
-          <t>Docs</t>
+          <t>Shipped table</t>
         </is>
       </c>
       <c r="C254" s="3" t="inlineStr">
         <is>
-          <t>Updated 2026-09-29: added Check 8 (spend vs stored budget) with both fixes and results</t>
+          <t>Regenerated 2026-09-29: the 2023/2024/2025 holiday flights (56 rows) trimmed to spend exactly their lifetime budgets; every other row identical</t>
         </is>
       </c>
       <c r="D254" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 13:54 PDT</t>
+          <t>2026-09-29 13:29 PDT</t>
         </is>
       </c>
     </row>
     <row r="255">
       <c r="A255" s="2" t="inlineStr">
         <is>
-          <t>generator/audit_cross_dataset_alignment.py</t>
+          <t>docs/cross_dataset_alignment_audit.md</t>
         </is>
       </c>
       <c r="B255" s="2" t="inlineStr">
         <is>
-          <t>Code</t>
+          <t>Docs</t>
         </is>
       </c>
       <c r="C255" s="3" t="inlineStr">
         <is>
-          <t>Updated 2026-09-29: Check 8's flight limit tightened from 1.05x to 1.0x now that flights are capped</t>
+          <t>Updated 2026-09-29: added Check 8 (spend vs stored budget) with both fixes and results</t>
         </is>
       </c>
       <c r="D255" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 13:30 PDT</t>
+          <t>2026-09-29 13:54 PDT</t>
         </is>
       </c>
     </row>
     <row r="256">
       <c r="A256" s="2" t="inlineStr">
         <is>
-          <t>dbt/models/staging/kinetic/stg_kinetic__snap_campaigns.sql</t>
+          <t>generator/audit_cross_dataset_alignment.py</t>
         </is>
       </c>
       <c r="B256" s="2" t="inlineStr">
@@ -6067,19 +6067,19 @@
       </c>
       <c r="C256" s="3" t="inlineStr">
         <is>
-          <t>Phase 2 staging (paid media: Snap): campaigns with ad_account_id renamed snap_ad_account_id, current budgets in micros and dollars</t>
+          <t>Updated 2026-09-29: Check 8's flight limit tightened from 1.05x to 1.0x now that flights are capped</t>
         </is>
       </c>
       <c r="D256" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 15:53 PDT</t>
+          <t>2026-09-29 13:30 PDT</t>
         </is>
       </c>
     </row>
     <row r="257">
       <c r="A257" s="2" t="inlineStr">
         <is>
-          <t>dbt/models/staging/kinetic/stg_kinetic__snap_ad_squads.sql</t>
+          <t>dbt/models/staging/kinetic/stg_kinetic__snap_campaigns.sql</t>
         </is>
       </c>
       <c r="B257" s="2" t="inlineStr">
@@ -6089,7 +6089,7 @@
       </c>
       <c r="C257" s="3" t="inlineStr">
         <is>
-          <t>Phase 2 staging (paid media: Snap): 1:1 pass-through of snap_ad_squads (Snap's ad set / ad group level)</t>
+          <t>Phase 2 staging (paid media: Snap): campaigns with ad_account_id renamed snap_ad_account_id, current budgets in micros and dollars</t>
         </is>
       </c>
       <c r="D257" s="2" t="inlineStr">
@@ -6101,7 +6101,7 @@
     <row r="258">
       <c r="A258" s="2" t="inlineStr">
         <is>
-          <t>dbt/models/staging/kinetic/stg_kinetic__snap_ads.sql</t>
+          <t>dbt/models/staging/kinetic/stg_kinetic__snap_ad_squads.sql</t>
         </is>
       </c>
       <c r="B258" s="2" t="inlineStr">
@@ -6111,7 +6111,7 @@
       </c>
       <c r="C258" s="3" t="inlineStr">
         <is>
-          <t>Phase 2 staging (paid media: Snap): 1:1 pass-through of snap_ads</t>
+          <t>Phase 2 staging (paid media: Snap): 1:1 pass-through of snap_ad_squads (Snap's ad set / ad group level)</t>
         </is>
       </c>
       <c r="D258" s="2" t="inlineStr">
@@ -6123,7 +6123,7 @@
     <row r="259">
       <c r="A259" s="2" t="inlineStr">
         <is>
-          <t>dbt/models/staging/kinetic/stg_kinetic__snap_stats_daily.sql</t>
+          <t>dbt/models/staging/kinetic/stg_kinetic__snap_ads.sql</t>
         </is>
       </c>
       <c r="B259" s="2" t="inlineStr">
@@ -6133,7 +6133,7 @@
       </c>
       <c r="C259" s="3" t="inlineStr">
         <is>
-          <t>Phase 2 staging (paid media: Snap): ad-day stats with combined ad_day_id key, spend in micros and dollars; documents swipes as Snap's clicks</t>
+          <t>Phase 2 staging (paid media: Snap): 1:1 pass-through of snap_ads</t>
         </is>
       </c>
       <c r="D259" s="2" t="inlineStr">
@@ -6145,7 +6145,7 @@
     <row r="260">
       <c r="A260" s="2" t="inlineStr">
         <is>
-          <t>dbt/models/staging/kinetic/_kinetic__staging.yml</t>
+          <t>dbt/models/staging/kinetic/stg_kinetic__snap_stats_daily.sql</t>
         </is>
       </c>
       <c r="B260" s="2" t="inlineStr">
@@ -6155,19 +6155,19 @@
       </c>
       <c r="C260" s="3" t="inlineStr">
         <is>
-          <t>Updated: tests for the 4 Snap staging models -- all hand-verified against live data first</t>
+          <t>Phase 2 staging (paid media: Snap): ad-day stats with combined ad_day_id key, spend in micros and dollars; documents swipes as Snap's clicks</t>
         </is>
       </c>
       <c r="D260" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 16:08 PDT</t>
+          <t>2026-09-29 15:53 PDT</t>
         </is>
       </c>
     </row>
     <row r="261">
       <c r="A261" s="2" t="inlineStr">
         <is>
-          <t>dbt/models/staging/kinetic/stg_kinetic__tiktok_campaigns.sql</t>
+          <t>dbt/models/staging/kinetic/_kinetic__staging.yml</t>
         </is>
       </c>
       <c r="B261" s="2" t="inlineStr">
@@ -6177,19 +6177,19 @@
       </c>
       <c r="C261" s="3" t="inlineStr">
         <is>
-          <t>Phase 2 staging (paid media: TikTok): campaigns with the single budget split into daily_budget_usd / lifetime_budget_usd by budget_mode (matching the other platforms), advertiser_id renamed tiktok_advertiser_id</t>
+          <t>Updated: tests for the 4 Snap staging models -- all hand-verified against live data first</t>
         </is>
       </c>
       <c r="D261" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 15:57 PDT</t>
+          <t>2026-09-29 16:08 PDT</t>
         </is>
       </c>
     </row>
     <row r="262">
       <c r="A262" s="2" t="inlineStr">
         <is>
-          <t>dbt/models/staging/kinetic/stg_kinetic__tiktok_adgroups.sql</t>
+          <t>dbt/models/staging/kinetic/stg_kinetic__tiktok_campaigns.sql</t>
         </is>
       </c>
       <c r="B262" s="2" t="inlineStr">
@@ -6199,7 +6199,7 @@
       </c>
       <c r="C262" s="3" t="inlineStr">
         <is>
-          <t>Phase 2 staging (paid media: TikTok): 1:1 pass-through of tiktok_adgroups</t>
+          <t>Phase 2 staging (paid media: TikTok): campaigns with the single budget split into daily_budget_usd / lifetime_budget_usd by budget_mode (matching the other platforms), advertiser_id renamed tiktok_advertiser_id</t>
         </is>
       </c>
       <c r="D262" s="2" t="inlineStr">
@@ -6211,7 +6211,7 @@
     <row r="263">
       <c r="A263" s="2" t="inlineStr">
         <is>
-          <t>dbt/models/staging/kinetic/stg_kinetic__tiktok_ads.sql</t>
+          <t>dbt/models/staging/kinetic/stg_kinetic__tiktok_adgroups.sql</t>
         </is>
       </c>
       <c r="B263" s="2" t="inlineStr">
@@ -6221,7 +6221,7 @@
       </c>
       <c r="C263" s="3" t="inlineStr">
         <is>
-          <t>Phase 2 staging (paid media: TikTok): 1:1 pass-through of tiktok_ads</t>
+          <t>Phase 2 staging (paid media: TikTok): 1:1 pass-through of tiktok_adgroups</t>
         </is>
       </c>
       <c r="D263" s="2" t="inlineStr">
@@ -6233,7 +6233,7 @@
     <row r="264">
       <c r="A264" s="2" t="inlineStr">
         <is>
-          <t>dbt/models/staging/kinetic/stg_kinetic__tiktok_reports_daily.sql</t>
+          <t>dbt/models/staging/kinetic/stg_kinetic__tiktok_ads.sql</t>
         </is>
       </c>
       <c r="B264" s="2" t="inlineStr">
@@ -6243,7 +6243,7 @@
       </c>
       <c r="C264" s="3" t="inlineStr">
         <is>
-          <t>Phase 2 staging (paid media: TikTok): ad-day reports with combined ad_day_id key, spend and CPM in micros and dollars, ctr_fraction</t>
+          <t>Phase 2 staging (paid media: TikTok): 1:1 pass-through of tiktok_ads</t>
         </is>
       </c>
       <c r="D264" s="2" t="inlineStr">
@@ -6255,7 +6255,7 @@
     <row r="265">
       <c r="A265" s="2" t="inlineStr">
         <is>
-          <t>dbt/models/staging/kinetic/stg_kinetic__product_variants.sql</t>
+          <t>dbt/models/staging/kinetic/stg_kinetic__tiktok_reports_daily.sql</t>
         </is>
       </c>
       <c r="B265" s="2" t="inlineStr">
@@ -6265,54 +6265,76 @@
       </c>
       <c r="C265" s="3" t="inlineStr">
         <is>
-          <t>Phase 2 staging (final table, 47 of 47): product variants with variant_option, price_adjustment_usd</t>
+          <t>Phase 2 staging (paid media: TikTok): ad-day reports with combined ad_day_id key, spend and CPM in micros and dollars, ctr_fraction</t>
         </is>
       </c>
       <c r="D265" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 16:08 PDT</t>
+          <t>2026-09-29 15:57 PDT</t>
         </is>
       </c>
     </row>
     <row r="266">
       <c r="A266" s="2" t="inlineStr">
         <is>
-          <t>HANDOFF.md</t>
+          <t>dbt/models/staging/kinetic/stg_kinetic__product_variants.sql</t>
         </is>
       </c>
       <c r="B266" s="2" t="inlineStr">
         <is>
-          <t>Doc</t>
+          <t>Code</t>
         </is>
       </c>
       <c r="C266" s="3" t="inlineStr">
         <is>
-          <t>Handoff note for starting a new chat/project: status, open decisions, prior decisions, pitfalls</t>
+          <t>Phase 2 staging (final table, 47 of 47): product variants with variant_option, price_adjustment_usd</t>
         </is>
       </c>
       <c r="D266" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 16:39 PDT</t>
+          <t>2026-09-29 16:08 PDT</t>
         </is>
       </c>
     </row>
     <row r="267">
       <c r="A267" s="2" t="inlineStr">
         <is>
+          <t>HANDOFF.md</t>
+        </is>
+      </c>
+      <c r="B267" s="2" t="inlineStr">
+        <is>
+          <t>Doc</t>
+        </is>
+      </c>
+      <c r="C267" s="3" t="inlineStr">
+        <is>
+          <t>Handoff note for starting a new chat/project: status, open decisions, prior decisions, pitfalls</t>
+        </is>
+      </c>
+      <c r="D267" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-29 16:43 PDT</t>
+        </is>
+      </c>
+    </row>
+    <row r="268">
+      <c r="A268" s="2" t="inlineStr">
+        <is>
           <t>dbt/models/staging/kinetic/_kinetic__staging.yml</t>
         </is>
       </c>
-      <c r="B267" s="2" t="inlineStr">
-        <is>
-          <t>Code</t>
-        </is>
-      </c>
-      <c r="C267" s="3" t="inlineStr">
+      <c r="B268" s="2" t="inlineStr">
+        <is>
+          <t>Code</t>
+        </is>
+      </c>
+      <c r="C268" s="3" t="inlineStr">
         <is>
           <t>Updated: tests for the 4 TikTok staging models -- all hand-verified against live data first</t>
         </is>
       </c>
-      <c r="D267" s="2" t="inlineStr">
+      <c r="D268" s="2" t="inlineStr">
         <is>
           <t>2026-09-29 16:08 PDT</t>
         </is>

</xml_diff>

<commit_message>
mart_mrr_monthly: stop at last month of data, add data_through; log marts built in dbt
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011iLTiTsTyvHcVHREQNUg8N
</commit_message>
<xml_diff>
--- a/File_Manifest.xlsx
+++ b/File_Manifest.xlsx
@@ -506,7 +506,7 @@
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 16:43 PDT</t>
+          <t>2026-09-29 17:03 PDT</t>
         </is>
       </c>
     </row>
@@ -748,7 +748,7 @@
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 16:43 PDT</t>
+          <t>2026-09-29 17:03 PDT</t>
         </is>
       </c>
     </row>
@@ -4576,7 +4576,7 @@
       </c>
       <c r="D188" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 16:08 PDT</t>
+          <t>2026-09-29 16:49 PDT</t>
         </is>
       </c>
     </row>
@@ -4620,7 +4620,7 @@
       </c>
       <c r="D190" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 16:39 PDT</t>
+          <t>2026-09-29 16:49 PDT</t>
         </is>
       </c>
     </row>
@@ -4642,7 +4642,7 @@
       </c>
       <c r="D191" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28 14:48 PDT</t>
+          <t>2026-09-29 17:02 PDT</t>
         </is>
       </c>
     </row>
@@ -4664,7 +4664,7 @@
       </c>
       <c r="D192" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28 14:53 PDT</t>
+          <t>2026-09-29 17:02 PDT</t>
         </is>
       </c>
     </row>
@@ -5016,7 +5016,7 @@
       </c>
       <c r="D208" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 16:08 PDT</t>
+          <t>2026-09-29 16:49 PDT</t>
         </is>
       </c>
     </row>
@@ -5126,7 +5126,7 @@
       </c>
       <c r="D213" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 16:08 PDT</t>
+          <t>2026-09-29 16:49 PDT</t>
         </is>
       </c>
     </row>
@@ -5236,7 +5236,7 @@
       </c>
       <c r="D218" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 16:08 PDT</t>
+          <t>2026-09-29 16:49 PDT</t>
         </is>
       </c>
     </row>
@@ -5346,7 +5346,7 @@
       </c>
       <c r="D223" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 16:08 PDT</t>
+          <t>2026-09-29 16:49 PDT</t>
         </is>
       </c>
     </row>
@@ -5456,7 +5456,7 @@
       </c>
       <c r="D228" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 16:08 PDT</t>
+          <t>2026-09-29 16:49 PDT</t>
         </is>
       </c>
     </row>
@@ -5544,7 +5544,7 @@
       </c>
       <c r="D232" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 16:08 PDT</t>
+          <t>2026-09-29 16:49 PDT</t>
         </is>
       </c>
     </row>
@@ -5632,7 +5632,7 @@
       </c>
       <c r="D236" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 16:08 PDT</t>
+          <t>2026-09-29 16:49 PDT</t>
         </is>
       </c>
     </row>
@@ -6182,7 +6182,7 @@
       </c>
       <c r="D261" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 16:08 PDT</t>
+          <t>2026-09-29 16:49 PDT</t>
         </is>
       </c>
     </row>
@@ -6314,7 +6314,7 @@
       </c>
       <c r="D267" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 16:43 PDT</t>
+          <t>2026-09-29 17:03 PDT</t>
         </is>
       </c>
     </row>
@@ -6336,7 +6336,7 @@
       </c>
       <c r="D268" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 16:08 PDT</t>
+          <t>2026-09-29 16:49 PDT</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
int_orders_net: per-order gross/discount/paid/refund/net with guest customer resolution; tests, manifest, changelog
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012MSGmVw4D6TxU8u8LSeA2e
</commit_message>
<xml_diff>
--- a/File_Manifest.xlsx
+++ b/File_Manifest.xlsx
@@ -435,7 +435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D268"/>
+  <dimension ref="A1:D272"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="48" customWidth="1" min="1" max="1"/>
@@ -506,7 +506,7 @@
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 17:03 PDT</t>
+          <t>2026-09-29 17:09 PDT</t>
         </is>
       </c>
     </row>
@@ -638,7 +638,7 @@
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 16:43 PDT</t>
+          <t>2026-09-29 17:18 PDT</t>
         </is>
       </c>
     </row>
@@ -748,7 +748,7 @@
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 17:03 PDT</t>
+          <t>2026-09-29 17:18 PDT</t>
         </is>
       </c>
     </row>
@@ -4620,7 +4620,7 @@
       </c>
       <c r="D190" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 16:49 PDT</t>
+          <t>2026-09-29 17:18 PDT</t>
         </is>
       </c>
     </row>
@@ -4847,7 +4847,7 @@
     <row r="201">
       <c r="A201" s="2" t="inlineStr">
         <is>
-          <t>dbt/models/marts/mart_storefront_revenue_monthly.sql</t>
+          <t>dbt/models/intermediate/int_orders_net.sql</t>
         </is>
       </c>
       <c r="B201" s="2" t="inlineStr">
@@ -4857,19 +4857,19 @@
       </c>
       <c r="C201" s="3" t="inlineStr">
         <is>
-          <t>Second canonical metric mart: non-subscription (course+merch) gross/net revenue, AOV, guest-checkout share, discount-usage share, refund rate by month -- validated against a hand-run equivalent query on the live database (2026-07: 246 orders, $13,843.71 gross revenue, $56.28 AOV)</t>
+          <t>Intermediate model: one row per order with gross (pre-discount), discount, paid, succeeded-refund and net amounts, plus customer_id resolved for guest orders via email match</t>
         </is>
       </c>
       <c r="D201" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28 14:53 PDT</t>
+          <t>2026-09-29 17:18 PDT</t>
         </is>
       </c>
     </row>
     <row r="202">
       <c r="A202" s="2" t="inlineStr">
         <is>
-          <t>dbt/models/staging/kinetic/stg_kinetic__customer_addresses.sql</t>
+          <t>dbt/tests/assert_int_orders_net_no_negative_net.sql</t>
         </is>
       </c>
       <c r="B202" s="2" t="inlineStr">
@@ -4879,19 +4879,19 @@
       </c>
       <c r="C202" s="3" t="inlineStr">
         <is>
-          <t>Phase 2 staging (Customer 360): 1:1 pass-through of customer_addresses</t>
+          <t>dbt test: fails if any order's net is below zero (net is deliberately not floored)</t>
         </is>
       </c>
       <c r="D202" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 10:26 PDT</t>
+          <t>2026-09-29 17:18 PDT</t>
         </is>
       </c>
     </row>
     <row r="203">
       <c r="A203" s="2" t="inlineStr">
         <is>
-          <t>dbt/models/staging/kinetic/stg_kinetic__devices.sql</t>
+          <t>dbt/tests/assert_int_orders_net_money_reconciles.sql</t>
         </is>
       </c>
       <c r="B203" s="2" t="inlineStr">
@@ -4901,19 +4901,19 @@
       </c>
       <c r="C203" s="3" t="inlineStr">
         <is>
-          <t>Phase 2 staging (Customer 360): 1:1 pass-through of devices, plus is_anonymous_device flag (customer_id null for ~94% of devices by design)</t>
+          <t>dbt test: gross - discount = paid and paid - refund = net on every order</t>
         </is>
       </c>
       <c r="D203" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 10:26 PDT</t>
+          <t>2026-09-29 17:18 PDT</t>
         </is>
       </c>
     </row>
     <row r="204">
       <c r="A204" s="2" t="inlineStr">
         <is>
-          <t>dbt/models/staging/kinetic/stg_kinetic__identity_map.sql</t>
+          <t>dbt/tests/assert_int_orders_net_refunds_match_source.sql</t>
         </is>
       </c>
       <c r="B204" s="2" t="inlineStr">
@@ -4923,19 +4923,19 @@
       </c>
       <c r="C204" s="3" t="inlineStr">
         <is>
-          <t>Phase 2 staging (Customer 360): 1:1 pass-through of identity_map</t>
+          <t>dbt test: total refunds in int_orders_net equal total succeeded refunds in int_orders_refunded</t>
         </is>
       </c>
       <c r="D204" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 10:26 PDT</t>
+          <t>2026-09-29 17:18 PDT</t>
         </is>
       </c>
     </row>
     <row r="205">
       <c r="A205" s="2" t="inlineStr">
         <is>
-          <t>dbt/models/staging/kinetic/stg_kinetic__segments.sql</t>
+          <t>dbt/models/marts/mart_storefront_revenue_monthly.sql</t>
         </is>
       </c>
       <c r="B205" s="2" t="inlineStr">
@@ -4945,19 +4945,19 @@
       </c>
       <c r="C205" s="3" t="inlineStr">
         <is>
-          <t>Phase 2 staging (Customer 360): 1:1 pass-through of segments</t>
+          <t>Second canonical metric mart: non-subscription (course+merch) gross/net revenue, AOV, guest-checkout share, discount-usage share, refund rate by month -- validated against a hand-run equivalent query on the live database (2026-07: 246 orders, $13,843.71 gross revenue, $56.28 AOV)</t>
         </is>
       </c>
       <c r="D205" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 10:26 PDT</t>
+          <t>2026-09-28 14:53 PDT</t>
         </is>
       </c>
     </row>
     <row r="206">
       <c r="A206" s="2" t="inlineStr">
         <is>
-          <t>dbt/models/staging/kinetic/stg_kinetic__customer_segment_membership.sql</t>
+          <t>dbt/models/staging/kinetic/stg_kinetic__customer_addresses.sql</t>
         </is>
       </c>
       <c r="B206" s="2" t="inlineStr">
@@ -4967,7 +4967,7 @@
       </c>
       <c r="C206" s="3" t="inlineStr">
         <is>
-          <t>Phase 2 staging (Customer 360): 1:1 pass-through of customer_segment_membership, plus is_current_member flag</t>
+          <t>Phase 2 staging (Customer 360): 1:1 pass-through of customer_addresses</t>
         </is>
       </c>
       <c r="D206" s="2" t="inlineStr">
@@ -4979,7 +4979,7 @@
     <row r="207">
       <c r="A207" s="2" t="inlineStr">
         <is>
-          <t>dbt/models/staging/kinetic/stg_kinetic__subscription_events.sql</t>
+          <t>dbt/models/staging/kinetic/stg_kinetic__devices.sql</t>
         </is>
       </c>
       <c r="B207" s="2" t="inlineStr">
@@ -4989,7 +4989,7 @@
       </c>
       <c r="C207" s="3" t="inlineStr">
         <is>
-          <t>Phase 2 staging (Customer 360): 1:1 pass-through of subscription_events; old_plan/new_plan renamed to old_plan_id/new_plan_id</t>
+          <t>Phase 2 staging (Customer 360): 1:1 pass-through of devices, plus is_anonymous_device flag (customer_id null for ~94% of devices by design)</t>
         </is>
       </c>
       <c r="D207" s="2" t="inlineStr">
@@ -5001,7 +5001,7 @@
     <row r="208">
       <c r="A208" s="2" t="inlineStr">
         <is>
-          <t>dbt/models/staging/kinetic/_kinetic__staging.yml</t>
+          <t>dbt/models/staging/kinetic/stg_kinetic__identity_map.sql</t>
         </is>
       </c>
       <c r="B208" s="2" t="inlineStr">
@@ -5011,19 +5011,19 @@
       </c>
       <c r="C208" s="3" t="inlineStr">
         <is>
-          <t>Updated: tests for the 6 Customer 360 staging models (PK not_null/unique, FK relationships) -- all hand-verified against live data first</t>
+          <t>Phase 2 staging (Customer 360): 1:1 pass-through of identity_map</t>
         </is>
       </c>
       <c r="D208" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 16:49 PDT</t>
+          <t>2026-09-29 10:26 PDT</t>
         </is>
       </c>
     </row>
     <row r="209">
       <c r="A209" s="2" t="inlineStr">
         <is>
-          <t>dbt/models/staging/kinetic/stg_kinetic__web_sessions.sql</t>
+          <t>dbt/models/staging/kinetic/stg_kinetic__segments.sql</t>
         </is>
       </c>
       <c r="B209" s="2" t="inlineStr">
@@ -5033,19 +5033,19 @@
       </c>
       <c r="C209" s="3" t="inlineStr">
         <is>
-          <t>Phase 2 staging (web/app engagement): 1:1 pass-through of web_sessions, plus is_known_customer flag (customer_id null for ~79% of sessions by design)</t>
+          <t>Phase 2 staging (Customer 360): 1:1 pass-through of segments</t>
         </is>
       </c>
       <c r="D209" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 12:58 PDT</t>
+          <t>2026-09-29 10:26 PDT</t>
         </is>
       </c>
     </row>
     <row r="210">
       <c r="A210" s="2" t="inlineStr">
         <is>
-          <t>dbt/models/staging/kinetic/stg_kinetic__web_events.sql</t>
+          <t>dbt/models/staging/kinetic/stg_kinetic__customer_segment_membership.sql</t>
         </is>
       </c>
       <c r="B210" s="2" t="inlineStr">
@@ -5055,19 +5055,19 @@
       </c>
       <c r="C210" s="3" t="inlineStr">
         <is>
-          <t>Phase 2 staging (web/app engagement): 1:1 pass-through of web_events</t>
+          <t>Phase 2 staging (Customer 360): 1:1 pass-through of customer_segment_membership, plus is_current_member flag</t>
         </is>
       </c>
       <c r="D210" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 12:58 PDT</t>
+          <t>2026-09-29 10:26 PDT</t>
         </is>
       </c>
     </row>
     <row r="211">
       <c r="A211" s="2" t="inlineStr">
         <is>
-          <t>dbt/models/staging/kinetic/stg_kinetic__app_sessions.sql</t>
+          <t>dbt/models/staging/kinetic/stg_kinetic__subscription_events.sql</t>
         </is>
       </c>
       <c r="B211" s="2" t="inlineStr">
@@ -5077,19 +5077,19 @@
       </c>
       <c r="C211" s="3" t="inlineStr">
         <is>
-          <t>Phase 2 staging (web/app engagement): 1:1 pass-through of app_sessions</t>
+          <t>Phase 2 staging (Customer 360): 1:1 pass-through of subscription_events; old_plan/new_plan renamed to old_plan_id/new_plan_id</t>
         </is>
       </c>
       <c r="D211" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 12:58 PDT</t>
+          <t>2026-09-29 10:26 PDT</t>
         </is>
       </c>
     </row>
     <row r="212">
       <c r="A212" s="2" t="inlineStr">
         <is>
-          <t>dbt/models/staging/kinetic/stg_kinetic__app_events.sql</t>
+          <t>dbt/models/staging/kinetic/_kinetic__staging.yml</t>
         </is>
       </c>
       <c r="B212" s="2" t="inlineStr">
@@ -5099,19 +5099,19 @@
       </c>
       <c r="C212" s="3" t="inlineStr">
         <is>
-          <t>Phase 2 staging (web/app engagement): 1:1 pass-through of app_events</t>
+          <t>Updated: tests for the 6 Customer 360 staging models (PK not_null/unique, FK relationships) -- all hand-verified against live data first</t>
         </is>
       </c>
       <c r="D212" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 12:58 PDT</t>
+          <t>2026-09-29 16:49 PDT</t>
         </is>
       </c>
     </row>
     <row r="213">
       <c r="A213" s="2" t="inlineStr">
         <is>
-          <t>dbt/models/staging/kinetic/_kinetic__staging.yml</t>
+          <t>dbt/models/staging/kinetic/stg_kinetic__web_sessions.sql</t>
         </is>
       </c>
       <c r="B213" s="2" t="inlineStr">
@@ -5121,19 +5121,19 @@
       </c>
       <c r="C213" s="3" t="inlineStr">
         <is>
-          <t>Updated: tests for the 4 web/app engagement staging models -- all hand-verified against live data first</t>
+          <t>Phase 2 staging (web/app engagement): 1:1 pass-through of web_sessions, plus is_known_customer flag (customer_id null for ~79% of sessions by design)</t>
         </is>
       </c>
       <c r="D213" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 16:49 PDT</t>
+          <t>2026-09-29 12:58 PDT</t>
         </is>
       </c>
     </row>
     <row r="214">
       <c r="A214" s="2" t="inlineStr">
         <is>
-          <t>dbt/models/staging/kinetic/stg_kinetic__braze_email_campaigns.sql</t>
+          <t>dbt/models/staging/kinetic/stg_kinetic__web_events.sql</t>
         </is>
       </c>
       <c r="B214" s="2" t="inlineStr">
@@ -5143,19 +5143,19 @@
       </c>
       <c r="C214" s="3" t="inlineStr">
         <is>
-          <t>Phase 2 staging (email/push): 1:1 pass-through of braze_email_campaigns</t>
+          <t>Phase 2 staging (web/app engagement): 1:1 pass-through of web_events</t>
         </is>
       </c>
       <c r="D214" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 12:59 PDT</t>
+          <t>2026-09-29 12:58 PDT</t>
         </is>
       </c>
     </row>
     <row r="215">
       <c r="A215" s="2" t="inlineStr">
         <is>
-          <t>dbt/models/staging/kinetic/stg_kinetic__braze_push_campaigns.sql</t>
+          <t>dbt/models/staging/kinetic/stg_kinetic__app_sessions.sql</t>
         </is>
       </c>
       <c r="B215" s="2" t="inlineStr">
@@ -5165,19 +5165,19 @@
       </c>
       <c r="C215" s="3" t="inlineStr">
         <is>
-          <t>Phase 2 staging (email/push): 1:1 pass-through of braze_push_campaigns</t>
+          <t>Phase 2 staging (web/app engagement): 1:1 pass-through of app_sessions</t>
         </is>
       </c>
       <c r="D215" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 12:59 PDT</t>
+          <t>2026-09-29 12:58 PDT</t>
         </is>
       </c>
     </row>
     <row r="216">
       <c r="A216" s="2" t="inlineStr">
         <is>
-          <t>dbt/models/staging/kinetic/stg_kinetic__braze_email_events.sql</t>
+          <t>dbt/models/staging/kinetic/stg_kinetic__app_events.sql</t>
         </is>
       </c>
       <c r="B216" s="2" t="inlineStr">
@@ -5187,19 +5187,19 @@
       </c>
       <c r="C216" s="3" t="inlineStr">
         <is>
-          <t>Phase 2 staging (email/push): braze_email_events with external_user_id renamed to customer_id and a short event_name (send/open/click/bounce/unsubscribe) alongside Braze's raw event_type</t>
+          <t>Phase 2 staging (web/app engagement): 1:1 pass-through of app_events</t>
         </is>
       </c>
       <c r="D216" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 12:59 PDT</t>
+          <t>2026-09-29 12:58 PDT</t>
         </is>
       </c>
     </row>
     <row r="217">
       <c r="A217" s="2" t="inlineStr">
         <is>
-          <t>dbt/models/staging/kinetic/stg_kinetic__braze_push_events.sql</t>
+          <t>dbt/models/staging/kinetic/_kinetic__staging.yml</t>
         </is>
       </c>
       <c r="B217" s="2" t="inlineStr">
@@ -5209,19 +5209,19 @@
       </c>
       <c r="C217" s="3" t="inlineStr">
         <is>
-          <t>Phase 2 staging (email/push): braze_push_events with external_user_id renamed to customer_id and a short event_name alongside Braze's raw event_type</t>
+          <t>Updated: tests for the 4 web/app engagement staging models -- all hand-verified against live data first</t>
         </is>
       </c>
       <c r="D217" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 12:59 PDT</t>
+          <t>2026-09-29 16:49 PDT</t>
         </is>
       </c>
     </row>
     <row r="218">
       <c r="A218" s="2" t="inlineStr">
         <is>
-          <t>dbt/models/staging/kinetic/_kinetic__staging.yml</t>
+          <t>dbt/models/staging/kinetic/stg_kinetic__braze_email_campaigns.sql</t>
         </is>
       </c>
       <c r="B218" s="2" t="inlineStr">
@@ -5231,19 +5231,19 @@
       </c>
       <c r="C218" s="3" t="inlineStr">
         <is>
-          <t>Updated: tests for the 4 Braze staging models, incl. accepted_values on event_name -- all hand-verified against live data first</t>
+          <t>Phase 2 staging (email/push): 1:1 pass-through of braze_email_campaigns</t>
         </is>
       </c>
       <c r="D218" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 16:49 PDT</t>
+          <t>2026-09-29 12:59 PDT</t>
         </is>
       </c>
     </row>
     <row r="219">
       <c r="A219" s="2" t="inlineStr">
         <is>
-          <t>dbt/models/staging/kinetic/stg_kinetic__meta_campaigns.sql</t>
+          <t>dbt/models/staging/kinetic/stg_kinetic__braze_push_campaigns.sql</t>
         </is>
       </c>
       <c r="B219" s="2" t="inlineStr">
@@ -5253,19 +5253,19 @@
       </c>
       <c r="C219" s="3" t="inlineStr">
         <is>
-          <t>Phase 2 staging (paid media: Meta): meta_campaigns with budgets in both raw cents and dollars (Meta API stores budgets in cents)</t>
+          <t>Phase 2 staging (email/push): 1:1 pass-through of braze_push_campaigns</t>
         </is>
       </c>
       <c r="D219" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 13:02 PDT</t>
+          <t>2026-09-29 12:59 PDT</t>
         </is>
       </c>
     </row>
     <row r="220">
       <c r="A220" s="2" t="inlineStr">
         <is>
-          <t>dbt/models/staging/kinetic/stg_kinetic__meta_ads.sql</t>
+          <t>dbt/models/staging/kinetic/stg_kinetic__braze_email_events.sql</t>
         </is>
       </c>
       <c r="B220" s="2" t="inlineStr">
@@ -5275,19 +5275,19 @@
       </c>
       <c r="C220" s="3" t="inlineStr">
         <is>
-          <t>Phase 2 staging (paid media: Meta): 1:1 pass-through of meta_ads</t>
+          <t>Phase 2 staging (email/push): braze_email_events with external_user_id renamed to customer_id and a short event_name (send/open/click/bounce/unsubscribe) alongside Braze's raw event_type</t>
         </is>
       </c>
       <c r="D220" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 13:02 PDT</t>
+          <t>2026-09-29 12:59 PDT</t>
         </is>
       </c>
     </row>
     <row r="221">
       <c r="A221" s="2" t="inlineStr">
         <is>
-          <t>dbt/models/staging/kinetic/stg_kinetic__meta_ad_insights_daily.sql</t>
+          <t>dbt/models/staging/kinetic/stg_kinetic__braze_push_events.sql</t>
         </is>
       </c>
       <c r="B221" s="2" t="inlineStr">
@@ -5297,19 +5297,19 @@
       </c>
       <c r="C221" s="3" t="inlineStr">
         <is>
-          <t>Phase 2 staging (paid media: Meta): meta_ad_insights_daily with a combined ad_day_id key, unit-suffixed columns (spend_usd, cpm_usd, cpc_usd) and ctr renamed ctr_fraction (0.017 = 1.7%)</t>
+          <t>Phase 2 staging (email/push): braze_push_events with external_user_id renamed to customer_id and a short event_name alongside Braze's raw event_type</t>
         </is>
       </c>
       <c r="D221" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 13:02 PDT</t>
+          <t>2026-09-29 12:59 PDT</t>
         </is>
       </c>
     </row>
     <row r="222">
       <c r="A222" s="2" t="inlineStr">
         <is>
-          <t>dbt/models/staging/kinetic/stg_kinetic__meta_ad_actions_daily.sql</t>
+          <t>dbt/models/staging/kinetic/_kinetic__staging.yml</t>
         </is>
       </c>
       <c r="B222" s="2" t="inlineStr">
@@ -5319,19 +5319,19 @@
       </c>
       <c r="C222" s="3" t="inlineStr">
         <is>
-          <t>Phase 2 staging (paid media: Meta): meta_ad_actions_daily with a combined ad_day_action_id key; value renamed action_count</t>
+          <t>Updated: tests for the 4 Braze staging models, incl. accepted_values on event_name -- all hand-verified against live data first</t>
         </is>
       </c>
       <c r="D222" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 13:02 PDT</t>
+          <t>2026-09-29 16:49 PDT</t>
         </is>
       </c>
     </row>
     <row r="223">
       <c r="A223" s="2" t="inlineStr">
         <is>
-          <t>dbt/models/staging/kinetic/_kinetic__staging.yml</t>
+          <t>dbt/models/staging/kinetic/stg_kinetic__meta_campaigns.sql</t>
         </is>
       </c>
       <c r="B223" s="2" t="inlineStr">
@@ -5341,19 +5341,19 @@
       </c>
       <c r="C223" s="3" t="inlineStr">
         <is>
-          <t>Updated: tests for the 4 Meta staging models, incl. uniqueness of the combined daily keys -- all hand-verified against live data first</t>
+          <t>Phase 2 staging (paid media: Meta): meta_campaigns with budgets in both raw cents and dollars (Meta API stores budgets in cents)</t>
         </is>
       </c>
       <c r="D223" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 16:49 PDT</t>
+          <t>2026-09-29 13:02 PDT</t>
         </is>
       </c>
     </row>
     <row r="224">
       <c r="A224" s="2" t="inlineStr">
         <is>
-          <t>dbt/models/staging/kinetic/stg_kinetic__google_search_campaigns.sql</t>
+          <t>dbt/models/staging/kinetic/stg_kinetic__meta_ads.sql</t>
         </is>
       </c>
       <c r="B224" s="2" t="inlineStr">
@@ -5363,19 +5363,19 @@
       </c>
       <c r="C224" s="3" t="inlineStr">
         <is>
-          <t>Phase 2 staging (paid media: Google Search): campaigns with the raw customer_id renamed google_ads_account_id (it's the Google Ads account number, not a Kinetic customer), daily budget in micros and dollars, end_date cast back to a date</t>
+          <t>Phase 2 staging (paid media: Meta): 1:1 pass-through of meta_ads</t>
         </is>
       </c>
       <c r="D224" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 13:13 PDT</t>
+          <t>2026-09-29 13:02 PDT</t>
         </is>
       </c>
     </row>
     <row r="225">
       <c r="A225" s="2" t="inlineStr">
         <is>
-          <t>dbt/models/staging/kinetic/stg_kinetic__google_search_ad_groups.sql</t>
+          <t>dbt/models/staging/kinetic/stg_kinetic__meta_ad_insights_daily.sql</t>
         </is>
       </c>
       <c r="B225" s="2" t="inlineStr">
@@ -5385,19 +5385,19 @@
       </c>
       <c r="C225" s="3" t="inlineStr">
         <is>
-          <t>Phase 2 staging (paid media: Google Search): ad groups; cpc_bid_micros cast back to a number (always empty -- automated bidding)</t>
+          <t>Phase 2 staging (paid media: Meta): meta_ad_insights_daily with a combined ad_day_id key, unit-suffixed columns (spend_usd, cpm_usd, cpc_usd) and ctr renamed ctr_fraction (0.017 = 1.7%)</t>
         </is>
       </c>
       <c r="D225" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 13:13 PDT</t>
+          <t>2026-09-29 13:02 PDT</t>
         </is>
       </c>
     </row>
     <row r="226">
       <c r="A226" s="2" t="inlineStr">
         <is>
-          <t>dbt/models/staging/kinetic/stg_kinetic__google_search_performance_daily.sql</t>
+          <t>dbt/models/staging/kinetic/stg_kinetic__meta_ad_actions_daily.sql</t>
         </is>
       </c>
       <c r="B226" s="2" t="inlineStr">
@@ -5407,19 +5407,19 @@
       </c>
       <c r="C226" s="3" t="inlineStr">
         <is>
-          <t>Phase 2 staging (paid media: Google Search): ad-group-day performance with combined ad_group_day_id key, cost converted from micros to dollars, ctr_fraction. The keyword table rolled up -- never add the two together</t>
+          <t>Phase 2 staging (paid media: Meta): meta_ad_actions_daily with a combined ad_day_action_id key; value renamed action_count</t>
         </is>
       </c>
       <c r="D226" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 13:13 PDT</t>
+          <t>2026-09-29 13:02 PDT</t>
         </is>
       </c>
     </row>
     <row r="227">
       <c r="A227" s="2" t="inlineStr">
         <is>
-          <t>dbt/models/staging/kinetic/stg_kinetic__google_search_keyword_performance_daily.sql</t>
+          <t>dbt/models/staging/kinetic/_kinetic__staging.yml</t>
         </is>
       </c>
       <c r="B227" s="2" t="inlineStr">
@@ -5429,19 +5429,19 @@
       </c>
       <c r="C227" s="3" t="inlineStr">
         <is>
-          <t>Phase 2 staging (paid media: Google Search): keyword-day performance with combined keyword_day_id key, cost converted from micros to dollars, ctr_fraction</t>
+          <t>Updated: tests for the 4 Meta staging models, incl. uniqueness of the combined daily keys -- all hand-verified against live data first</t>
         </is>
       </c>
       <c r="D227" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 13:13 PDT</t>
+          <t>2026-09-29 16:49 PDT</t>
         </is>
       </c>
     </row>
     <row r="228">
       <c r="A228" s="2" t="inlineStr">
         <is>
-          <t>dbt/models/staging/kinetic/_kinetic__staging.yml</t>
+          <t>dbt/models/staging/kinetic/stg_kinetic__google_search_campaigns.sql</t>
         </is>
       </c>
       <c r="B228" s="2" t="inlineStr">
@@ -5451,19 +5451,19 @@
       </c>
       <c r="C228" s="3" t="inlineStr">
         <is>
-          <t>Updated: tests for the 4 Google Search staging models -- all hand-verified against live data first</t>
+          <t>Phase 2 staging (paid media: Google Search): campaigns with the raw customer_id renamed google_ads_account_id (it's the Google Ads account number, not a Kinetic customer), daily budget in micros and dollars, end_date cast back to a date</t>
         </is>
       </c>
       <c r="D228" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 16:49 PDT</t>
+          <t>2026-09-29 13:13 PDT</t>
         </is>
       </c>
     </row>
     <row r="229">
       <c r="A229" s="2" t="inlineStr">
         <is>
-          <t>dbt/models/staging/kinetic/stg_kinetic__youtube_campaigns.sql</t>
+          <t>dbt/models/staging/kinetic/stg_kinetic__google_search_ad_groups.sql</t>
         </is>
       </c>
       <c r="B229" s="2" t="inlineStr">
@@ -5473,19 +5473,19 @@
       </c>
       <c r="C229" s="3" t="inlineStr">
         <is>
-          <t>Phase 2 staging (paid media: YouTube): campaigns with customer_id renamed google_ads_account_id (the ad account, not a Kinetic customer), budgets in micros and dollars</t>
+          <t>Phase 2 staging (paid media: Google Search): ad groups; cpc_bid_micros cast back to a number (always empty -- automated bidding)</t>
         </is>
       </c>
       <c r="D229" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 13:14 PDT</t>
+          <t>2026-09-29 13:13 PDT</t>
         </is>
       </c>
     </row>
     <row r="230">
       <c r="A230" s="2" t="inlineStr">
         <is>
-          <t>dbt/models/staging/kinetic/stg_kinetic__youtube_ad_groups.sql</t>
+          <t>dbt/models/staging/kinetic/stg_kinetic__google_search_performance_daily.sql</t>
         </is>
       </c>
       <c r="B230" s="2" t="inlineStr">
@@ -5495,19 +5495,19 @@
       </c>
       <c r="C230" s="3" t="inlineStr">
         <is>
-          <t>Phase 2 staging (paid media: YouTube): 1:1 pass-through of youtube_ad_groups</t>
+          <t>Phase 2 staging (paid media: Google Search): ad-group-day performance with combined ad_group_day_id key, cost converted from micros to dollars, ctr_fraction. The keyword table rolled up -- never add the two together</t>
         </is>
       </c>
       <c r="D230" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 13:14 PDT</t>
+          <t>2026-09-29 13:13 PDT</t>
         </is>
       </c>
     </row>
     <row r="231">
       <c r="A231" s="2" t="inlineStr">
         <is>
-          <t>dbt/models/staging/kinetic/stg_kinetic__youtube_performance_daily.sql</t>
+          <t>dbt/models/staging/kinetic/stg_kinetic__google_search_keyword_performance_daily.sql</t>
         </is>
       </c>
       <c r="B231" s="2" t="inlineStr">
@@ -5517,12 +5517,12 @@
       </c>
       <c r="C231" s="3" t="inlineStr">
         <is>
-          <t>Phase 2 staging (paid media: YouTube): ad-group-day performance with combined ad_group_day_id key, cost and cost-per-view converted from micros to dollars, video_view_rate_fraction</t>
+          <t>Phase 2 staging (paid media: Google Search): keyword-day performance with combined keyword_day_id key, cost converted from micros to dollars, ctr_fraction</t>
         </is>
       </c>
       <c r="D231" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 13:14 PDT</t>
+          <t>2026-09-29 13:13 PDT</t>
         </is>
       </c>
     </row>
@@ -5539,7 +5539,7 @@
       </c>
       <c r="C232" s="3" t="inlineStr">
         <is>
-          <t>Updated: tests for the 3 YouTube staging models -- all hand-verified against live data first</t>
+          <t>Updated: tests for the 4 Google Search staging models -- all hand-verified against live data first</t>
         </is>
       </c>
       <c r="D232" s="2" t="inlineStr">
@@ -5551,7 +5551,7 @@
     <row r="233">
       <c r="A233" s="2" t="inlineStr">
         <is>
-          <t>dbt/models/staging/kinetic/stg_kinetic__dv360_insertion_orders.sql</t>
+          <t>dbt/models/staging/kinetic/stg_kinetic__youtube_campaigns.sql</t>
         </is>
       </c>
       <c r="B233" s="2" t="inlineStr">
@@ -5561,19 +5561,19 @@
       </c>
       <c r="C233" s="3" t="inlineStr">
         <is>
-          <t>Phase 2 staging (paid media: DV360): insertion orders with budget_micros named monthly_budget_* (it's a monthly budget), end_date cast back to a date; flags the flat-budget-vs-growing-spend known issue</t>
+          <t>Phase 2 staging (paid media: YouTube): campaigns with customer_id renamed google_ads_account_id (the ad account, not a Kinetic customer), budgets in micros and dollars</t>
         </is>
       </c>
       <c r="D233" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 13:27 PDT</t>
+          <t>2026-09-29 13:14 PDT</t>
         </is>
       </c>
     </row>
     <row r="234">
       <c r="A234" s="2" t="inlineStr">
         <is>
-          <t>dbt/models/staging/kinetic/stg_kinetic__dv360_line_items.sql</t>
+          <t>dbt/models/staging/kinetic/stg_kinetic__youtube_ad_groups.sql</t>
         </is>
       </c>
       <c r="B234" s="2" t="inlineStr">
@@ -5583,19 +5583,19 @@
       </c>
       <c r="C234" s="3" t="inlineStr">
         <is>
-          <t>Phase 2 staging (paid media: DV360): 1:1 pass-through of dv360_line_items</t>
+          <t>Phase 2 staging (paid media: YouTube): 1:1 pass-through of youtube_ad_groups</t>
         </is>
       </c>
       <c r="D234" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 13:19 PDT</t>
+          <t>2026-09-29 13:14 PDT</t>
         </is>
       </c>
     </row>
     <row r="235">
       <c r="A235" s="2" t="inlineStr">
         <is>
-          <t>dbt/models/staging/kinetic/stg_kinetic__dv360_performance_daily.sql</t>
+          <t>dbt/models/staging/kinetic/stg_kinetic__youtube_performance_daily.sql</t>
         </is>
       </c>
       <c r="B235" s="2" t="inlineStr">
@@ -5605,12 +5605,12 @@
       </c>
       <c r="C235" s="3" t="inlineStr">
         <is>
-          <t>Phase 2 staging (paid media: DV360): line-item x day x exchange x environment performance with combined line_item_day_slice_id key, micros converted to dollars, ctr_fraction</t>
+          <t>Phase 2 staging (paid media: YouTube): ad-group-day performance with combined ad_group_day_id key, cost and cost-per-view converted from micros to dollars, video_view_rate_fraction</t>
         </is>
       </c>
       <c r="D235" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 13:19 PDT</t>
+          <t>2026-09-29 13:14 PDT</t>
         </is>
       </c>
     </row>
@@ -5627,7 +5627,7 @@
       </c>
       <c r="C236" s="3" t="inlineStr">
         <is>
-          <t>Updated: tests for the 3 DV360 staging models, incl. accepted_values on exchange and environment -- all hand-verified against live data first</t>
+          <t>Updated: tests for the 3 YouTube staging models -- all hand-verified against live data first</t>
         </is>
       </c>
       <c r="D236" s="2" t="inlineStr">
@@ -5639,7 +5639,7 @@
     <row r="237">
       <c r="A237" s="2" t="inlineStr">
         <is>
-          <t>generator/params.py</t>
+          <t>dbt/models/staging/kinetic/stg_kinetic__dv360_insertion_orders.sql</t>
         </is>
       </c>
       <c r="B237" s="2" t="inlineStr">
@@ -5649,107 +5649,107 @@
       </c>
       <c r="C237" s="3" t="inlineStr">
         <is>
-          <t>Updated 2026-09-29: every evergreen ad budget on all 6 platforms is now the campaign's CURRENT budget, sized from realized spend (weekly average &lt;= budget, no day &gt; 1.75x; DV360 monthly &gt;= highest month). The old flat 'typical day' budgets let later months spend up to ~20x the stored budget</t>
+          <t>Phase 2 staging (paid media: DV360): insertion orders with budget_micros named monthly_budget_* (it's a monthly budget), end_date cast back to a date; flags the flat-budget-vs-growing-spend known issue</t>
         </is>
       </c>
       <c r="D237" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 13:23 PDT</t>
+          <t>2026-09-29 13:27 PDT</t>
         </is>
       </c>
     </row>
     <row r="238">
       <c r="A238" s="2" t="inlineStr">
         <is>
-          <t>data/meta_campaigns.csv</t>
+          <t>dbt/models/staging/kinetic/stg_kinetic__dv360_line_items.sql</t>
         </is>
       </c>
       <c r="B238" s="2" t="inlineStr">
         <is>
-          <t>Shipped table</t>
+          <t>Code</t>
         </is>
       </c>
       <c r="C238" s="3" t="inlineStr">
         <is>
-          <t>Regenerated 2026-09-29: evergreen daily_budget values updated to current budgets (only that column, only the 4 evergreen rows changed)</t>
+          <t>Phase 2 staging (paid media: DV360): 1:1 pass-through of dv360_line_items</t>
         </is>
       </c>
       <c r="D238" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 13:24 PDT</t>
+          <t>2026-09-29 13:19 PDT</t>
         </is>
       </c>
     </row>
     <row r="239">
       <c r="A239" s="2" t="inlineStr">
         <is>
-          <t>data/google_search_campaigns.csv</t>
+          <t>dbt/models/staging/kinetic/stg_kinetic__dv360_performance_daily.sql</t>
         </is>
       </c>
       <c r="B239" s="2" t="inlineStr">
         <is>
-          <t>Shipped table</t>
+          <t>Code</t>
         </is>
       </c>
       <c r="C239" s="3" t="inlineStr">
         <is>
-          <t>Regenerated 2026-09-29: campaign_budget_micros updated to current budgets (only that column changed)</t>
+          <t>Phase 2 staging (paid media: DV360): line-item x day x exchange x environment performance with combined line_item_day_slice_id key, micros converted to dollars, ctr_fraction</t>
         </is>
       </c>
       <c r="D239" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 13:24 PDT</t>
+          <t>2026-09-29 13:19 PDT</t>
         </is>
       </c>
     </row>
     <row r="240">
       <c r="A240" s="2" t="inlineStr">
         <is>
-          <t>data/youtube_campaigns.csv</t>
+          <t>dbt/models/staging/kinetic/_kinetic__staging.yml</t>
         </is>
       </c>
       <c r="B240" s="2" t="inlineStr">
         <is>
-          <t>Shipped table</t>
+          <t>Code</t>
         </is>
       </c>
       <c r="C240" s="3" t="inlineStr">
         <is>
-          <t>Regenerated 2026-09-29: evergreen campaign_budget_micros updated to current budgets (only that column, only the 4 evergreen rows changed)</t>
+          <t>Updated: tests for the 3 DV360 staging models, incl. accepted_values on exchange and environment -- all hand-verified against live data first</t>
         </is>
       </c>
       <c r="D240" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 13:24 PDT</t>
+          <t>2026-09-29 16:49 PDT</t>
         </is>
       </c>
     </row>
     <row r="241">
       <c r="A241" s="2" t="inlineStr">
         <is>
-          <t>data/dv360_insertion_orders.csv</t>
+          <t>generator/params.py</t>
         </is>
       </c>
       <c r="B241" s="2" t="inlineStr">
         <is>
-          <t>Shipped table</t>
+          <t>Code</t>
         </is>
       </c>
       <c r="C241" s="3" t="inlineStr">
         <is>
-          <t>Regenerated 2026-09-29: monthly budget_micros updated to current budgets (only that column changed)</t>
+          <t>Updated 2026-09-29: every evergreen ad budget on all 6 platforms is now the campaign's CURRENT budget, sized from realized spend (weekly average &lt;= budget, no day &gt; 1.75x; DV360 monthly &gt;= highest month). The old flat 'typical day' budgets let later months spend up to ~20x the stored budget</t>
         </is>
       </c>
       <c r="D241" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 13:24 PDT</t>
+          <t>2026-09-29 13:23 PDT</t>
         </is>
       </c>
     </row>
     <row r="242">
       <c r="A242" s="2" t="inlineStr">
         <is>
-          <t>data/snap_campaigns.csv</t>
+          <t>data/meta_campaigns.csv</t>
         </is>
       </c>
       <c r="B242" s="2" t="inlineStr">
@@ -5759,7 +5759,7 @@
       </c>
       <c r="C242" s="3" t="inlineStr">
         <is>
-          <t>Regenerated 2026-09-29: evergreen daily_budget_micro updated to current budgets (only that column, only the 4 evergreen rows changed)</t>
+          <t>Regenerated 2026-09-29: evergreen daily_budget values updated to current budgets (only that column, only the 4 evergreen rows changed)</t>
         </is>
       </c>
       <c r="D242" s="2" t="inlineStr">
@@ -5771,7 +5771,7 @@
     <row r="243">
       <c r="A243" s="2" t="inlineStr">
         <is>
-          <t>data/tiktok_campaigns.csv</t>
+          <t>data/google_search_campaigns.csv</t>
         </is>
       </c>
       <c r="B243" s="2" t="inlineStr">
@@ -5781,7 +5781,7 @@
       </c>
       <c r="C243" s="3" t="inlineStr">
         <is>
-          <t>Regenerated 2026-09-29: BUDGET_MODE_DAY budget_micro updated to current budgets (only that column, only the 4 evergreen rows changed)</t>
+          <t>Regenerated 2026-09-29: campaign_budget_micros updated to current budgets (only that column changed)</t>
         </is>
       </c>
       <c r="D243" s="2" t="inlineStr">
@@ -5793,95 +5793,95 @@
     <row r="244">
       <c r="A244" s="2" t="inlineStr">
         <is>
-          <t>generator/audit_cross_dataset_alignment.py</t>
+          <t>data/youtube_campaigns.csv</t>
         </is>
       </c>
       <c r="B244" s="2" t="inlineStr">
         <is>
-          <t>Code</t>
+          <t>Shipped table</t>
         </is>
       </c>
       <c r="C244" s="3" t="inlineStr">
         <is>
-          <t>Updated 2026-09-29: new Check 8 -- spend vs stored budget for every campaign on all 6 platforms (weekly/daily limits for daily budgets, monthly for DV360, total for holiday flights)</t>
+          <t>Regenerated 2026-09-29: evergreen campaign_budget_micros updated to current budgets (only that column, only the 4 evergreen rows changed)</t>
         </is>
       </c>
       <c r="D244" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 13:30 PDT</t>
+          <t>2026-09-29 13:24 PDT</t>
         </is>
       </c>
     </row>
     <row r="245">
       <c r="A245" s="2" t="inlineStr">
         <is>
-          <t>dbt/models/staging/kinetic/stg_kinetic__dv360_insertion_orders.sql</t>
+          <t>data/dv360_insertion_orders.csv</t>
         </is>
       </c>
       <c r="B245" s="2" t="inlineStr">
         <is>
-          <t>Code</t>
+          <t>Shipped table</t>
         </is>
       </c>
       <c r="C245" s="3" t="inlineStr">
         <is>
-          <t>Updated: budget known-issue note replaced -- budgets are now current budgets</t>
+          <t>Regenerated 2026-09-29: monthly budget_micros updated to current budgets (only that column changed)</t>
         </is>
       </c>
       <c r="D245" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 13:27 PDT</t>
+          <t>2026-09-29 13:24 PDT</t>
         </is>
       </c>
     </row>
     <row r="246">
       <c r="A246" s="2" t="inlineStr">
         <is>
-          <t>generator/paid_media_common.py</t>
+          <t>data/snap_campaigns.csv</t>
         </is>
       </c>
       <c r="B246" s="2" t="inlineStr">
         <is>
-          <t>Code</t>
+          <t>Shipped table</t>
         </is>
       </c>
       <c r="C246" s="3" t="inlineStr">
         <is>
-          <t>Updated 2026-09-29: new cap_flight_at_budget() -- rescales a holiday flight's days so it never spends past its lifetime budget, replaying the same random rates so every other row is unchanged</t>
+          <t>Regenerated 2026-09-29: evergreen daily_budget_micro updated to current budgets (only that column, only the 4 evergreen rows changed)</t>
         </is>
       </c>
       <c r="D246" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 13:29 PDT</t>
+          <t>2026-09-29 13:24 PDT</t>
         </is>
       </c>
     </row>
     <row r="247">
       <c r="A247" s="2" t="inlineStr">
         <is>
-          <t>generator/build_meta_ad_insights_daily.py</t>
+          <t>data/tiktok_campaigns.csv</t>
         </is>
       </c>
       <c r="B247" s="2" t="inlineStr">
         <is>
-          <t>Code</t>
+          <t>Shipped table</t>
         </is>
       </c>
       <c r="C247" s="3" t="inlineStr">
         <is>
-          <t>Updated 2026-09-29: holiday flights capped at their lifetime budget via cap_flight_at_budget()</t>
+          <t>Regenerated 2026-09-29: BUDGET_MODE_DAY budget_micro updated to current budgets (only that column, only the 4 evergreen rows changed)</t>
         </is>
       </c>
       <c r="D247" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 13:29 PDT</t>
+          <t>2026-09-29 13:24 PDT</t>
         </is>
       </c>
     </row>
     <row r="248">
       <c r="A248" s="2" t="inlineStr">
         <is>
-          <t>generator/build_snap_stats_daily.py</t>
+          <t>generator/audit_cross_dataset_alignment.py</t>
         </is>
       </c>
       <c r="B248" s="2" t="inlineStr">
@@ -5891,19 +5891,19 @@
       </c>
       <c r="C248" s="3" t="inlineStr">
         <is>
-          <t>Updated 2026-09-29: holiday flights capped at their lifetime budget via cap_flight_at_budget()</t>
+          <t>Updated 2026-09-29: new Check 8 -- spend vs stored budget for every campaign on all 6 platforms (weekly/daily limits for daily budgets, monthly for DV360, total for holiday flights)</t>
         </is>
       </c>
       <c r="D248" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 13:29 PDT</t>
+          <t>2026-09-29 13:30 PDT</t>
         </is>
       </c>
     </row>
     <row r="249">
       <c r="A249" s="2" t="inlineStr">
         <is>
-          <t>generator/build_tiktok_reports_daily.py</t>
+          <t>dbt/models/staging/kinetic/stg_kinetic__dv360_insertion_orders.sql</t>
         </is>
       </c>
       <c r="B249" s="2" t="inlineStr">
@@ -5913,19 +5913,19 @@
       </c>
       <c r="C249" s="3" t="inlineStr">
         <is>
-          <t>Updated 2026-09-29: holiday flights capped at their lifetime budget via cap_flight_at_budget()</t>
+          <t>Updated: budget known-issue note replaced -- budgets are now current budgets</t>
         </is>
       </c>
       <c r="D249" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 13:29 PDT</t>
+          <t>2026-09-29 13:27 PDT</t>
         </is>
       </c>
     </row>
     <row r="250">
       <c r="A250" s="2" t="inlineStr">
         <is>
-          <t>generator/build_youtube_performance_daily.py</t>
+          <t>generator/paid_media_common.py</t>
         </is>
       </c>
       <c r="B250" s="2" t="inlineStr">
@@ -5935,7 +5935,7 @@
       </c>
       <c r="C250" s="3" t="inlineStr">
         <is>
-          <t>Updated 2026-09-29: holiday flights capped at their lifetime budget via cap_flight_at_budget() (no-op today -- all YouTube flights were already under budget)</t>
+          <t>Updated 2026-09-29: new cap_flight_at_budget() -- rescales a holiday flight's days so it never spends past its lifetime budget, replaying the same random rates so every other row is unchanged</t>
         </is>
       </c>
       <c r="D250" s="2" t="inlineStr">
@@ -5947,17 +5947,17 @@
     <row r="251">
       <c r="A251" s="2" t="inlineStr">
         <is>
-          <t>data/meta_ad_insights_daily.csv</t>
+          <t>generator/build_meta_ad_insights_daily.py</t>
         </is>
       </c>
       <c r="B251" s="2" t="inlineStr">
         <is>
-          <t>Shipped table</t>
+          <t>Code</t>
         </is>
       </c>
       <c r="C251" s="3" t="inlineStr">
         <is>
-          <t>Regenerated 2026-09-29: the 2023 and 2024 holiday flights (38 rows) trimmed to spend exactly their lifetime budget; every other row identical</t>
+          <t>Updated 2026-09-29: holiday flights capped at their lifetime budget via cap_flight_at_budget()</t>
         </is>
       </c>
       <c r="D251" s="2" t="inlineStr">
@@ -5969,17 +5969,17 @@
     <row r="252">
       <c r="A252" s="2" t="inlineStr">
         <is>
-          <t>data/meta_ad_actions_daily.csv</t>
+          <t>generator/build_snap_stats_daily.py</t>
         </is>
       </c>
       <c r="B252" s="2" t="inlineStr">
         <is>
-          <t>Shipped table</t>
+          <t>Code</t>
         </is>
       </c>
       <c r="C252" s="3" t="inlineStr">
         <is>
-          <t>Regenerated 2026-09-29: re-derived from the trimmed insights rows -- only the 2023/2024 holiday flights' action rows changed (one initiate_checkout row on 2024-11-15 dropped to zero and is no longer emitted)</t>
+          <t>Updated 2026-09-29: holiday flights capped at their lifetime budget via cap_flight_at_budget()</t>
         </is>
       </c>
       <c r="D252" s="2" t="inlineStr">
@@ -5991,17 +5991,17 @@
     <row r="253">
       <c r="A253" s="2" t="inlineStr">
         <is>
-          <t>data/snap_stats_daily.csv</t>
+          <t>generator/build_tiktok_reports_daily.py</t>
         </is>
       </c>
       <c r="B253" s="2" t="inlineStr">
         <is>
-          <t>Shipped table</t>
+          <t>Code</t>
         </is>
       </c>
       <c r="C253" s="3" t="inlineStr">
         <is>
-          <t>Regenerated 2026-09-29: the 2024 holiday flight (19 rows) trimmed to spend exactly its lifetime budget; every other row identical</t>
+          <t>Updated 2026-09-29: holiday flights capped at their lifetime budget via cap_flight_at_budget()</t>
         </is>
       </c>
       <c r="D253" s="2" t="inlineStr">
@@ -6013,17 +6013,17 @@
     <row r="254">
       <c r="A254" s="2" t="inlineStr">
         <is>
-          <t>data/tiktok_reports_daily.csv</t>
+          <t>generator/build_youtube_performance_daily.py</t>
         </is>
       </c>
       <c r="B254" s="2" t="inlineStr">
         <is>
-          <t>Shipped table</t>
+          <t>Code</t>
         </is>
       </c>
       <c r="C254" s="3" t="inlineStr">
         <is>
-          <t>Regenerated 2026-09-29: the 2023/2024/2025 holiday flights (56 rows) trimmed to spend exactly their lifetime budgets; every other row identical</t>
+          <t>Updated 2026-09-29: holiday flights capped at their lifetime budget via cap_flight_at_budget() (no-op today -- all YouTube flights were already under budget)</t>
         </is>
       </c>
       <c r="D254" s="2" t="inlineStr">
@@ -6035,117 +6035,117 @@
     <row r="255">
       <c r="A255" s="2" t="inlineStr">
         <is>
-          <t>docs/cross_dataset_alignment_audit.md</t>
+          <t>data/meta_ad_insights_daily.csv</t>
         </is>
       </c>
       <c r="B255" s="2" t="inlineStr">
         <is>
-          <t>Docs</t>
+          <t>Shipped table</t>
         </is>
       </c>
       <c r="C255" s="3" t="inlineStr">
         <is>
-          <t>Updated 2026-09-29: added Check 8 (spend vs stored budget) with both fixes and results</t>
+          <t>Regenerated 2026-09-29: the 2023 and 2024 holiday flights (38 rows) trimmed to spend exactly their lifetime budget; every other row identical</t>
         </is>
       </c>
       <c r="D255" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 13:54 PDT</t>
+          <t>2026-09-29 13:29 PDT</t>
         </is>
       </c>
     </row>
     <row r="256">
       <c r="A256" s="2" t="inlineStr">
         <is>
-          <t>generator/audit_cross_dataset_alignment.py</t>
+          <t>data/meta_ad_actions_daily.csv</t>
         </is>
       </c>
       <c r="B256" s="2" t="inlineStr">
         <is>
-          <t>Code</t>
+          <t>Shipped table</t>
         </is>
       </c>
       <c r="C256" s="3" t="inlineStr">
         <is>
-          <t>Updated 2026-09-29: Check 8's flight limit tightened from 1.05x to 1.0x now that flights are capped</t>
+          <t>Regenerated 2026-09-29: re-derived from the trimmed insights rows -- only the 2023/2024 holiday flights' action rows changed (one initiate_checkout row on 2024-11-15 dropped to zero and is no longer emitted)</t>
         </is>
       </c>
       <c r="D256" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 13:30 PDT</t>
+          <t>2026-09-29 13:29 PDT</t>
         </is>
       </c>
     </row>
     <row r="257">
       <c r="A257" s="2" t="inlineStr">
         <is>
-          <t>dbt/models/staging/kinetic/stg_kinetic__snap_campaigns.sql</t>
+          <t>data/snap_stats_daily.csv</t>
         </is>
       </c>
       <c r="B257" s="2" t="inlineStr">
         <is>
-          <t>Code</t>
+          <t>Shipped table</t>
         </is>
       </c>
       <c r="C257" s="3" t="inlineStr">
         <is>
-          <t>Phase 2 staging (paid media: Snap): campaigns with ad_account_id renamed snap_ad_account_id, current budgets in micros and dollars</t>
+          <t>Regenerated 2026-09-29: the 2024 holiday flight (19 rows) trimmed to spend exactly its lifetime budget; every other row identical</t>
         </is>
       </c>
       <c r="D257" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 15:53 PDT</t>
+          <t>2026-09-29 13:29 PDT</t>
         </is>
       </c>
     </row>
     <row r="258">
       <c r="A258" s="2" t="inlineStr">
         <is>
-          <t>dbt/models/staging/kinetic/stg_kinetic__snap_ad_squads.sql</t>
+          <t>data/tiktok_reports_daily.csv</t>
         </is>
       </c>
       <c r="B258" s="2" t="inlineStr">
         <is>
-          <t>Code</t>
+          <t>Shipped table</t>
         </is>
       </c>
       <c r="C258" s="3" t="inlineStr">
         <is>
-          <t>Phase 2 staging (paid media: Snap): 1:1 pass-through of snap_ad_squads (Snap's ad set / ad group level)</t>
+          <t>Regenerated 2026-09-29: the 2023/2024/2025 holiday flights (56 rows) trimmed to spend exactly their lifetime budgets; every other row identical</t>
         </is>
       </c>
       <c r="D258" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 15:53 PDT</t>
+          <t>2026-09-29 13:29 PDT</t>
         </is>
       </c>
     </row>
     <row r="259">
       <c r="A259" s="2" t="inlineStr">
         <is>
-          <t>dbt/models/staging/kinetic/stg_kinetic__snap_ads.sql</t>
+          <t>docs/cross_dataset_alignment_audit.md</t>
         </is>
       </c>
       <c r="B259" s="2" t="inlineStr">
         <is>
-          <t>Code</t>
+          <t>Docs</t>
         </is>
       </c>
       <c r="C259" s="3" t="inlineStr">
         <is>
-          <t>Phase 2 staging (paid media: Snap): 1:1 pass-through of snap_ads</t>
+          <t>Updated 2026-09-29: added Check 8 (spend vs stored budget) with both fixes and results</t>
         </is>
       </c>
       <c r="D259" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 15:53 PDT</t>
+          <t>2026-09-29 13:54 PDT</t>
         </is>
       </c>
     </row>
     <row r="260">
       <c r="A260" s="2" t="inlineStr">
         <is>
-          <t>dbt/models/staging/kinetic/stg_kinetic__snap_stats_daily.sql</t>
+          <t>generator/audit_cross_dataset_alignment.py</t>
         </is>
       </c>
       <c r="B260" s="2" t="inlineStr">
@@ -6155,19 +6155,19 @@
       </c>
       <c r="C260" s="3" t="inlineStr">
         <is>
-          <t>Phase 2 staging (paid media: Snap): ad-day stats with combined ad_day_id key, spend in micros and dollars; documents swipes as Snap's clicks</t>
+          <t>Updated 2026-09-29: Check 8's flight limit tightened from 1.05x to 1.0x now that flights are capped</t>
         </is>
       </c>
       <c r="D260" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 15:53 PDT</t>
+          <t>2026-09-29 13:30 PDT</t>
         </is>
       </c>
     </row>
     <row r="261">
       <c r="A261" s="2" t="inlineStr">
         <is>
-          <t>dbt/models/staging/kinetic/_kinetic__staging.yml</t>
+          <t>dbt/models/staging/kinetic/stg_kinetic__snap_campaigns.sql</t>
         </is>
       </c>
       <c r="B261" s="2" t="inlineStr">
@@ -6177,19 +6177,19 @@
       </c>
       <c r="C261" s="3" t="inlineStr">
         <is>
-          <t>Updated: tests for the 4 Snap staging models -- all hand-verified against live data first</t>
+          <t>Phase 2 staging (paid media: Snap): campaigns with ad_account_id renamed snap_ad_account_id, current budgets in micros and dollars</t>
         </is>
       </c>
       <c r="D261" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 16:49 PDT</t>
+          <t>2026-09-29 15:53 PDT</t>
         </is>
       </c>
     </row>
     <row r="262">
       <c r="A262" s="2" t="inlineStr">
         <is>
-          <t>dbt/models/staging/kinetic/stg_kinetic__tiktok_campaigns.sql</t>
+          <t>dbt/models/staging/kinetic/stg_kinetic__snap_ad_squads.sql</t>
         </is>
       </c>
       <c r="B262" s="2" t="inlineStr">
@@ -6199,19 +6199,19 @@
       </c>
       <c r="C262" s="3" t="inlineStr">
         <is>
-          <t>Phase 2 staging (paid media: TikTok): campaigns with the single budget split into daily_budget_usd / lifetime_budget_usd by budget_mode (matching the other platforms), advertiser_id renamed tiktok_advertiser_id</t>
+          <t>Phase 2 staging (paid media: Snap): 1:1 pass-through of snap_ad_squads (Snap's ad set / ad group level)</t>
         </is>
       </c>
       <c r="D262" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 15:57 PDT</t>
+          <t>2026-09-29 15:53 PDT</t>
         </is>
       </c>
     </row>
     <row r="263">
       <c r="A263" s="2" t="inlineStr">
         <is>
-          <t>dbt/models/staging/kinetic/stg_kinetic__tiktok_adgroups.sql</t>
+          <t>dbt/models/staging/kinetic/stg_kinetic__snap_ads.sql</t>
         </is>
       </c>
       <c r="B263" s="2" t="inlineStr">
@@ -6221,19 +6221,19 @@
       </c>
       <c r="C263" s="3" t="inlineStr">
         <is>
-          <t>Phase 2 staging (paid media: TikTok): 1:1 pass-through of tiktok_adgroups</t>
+          <t>Phase 2 staging (paid media: Snap): 1:1 pass-through of snap_ads</t>
         </is>
       </c>
       <c r="D263" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 15:57 PDT</t>
+          <t>2026-09-29 15:53 PDT</t>
         </is>
       </c>
     </row>
     <row r="264">
       <c r="A264" s="2" t="inlineStr">
         <is>
-          <t>dbt/models/staging/kinetic/stg_kinetic__tiktok_ads.sql</t>
+          <t>dbt/models/staging/kinetic/stg_kinetic__snap_stats_daily.sql</t>
         </is>
       </c>
       <c r="B264" s="2" t="inlineStr">
@@ -6243,19 +6243,19 @@
       </c>
       <c r="C264" s="3" t="inlineStr">
         <is>
-          <t>Phase 2 staging (paid media: TikTok): 1:1 pass-through of tiktok_ads</t>
+          <t>Phase 2 staging (paid media: Snap): ad-day stats with combined ad_day_id key, spend in micros and dollars; documents swipes as Snap's clicks</t>
         </is>
       </c>
       <c r="D264" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 15:57 PDT</t>
+          <t>2026-09-29 15:53 PDT</t>
         </is>
       </c>
     </row>
     <row r="265">
       <c r="A265" s="2" t="inlineStr">
         <is>
-          <t>dbt/models/staging/kinetic/stg_kinetic__tiktok_reports_daily.sql</t>
+          <t>dbt/models/staging/kinetic/_kinetic__staging.yml</t>
         </is>
       </c>
       <c r="B265" s="2" t="inlineStr">
@@ -6265,19 +6265,19 @@
       </c>
       <c r="C265" s="3" t="inlineStr">
         <is>
-          <t>Phase 2 staging (paid media: TikTok): ad-day reports with combined ad_day_id key, spend and CPM in micros and dollars, ctr_fraction</t>
+          <t>Updated: tests for the 4 Snap staging models -- all hand-verified against live data first</t>
         </is>
       </c>
       <c r="D265" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 15:57 PDT</t>
+          <t>2026-09-29 16:49 PDT</t>
         </is>
       </c>
     </row>
     <row r="266">
       <c r="A266" s="2" t="inlineStr">
         <is>
-          <t>dbt/models/staging/kinetic/stg_kinetic__product_variants.sql</t>
+          <t>dbt/models/staging/kinetic/stg_kinetic__tiktok_campaigns.sql</t>
         </is>
       </c>
       <c r="B266" s="2" t="inlineStr">
@@ -6287,54 +6287,142 @@
       </c>
       <c r="C266" s="3" t="inlineStr">
         <is>
-          <t>Phase 2 staging (final table, 47 of 47): product variants with variant_option, price_adjustment_usd</t>
+          <t>Phase 2 staging (paid media: TikTok): campaigns with the single budget split into daily_budget_usd / lifetime_budget_usd by budget_mode (matching the other platforms), advertiser_id renamed tiktok_advertiser_id</t>
         </is>
       </c>
       <c r="D266" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 16:08 PDT</t>
+          <t>2026-09-29 15:57 PDT</t>
         </is>
       </c>
     </row>
     <row r="267">
       <c r="A267" s="2" t="inlineStr">
         <is>
-          <t>HANDOFF.md</t>
+          <t>dbt/models/staging/kinetic/stg_kinetic__tiktok_adgroups.sql</t>
         </is>
       </c>
       <c r="B267" s="2" t="inlineStr">
         <is>
-          <t>Doc</t>
+          <t>Code</t>
         </is>
       </c>
       <c r="C267" s="3" t="inlineStr">
         <is>
-          <t>Handoff note for starting a new chat/project: status, open decisions, prior decisions, pitfalls</t>
+          <t>Phase 2 staging (paid media: TikTok): 1:1 pass-through of tiktok_adgroups</t>
         </is>
       </c>
       <c r="D267" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 17:03 PDT</t>
+          <t>2026-09-29 15:57 PDT</t>
         </is>
       </c>
     </row>
     <row r="268">
       <c r="A268" s="2" t="inlineStr">
         <is>
+          <t>dbt/models/staging/kinetic/stg_kinetic__tiktok_ads.sql</t>
+        </is>
+      </c>
+      <c r="B268" s="2" t="inlineStr">
+        <is>
+          <t>Code</t>
+        </is>
+      </c>
+      <c r="C268" s="3" t="inlineStr">
+        <is>
+          <t>Phase 2 staging (paid media: TikTok): 1:1 pass-through of tiktok_ads</t>
+        </is>
+      </c>
+      <c r="D268" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-29 15:57 PDT</t>
+        </is>
+      </c>
+    </row>
+    <row r="269">
+      <c r="A269" s="2" t="inlineStr">
+        <is>
+          <t>dbt/models/staging/kinetic/stg_kinetic__tiktok_reports_daily.sql</t>
+        </is>
+      </c>
+      <c r="B269" s="2" t="inlineStr">
+        <is>
+          <t>Code</t>
+        </is>
+      </c>
+      <c r="C269" s="3" t="inlineStr">
+        <is>
+          <t>Phase 2 staging (paid media: TikTok): ad-day reports with combined ad_day_id key, spend and CPM in micros and dollars, ctr_fraction</t>
+        </is>
+      </c>
+      <c r="D269" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-29 15:57 PDT</t>
+        </is>
+      </c>
+    </row>
+    <row r="270">
+      <c r="A270" s="2" t="inlineStr">
+        <is>
+          <t>dbt/models/staging/kinetic/stg_kinetic__product_variants.sql</t>
+        </is>
+      </c>
+      <c r="B270" s="2" t="inlineStr">
+        <is>
+          <t>Code</t>
+        </is>
+      </c>
+      <c r="C270" s="3" t="inlineStr">
+        <is>
+          <t>Phase 2 staging (final table, 47 of 47): product variants with variant_option, price_adjustment_usd</t>
+        </is>
+      </c>
+      <c r="D270" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-29 16:08 PDT</t>
+        </is>
+      </c>
+    </row>
+    <row r="271">
+      <c r="A271" s="2" t="inlineStr">
+        <is>
+          <t>HANDOFF.md</t>
+        </is>
+      </c>
+      <c r="B271" s="2" t="inlineStr">
+        <is>
+          <t>Doc</t>
+        </is>
+      </c>
+      <c r="C271" s="3" t="inlineStr">
+        <is>
+          <t>Handoff note for starting a new chat/project: status, open decisions, prior decisions, pitfalls</t>
+        </is>
+      </c>
+      <c r="D271" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-29 17:09 PDT</t>
+        </is>
+      </c>
+    </row>
+    <row r="272">
+      <c r="A272" s="2" t="inlineStr">
+        <is>
           <t>dbt/models/staging/kinetic/_kinetic__staging.yml</t>
         </is>
       </c>
-      <c r="B268" s="2" t="inlineStr">
-        <is>
-          <t>Code</t>
-        </is>
-      </c>
-      <c r="C268" s="3" t="inlineStr">
+      <c r="B272" s="2" t="inlineStr">
+        <is>
+          <t>Code</t>
+        </is>
+      </c>
+      <c r="C272" s="3" t="inlineStr">
         <is>
           <t>Updated: tests for the 4 TikTok staging models -- all hand-verified against live data first</t>
         </is>
       </c>
-      <c r="D268" s="2" t="inlineStr">
+      <c r="D272" s="2" t="inlineStr">
         <is>
           <t>2026-09-29 16:49 PDT</t>
         </is>

</xml_diff>

<commit_message>
int_sessions_unified: unified web+app sessions with back-filled customer; tests, manifest, changelog
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012MSGmVw4D6TxU8u8LSeA2e
</commit_message>
<xml_diff>
--- a/File_Manifest.xlsx
+++ b/File_Manifest.xlsx
@@ -435,7 +435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D272"/>
+  <dimension ref="A1:D276"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="48" customWidth="1" min="1" max="1"/>
@@ -506,7 +506,7 @@
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 17:09 PDT</t>
+          <t>2026-09-29 17:20 PDT</t>
         </is>
       </c>
     </row>
@@ -638,7 +638,7 @@
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 17:18 PDT</t>
+          <t>2026-09-29 17:23 PDT</t>
         </is>
       </c>
     </row>
@@ -748,7 +748,7 @@
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 17:18 PDT</t>
+          <t>2026-09-29 17:23 PDT</t>
         </is>
       </c>
     </row>
@@ -4620,7 +4620,7 @@
       </c>
       <c r="D190" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 17:18 PDT</t>
+          <t>2026-09-29 17:23 PDT</t>
         </is>
       </c>
     </row>
@@ -4935,7 +4935,7 @@
     <row r="205">
       <c r="A205" s="2" t="inlineStr">
         <is>
-          <t>dbt/models/marts/mart_storefront_revenue_monthly.sql</t>
+          <t>dbt/models/intermediate/int_sessions_unified.sql</t>
         </is>
       </c>
       <c r="B205" s="2" t="inlineStr">
@@ -4945,19 +4945,19 @@
       </c>
       <c r="C205" s="3" t="inlineStr">
         <is>
-          <t>Second canonical metric mart: non-subscription (course+merch) gross/net revenue, AOV, guest-checkout share, discount-usage share, refund rate by month -- validated against a hand-run equivalent query on the live database (2026-07: 246 orders, $13,843.71 gross revenue, $56.28 AOV)</t>
+          <t>Intermediate model: one row per web or app session, with customer_id resolved (known at the time, or back-filled from the visitor's anonymous_id via int_customer_identity)</t>
         </is>
       </c>
       <c r="D205" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28 14:53 PDT</t>
+          <t>2026-09-29 17:23 PDT</t>
         </is>
       </c>
     </row>
     <row r="206">
       <c r="A206" s="2" t="inlineStr">
         <is>
-          <t>dbt/models/staging/kinetic/stg_kinetic__customer_addresses.sql</t>
+          <t>dbt/tests/assert_int_sessions_unified_customer_matches_resolution.sql</t>
         </is>
       </c>
       <c r="B206" s="2" t="inlineStr">
@@ -4967,19 +4967,19 @@
       </c>
       <c r="C206" s="3" t="inlineStr">
         <is>
-          <t>Phase 2 staging (Customer 360): 1:1 pass-through of customer_addresses</t>
+          <t>dbt test: customer_id is null exactly when a session is anonymous</t>
         </is>
       </c>
       <c r="D206" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 10:26 PDT</t>
+          <t>2026-09-29 17:23 PDT</t>
         </is>
       </c>
     </row>
     <row r="207">
       <c r="A207" s="2" t="inlineStr">
         <is>
-          <t>dbt/models/staging/kinetic/stg_kinetic__devices.sql</t>
+          <t>dbt/tests/assert_int_sessions_unified_counts_match_sources.sql</t>
         </is>
       </c>
       <c r="B207" s="2" t="inlineStr">
@@ -4989,19 +4989,19 @@
       </c>
       <c r="C207" s="3" t="inlineStr">
         <is>
-          <t>Phase 2 staging (Customer 360): 1:1 pass-through of devices, plus is_anonymous_device flag (customer_id null for ~94% of devices by design)</t>
+          <t>dbt test: unified session count equals web + app session counts</t>
         </is>
       </c>
       <c r="D207" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 10:26 PDT</t>
+          <t>2026-09-29 17:23 PDT</t>
         </is>
       </c>
     </row>
     <row r="208">
       <c r="A208" s="2" t="inlineStr">
         <is>
-          <t>dbt/models/staging/kinetic/stg_kinetic__identity_map.sql</t>
+          <t>dbt/tests/assert_int_sessions_unified_no_negative_duration.sql</t>
         </is>
       </c>
       <c r="B208" s="2" t="inlineStr">
@@ -5011,19 +5011,19 @@
       </c>
       <c r="C208" s="3" t="inlineStr">
         <is>
-          <t>Phase 2 staging (Customer 360): 1:1 pass-through of identity_map</t>
+          <t>dbt test: no session ends before it starts</t>
         </is>
       </c>
       <c r="D208" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 10:26 PDT</t>
+          <t>2026-09-29 17:23 PDT</t>
         </is>
       </c>
     </row>
     <row r="209">
       <c r="A209" s="2" t="inlineStr">
         <is>
-          <t>dbt/models/staging/kinetic/stg_kinetic__segments.sql</t>
+          <t>dbt/models/marts/mart_storefront_revenue_monthly.sql</t>
         </is>
       </c>
       <c r="B209" s="2" t="inlineStr">
@@ -5033,19 +5033,19 @@
       </c>
       <c r="C209" s="3" t="inlineStr">
         <is>
-          <t>Phase 2 staging (Customer 360): 1:1 pass-through of segments</t>
+          <t>Second canonical metric mart: non-subscription (course+merch) gross/net revenue, AOV, guest-checkout share, discount-usage share, refund rate by month -- validated against a hand-run equivalent query on the live database (2026-07: 246 orders, $13,843.71 gross revenue, $56.28 AOV)</t>
         </is>
       </c>
       <c r="D209" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 10:26 PDT</t>
+          <t>2026-09-28 14:53 PDT</t>
         </is>
       </c>
     </row>
     <row r="210">
       <c r="A210" s="2" t="inlineStr">
         <is>
-          <t>dbt/models/staging/kinetic/stg_kinetic__customer_segment_membership.sql</t>
+          <t>dbt/models/staging/kinetic/stg_kinetic__customer_addresses.sql</t>
         </is>
       </c>
       <c r="B210" s="2" t="inlineStr">
@@ -5055,7 +5055,7 @@
       </c>
       <c r="C210" s="3" t="inlineStr">
         <is>
-          <t>Phase 2 staging (Customer 360): 1:1 pass-through of customer_segment_membership, plus is_current_member flag</t>
+          <t>Phase 2 staging (Customer 360): 1:1 pass-through of customer_addresses</t>
         </is>
       </c>
       <c r="D210" s="2" t="inlineStr">
@@ -5067,7 +5067,7 @@
     <row r="211">
       <c r="A211" s="2" t="inlineStr">
         <is>
-          <t>dbt/models/staging/kinetic/stg_kinetic__subscription_events.sql</t>
+          <t>dbt/models/staging/kinetic/stg_kinetic__devices.sql</t>
         </is>
       </c>
       <c r="B211" s="2" t="inlineStr">
@@ -5077,7 +5077,7 @@
       </c>
       <c r="C211" s="3" t="inlineStr">
         <is>
-          <t>Phase 2 staging (Customer 360): 1:1 pass-through of subscription_events; old_plan/new_plan renamed to old_plan_id/new_plan_id</t>
+          <t>Phase 2 staging (Customer 360): 1:1 pass-through of devices, plus is_anonymous_device flag (customer_id null for ~94% of devices by design)</t>
         </is>
       </c>
       <c r="D211" s="2" t="inlineStr">
@@ -5089,7 +5089,7 @@
     <row r="212">
       <c r="A212" s="2" t="inlineStr">
         <is>
-          <t>dbt/models/staging/kinetic/_kinetic__staging.yml</t>
+          <t>dbt/models/staging/kinetic/stg_kinetic__identity_map.sql</t>
         </is>
       </c>
       <c r="B212" s="2" t="inlineStr">
@@ -5099,19 +5099,19 @@
       </c>
       <c r="C212" s="3" t="inlineStr">
         <is>
-          <t>Updated: tests for the 6 Customer 360 staging models (PK not_null/unique, FK relationships) -- all hand-verified against live data first</t>
+          <t>Phase 2 staging (Customer 360): 1:1 pass-through of identity_map</t>
         </is>
       </c>
       <c r="D212" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 16:49 PDT</t>
+          <t>2026-09-29 10:26 PDT</t>
         </is>
       </c>
     </row>
     <row r="213">
       <c r="A213" s="2" t="inlineStr">
         <is>
-          <t>dbt/models/staging/kinetic/stg_kinetic__web_sessions.sql</t>
+          <t>dbt/models/staging/kinetic/stg_kinetic__segments.sql</t>
         </is>
       </c>
       <c r="B213" s="2" t="inlineStr">
@@ -5121,19 +5121,19 @@
       </c>
       <c r="C213" s="3" t="inlineStr">
         <is>
-          <t>Phase 2 staging (web/app engagement): 1:1 pass-through of web_sessions, plus is_known_customer flag (customer_id null for ~79% of sessions by design)</t>
+          <t>Phase 2 staging (Customer 360): 1:1 pass-through of segments</t>
         </is>
       </c>
       <c r="D213" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 12:58 PDT</t>
+          <t>2026-09-29 10:26 PDT</t>
         </is>
       </c>
     </row>
     <row r="214">
       <c r="A214" s="2" t="inlineStr">
         <is>
-          <t>dbt/models/staging/kinetic/stg_kinetic__web_events.sql</t>
+          <t>dbt/models/staging/kinetic/stg_kinetic__customer_segment_membership.sql</t>
         </is>
       </c>
       <c r="B214" s="2" t="inlineStr">
@@ -5143,19 +5143,19 @@
       </c>
       <c r="C214" s="3" t="inlineStr">
         <is>
-          <t>Phase 2 staging (web/app engagement): 1:1 pass-through of web_events</t>
+          <t>Phase 2 staging (Customer 360): 1:1 pass-through of customer_segment_membership, plus is_current_member flag</t>
         </is>
       </c>
       <c r="D214" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 12:58 PDT</t>
+          <t>2026-09-29 10:26 PDT</t>
         </is>
       </c>
     </row>
     <row r="215">
       <c r="A215" s="2" t="inlineStr">
         <is>
-          <t>dbt/models/staging/kinetic/stg_kinetic__app_sessions.sql</t>
+          <t>dbt/models/staging/kinetic/stg_kinetic__subscription_events.sql</t>
         </is>
       </c>
       <c r="B215" s="2" t="inlineStr">
@@ -5165,19 +5165,19 @@
       </c>
       <c r="C215" s="3" t="inlineStr">
         <is>
-          <t>Phase 2 staging (web/app engagement): 1:1 pass-through of app_sessions</t>
+          <t>Phase 2 staging (Customer 360): 1:1 pass-through of subscription_events; old_plan/new_plan renamed to old_plan_id/new_plan_id</t>
         </is>
       </c>
       <c r="D215" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 12:58 PDT</t>
+          <t>2026-09-29 10:26 PDT</t>
         </is>
       </c>
     </row>
     <row r="216">
       <c r="A216" s="2" t="inlineStr">
         <is>
-          <t>dbt/models/staging/kinetic/stg_kinetic__app_events.sql</t>
+          <t>dbt/models/staging/kinetic/_kinetic__staging.yml</t>
         </is>
       </c>
       <c r="B216" s="2" t="inlineStr">
@@ -5187,19 +5187,19 @@
       </c>
       <c r="C216" s="3" t="inlineStr">
         <is>
-          <t>Phase 2 staging (web/app engagement): 1:1 pass-through of app_events</t>
+          <t>Updated: tests for the 6 Customer 360 staging models (PK not_null/unique, FK relationships) -- all hand-verified against live data first</t>
         </is>
       </c>
       <c r="D216" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 12:58 PDT</t>
+          <t>2026-09-29 16:49 PDT</t>
         </is>
       </c>
     </row>
     <row r="217">
       <c r="A217" s="2" t="inlineStr">
         <is>
-          <t>dbt/models/staging/kinetic/_kinetic__staging.yml</t>
+          <t>dbt/models/staging/kinetic/stg_kinetic__web_sessions.sql</t>
         </is>
       </c>
       <c r="B217" s="2" t="inlineStr">
@@ -5209,19 +5209,19 @@
       </c>
       <c r="C217" s="3" t="inlineStr">
         <is>
-          <t>Updated: tests for the 4 web/app engagement staging models -- all hand-verified against live data first</t>
+          <t>Phase 2 staging (web/app engagement): 1:1 pass-through of web_sessions, plus is_known_customer flag (customer_id null for ~79% of sessions by design)</t>
         </is>
       </c>
       <c r="D217" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 16:49 PDT</t>
+          <t>2026-09-29 12:58 PDT</t>
         </is>
       </c>
     </row>
     <row r="218">
       <c r="A218" s="2" t="inlineStr">
         <is>
-          <t>dbt/models/staging/kinetic/stg_kinetic__braze_email_campaigns.sql</t>
+          <t>dbt/models/staging/kinetic/stg_kinetic__web_events.sql</t>
         </is>
       </c>
       <c r="B218" s="2" t="inlineStr">
@@ -5231,19 +5231,19 @@
       </c>
       <c r="C218" s="3" t="inlineStr">
         <is>
-          <t>Phase 2 staging (email/push): 1:1 pass-through of braze_email_campaigns</t>
+          <t>Phase 2 staging (web/app engagement): 1:1 pass-through of web_events</t>
         </is>
       </c>
       <c r="D218" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 12:59 PDT</t>
+          <t>2026-09-29 12:58 PDT</t>
         </is>
       </c>
     </row>
     <row r="219">
       <c r="A219" s="2" t="inlineStr">
         <is>
-          <t>dbt/models/staging/kinetic/stg_kinetic__braze_push_campaigns.sql</t>
+          <t>dbt/models/staging/kinetic/stg_kinetic__app_sessions.sql</t>
         </is>
       </c>
       <c r="B219" s="2" t="inlineStr">
@@ -5253,19 +5253,19 @@
       </c>
       <c r="C219" s="3" t="inlineStr">
         <is>
-          <t>Phase 2 staging (email/push): 1:1 pass-through of braze_push_campaigns</t>
+          <t>Phase 2 staging (web/app engagement): 1:1 pass-through of app_sessions</t>
         </is>
       </c>
       <c r="D219" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 12:59 PDT</t>
+          <t>2026-09-29 12:58 PDT</t>
         </is>
       </c>
     </row>
     <row r="220">
       <c r="A220" s="2" t="inlineStr">
         <is>
-          <t>dbt/models/staging/kinetic/stg_kinetic__braze_email_events.sql</t>
+          <t>dbt/models/staging/kinetic/stg_kinetic__app_events.sql</t>
         </is>
       </c>
       <c r="B220" s="2" t="inlineStr">
@@ -5275,19 +5275,19 @@
       </c>
       <c r="C220" s="3" t="inlineStr">
         <is>
-          <t>Phase 2 staging (email/push): braze_email_events with external_user_id renamed to customer_id and a short event_name (send/open/click/bounce/unsubscribe) alongside Braze's raw event_type</t>
+          <t>Phase 2 staging (web/app engagement): 1:1 pass-through of app_events</t>
         </is>
       </c>
       <c r="D220" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 12:59 PDT</t>
+          <t>2026-09-29 12:58 PDT</t>
         </is>
       </c>
     </row>
     <row r="221">
       <c r="A221" s="2" t="inlineStr">
         <is>
-          <t>dbt/models/staging/kinetic/stg_kinetic__braze_push_events.sql</t>
+          <t>dbt/models/staging/kinetic/_kinetic__staging.yml</t>
         </is>
       </c>
       <c r="B221" s="2" t="inlineStr">
@@ -5297,19 +5297,19 @@
       </c>
       <c r="C221" s="3" t="inlineStr">
         <is>
-          <t>Phase 2 staging (email/push): braze_push_events with external_user_id renamed to customer_id and a short event_name alongside Braze's raw event_type</t>
+          <t>Updated: tests for the 4 web/app engagement staging models -- all hand-verified against live data first</t>
         </is>
       </c>
       <c r="D221" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 12:59 PDT</t>
+          <t>2026-09-29 16:49 PDT</t>
         </is>
       </c>
     </row>
     <row r="222">
       <c r="A222" s="2" t="inlineStr">
         <is>
-          <t>dbt/models/staging/kinetic/_kinetic__staging.yml</t>
+          <t>dbt/models/staging/kinetic/stg_kinetic__braze_email_campaigns.sql</t>
         </is>
       </c>
       <c r="B222" s="2" t="inlineStr">
@@ -5319,19 +5319,19 @@
       </c>
       <c r="C222" s="3" t="inlineStr">
         <is>
-          <t>Updated: tests for the 4 Braze staging models, incl. accepted_values on event_name -- all hand-verified against live data first</t>
+          <t>Phase 2 staging (email/push): 1:1 pass-through of braze_email_campaigns</t>
         </is>
       </c>
       <c r="D222" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 16:49 PDT</t>
+          <t>2026-09-29 12:59 PDT</t>
         </is>
       </c>
     </row>
     <row r="223">
       <c r="A223" s="2" t="inlineStr">
         <is>
-          <t>dbt/models/staging/kinetic/stg_kinetic__meta_campaigns.sql</t>
+          <t>dbt/models/staging/kinetic/stg_kinetic__braze_push_campaigns.sql</t>
         </is>
       </c>
       <c r="B223" s="2" t="inlineStr">
@@ -5341,19 +5341,19 @@
       </c>
       <c r="C223" s="3" t="inlineStr">
         <is>
-          <t>Phase 2 staging (paid media: Meta): meta_campaigns with budgets in both raw cents and dollars (Meta API stores budgets in cents)</t>
+          <t>Phase 2 staging (email/push): 1:1 pass-through of braze_push_campaigns</t>
         </is>
       </c>
       <c r="D223" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 13:02 PDT</t>
+          <t>2026-09-29 12:59 PDT</t>
         </is>
       </c>
     </row>
     <row r="224">
       <c r="A224" s="2" t="inlineStr">
         <is>
-          <t>dbt/models/staging/kinetic/stg_kinetic__meta_ads.sql</t>
+          <t>dbt/models/staging/kinetic/stg_kinetic__braze_email_events.sql</t>
         </is>
       </c>
       <c r="B224" s="2" t="inlineStr">
@@ -5363,19 +5363,19 @@
       </c>
       <c r="C224" s="3" t="inlineStr">
         <is>
-          <t>Phase 2 staging (paid media: Meta): 1:1 pass-through of meta_ads</t>
+          <t>Phase 2 staging (email/push): braze_email_events with external_user_id renamed to customer_id and a short event_name (send/open/click/bounce/unsubscribe) alongside Braze's raw event_type</t>
         </is>
       </c>
       <c r="D224" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 13:02 PDT</t>
+          <t>2026-09-29 12:59 PDT</t>
         </is>
       </c>
     </row>
     <row r="225">
       <c r="A225" s="2" t="inlineStr">
         <is>
-          <t>dbt/models/staging/kinetic/stg_kinetic__meta_ad_insights_daily.sql</t>
+          <t>dbt/models/staging/kinetic/stg_kinetic__braze_push_events.sql</t>
         </is>
       </c>
       <c r="B225" s="2" t="inlineStr">
@@ -5385,19 +5385,19 @@
       </c>
       <c r="C225" s="3" t="inlineStr">
         <is>
-          <t>Phase 2 staging (paid media: Meta): meta_ad_insights_daily with a combined ad_day_id key, unit-suffixed columns (spend_usd, cpm_usd, cpc_usd) and ctr renamed ctr_fraction (0.017 = 1.7%)</t>
+          <t>Phase 2 staging (email/push): braze_push_events with external_user_id renamed to customer_id and a short event_name alongside Braze's raw event_type</t>
         </is>
       </c>
       <c r="D225" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 13:02 PDT</t>
+          <t>2026-09-29 12:59 PDT</t>
         </is>
       </c>
     </row>
     <row r="226">
       <c r="A226" s="2" t="inlineStr">
         <is>
-          <t>dbt/models/staging/kinetic/stg_kinetic__meta_ad_actions_daily.sql</t>
+          <t>dbt/models/staging/kinetic/_kinetic__staging.yml</t>
         </is>
       </c>
       <c r="B226" s="2" t="inlineStr">
@@ -5407,19 +5407,19 @@
       </c>
       <c r="C226" s="3" t="inlineStr">
         <is>
-          <t>Phase 2 staging (paid media: Meta): meta_ad_actions_daily with a combined ad_day_action_id key; value renamed action_count</t>
+          <t>Updated: tests for the 4 Braze staging models, incl. accepted_values on event_name -- all hand-verified against live data first</t>
         </is>
       </c>
       <c r="D226" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 13:02 PDT</t>
+          <t>2026-09-29 16:49 PDT</t>
         </is>
       </c>
     </row>
     <row r="227">
       <c r="A227" s="2" t="inlineStr">
         <is>
-          <t>dbt/models/staging/kinetic/_kinetic__staging.yml</t>
+          <t>dbt/models/staging/kinetic/stg_kinetic__meta_campaigns.sql</t>
         </is>
       </c>
       <c r="B227" s="2" t="inlineStr">
@@ -5429,19 +5429,19 @@
       </c>
       <c r="C227" s="3" t="inlineStr">
         <is>
-          <t>Updated: tests for the 4 Meta staging models, incl. uniqueness of the combined daily keys -- all hand-verified against live data first</t>
+          <t>Phase 2 staging (paid media: Meta): meta_campaigns with budgets in both raw cents and dollars (Meta API stores budgets in cents)</t>
         </is>
       </c>
       <c r="D227" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 16:49 PDT</t>
+          <t>2026-09-29 13:02 PDT</t>
         </is>
       </c>
     </row>
     <row r="228">
       <c r="A228" s="2" t="inlineStr">
         <is>
-          <t>dbt/models/staging/kinetic/stg_kinetic__google_search_campaigns.sql</t>
+          <t>dbt/models/staging/kinetic/stg_kinetic__meta_ads.sql</t>
         </is>
       </c>
       <c r="B228" s="2" t="inlineStr">
@@ -5451,19 +5451,19 @@
       </c>
       <c r="C228" s="3" t="inlineStr">
         <is>
-          <t>Phase 2 staging (paid media: Google Search): campaigns with the raw customer_id renamed google_ads_account_id (it's the Google Ads account number, not a Kinetic customer), daily budget in micros and dollars, end_date cast back to a date</t>
+          <t>Phase 2 staging (paid media: Meta): 1:1 pass-through of meta_ads</t>
         </is>
       </c>
       <c r="D228" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 13:13 PDT</t>
+          <t>2026-09-29 13:02 PDT</t>
         </is>
       </c>
     </row>
     <row r="229">
       <c r="A229" s="2" t="inlineStr">
         <is>
-          <t>dbt/models/staging/kinetic/stg_kinetic__google_search_ad_groups.sql</t>
+          <t>dbt/models/staging/kinetic/stg_kinetic__meta_ad_insights_daily.sql</t>
         </is>
       </c>
       <c r="B229" s="2" t="inlineStr">
@@ -5473,19 +5473,19 @@
       </c>
       <c r="C229" s="3" t="inlineStr">
         <is>
-          <t>Phase 2 staging (paid media: Google Search): ad groups; cpc_bid_micros cast back to a number (always empty -- automated bidding)</t>
+          <t>Phase 2 staging (paid media: Meta): meta_ad_insights_daily with a combined ad_day_id key, unit-suffixed columns (spend_usd, cpm_usd, cpc_usd) and ctr renamed ctr_fraction (0.017 = 1.7%)</t>
         </is>
       </c>
       <c r="D229" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 13:13 PDT</t>
+          <t>2026-09-29 13:02 PDT</t>
         </is>
       </c>
     </row>
     <row r="230">
       <c r="A230" s="2" t="inlineStr">
         <is>
-          <t>dbt/models/staging/kinetic/stg_kinetic__google_search_performance_daily.sql</t>
+          <t>dbt/models/staging/kinetic/stg_kinetic__meta_ad_actions_daily.sql</t>
         </is>
       </c>
       <c r="B230" s="2" t="inlineStr">
@@ -5495,19 +5495,19 @@
       </c>
       <c r="C230" s="3" t="inlineStr">
         <is>
-          <t>Phase 2 staging (paid media: Google Search): ad-group-day performance with combined ad_group_day_id key, cost converted from micros to dollars, ctr_fraction. The keyword table rolled up -- never add the two together</t>
+          <t>Phase 2 staging (paid media: Meta): meta_ad_actions_daily with a combined ad_day_action_id key; value renamed action_count</t>
         </is>
       </c>
       <c r="D230" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 13:13 PDT</t>
+          <t>2026-09-29 13:02 PDT</t>
         </is>
       </c>
     </row>
     <row r="231">
       <c r="A231" s="2" t="inlineStr">
         <is>
-          <t>dbt/models/staging/kinetic/stg_kinetic__google_search_keyword_performance_daily.sql</t>
+          <t>dbt/models/staging/kinetic/_kinetic__staging.yml</t>
         </is>
       </c>
       <c r="B231" s="2" t="inlineStr">
@@ -5517,19 +5517,19 @@
       </c>
       <c r="C231" s="3" t="inlineStr">
         <is>
-          <t>Phase 2 staging (paid media: Google Search): keyword-day performance with combined keyword_day_id key, cost converted from micros to dollars, ctr_fraction</t>
+          <t>Updated: tests for the 4 Meta staging models, incl. uniqueness of the combined daily keys -- all hand-verified against live data first</t>
         </is>
       </c>
       <c r="D231" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 13:13 PDT</t>
+          <t>2026-09-29 16:49 PDT</t>
         </is>
       </c>
     </row>
     <row r="232">
       <c r="A232" s="2" t="inlineStr">
         <is>
-          <t>dbt/models/staging/kinetic/_kinetic__staging.yml</t>
+          <t>dbt/models/staging/kinetic/stg_kinetic__google_search_campaigns.sql</t>
         </is>
       </c>
       <c r="B232" s="2" t="inlineStr">
@@ -5539,19 +5539,19 @@
       </c>
       <c r="C232" s="3" t="inlineStr">
         <is>
-          <t>Updated: tests for the 4 Google Search staging models -- all hand-verified against live data first</t>
+          <t>Phase 2 staging (paid media: Google Search): campaigns with the raw customer_id renamed google_ads_account_id (it's the Google Ads account number, not a Kinetic customer), daily budget in micros and dollars, end_date cast back to a date</t>
         </is>
       </c>
       <c r="D232" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 16:49 PDT</t>
+          <t>2026-09-29 13:13 PDT</t>
         </is>
       </c>
     </row>
     <row r="233">
       <c r="A233" s="2" t="inlineStr">
         <is>
-          <t>dbt/models/staging/kinetic/stg_kinetic__youtube_campaigns.sql</t>
+          <t>dbt/models/staging/kinetic/stg_kinetic__google_search_ad_groups.sql</t>
         </is>
       </c>
       <c r="B233" s="2" t="inlineStr">
@@ -5561,19 +5561,19 @@
       </c>
       <c r="C233" s="3" t="inlineStr">
         <is>
-          <t>Phase 2 staging (paid media: YouTube): campaigns with customer_id renamed google_ads_account_id (the ad account, not a Kinetic customer), budgets in micros and dollars</t>
+          <t>Phase 2 staging (paid media: Google Search): ad groups; cpc_bid_micros cast back to a number (always empty -- automated bidding)</t>
         </is>
       </c>
       <c r="D233" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 13:14 PDT</t>
+          <t>2026-09-29 13:13 PDT</t>
         </is>
       </c>
     </row>
     <row r="234">
       <c r="A234" s="2" t="inlineStr">
         <is>
-          <t>dbt/models/staging/kinetic/stg_kinetic__youtube_ad_groups.sql</t>
+          <t>dbt/models/staging/kinetic/stg_kinetic__google_search_performance_daily.sql</t>
         </is>
       </c>
       <c r="B234" s="2" t="inlineStr">
@@ -5583,19 +5583,19 @@
       </c>
       <c r="C234" s="3" t="inlineStr">
         <is>
-          <t>Phase 2 staging (paid media: YouTube): 1:1 pass-through of youtube_ad_groups</t>
+          <t>Phase 2 staging (paid media: Google Search): ad-group-day performance with combined ad_group_day_id key, cost converted from micros to dollars, ctr_fraction. The keyword table rolled up -- never add the two together</t>
         </is>
       </c>
       <c r="D234" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 13:14 PDT</t>
+          <t>2026-09-29 13:13 PDT</t>
         </is>
       </c>
     </row>
     <row r="235">
       <c r="A235" s="2" t="inlineStr">
         <is>
-          <t>dbt/models/staging/kinetic/stg_kinetic__youtube_performance_daily.sql</t>
+          <t>dbt/models/staging/kinetic/stg_kinetic__google_search_keyword_performance_daily.sql</t>
         </is>
       </c>
       <c r="B235" s="2" t="inlineStr">
@@ -5605,12 +5605,12 @@
       </c>
       <c r="C235" s="3" t="inlineStr">
         <is>
-          <t>Phase 2 staging (paid media: YouTube): ad-group-day performance with combined ad_group_day_id key, cost and cost-per-view converted from micros to dollars, video_view_rate_fraction</t>
+          <t>Phase 2 staging (paid media: Google Search): keyword-day performance with combined keyword_day_id key, cost converted from micros to dollars, ctr_fraction</t>
         </is>
       </c>
       <c r="D235" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 13:14 PDT</t>
+          <t>2026-09-29 13:13 PDT</t>
         </is>
       </c>
     </row>
@@ -5627,7 +5627,7 @@
       </c>
       <c r="C236" s="3" t="inlineStr">
         <is>
-          <t>Updated: tests for the 3 YouTube staging models -- all hand-verified against live data first</t>
+          <t>Updated: tests for the 4 Google Search staging models -- all hand-verified against live data first</t>
         </is>
       </c>
       <c r="D236" s="2" t="inlineStr">
@@ -5639,7 +5639,7 @@
     <row r="237">
       <c r="A237" s="2" t="inlineStr">
         <is>
-          <t>dbt/models/staging/kinetic/stg_kinetic__dv360_insertion_orders.sql</t>
+          <t>dbt/models/staging/kinetic/stg_kinetic__youtube_campaigns.sql</t>
         </is>
       </c>
       <c r="B237" s="2" t="inlineStr">
@@ -5649,19 +5649,19 @@
       </c>
       <c r="C237" s="3" t="inlineStr">
         <is>
-          <t>Phase 2 staging (paid media: DV360): insertion orders with budget_micros named monthly_budget_* (it's a monthly budget), end_date cast back to a date; flags the flat-budget-vs-growing-spend known issue</t>
+          <t>Phase 2 staging (paid media: YouTube): campaigns with customer_id renamed google_ads_account_id (the ad account, not a Kinetic customer), budgets in micros and dollars</t>
         </is>
       </c>
       <c r="D237" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 13:27 PDT</t>
+          <t>2026-09-29 13:14 PDT</t>
         </is>
       </c>
     </row>
     <row r="238">
       <c r="A238" s="2" t="inlineStr">
         <is>
-          <t>dbt/models/staging/kinetic/stg_kinetic__dv360_line_items.sql</t>
+          <t>dbt/models/staging/kinetic/stg_kinetic__youtube_ad_groups.sql</t>
         </is>
       </c>
       <c r="B238" s="2" t="inlineStr">
@@ -5671,19 +5671,19 @@
       </c>
       <c r="C238" s="3" t="inlineStr">
         <is>
-          <t>Phase 2 staging (paid media: DV360): 1:1 pass-through of dv360_line_items</t>
+          <t>Phase 2 staging (paid media: YouTube): 1:1 pass-through of youtube_ad_groups</t>
         </is>
       </c>
       <c r="D238" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 13:19 PDT</t>
+          <t>2026-09-29 13:14 PDT</t>
         </is>
       </c>
     </row>
     <row r="239">
       <c r="A239" s="2" t="inlineStr">
         <is>
-          <t>dbt/models/staging/kinetic/stg_kinetic__dv360_performance_daily.sql</t>
+          <t>dbt/models/staging/kinetic/stg_kinetic__youtube_performance_daily.sql</t>
         </is>
       </c>
       <c r="B239" s="2" t="inlineStr">
@@ -5693,12 +5693,12 @@
       </c>
       <c r="C239" s="3" t="inlineStr">
         <is>
-          <t>Phase 2 staging (paid media: DV360): line-item x day x exchange x environment performance with combined line_item_day_slice_id key, micros converted to dollars, ctr_fraction</t>
+          <t>Phase 2 staging (paid media: YouTube): ad-group-day performance with combined ad_group_day_id key, cost and cost-per-view converted from micros to dollars, video_view_rate_fraction</t>
         </is>
       </c>
       <c r="D239" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 13:19 PDT</t>
+          <t>2026-09-29 13:14 PDT</t>
         </is>
       </c>
     </row>
@@ -5715,7 +5715,7 @@
       </c>
       <c r="C240" s="3" t="inlineStr">
         <is>
-          <t>Updated: tests for the 3 DV360 staging models, incl. accepted_values on exchange and environment -- all hand-verified against live data first</t>
+          <t>Updated: tests for the 3 YouTube staging models -- all hand-verified against live data first</t>
         </is>
       </c>
       <c r="D240" s="2" t="inlineStr">
@@ -5727,7 +5727,7 @@
     <row r="241">
       <c r="A241" s="2" t="inlineStr">
         <is>
-          <t>generator/params.py</t>
+          <t>dbt/models/staging/kinetic/stg_kinetic__dv360_insertion_orders.sql</t>
         </is>
       </c>
       <c r="B241" s="2" t="inlineStr">
@@ -5737,107 +5737,107 @@
       </c>
       <c r="C241" s="3" t="inlineStr">
         <is>
-          <t>Updated 2026-09-29: every evergreen ad budget on all 6 platforms is now the campaign's CURRENT budget, sized from realized spend (weekly average &lt;= budget, no day &gt; 1.75x; DV360 monthly &gt;= highest month). The old flat 'typical day' budgets let later months spend up to ~20x the stored budget</t>
+          <t>Phase 2 staging (paid media: DV360): insertion orders with budget_micros named monthly_budget_* (it's a monthly budget), end_date cast back to a date; flags the flat-budget-vs-growing-spend known issue</t>
         </is>
       </c>
       <c r="D241" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 13:23 PDT</t>
+          <t>2026-09-29 13:27 PDT</t>
         </is>
       </c>
     </row>
     <row r="242">
       <c r="A242" s="2" t="inlineStr">
         <is>
-          <t>data/meta_campaigns.csv</t>
+          <t>dbt/models/staging/kinetic/stg_kinetic__dv360_line_items.sql</t>
         </is>
       </c>
       <c r="B242" s="2" t="inlineStr">
         <is>
-          <t>Shipped table</t>
+          <t>Code</t>
         </is>
       </c>
       <c r="C242" s="3" t="inlineStr">
         <is>
-          <t>Regenerated 2026-09-29: evergreen daily_budget values updated to current budgets (only that column, only the 4 evergreen rows changed)</t>
+          <t>Phase 2 staging (paid media: DV360): 1:1 pass-through of dv360_line_items</t>
         </is>
       </c>
       <c r="D242" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 13:24 PDT</t>
+          <t>2026-09-29 13:19 PDT</t>
         </is>
       </c>
     </row>
     <row r="243">
       <c r="A243" s="2" t="inlineStr">
         <is>
-          <t>data/google_search_campaigns.csv</t>
+          <t>dbt/models/staging/kinetic/stg_kinetic__dv360_performance_daily.sql</t>
         </is>
       </c>
       <c r="B243" s="2" t="inlineStr">
         <is>
-          <t>Shipped table</t>
+          <t>Code</t>
         </is>
       </c>
       <c r="C243" s="3" t="inlineStr">
         <is>
-          <t>Regenerated 2026-09-29: campaign_budget_micros updated to current budgets (only that column changed)</t>
+          <t>Phase 2 staging (paid media: DV360): line-item x day x exchange x environment performance with combined line_item_day_slice_id key, micros converted to dollars, ctr_fraction</t>
         </is>
       </c>
       <c r="D243" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 13:24 PDT</t>
+          <t>2026-09-29 13:19 PDT</t>
         </is>
       </c>
     </row>
     <row r="244">
       <c r="A244" s="2" t="inlineStr">
         <is>
-          <t>data/youtube_campaigns.csv</t>
+          <t>dbt/models/staging/kinetic/_kinetic__staging.yml</t>
         </is>
       </c>
       <c r="B244" s="2" t="inlineStr">
         <is>
-          <t>Shipped table</t>
+          <t>Code</t>
         </is>
       </c>
       <c r="C244" s="3" t="inlineStr">
         <is>
-          <t>Regenerated 2026-09-29: evergreen campaign_budget_micros updated to current budgets (only that column, only the 4 evergreen rows changed)</t>
+          <t>Updated: tests for the 3 DV360 staging models, incl. accepted_values on exchange and environment -- all hand-verified against live data first</t>
         </is>
       </c>
       <c r="D244" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 13:24 PDT</t>
+          <t>2026-09-29 16:49 PDT</t>
         </is>
       </c>
     </row>
     <row r="245">
       <c r="A245" s="2" t="inlineStr">
         <is>
-          <t>data/dv360_insertion_orders.csv</t>
+          <t>generator/params.py</t>
         </is>
       </c>
       <c r="B245" s="2" t="inlineStr">
         <is>
-          <t>Shipped table</t>
+          <t>Code</t>
         </is>
       </c>
       <c r="C245" s="3" t="inlineStr">
         <is>
-          <t>Regenerated 2026-09-29: monthly budget_micros updated to current budgets (only that column changed)</t>
+          <t>Updated 2026-09-29: every evergreen ad budget on all 6 platforms is now the campaign's CURRENT budget, sized from realized spend (weekly average &lt;= budget, no day &gt; 1.75x; DV360 monthly &gt;= highest month). The old flat 'typical day' budgets let later months spend up to ~20x the stored budget</t>
         </is>
       </c>
       <c r="D245" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 13:24 PDT</t>
+          <t>2026-09-29 13:23 PDT</t>
         </is>
       </c>
     </row>
     <row r="246">
       <c r="A246" s="2" t="inlineStr">
         <is>
-          <t>data/snap_campaigns.csv</t>
+          <t>data/meta_campaigns.csv</t>
         </is>
       </c>
       <c r="B246" s="2" t="inlineStr">
@@ -5847,7 +5847,7 @@
       </c>
       <c r="C246" s="3" t="inlineStr">
         <is>
-          <t>Regenerated 2026-09-29: evergreen daily_budget_micro updated to current budgets (only that column, only the 4 evergreen rows changed)</t>
+          <t>Regenerated 2026-09-29: evergreen daily_budget values updated to current budgets (only that column, only the 4 evergreen rows changed)</t>
         </is>
       </c>
       <c r="D246" s="2" t="inlineStr">
@@ -5859,7 +5859,7 @@
     <row r="247">
       <c r="A247" s="2" t="inlineStr">
         <is>
-          <t>data/tiktok_campaigns.csv</t>
+          <t>data/google_search_campaigns.csv</t>
         </is>
       </c>
       <c r="B247" s="2" t="inlineStr">
@@ -5869,7 +5869,7 @@
       </c>
       <c r="C247" s="3" t="inlineStr">
         <is>
-          <t>Regenerated 2026-09-29: BUDGET_MODE_DAY budget_micro updated to current budgets (only that column, only the 4 evergreen rows changed)</t>
+          <t>Regenerated 2026-09-29: campaign_budget_micros updated to current budgets (only that column changed)</t>
         </is>
       </c>
       <c r="D247" s="2" t="inlineStr">
@@ -5881,95 +5881,95 @@
     <row r="248">
       <c r="A248" s="2" t="inlineStr">
         <is>
-          <t>generator/audit_cross_dataset_alignment.py</t>
+          <t>data/youtube_campaigns.csv</t>
         </is>
       </c>
       <c r="B248" s="2" t="inlineStr">
         <is>
-          <t>Code</t>
+          <t>Shipped table</t>
         </is>
       </c>
       <c r="C248" s="3" t="inlineStr">
         <is>
-          <t>Updated 2026-09-29: new Check 8 -- spend vs stored budget for every campaign on all 6 platforms (weekly/daily limits for daily budgets, monthly for DV360, total for holiday flights)</t>
+          <t>Regenerated 2026-09-29: evergreen campaign_budget_micros updated to current budgets (only that column, only the 4 evergreen rows changed)</t>
         </is>
       </c>
       <c r="D248" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 13:30 PDT</t>
+          <t>2026-09-29 13:24 PDT</t>
         </is>
       </c>
     </row>
     <row r="249">
       <c r="A249" s="2" t="inlineStr">
         <is>
-          <t>dbt/models/staging/kinetic/stg_kinetic__dv360_insertion_orders.sql</t>
+          <t>data/dv360_insertion_orders.csv</t>
         </is>
       </c>
       <c r="B249" s="2" t="inlineStr">
         <is>
-          <t>Code</t>
+          <t>Shipped table</t>
         </is>
       </c>
       <c r="C249" s="3" t="inlineStr">
         <is>
-          <t>Updated: budget known-issue note replaced -- budgets are now current budgets</t>
+          <t>Regenerated 2026-09-29: monthly budget_micros updated to current budgets (only that column changed)</t>
         </is>
       </c>
       <c r="D249" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 13:27 PDT</t>
+          <t>2026-09-29 13:24 PDT</t>
         </is>
       </c>
     </row>
     <row r="250">
       <c r="A250" s="2" t="inlineStr">
         <is>
-          <t>generator/paid_media_common.py</t>
+          <t>data/snap_campaigns.csv</t>
         </is>
       </c>
       <c r="B250" s="2" t="inlineStr">
         <is>
-          <t>Code</t>
+          <t>Shipped table</t>
         </is>
       </c>
       <c r="C250" s="3" t="inlineStr">
         <is>
-          <t>Updated 2026-09-29: new cap_flight_at_budget() -- rescales a holiday flight's days so it never spends past its lifetime budget, replaying the same random rates so every other row is unchanged</t>
+          <t>Regenerated 2026-09-29: evergreen daily_budget_micro updated to current budgets (only that column, only the 4 evergreen rows changed)</t>
         </is>
       </c>
       <c r="D250" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 13:29 PDT</t>
+          <t>2026-09-29 13:24 PDT</t>
         </is>
       </c>
     </row>
     <row r="251">
       <c r="A251" s="2" t="inlineStr">
         <is>
-          <t>generator/build_meta_ad_insights_daily.py</t>
+          <t>data/tiktok_campaigns.csv</t>
         </is>
       </c>
       <c r="B251" s="2" t="inlineStr">
         <is>
-          <t>Code</t>
+          <t>Shipped table</t>
         </is>
       </c>
       <c r="C251" s="3" t="inlineStr">
         <is>
-          <t>Updated 2026-09-29: holiday flights capped at their lifetime budget via cap_flight_at_budget()</t>
+          <t>Regenerated 2026-09-29: BUDGET_MODE_DAY budget_micro updated to current budgets (only that column, only the 4 evergreen rows changed)</t>
         </is>
       </c>
       <c r="D251" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 13:29 PDT</t>
+          <t>2026-09-29 13:24 PDT</t>
         </is>
       </c>
     </row>
     <row r="252">
       <c r="A252" s="2" t="inlineStr">
         <is>
-          <t>generator/build_snap_stats_daily.py</t>
+          <t>generator/audit_cross_dataset_alignment.py</t>
         </is>
       </c>
       <c r="B252" s="2" t="inlineStr">
@@ -5979,19 +5979,19 @@
       </c>
       <c r="C252" s="3" t="inlineStr">
         <is>
-          <t>Updated 2026-09-29: holiday flights capped at their lifetime budget via cap_flight_at_budget()</t>
+          <t>Updated 2026-09-29: new Check 8 -- spend vs stored budget for every campaign on all 6 platforms (weekly/daily limits for daily budgets, monthly for DV360, total for holiday flights)</t>
         </is>
       </c>
       <c r="D252" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 13:29 PDT</t>
+          <t>2026-09-29 13:30 PDT</t>
         </is>
       </c>
     </row>
     <row r="253">
       <c r="A253" s="2" t="inlineStr">
         <is>
-          <t>generator/build_tiktok_reports_daily.py</t>
+          <t>dbt/models/staging/kinetic/stg_kinetic__dv360_insertion_orders.sql</t>
         </is>
       </c>
       <c r="B253" s="2" t="inlineStr">
@@ -6001,19 +6001,19 @@
       </c>
       <c r="C253" s="3" t="inlineStr">
         <is>
-          <t>Updated 2026-09-29: holiday flights capped at their lifetime budget via cap_flight_at_budget()</t>
+          <t>Updated: budget known-issue note replaced -- budgets are now current budgets</t>
         </is>
       </c>
       <c r="D253" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 13:29 PDT</t>
+          <t>2026-09-29 13:27 PDT</t>
         </is>
       </c>
     </row>
     <row r="254">
       <c r="A254" s="2" t="inlineStr">
         <is>
-          <t>generator/build_youtube_performance_daily.py</t>
+          <t>generator/paid_media_common.py</t>
         </is>
       </c>
       <c r="B254" s="2" t="inlineStr">
@@ -6023,7 +6023,7 @@
       </c>
       <c r="C254" s="3" t="inlineStr">
         <is>
-          <t>Updated 2026-09-29: holiday flights capped at their lifetime budget via cap_flight_at_budget() (no-op today -- all YouTube flights were already under budget)</t>
+          <t>Updated 2026-09-29: new cap_flight_at_budget() -- rescales a holiday flight's days so it never spends past its lifetime budget, replaying the same random rates so every other row is unchanged</t>
         </is>
       </c>
       <c r="D254" s="2" t="inlineStr">
@@ -6035,17 +6035,17 @@
     <row r="255">
       <c r="A255" s="2" t="inlineStr">
         <is>
-          <t>data/meta_ad_insights_daily.csv</t>
+          <t>generator/build_meta_ad_insights_daily.py</t>
         </is>
       </c>
       <c r="B255" s="2" t="inlineStr">
         <is>
-          <t>Shipped table</t>
+          <t>Code</t>
         </is>
       </c>
       <c r="C255" s="3" t="inlineStr">
         <is>
-          <t>Regenerated 2026-09-29: the 2023 and 2024 holiday flights (38 rows) trimmed to spend exactly their lifetime budget; every other row identical</t>
+          <t>Updated 2026-09-29: holiday flights capped at their lifetime budget via cap_flight_at_budget()</t>
         </is>
       </c>
       <c r="D255" s="2" t="inlineStr">
@@ -6057,17 +6057,17 @@
     <row r="256">
       <c r="A256" s="2" t="inlineStr">
         <is>
-          <t>data/meta_ad_actions_daily.csv</t>
+          <t>generator/build_snap_stats_daily.py</t>
         </is>
       </c>
       <c r="B256" s="2" t="inlineStr">
         <is>
-          <t>Shipped table</t>
+          <t>Code</t>
         </is>
       </c>
       <c r="C256" s="3" t="inlineStr">
         <is>
-          <t>Regenerated 2026-09-29: re-derived from the trimmed insights rows -- only the 2023/2024 holiday flights' action rows changed (one initiate_checkout row on 2024-11-15 dropped to zero and is no longer emitted)</t>
+          <t>Updated 2026-09-29: holiday flights capped at their lifetime budget via cap_flight_at_budget()</t>
         </is>
       </c>
       <c r="D256" s="2" t="inlineStr">
@@ -6079,17 +6079,17 @@
     <row r="257">
       <c r="A257" s="2" t="inlineStr">
         <is>
-          <t>data/snap_stats_daily.csv</t>
+          <t>generator/build_tiktok_reports_daily.py</t>
         </is>
       </c>
       <c r="B257" s="2" t="inlineStr">
         <is>
-          <t>Shipped table</t>
+          <t>Code</t>
         </is>
       </c>
       <c r="C257" s="3" t="inlineStr">
         <is>
-          <t>Regenerated 2026-09-29: the 2024 holiday flight (19 rows) trimmed to spend exactly its lifetime budget; every other row identical</t>
+          <t>Updated 2026-09-29: holiday flights capped at their lifetime budget via cap_flight_at_budget()</t>
         </is>
       </c>
       <c r="D257" s="2" t="inlineStr">
@@ -6101,17 +6101,17 @@
     <row r="258">
       <c r="A258" s="2" t="inlineStr">
         <is>
-          <t>data/tiktok_reports_daily.csv</t>
+          <t>generator/build_youtube_performance_daily.py</t>
         </is>
       </c>
       <c r="B258" s="2" t="inlineStr">
         <is>
-          <t>Shipped table</t>
+          <t>Code</t>
         </is>
       </c>
       <c r="C258" s="3" t="inlineStr">
         <is>
-          <t>Regenerated 2026-09-29: the 2023/2024/2025 holiday flights (56 rows) trimmed to spend exactly their lifetime budgets; every other row identical</t>
+          <t>Updated 2026-09-29: holiday flights capped at their lifetime budget via cap_flight_at_budget() (no-op today -- all YouTube flights were already under budget)</t>
         </is>
       </c>
       <c r="D258" s="2" t="inlineStr">
@@ -6123,117 +6123,117 @@
     <row r="259">
       <c r="A259" s="2" t="inlineStr">
         <is>
-          <t>docs/cross_dataset_alignment_audit.md</t>
+          <t>data/meta_ad_insights_daily.csv</t>
         </is>
       </c>
       <c r="B259" s="2" t="inlineStr">
         <is>
-          <t>Docs</t>
+          <t>Shipped table</t>
         </is>
       </c>
       <c r="C259" s="3" t="inlineStr">
         <is>
-          <t>Updated 2026-09-29: added Check 8 (spend vs stored budget) with both fixes and results</t>
+          <t>Regenerated 2026-09-29: the 2023 and 2024 holiday flights (38 rows) trimmed to spend exactly their lifetime budget; every other row identical</t>
         </is>
       </c>
       <c r="D259" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 13:54 PDT</t>
+          <t>2026-09-29 13:29 PDT</t>
         </is>
       </c>
     </row>
     <row r="260">
       <c r="A260" s="2" t="inlineStr">
         <is>
-          <t>generator/audit_cross_dataset_alignment.py</t>
+          <t>data/meta_ad_actions_daily.csv</t>
         </is>
       </c>
       <c r="B260" s="2" t="inlineStr">
         <is>
-          <t>Code</t>
+          <t>Shipped table</t>
         </is>
       </c>
       <c r="C260" s="3" t="inlineStr">
         <is>
-          <t>Updated 2026-09-29: Check 8's flight limit tightened from 1.05x to 1.0x now that flights are capped</t>
+          <t>Regenerated 2026-09-29: re-derived from the trimmed insights rows -- only the 2023/2024 holiday flights' action rows changed (one initiate_checkout row on 2024-11-15 dropped to zero and is no longer emitted)</t>
         </is>
       </c>
       <c r="D260" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 13:30 PDT</t>
+          <t>2026-09-29 13:29 PDT</t>
         </is>
       </c>
     </row>
     <row r="261">
       <c r="A261" s="2" t="inlineStr">
         <is>
-          <t>dbt/models/staging/kinetic/stg_kinetic__snap_campaigns.sql</t>
+          <t>data/snap_stats_daily.csv</t>
         </is>
       </c>
       <c r="B261" s="2" t="inlineStr">
         <is>
-          <t>Code</t>
+          <t>Shipped table</t>
         </is>
       </c>
       <c r="C261" s="3" t="inlineStr">
         <is>
-          <t>Phase 2 staging (paid media: Snap): campaigns with ad_account_id renamed snap_ad_account_id, current budgets in micros and dollars</t>
+          <t>Regenerated 2026-09-29: the 2024 holiday flight (19 rows) trimmed to spend exactly its lifetime budget; every other row identical</t>
         </is>
       </c>
       <c r="D261" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 15:53 PDT</t>
+          <t>2026-09-29 13:29 PDT</t>
         </is>
       </c>
     </row>
     <row r="262">
       <c r="A262" s="2" t="inlineStr">
         <is>
-          <t>dbt/models/staging/kinetic/stg_kinetic__snap_ad_squads.sql</t>
+          <t>data/tiktok_reports_daily.csv</t>
         </is>
       </c>
       <c r="B262" s="2" t="inlineStr">
         <is>
-          <t>Code</t>
+          <t>Shipped table</t>
         </is>
       </c>
       <c r="C262" s="3" t="inlineStr">
         <is>
-          <t>Phase 2 staging (paid media: Snap): 1:1 pass-through of snap_ad_squads (Snap's ad set / ad group level)</t>
+          <t>Regenerated 2026-09-29: the 2023/2024/2025 holiday flights (56 rows) trimmed to spend exactly their lifetime budgets; every other row identical</t>
         </is>
       </c>
       <c r="D262" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 15:53 PDT</t>
+          <t>2026-09-29 13:29 PDT</t>
         </is>
       </c>
     </row>
     <row r="263">
       <c r="A263" s="2" t="inlineStr">
         <is>
-          <t>dbt/models/staging/kinetic/stg_kinetic__snap_ads.sql</t>
+          <t>docs/cross_dataset_alignment_audit.md</t>
         </is>
       </c>
       <c r="B263" s="2" t="inlineStr">
         <is>
-          <t>Code</t>
+          <t>Docs</t>
         </is>
       </c>
       <c r="C263" s="3" t="inlineStr">
         <is>
-          <t>Phase 2 staging (paid media: Snap): 1:1 pass-through of snap_ads</t>
+          <t>Updated 2026-09-29: added Check 8 (spend vs stored budget) with both fixes and results</t>
         </is>
       </c>
       <c r="D263" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 15:53 PDT</t>
+          <t>2026-09-29 13:54 PDT</t>
         </is>
       </c>
     </row>
     <row r="264">
       <c r="A264" s="2" t="inlineStr">
         <is>
-          <t>dbt/models/staging/kinetic/stg_kinetic__snap_stats_daily.sql</t>
+          <t>generator/audit_cross_dataset_alignment.py</t>
         </is>
       </c>
       <c r="B264" s="2" t="inlineStr">
@@ -6243,19 +6243,19 @@
       </c>
       <c r="C264" s="3" t="inlineStr">
         <is>
-          <t>Phase 2 staging (paid media: Snap): ad-day stats with combined ad_day_id key, spend in micros and dollars; documents swipes as Snap's clicks</t>
+          <t>Updated 2026-09-29: Check 8's flight limit tightened from 1.05x to 1.0x now that flights are capped</t>
         </is>
       </c>
       <c r="D264" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 15:53 PDT</t>
+          <t>2026-09-29 13:30 PDT</t>
         </is>
       </c>
     </row>
     <row r="265">
       <c r="A265" s="2" t="inlineStr">
         <is>
-          <t>dbt/models/staging/kinetic/_kinetic__staging.yml</t>
+          <t>dbt/models/staging/kinetic/stg_kinetic__snap_campaigns.sql</t>
         </is>
       </c>
       <c r="B265" s="2" t="inlineStr">
@@ -6265,19 +6265,19 @@
       </c>
       <c r="C265" s="3" t="inlineStr">
         <is>
-          <t>Updated: tests for the 4 Snap staging models -- all hand-verified against live data first</t>
+          <t>Phase 2 staging (paid media: Snap): campaigns with ad_account_id renamed snap_ad_account_id, current budgets in micros and dollars</t>
         </is>
       </c>
       <c r="D265" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 16:49 PDT</t>
+          <t>2026-09-29 15:53 PDT</t>
         </is>
       </c>
     </row>
     <row r="266">
       <c r="A266" s="2" t="inlineStr">
         <is>
-          <t>dbt/models/staging/kinetic/stg_kinetic__tiktok_campaigns.sql</t>
+          <t>dbt/models/staging/kinetic/stg_kinetic__snap_ad_squads.sql</t>
         </is>
       </c>
       <c r="B266" s="2" t="inlineStr">
@@ -6287,19 +6287,19 @@
       </c>
       <c r="C266" s="3" t="inlineStr">
         <is>
-          <t>Phase 2 staging (paid media: TikTok): campaigns with the single budget split into daily_budget_usd / lifetime_budget_usd by budget_mode (matching the other platforms), advertiser_id renamed tiktok_advertiser_id</t>
+          <t>Phase 2 staging (paid media: Snap): 1:1 pass-through of snap_ad_squads (Snap's ad set / ad group level)</t>
         </is>
       </c>
       <c r="D266" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 15:57 PDT</t>
+          <t>2026-09-29 15:53 PDT</t>
         </is>
       </c>
     </row>
     <row r="267">
       <c r="A267" s="2" t="inlineStr">
         <is>
-          <t>dbt/models/staging/kinetic/stg_kinetic__tiktok_adgroups.sql</t>
+          <t>dbt/models/staging/kinetic/stg_kinetic__snap_ads.sql</t>
         </is>
       </c>
       <c r="B267" s="2" t="inlineStr">
@@ -6309,19 +6309,19 @@
       </c>
       <c r="C267" s="3" t="inlineStr">
         <is>
-          <t>Phase 2 staging (paid media: TikTok): 1:1 pass-through of tiktok_adgroups</t>
+          <t>Phase 2 staging (paid media: Snap): 1:1 pass-through of snap_ads</t>
         </is>
       </c>
       <c r="D267" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 15:57 PDT</t>
+          <t>2026-09-29 15:53 PDT</t>
         </is>
       </c>
     </row>
     <row r="268">
       <c r="A268" s="2" t="inlineStr">
         <is>
-          <t>dbt/models/staging/kinetic/stg_kinetic__tiktok_ads.sql</t>
+          <t>dbt/models/staging/kinetic/stg_kinetic__snap_stats_daily.sql</t>
         </is>
       </c>
       <c r="B268" s="2" t="inlineStr">
@@ -6331,19 +6331,19 @@
       </c>
       <c r="C268" s="3" t="inlineStr">
         <is>
-          <t>Phase 2 staging (paid media: TikTok): 1:1 pass-through of tiktok_ads</t>
+          <t>Phase 2 staging (paid media: Snap): ad-day stats with combined ad_day_id key, spend in micros and dollars; documents swipes as Snap's clicks</t>
         </is>
       </c>
       <c r="D268" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 15:57 PDT</t>
+          <t>2026-09-29 15:53 PDT</t>
         </is>
       </c>
     </row>
     <row r="269">
       <c r="A269" s="2" t="inlineStr">
         <is>
-          <t>dbt/models/staging/kinetic/stg_kinetic__tiktok_reports_daily.sql</t>
+          <t>dbt/models/staging/kinetic/_kinetic__staging.yml</t>
         </is>
       </c>
       <c r="B269" s="2" t="inlineStr">
@@ -6353,19 +6353,19 @@
       </c>
       <c r="C269" s="3" t="inlineStr">
         <is>
-          <t>Phase 2 staging (paid media: TikTok): ad-day reports with combined ad_day_id key, spend and CPM in micros and dollars, ctr_fraction</t>
+          <t>Updated: tests for the 4 Snap staging models -- all hand-verified against live data first</t>
         </is>
       </c>
       <c r="D269" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 15:57 PDT</t>
+          <t>2026-09-29 16:49 PDT</t>
         </is>
       </c>
     </row>
     <row r="270">
       <c r="A270" s="2" t="inlineStr">
         <is>
-          <t>dbt/models/staging/kinetic/stg_kinetic__product_variants.sql</t>
+          <t>dbt/models/staging/kinetic/stg_kinetic__tiktok_campaigns.sql</t>
         </is>
       </c>
       <c r="B270" s="2" t="inlineStr">
@@ -6375,54 +6375,142 @@
       </c>
       <c r="C270" s="3" t="inlineStr">
         <is>
-          <t>Phase 2 staging (final table, 47 of 47): product variants with variant_option, price_adjustment_usd</t>
+          <t>Phase 2 staging (paid media: TikTok): campaigns with the single budget split into daily_budget_usd / lifetime_budget_usd by budget_mode (matching the other platforms), advertiser_id renamed tiktok_advertiser_id</t>
         </is>
       </c>
       <c r="D270" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 16:08 PDT</t>
+          <t>2026-09-29 15:57 PDT</t>
         </is>
       </c>
     </row>
     <row r="271">
       <c r="A271" s="2" t="inlineStr">
         <is>
-          <t>HANDOFF.md</t>
+          <t>dbt/models/staging/kinetic/stg_kinetic__tiktok_adgroups.sql</t>
         </is>
       </c>
       <c r="B271" s="2" t="inlineStr">
         <is>
-          <t>Doc</t>
+          <t>Code</t>
         </is>
       </c>
       <c r="C271" s="3" t="inlineStr">
         <is>
-          <t>Handoff note for starting a new chat/project: status, open decisions, prior decisions, pitfalls</t>
+          <t>Phase 2 staging (paid media: TikTok): 1:1 pass-through of tiktok_adgroups</t>
         </is>
       </c>
       <c r="D271" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 17:09 PDT</t>
+          <t>2026-09-29 15:57 PDT</t>
         </is>
       </c>
     </row>
     <row r="272">
       <c r="A272" s="2" t="inlineStr">
         <is>
+          <t>dbt/models/staging/kinetic/stg_kinetic__tiktok_ads.sql</t>
+        </is>
+      </c>
+      <c r="B272" s="2" t="inlineStr">
+        <is>
+          <t>Code</t>
+        </is>
+      </c>
+      <c r="C272" s="3" t="inlineStr">
+        <is>
+          <t>Phase 2 staging (paid media: TikTok): 1:1 pass-through of tiktok_ads</t>
+        </is>
+      </c>
+      <c r="D272" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-29 15:57 PDT</t>
+        </is>
+      </c>
+    </row>
+    <row r="273">
+      <c r="A273" s="2" t="inlineStr">
+        <is>
+          <t>dbt/models/staging/kinetic/stg_kinetic__tiktok_reports_daily.sql</t>
+        </is>
+      </c>
+      <c r="B273" s="2" t="inlineStr">
+        <is>
+          <t>Code</t>
+        </is>
+      </c>
+      <c r="C273" s="3" t="inlineStr">
+        <is>
+          <t>Phase 2 staging (paid media: TikTok): ad-day reports with combined ad_day_id key, spend and CPM in micros and dollars, ctr_fraction</t>
+        </is>
+      </c>
+      <c r="D273" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-29 15:57 PDT</t>
+        </is>
+      </c>
+    </row>
+    <row r="274">
+      <c r="A274" s="2" t="inlineStr">
+        <is>
+          <t>dbt/models/staging/kinetic/stg_kinetic__product_variants.sql</t>
+        </is>
+      </c>
+      <c r="B274" s="2" t="inlineStr">
+        <is>
+          <t>Code</t>
+        </is>
+      </c>
+      <c r="C274" s="3" t="inlineStr">
+        <is>
+          <t>Phase 2 staging (final table, 47 of 47): product variants with variant_option, price_adjustment_usd</t>
+        </is>
+      </c>
+      <c r="D274" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-29 16:08 PDT</t>
+        </is>
+      </c>
+    </row>
+    <row r="275">
+      <c r="A275" s="2" t="inlineStr">
+        <is>
+          <t>HANDOFF.md</t>
+        </is>
+      </c>
+      <c r="B275" s="2" t="inlineStr">
+        <is>
+          <t>Doc</t>
+        </is>
+      </c>
+      <c r="C275" s="3" t="inlineStr">
+        <is>
+          <t>Handoff note for starting a new chat/project: status, open decisions, prior decisions, pitfalls</t>
+        </is>
+      </c>
+      <c r="D275" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-29 17:20 PDT</t>
+        </is>
+      </c>
+    </row>
+    <row r="276">
+      <c r="A276" s="2" t="inlineStr">
+        <is>
           <t>dbt/models/staging/kinetic/_kinetic__staging.yml</t>
         </is>
       </c>
-      <c r="B272" s="2" t="inlineStr">
-        <is>
-          <t>Code</t>
-        </is>
-      </c>
-      <c r="C272" s="3" t="inlineStr">
+      <c r="B276" s="2" t="inlineStr">
+        <is>
+          <t>Code</t>
+        </is>
+      </c>
+      <c r="C276" s="3" t="inlineStr">
         <is>
           <t>Updated: tests for the 4 TikTok staging models -- all hand-verified against live data first</t>
         </is>
       </c>
-      <c r="D272" s="2" t="inlineStr">
+      <c r="D276" s="2" t="inlineStr">
         <is>
           <t>2026-09-29 16:49 PDT</t>
         </is>

</xml_diff>

<commit_message>
Add OVERNIGHT_PLAN.md runbook for unattended run
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012MSGmVw4D6TxU8u8LSeA2e
</commit_message>
<xml_diff>
--- a/File_Manifest.xlsx
+++ b/File_Manifest.xlsx
@@ -435,7 +435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D276"/>
+  <dimension ref="A1:D277"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="48" customWidth="1" min="1" max="1"/>
@@ -506,7 +506,7 @@
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 17:20 PDT</t>
+          <t>2026-09-29 17:25 PDT</t>
         </is>
       </c>
     </row>
@@ -638,7 +638,7 @@
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 17:23 PDT</t>
+          <t>2026-09-29 18:17 PDT</t>
         </is>
       </c>
     </row>
@@ -748,7 +748,7 @@
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 17:23 PDT</t>
+          <t>2026-09-29 18:17 PDT</t>
         </is>
       </c>
     </row>
@@ -5023,29 +5023,29 @@
     <row r="209">
       <c r="A209" s="2" t="inlineStr">
         <is>
-          <t>dbt/models/marts/mart_storefront_revenue_monthly.sql</t>
+          <t>OVERNIGHT_PLAN.md</t>
         </is>
       </c>
       <c r="B209" s="2" t="inlineStr">
         <is>
-          <t>Code</t>
+          <t>Doc</t>
         </is>
       </c>
       <c r="C209" s="3" t="inlineStr">
         <is>
-          <t>Second canonical metric mart: non-subscription (course+merch) gross/net revenue, AOV, guest-checkout share, discount-usage share, refund rate by month -- validated against a hand-run equivalent query on the live database (2026-07: 246 orders, $13,843.71 gross revenue, $56.28 AOV)</t>
+          <t>Runbook for the unattended overnight run: queue, rules, stop rules, morning list format</t>
         </is>
       </c>
       <c r="D209" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28 14:53 PDT</t>
+          <t>2026-09-29 18:17 PDT</t>
         </is>
       </c>
     </row>
     <row r="210">
       <c r="A210" s="2" t="inlineStr">
         <is>
-          <t>dbt/models/staging/kinetic/stg_kinetic__customer_addresses.sql</t>
+          <t>dbt/models/marts/mart_storefront_revenue_monthly.sql</t>
         </is>
       </c>
       <c r="B210" s="2" t="inlineStr">
@@ -5055,19 +5055,19 @@
       </c>
       <c r="C210" s="3" t="inlineStr">
         <is>
-          <t>Phase 2 staging (Customer 360): 1:1 pass-through of customer_addresses</t>
+          <t>Second canonical metric mart: non-subscription (course+merch) gross/net revenue, AOV, guest-checkout share, discount-usage share, refund rate by month -- validated against a hand-run equivalent query on the live database (2026-07: 246 orders, $13,843.71 gross revenue, $56.28 AOV)</t>
         </is>
       </c>
       <c r="D210" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 10:26 PDT</t>
+          <t>2026-09-28 14:53 PDT</t>
         </is>
       </c>
     </row>
     <row r="211">
       <c r="A211" s="2" t="inlineStr">
         <is>
-          <t>dbt/models/staging/kinetic/stg_kinetic__devices.sql</t>
+          <t>dbt/models/staging/kinetic/stg_kinetic__customer_addresses.sql</t>
         </is>
       </c>
       <c r="B211" s="2" t="inlineStr">
@@ -5077,7 +5077,7 @@
       </c>
       <c r="C211" s="3" t="inlineStr">
         <is>
-          <t>Phase 2 staging (Customer 360): 1:1 pass-through of devices, plus is_anonymous_device flag (customer_id null for ~94% of devices by design)</t>
+          <t>Phase 2 staging (Customer 360): 1:1 pass-through of customer_addresses</t>
         </is>
       </c>
       <c r="D211" s="2" t="inlineStr">
@@ -5089,7 +5089,7 @@
     <row r="212">
       <c r="A212" s="2" t="inlineStr">
         <is>
-          <t>dbt/models/staging/kinetic/stg_kinetic__identity_map.sql</t>
+          <t>dbt/models/staging/kinetic/stg_kinetic__devices.sql</t>
         </is>
       </c>
       <c r="B212" s="2" t="inlineStr">
@@ -5099,7 +5099,7 @@
       </c>
       <c r="C212" s="3" t="inlineStr">
         <is>
-          <t>Phase 2 staging (Customer 360): 1:1 pass-through of identity_map</t>
+          <t>Phase 2 staging (Customer 360): 1:1 pass-through of devices, plus is_anonymous_device flag (customer_id null for ~94% of devices by design)</t>
         </is>
       </c>
       <c r="D212" s="2" t="inlineStr">
@@ -5111,7 +5111,7 @@
     <row r="213">
       <c r="A213" s="2" t="inlineStr">
         <is>
-          <t>dbt/models/staging/kinetic/stg_kinetic__segments.sql</t>
+          <t>dbt/models/staging/kinetic/stg_kinetic__identity_map.sql</t>
         </is>
       </c>
       <c r="B213" s="2" t="inlineStr">
@@ -5121,7 +5121,7 @@
       </c>
       <c r="C213" s="3" t="inlineStr">
         <is>
-          <t>Phase 2 staging (Customer 360): 1:1 pass-through of segments</t>
+          <t>Phase 2 staging (Customer 360): 1:1 pass-through of identity_map</t>
         </is>
       </c>
       <c r="D213" s="2" t="inlineStr">
@@ -5133,7 +5133,7 @@
     <row r="214">
       <c r="A214" s="2" t="inlineStr">
         <is>
-          <t>dbt/models/staging/kinetic/stg_kinetic__customer_segment_membership.sql</t>
+          <t>dbt/models/staging/kinetic/stg_kinetic__segments.sql</t>
         </is>
       </c>
       <c r="B214" s="2" t="inlineStr">
@@ -5143,7 +5143,7 @@
       </c>
       <c r="C214" s="3" t="inlineStr">
         <is>
-          <t>Phase 2 staging (Customer 360): 1:1 pass-through of customer_segment_membership, plus is_current_member flag</t>
+          <t>Phase 2 staging (Customer 360): 1:1 pass-through of segments</t>
         </is>
       </c>
       <c r="D214" s="2" t="inlineStr">
@@ -5155,7 +5155,7 @@
     <row r="215">
       <c r="A215" s="2" t="inlineStr">
         <is>
-          <t>dbt/models/staging/kinetic/stg_kinetic__subscription_events.sql</t>
+          <t>dbt/models/staging/kinetic/stg_kinetic__customer_segment_membership.sql</t>
         </is>
       </c>
       <c r="B215" s="2" t="inlineStr">
@@ -5165,7 +5165,7 @@
       </c>
       <c r="C215" s="3" t="inlineStr">
         <is>
-          <t>Phase 2 staging (Customer 360): 1:1 pass-through of subscription_events; old_plan/new_plan renamed to old_plan_id/new_plan_id</t>
+          <t>Phase 2 staging (Customer 360): 1:1 pass-through of customer_segment_membership, plus is_current_member flag</t>
         </is>
       </c>
       <c r="D215" s="2" t="inlineStr">
@@ -5177,7 +5177,7 @@
     <row r="216">
       <c r="A216" s="2" t="inlineStr">
         <is>
-          <t>dbt/models/staging/kinetic/_kinetic__staging.yml</t>
+          <t>dbt/models/staging/kinetic/stg_kinetic__subscription_events.sql</t>
         </is>
       </c>
       <c r="B216" s="2" t="inlineStr">
@@ -5187,19 +5187,19 @@
       </c>
       <c r="C216" s="3" t="inlineStr">
         <is>
-          <t>Updated: tests for the 6 Customer 360 staging models (PK not_null/unique, FK relationships) -- all hand-verified against live data first</t>
+          <t>Phase 2 staging (Customer 360): 1:1 pass-through of subscription_events; old_plan/new_plan renamed to old_plan_id/new_plan_id</t>
         </is>
       </c>
       <c r="D216" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 16:49 PDT</t>
+          <t>2026-09-29 10:26 PDT</t>
         </is>
       </c>
     </row>
     <row r="217">
       <c r="A217" s="2" t="inlineStr">
         <is>
-          <t>dbt/models/staging/kinetic/stg_kinetic__web_sessions.sql</t>
+          <t>dbt/models/staging/kinetic/_kinetic__staging.yml</t>
         </is>
       </c>
       <c r="B217" s="2" t="inlineStr">
@@ -5209,19 +5209,19 @@
       </c>
       <c r="C217" s="3" t="inlineStr">
         <is>
-          <t>Phase 2 staging (web/app engagement): 1:1 pass-through of web_sessions, plus is_known_customer flag (customer_id null for ~79% of sessions by design)</t>
+          <t>Updated: tests for the 6 Customer 360 staging models (PK not_null/unique, FK relationships) -- all hand-verified against live data first</t>
         </is>
       </c>
       <c r="D217" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 12:58 PDT</t>
+          <t>2026-09-29 16:49 PDT</t>
         </is>
       </c>
     </row>
     <row r="218">
       <c r="A218" s="2" t="inlineStr">
         <is>
-          <t>dbt/models/staging/kinetic/stg_kinetic__web_events.sql</t>
+          <t>dbt/models/staging/kinetic/stg_kinetic__web_sessions.sql</t>
         </is>
       </c>
       <c r="B218" s="2" t="inlineStr">
@@ -5231,7 +5231,7 @@
       </c>
       <c r="C218" s="3" t="inlineStr">
         <is>
-          <t>Phase 2 staging (web/app engagement): 1:1 pass-through of web_events</t>
+          <t>Phase 2 staging (web/app engagement): 1:1 pass-through of web_sessions, plus is_known_customer flag (customer_id null for ~79% of sessions by design)</t>
         </is>
       </c>
       <c r="D218" s="2" t="inlineStr">
@@ -5243,7 +5243,7 @@
     <row r="219">
       <c r="A219" s="2" t="inlineStr">
         <is>
-          <t>dbt/models/staging/kinetic/stg_kinetic__app_sessions.sql</t>
+          <t>dbt/models/staging/kinetic/stg_kinetic__web_events.sql</t>
         </is>
       </c>
       <c r="B219" s="2" t="inlineStr">
@@ -5253,7 +5253,7 @@
       </c>
       <c r="C219" s="3" t="inlineStr">
         <is>
-          <t>Phase 2 staging (web/app engagement): 1:1 pass-through of app_sessions</t>
+          <t>Phase 2 staging (web/app engagement): 1:1 pass-through of web_events</t>
         </is>
       </c>
       <c r="D219" s="2" t="inlineStr">
@@ -5265,7 +5265,7 @@
     <row r="220">
       <c r="A220" s="2" t="inlineStr">
         <is>
-          <t>dbt/models/staging/kinetic/stg_kinetic__app_events.sql</t>
+          <t>dbt/models/staging/kinetic/stg_kinetic__app_sessions.sql</t>
         </is>
       </c>
       <c r="B220" s="2" t="inlineStr">
@@ -5275,7 +5275,7 @@
       </c>
       <c r="C220" s="3" t="inlineStr">
         <is>
-          <t>Phase 2 staging (web/app engagement): 1:1 pass-through of app_events</t>
+          <t>Phase 2 staging (web/app engagement): 1:1 pass-through of app_sessions</t>
         </is>
       </c>
       <c r="D220" s="2" t="inlineStr">
@@ -5287,7 +5287,7 @@
     <row r="221">
       <c r="A221" s="2" t="inlineStr">
         <is>
-          <t>dbt/models/staging/kinetic/_kinetic__staging.yml</t>
+          <t>dbt/models/staging/kinetic/stg_kinetic__app_events.sql</t>
         </is>
       </c>
       <c r="B221" s="2" t="inlineStr">
@@ -5297,19 +5297,19 @@
       </c>
       <c r="C221" s="3" t="inlineStr">
         <is>
-          <t>Updated: tests for the 4 web/app engagement staging models -- all hand-verified against live data first</t>
+          <t>Phase 2 staging (web/app engagement): 1:1 pass-through of app_events</t>
         </is>
       </c>
       <c r="D221" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 16:49 PDT</t>
+          <t>2026-09-29 12:58 PDT</t>
         </is>
       </c>
     </row>
     <row r="222">
       <c r="A222" s="2" t="inlineStr">
         <is>
-          <t>dbt/models/staging/kinetic/stg_kinetic__braze_email_campaigns.sql</t>
+          <t>dbt/models/staging/kinetic/_kinetic__staging.yml</t>
         </is>
       </c>
       <c r="B222" s="2" t="inlineStr">
@@ -5319,19 +5319,19 @@
       </c>
       <c r="C222" s="3" t="inlineStr">
         <is>
-          <t>Phase 2 staging (email/push): 1:1 pass-through of braze_email_campaigns</t>
+          <t>Updated: tests for the 4 web/app engagement staging models -- all hand-verified against live data first</t>
         </is>
       </c>
       <c r="D222" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 12:59 PDT</t>
+          <t>2026-09-29 16:49 PDT</t>
         </is>
       </c>
     </row>
     <row r="223">
       <c r="A223" s="2" t="inlineStr">
         <is>
-          <t>dbt/models/staging/kinetic/stg_kinetic__braze_push_campaigns.sql</t>
+          <t>dbt/models/staging/kinetic/stg_kinetic__braze_email_campaigns.sql</t>
         </is>
       </c>
       <c r="B223" s="2" t="inlineStr">
@@ -5341,7 +5341,7 @@
       </c>
       <c r="C223" s="3" t="inlineStr">
         <is>
-          <t>Phase 2 staging (email/push): 1:1 pass-through of braze_push_campaigns</t>
+          <t>Phase 2 staging (email/push): 1:1 pass-through of braze_email_campaigns</t>
         </is>
       </c>
       <c r="D223" s="2" t="inlineStr">
@@ -5353,7 +5353,7 @@
     <row r="224">
       <c r="A224" s="2" t="inlineStr">
         <is>
-          <t>dbt/models/staging/kinetic/stg_kinetic__braze_email_events.sql</t>
+          <t>dbt/models/staging/kinetic/stg_kinetic__braze_push_campaigns.sql</t>
         </is>
       </c>
       <c r="B224" s="2" t="inlineStr">
@@ -5363,7 +5363,7 @@
       </c>
       <c r="C224" s="3" t="inlineStr">
         <is>
-          <t>Phase 2 staging (email/push): braze_email_events with external_user_id renamed to customer_id and a short event_name (send/open/click/bounce/unsubscribe) alongside Braze's raw event_type</t>
+          <t>Phase 2 staging (email/push): 1:1 pass-through of braze_push_campaigns</t>
         </is>
       </c>
       <c r="D224" s="2" t="inlineStr">
@@ -5375,7 +5375,7 @@
     <row r="225">
       <c r="A225" s="2" t="inlineStr">
         <is>
-          <t>dbt/models/staging/kinetic/stg_kinetic__braze_push_events.sql</t>
+          <t>dbt/models/staging/kinetic/stg_kinetic__braze_email_events.sql</t>
         </is>
       </c>
       <c r="B225" s="2" t="inlineStr">
@@ -5385,7 +5385,7 @@
       </c>
       <c r="C225" s="3" t="inlineStr">
         <is>
-          <t>Phase 2 staging (email/push): braze_push_events with external_user_id renamed to customer_id and a short event_name alongside Braze's raw event_type</t>
+          <t>Phase 2 staging (email/push): braze_email_events with external_user_id renamed to customer_id and a short event_name (send/open/click/bounce/unsubscribe) alongside Braze's raw event_type</t>
         </is>
       </c>
       <c r="D225" s="2" t="inlineStr">
@@ -5397,7 +5397,7 @@
     <row r="226">
       <c r="A226" s="2" t="inlineStr">
         <is>
-          <t>dbt/models/staging/kinetic/_kinetic__staging.yml</t>
+          <t>dbt/models/staging/kinetic/stg_kinetic__braze_push_events.sql</t>
         </is>
       </c>
       <c r="B226" s="2" t="inlineStr">
@@ -5407,19 +5407,19 @@
       </c>
       <c r="C226" s="3" t="inlineStr">
         <is>
-          <t>Updated: tests for the 4 Braze staging models, incl. accepted_values on event_name -- all hand-verified against live data first</t>
+          <t>Phase 2 staging (email/push): braze_push_events with external_user_id renamed to customer_id and a short event_name alongside Braze's raw event_type</t>
         </is>
       </c>
       <c r="D226" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 16:49 PDT</t>
+          <t>2026-09-29 12:59 PDT</t>
         </is>
       </c>
     </row>
     <row r="227">
       <c r="A227" s="2" t="inlineStr">
         <is>
-          <t>dbt/models/staging/kinetic/stg_kinetic__meta_campaigns.sql</t>
+          <t>dbt/models/staging/kinetic/_kinetic__staging.yml</t>
         </is>
       </c>
       <c r="B227" s="2" t="inlineStr">
@@ -5429,19 +5429,19 @@
       </c>
       <c r="C227" s="3" t="inlineStr">
         <is>
-          <t>Phase 2 staging (paid media: Meta): meta_campaigns with budgets in both raw cents and dollars (Meta API stores budgets in cents)</t>
+          <t>Updated: tests for the 4 Braze staging models, incl. accepted_values on event_name -- all hand-verified against live data first</t>
         </is>
       </c>
       <c r="D227" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 13:02 PDT</t>
+          <t>2026-09-29 16:49 PDT</t>
         </is>
       </c>
     </row>
     <row r="228">
       <c r="A228" s="2" t="inlineStr">
         <is>
-          <t>dbt/models/staging/kinetic/stg_kinetic__meta_ads.sql</t>
+          <t>dbt/models/staging/kinetic/stg_kinetic__meta_campaigns.sql</t>
         </is>
       </c>
       <c r="B228" s="2" t="inlineStr">
@@ -5451,7 +5451,7 @@
       </c>
       <c r="C228" s="3" t="inlineStr">
         <is>
-          <t>Phase 2 staging (paid media: Meta): 1:1 pass-through of meta_ads</t>
+          <t>Phase 2 staging (paid media: Meta): meta_campaigns with budgets in both raw cents and dollars (Meta API stores budgets in cents)</t>
         </is>
       </c>
       <c r="D228" s="2" t="inlineStr">
@@ -5463,7 +5463,7 @@
     <row r="229">
       <c r="A229" s="2" t="inlineStr">
         <is>
-          <t>dbt/models/staging/kinetic/stg_kinetic__meta_ad_insights_daily.sql</t>
+          <t>dbt/models/staging/kinetic/stg_kinetic__meta_ads.sql</t>
         </is>
       </c>
       <c r="B229" s="2" t="inlineStr">
@@ -5473,7 +5473,7 @@
       </c>
       <c r="C229" s="3" t="inlineStr">
         <is>
-          <t>Phase 2 staging (paid media: Meta): meta_ad_insights_daily with a combined ad_day_id key, unit-suffixed columns (spend_usd, cpm_usd, cpc_usd) and ctr renamed ctr_fraction (0.017 = 1.7%)</t>
+          <t>Phase 2 staging (paid media: Meta): 1:1 pass-through of meta_ads</t>
         </is>
       </c>
       <c r="D229" s="2" t="inlineStr">
@@ -5485,7 +5485,7 @@
     <row r="230">
       <c r="A230" s="2" t="inlineStr">
         <is>
-          <t>dbt/models/staging/kinetic/stg_kinetic__meta_ad_actions_daily.sql</t>
+          <t>dbt/models/staging/kinetic/stg_kinetic__meta_ad_insights_daily.sql</t>
         </is>
       </c>
       <c r="B230" s="2" t="inlineStr">
@@ -5495,7 +5495,7 @@
       </c>
       <c r="C230" s="3" t="inlineStr">
         <is>
-          <t>Phase 2 staging (paid media: Meta): meta_ad_actions_daily with a combined ad_day_action_id key; value renamed action_count</t>
+          <t>Phase 2 staging (paid media: Meta): meta_ad_insights_daily with a combined ad_day_id key, unit-suffixed columns (spend_usd, cpm_usd, cpc_usd) and ctr renamed ctr_fraction (0.017 = 1.7%)</t>
         </is>
       </c>
       <c r="D230" s="2" t="inlineStr">
@@ -5507,7 +5507,7 @@
     <row r="231">
       <c r="A231" s="2" t="inlineStr">
         <is>
-          <t>dbt/models/staging/kinetic/_kinetic__staging.yml</t>
+          <t>dbt/models/staging/kinetic/stg_kinetic__meta_ad_actions_daily.sql</t>
         </is>
       </c>
       <c r="B231" s="2" t="inlineStr">
@@ -5517,19 +5517,19 @@
       </c>
       <c r="C231" s="3" t="inlineStr">
         <is>
-          <t>Updated: tests for the 4 Meta staging models, incl. uniqueness of the combined daily keys -- all hand-verified against live data first</t>
+          <t>Phase 2 staging (paid media: Meta): meta_ad_actions_daily with a combined ad_day_action_id key; value renamed action_count</t>
         </is>
       </c>
       <c r="D231" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 16:49 PDT</t>
+          <t>2026-09-29 13:02 PDT</t>
         </is>
       </c>
     </row>
     <row r="232">
       <c r="A232" s="2" t="inlineStr">
         <is>
-          <t>dbt/models/staging/kinetic/stg_kinetic__google_search_campaigns.sql</t>
+          <t>dbt/models/staging/kinetic/_kinetic__staging.yml</t>
         </is>
       </c>
       <c r="B232" s="2" t="inlineStr">
@@ -5539,19 +5539,19 @@
       </c>
       <c r="C232" s="3" t="inlineStr">
         <is>
-          <t>Phase 2 staging (paid media: Google Search): campaigns with the raw customer_id renamed google_ads_account_id (it's the Google Ads account number, not a Kinetic customer), daily budget in micros and dollars, end_date cast back to a date</t>
+          <t>Updated: tests for the 4 Meta staging models, incl. uniqueness of the combined daily keys -- all hand-verified against live data first</t>
         </is>
       </c>
       <c r="D232" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 13:13 PDT</t>
+          <t>2026-09-29 16:49 PDT</t>
         </is>
       </c>
     </row>
     <row r="233">
       <c r="A233" s="2" t="inlineStr">
         <is>
-          <t>dbt/models/staging/kinetic/stg_kinetic__google_search_ad_groups.sql</t>
+          <t>dbt/models/staging/kinetic/stg_kinetic__google_search_campaigns.sql</t>
         </is>
       </c>
       <c r="B233" s="2" t="inlineStr">
@@ -5561,7 +5561,7 @@
       </c>
       <c r="C233" s="3" t="inlineStr">
         <is>
-          <t>Phase 2 staging (paid media: Google Search): ad groups; cpc_bid_micros cast back to a number (always empty -- automated bidding)</t>
+          <t>Phase 2 staging (paid media: Google Search): campaigns with the raw customer_id renamed google_ads_account_id (it's the Google Ads account number, not a Kinetic customer), daily budget in micros and dollars, end_date cast back to a date</t>
         </is>
       </c>
       <c r="D233" s="2" t="inlineStr">
@@ -5573,7 +5573,7 @@
     <row r="234">
       <c r="A234" s="2" t="inlineStr">
         <is>
-          <t>dbt/models/staging/kinetic/stg_kinetic__google_search_performance_daily.sql</t>
+          <t>dbt/models/staging/kinetic/stg_kinetic__google_search_ad_groups.sql</t>
         </is>
       </c>
       <c r="B234" s="2" t="inlineStr">
@@ -5583,7 +5583,7 @@
       </c>
       <c r="C234" s="3" t="inlineStr">
         <is>
-          <t>Phase 2 staging (paid media: Google Search): ad-group-day performance with combined ad_group_day_id key, cost converted from micros to dollars, ctr_fraction. The keyword table rolled up -- never add the two together</t>
+          <t>Phase 2 staging (paid media: Google Search): ad groups; cpc_bid_micros cast back to a number (always empty -- automated bidding)</t>
         </is>
       </c>
       <c r="D234" s="2" t="inlineStr">
@@ -5595,7 +5595,7 @@
     <row r="235">
       <c r="A235" s="2" t="inlineStr">
         <is>
-          <t>dbt/models/staging/kinetic/stg_kinetic__google_search_keyword_performance_daily.sql</t>
+          <t>dbt/models/staging/kinetic/stg_kinetic__google_search_performance_daily.sql</t>
         </is>
       </c>
       <c r="B235" s="2" t="inlineStr">
@@ -5605,7 +5605,7 @@
       </c>
       <c r="C235" s="3" t="inlineStr">
         <is>
-          <t>Phase 2 staging (paid media: Google Search): keyword-day performance with combined keyword_day_id key, cost converted from micros to dollars, ctr_fraction</t>
+          <t>Phase 2 staging (paid media: Google Search): ad-group-day performance with combined ad_group_day_id key, cost converted from micros to dollars, ctr_fraction. The keyword table rolled up -- never add the two together</t>
         </is>
       </c>
       <c r="D235" s="2" t="inlineStr">
@@ -5617,7 +5617,7 @@
     <row r="236">
       <c r="A236" s="2" t="inlineStr">
         <is>
-          <t>dbt/models/staging/kinetic/_kinetic__staging.yml</t>
+          <t>dbt/models/staging/kinetic/stg_kinetic__google_search_keyword_performance_daily.sql</t>
         </is>
       </c>
       <c r="B236" s="2" t="inlineStr">
@@ -5627,19 +5627,19 @@
       </c>
       <c r="C236" s="3" t="inlineStr">
         <is>
-          <t>Updated: tests for the 4 Google Search staging models -- all hand-verified against live data first</t>
+          <t>Phase 2 staging (paid media: Google Search): keyword-day performance with combined keyword_day_id key, cost converted from micros to dollars, ctr_fraction</t>
         </is>
       </c>
       <c r="D236" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 16:49 PDT</t>
+          <t>2026-09-29 13:13 PDT</t>
         </is>
       </c>
     </row>
     <row r="237">
       <c r="A237" s="2" t="inlineStr">
         <is>
-          <t>dbt/models/staging/kinetic/stg_kinetic__youtube_campaigns.sql</t>
+          <t>dbt/models/staging/kinetic/_kinetic__staging.yml</t>
         </is>
       </c>
       <c r="B237" s="2" t="inlineStr">
@@ -5649,19 +5649,19 @@
       </c>
       <c r="C237" s="3" t="inlineStr">
         <is>
-          <t>Phase 2 staging (paid media: YouTube): campaigns with customer_id renamed google_ads_account_id (the ad account, not a Kinetic customer), budgets in micros and dollars</t>
+          <t>Updated: tests for the 4 Google Search staging models -- all hand-verified against live data first</t>
         </is>
       </c>
       <c r="D237" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 13:14 PDT</t>
+          <t>2026-09-29 16:49 PDT</t>
         </is>
       </c>
     </row>
     <row r="238">
       <c r="A238" s="2" t="inlineStr">
         <is>
-          <t>dbt/models/staging/kinetic/stg_kinetic__youtube_ad_groups.sql</t>
+          <t>dbt/models/staging/kinetic/stg_kinetic__youtube_campaigns.sql</t>
         </is>
       </c>
       <c r="B238" s="2" t="inlineStr">
@@ -5671,7 +5671,7 @@
       </c>
       <c r="C238" s="3" t="inlineStr">
         <is>
-          <t>Phase 2 staging (paid media: YouTube): 1:1 pass-through of youtube_ad_groups</t>
+          <t>Phase 2 staging (paid media: YouTube): campaigns with customer_id renamed google_ads_account_id (the ad account, not a Kinetic customer), budgets in micros and dollars</t>
         </is>
       </c>
       <c r="D238" s="2" t="inlineStr">
@@ -5683,7 +5683,7 @@
     <row r="239">
       <c r="A239" s="2" t="inlineStr">
         <is>
-          <t>dbt/models/staging/kinetic/stg_kinetic__youtube_performance_daily.sql</t>
+          <t>dbt/models/staging/kinetic/stg_kinetic__youtube_ad_groups.sql</t>
         </is>
       </c>
       <c r="B239" s="2" t="inlineStr">
@@ -5693,7 +5693,7 @@
       </c>
       <c r="C239" s="3" t="inlineStr">
         <is>
-          <t>Phase 2 staging (paid media: YouTube): ad-group-day performance with combined ad_group_day_id key, cost and cost-per-view converted from micros to dollars, video_view_rate_fraction</t>
+          <t>Phase 2 staging (paid media: YouTube): 1:1 pass-through of youtube_ad_groups</t>
         </is>
       </c>
       <c r="D239" s="2" t="inlineStr">
@@ -5705,7 +5705,7 @@
     <row r="240">
       <c r="A240" s="2" t="inlineStr">
         <is>
-          <t>dbt/models/staging/kinetic/_kinetic__staging.yml</t>
+          <t>dbt/models/staging/kinetic/stg_kinetic__youtube_performance_daily.sql</t>
         </is>
       </c>
       <c r="B240" s="2" t="inlineStr">
@@ -5715,19 +5715,19 @@
       </c>
       <c r="C240" s="3" t="inlineStr">
         <is>
-          <t>Updated: tests for the 3 YouTube staging models -- all hand-verified against live data first</t>
+          <t>Phase 2 staging (paid media: YouTube): ad-group-day performance with combined ad_group_day_id key, cost and cost-per-view converted from micros to dollars, video_view_rate_fraction</t>
         </is>
       </c>
       <c r="D240" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 16:49 PDT</t>
+          <t>2026-09-29 13:14 PDT</t>
         </is>
       </c>
     </row>
     <row r="241">
       <c r="A241" s="2" t="inlineStr">
         <is>
-          <t>dbt/models/staging/kinetic/stg_kinetic__dv360_insertion_orders.sql</t>
+          <t>dbt/models/staging/kinetic/_kinetic__staging.yml</t>
         </is>
       </c>
       <c r="B241" s="2" t="inlineStr">
@@ -5737,19 +5737,19 @@
       </c>
       <c r="C241" s="3" t="inlineStr">
         <is>
-          <t>Phase 2 staging (paid media: DV360): insertion orders with budget_micros named monthly_budget_* (it's a monthly budget), end_date cast back to a date; flags the flat-budget-vs-growing-spend known issue</t>
+          <t>Updated: tests for the 3 YouTube staging models -- all hand-verified against live data first</t>
         </is>
       </c>
       <c r="D241" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 13:27 PDT</t>
+          <t>2026-09-29 16:49 PDT</t>
         </is>
       </c>
     </row>
     <row r="242">
       <c r="A242" s="2" t="inlineStr">
         <is>
-          <t>dbt/models/staging/kinetic/stg_kinetic__dv360_line_items.sql</t>
+          <t>dbt/models/staging/kinetic/stg_kinetic__dv360_insertion_orders.sql</t>
         </is>
       </c>
       <c r="B242" s="2" t="inlineStr">
@@ -5759,19 +5759,19 @@
       </c>
       <c r="C242" s="3" t="inlineStr">
         <is>
-          <t>Phase 2 staging (paid media: DV360): 1:1 pass-through of dv360_line_items</t>
+          <t>Phase 2 staging (paid media: DV360): insertion orders with budget_micros named monthly_budget_* (it's a monthly budget), end_date cast back to a date; flags the flat-budget-vs-growing-spend known issue</t>
         </is>
       </c>
       <c r="D242" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 13:19 PDT</t>
+          <t>2026-09-29 13:27 PDT</t>
         </is>
       </c>
     </row>
     <row r="243">
       <c r="A243" s="2" t="inlineStr">
         <is>
-          <t>dbt/models/staging/kinetic/stg_kinetic__dv360_performance_daily.sql</t>
+          <t>dbt/models/staging/kinetic/stg_kinetic__dv360_line_items.sql</t>
         </is>
       </c>
       <c r="B243" s="2" t="inlineStr">
@@ -5781,7 +5781,7 @@
       </c>
       <c r="C243" s="3" t="inlineStr">
         <is>
-          <t>Phase 2 staging (paid media: DV360): line-item x day x exchange x environment performance with combined line_item_day_slice_id key, micros converted to dollars, ctr_fraction</t>
+          <t>Phase 2 staging (paid media: DV360): 1:1 pass-through of dv360_line_items</t>
         </is>
       </c>
       <c r="D243" s="2" t="inlineStr">
@@ -5793,7 +5793,7 @@
     <row r="244">
       <c r="A244" s="2" t="inlineStr">
         <is>
-          <t>dbt/models/staging/kinetic/_kinetic__staging.yml</t>
+          <t>dbt/models/staging/kinetic/stg_kinetic__dv360_performance_daily.sql</t>
         </is>
       </c>
       <c r="B244" s="2" t="inlineStr">
@@ -5803,19 +5803,19 @@
       </c>
       <c r="C244" s="3" t="inlineStr">
         <is>
-          <t>Updated: tests for the 3 DV360 staging models, incl. accepted_values on exchange and environment -- all hand-verified against live data first</t>
+          <t>Phase 2 staging (paid media: DV360): line-item x day x exchange x environment performance with combined line_item_day_slice_id key, micros converted to dollars, ctr_fraction</t>
         </is>
       </c>
       <c r="D244" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 16:49 PDT</t>
+          <t>2026-09-29 13:19 PDT</t>
         </is>
       </c>
     </row>
     <row r="245">
       <c r="A245" s="2" t="inlineStr">
         <is>
-          <t>generator/params.py</t>
+          <t>dbt/models/staging/kinetic/_kinetic__staging.yml</t>
         </is>
       </c>
       <c r="B245" s="2" t="inlineStr">
@@ -5825,41 +5825,41 @@
       </c>
       <c r="C245" s="3" t="inlineStr">
         <is>
-          <t>Updated 2026-09-29: every evergreen ad budget on all 6 platforms is now the campaign's CURRENT budget, sized from realized spend (weekly average &lt;= budget, no day &gt; 1.75x; DV360 monthly &gt;= highest month). The old flat 'typical day' budgets let later months spend up to ~20x the stored budget</t>
+          <t>Updated: tests for the 3 DV360 staging models, incl. accepted_values on exchange and environment -- all hand-verified against live data first</t>
         </is>
       </c>
       <c r="D245" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 13:23 PDT</t>
+          <t>2026-09-29 16:49 PDT</t>
         </is>
       </c>
     </row>
     <row r="246">
       <c r="A246" s="2" t="inlineStr">
         <is>
-          <t>data/meta_campaigns.csv</t>
+          <t>generator/params.py</t>
         </is>
       </c>
       <c r="B246" s="2" t="inlineStr">
         <is>
-          <t>Shipped table</t>
+          <t>Code</t>
         </is>
       </c>
       <c r="C246" s="3" t="inlineStr">
         <is>
-          <t>Regenerated 2026-09-29: evergreen daily_budget values updated to current budgets (only that column, only the 4 evergreen rows changed)</t>
+          <t>Updated 2026-09-29: every evergreen ad budget on all 6 platforms is now the campaign's CURRENT budget, sized from realized spend (weekly average &lt;= budget, no day &gt; 1.75x; DV360 monthly &gt;= highest month). The old flat 'typical day' budgets let later months spend up to ~20x the stored budget</t>
         </is>
       </c>
       <c r="D246" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 13:24 PDT</t>
+          <t>2026-09-29 13:23 PDT</t>
         </is>
       </c>
     </row>
     <row r="247">
       <c r="A247" s="2" t="inlineStr">
         <is>
-          <t>data/google_search_campaigns.csv</t>
+          <t>data/meta_campaigns.csv</t>
         </is>
       </c>
       <c r="B247" s="2" t="inlineStr">
@@ -5869,7 +5869,7 @@
       </c>
       <c r="C247" s="3" t="inlineStr">
         <is>
-          <t>Regenerated 2026-09-29: campaign_budget_micros updated to current budgets (only that column changed)</t>
+          <t>Regenerated 2026-09-29: evergreen daily_budget values updated to current budgets (only that column, only the 4 evergreen rows changed)</t>
         </is>
       </c>
       <c r="D247" s="2" t="inlineStr">
@@ -5881,7 +5881,7 @@
     <row r="248">
       <c r="A248" s="2" t="inlineStr">
         <is>
-          <t>data/youtube_campaigns.csv</t>
+          <t>data/google_search_campaigns.csv</t>
         </is>
       </c>
       <c r="B248" s="2" t="inlineStr">
@@ -5891,7 +5891,7 @@
       </c>
       <c r="C248" s="3" t="inlineStr">
         <is>
-          <t>Regenerated 2026-09-29: evergreen campaign_budget_micros updated to current budgets (only that column, only the 4 evergreen rows changed)</t>
+          <t>Regenerated 2026-09-29: campaign_budget_micros updated to current budgets (only that column changed)</t>
         </is>
       </c>
       <c r="D248" s="2" t="inlineStr">
@@ -5903,7 +5903,7 @@
     <row r="249">
       <c r="A249" s="2" t="inlineStr">
         <is>
-          <t>data/dv360_insertion_orders.csv</t>
+          <t>data/youtube_campaigns.csv</t>
         </is>
       </c>
       <c r="B249" s="2" t="inlineStr">
@@ -5913,7 +5913,7 @@
       </c>
       <c r="C249" s="3" t="inlineStr">
         <is>
-          <t>Regenerated 2026-09-29: monthly budget_micros updated to current budgets (only that column changed)</t>
+          <t>Regenerated 2026-09-29: evergreen campaign_budget_micros updated to current budgets (only that column, only the 4 evergreen rows changed)</t>
         </is>
       </c>
       <c r="D249" s="2" t="inlineStr">
@@ -5925,7 +5925,7 @@
     <row r="250">
       <c r="A250" s="2" t="inlineStr">
         <is>
-          <t>data/snap_campaigns.csv</t>
+          <t>data/dv360_insertion_orders.csv</t>
         </is>
       </c>
       <c r="B250" s="2" t="inlineStr">
@@ -5935,7 +5935,7 @@
       </c>
       <c r="C250" s="3" t="inlineStr">
         <is>
-          <t>Regenerated 2026-09-29: evergreen daily_budget_micro updated to current budgets (only that column, only the 4 evergreen rows changed)</t>
+          <t>Regenerated 2026-09-29: monthly budget_micros updated to current budgets (only that column changed)</t>
         </is>
       </c>
       <c r="D250" s="2" t="inlineStr">
@@ -5947,7 +5947,7 @@
     <row r="251">
       <c r="A251" s="2" t="inlineStr">
         <is>
-          <t>data/tiktok_campaigns.csv</t>
+          <t>data/snap_campaigns.csv</t>
         </is>
       </c>
       <c r="B251" s="2" t="inlineStr">
@@ -5957,7 +5957,7 @@
       </c>
       <c r="C251" s="3" t="inlineStr">
         <is>
-          <t>Regenerated 2026-09-29: BUDGET_MODE_DAY budget_micro updated to current budgets (only that column, only the 4 evergreen rows changed)</t>
+          <t>Regenerated 2026-09-29: evergreen daily_budget_micro updated to current budgets (only that column, only the 4 evergreen rows changed)</t>
         </is>
       </c>
       <c r="D251" s="2" t="inlineStr">
@@ -5969,29 +5969,29 @@
     <row r="252">
       <c r="A252" s="2" t="inlineStr">
         <is>
-          <t>generator/audit_cross_dataset_alignment.py</t>
+          <t>data/tiktok_campaigns.csv</t>
         </is>
       </c>
       <c r="B252" s="2" t="inlineStr">
         <is>
-          <t>Code</t>
+          <t>Shipped table</t>
         </is>
       </c>
       <c r="C252" s="3" t="inlineStr">
         <is>
-          <t>Updated 2026-09-29: new Check 8 -- spend vs stored budget for every campaign on all 6 platforms (weekly/daily limits for daily budgets, monthly for DV360, total for holiday flights)</t>
+          <t>Regenerated 2026-09-29: BUDGET_MODE_DAY budget_micro updated to current budgets (only that column, only the 4 evergreen rows changed)</t>
         </is>
       </c>
       <c r="D252" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 13:30 PDT</t>
+          <t>2026-09-29 13:24 PDT</t>
         </is>
       </c>
     </row>
     <row r="253">
       <c r="A253" s="2" t="inlineStr">
         <is>
-          <t>dbt/models/staging/kinetic/stg_kinetic__dv360_insertion_orders.sql</t>
+          <t>generator/audit_cross_dataset_alignment.py</t>
         </is>
       </c>
       <c r="B253" s="2" t="inlineStr">
@@ -6001,19 +6001,19 @@
       </c>
       <c r="C253" s="3" t="inlineStr">
         <is>
-          <t>Updated: budget known-issue note replaced -- budgets are now current budgets</t>
+          <t>Updated 2026-09-29: new Check 8 -- spend vs stored budget for every campaign on all 6 platforms (weekly/daily limits for daily budgets, monthly for DV360, total for holiday flights)</t>
         </is>
       </c>
       <c r="D253" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 13:27 PDT</t>
+          <t>2026-09-29 13:30 PDT</t>
         </is>
       </c>
     </row>
     <row r="254">
       <c r="A254" s="2" t="inlineStr">
         <is>
-          <t>generator/paid_media_common.py</t>
+          <t>dbt/models/staging/kinetic/stg_kinetic__dv360_insertion_orders.sql</t>
         </is>
       </c>
       <c r="B254" s="2" t="inlineStr">
@@ -6023,19 +6023,19 @@
       </c>
       <c r="C254" s="3" t="inlineStr">
         <is>
-          <t>Updated 2026-09-29: new cap_flight_at_budget() -- rescales a holiday flight's days so it never spends past its lifetime budget, replaying the same random rates so every other row is unchanged</t>
+          <t>Updated: budget known-issue note replaced -- budgets are now current budgets</t>
         </is>
       </c>
       <c r="D254" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 13:29 PDT</t>
+          <t>2026-09-29 13:27 PDT</t>
         </is>
       </c>
     </row>
     <row r="255">
       <c r="A255" s="2" t="inlineStr">
         <is>
-          <t>generator/build_meta_ad_insights_daily.py</t>
+          <t>generator/paid_media_common.py</t>
         </is>
       </c>
       <c r="B255" s="2" t="inlineStr">
@@ -6045,7 +6045,7 @@
       </c>
       <c r="C255" s="3" t="inlineStr">
         <is>
-          <t>Updated 2026-09-29: holiday flights capped at their lifetime budget via cap_flight_at_budget()</t>
+          <t>Updated 2026-09-29: new cap_flight_at_budget() -- rescales a holiday flight's days so it never spends past its lifetime budget, replaying the same random rates so every other row is unchanged</t>
         </is>
       </c>
       <c r="D255" s="2" t="inlineStr">
@@ -6057,7 +6057,7 @@
     <row r="256">
       <c r="A256" s="2" t="inlineStr">
         <is>
-          <t>generator/build_snap_stats_daily.py</t>
+          <t>generator/build_meta_ad_insights_daily.py</t>
         </is>
       </c>
       <c r="B256" s="2" t="inlineStr">
@@ -6079,7 +6079,7 @@
     <row r="257">
       <c r="A257" s="2" t="inlineStr">
         <is>
-          <t>generator/build_tiktok_reports_daily.py</t>
+          <t>generator/build_snap_stats_daily.py</t>
         </is>
       </c>
       <c r="B257" s="2" t="inlineStr">
@@ -6101,7 +6101,7 @@
     <row r="258">
       <c r="A258" s="2" t="inlineStr">
         <is>
-          <t>generator/build_youtube_performance_daily.py</t>
+          <t>generator/build_tiktok_reports_daily.py</t>
         </is>
       </c>
       <c r="B258" s="2" t="inlineStr">
@@ -6111,7 +6111,7 @@
       </c>
       <c r="C258" s="3" t="inlineStr">
         <is>
-          <t>Updated 2026-09-29: holiday flights capped at their lifetime budget via cap_flight_at_budget() (no-op today -- all YouTube flights were already under budget)</t>
+          <t>Updated 2026-09-29: holiday flights capped at their lifetime budget via cap_flight_at_budget()</t>
         </is>
       </c>
       <c r="D258" s="2" t="inlineStr">
@@ -6123,17 +6123,17 @@
     <row r="259">
       <c r="A259" s="2" t="inlineStr">
         <is>
-          <t>data/meta_ad_insights_daily.csv</t>
+          <t>generator/build_youtube_performance_daily.py</t>
         </is>
       </c>
       <c r="B259" s="2" t="inlineStr">
         <is>
-          <t>Shipped table</t>
+          <t>Code</t>
         </is>
       </c>
       <c r="C259" s="3" t="inlineStr">
         <is>
-          <t>Regenerated 2026-09-29: the 2023 and 2024 holiday flights (38 rows) trimmed to spend exactly their lifetime budget; every other row identical</t>
+          <t>Updated 2026-09-29: holiday flights capped at their lifetime budget via cap_flight_at_budget() (no-op today -- all YouTube flights were already under budget)</t>
         </is>
       </c>
       <c r="D259" s="2" t="inlineStr">
@@ -6145,7 +6145,7 @@
     <row r="260">
       <c r="A260" s="2" t="inlineStr">
         <is>
-          <t>data/meta_ad_actions_daily.csv</t>
+          <t>data/meta_ad_insights_daily.csv</t>
         </is>
       </c>
       <c r="B260" s="2" t="inlineStr">
@@ -6155,7 +6155,7 @@
       </c>
       <c r="C260" s="3" t="inlineStr">
         <is>
-          <t>Regenerated 2026-09-29: re-derived from the trimmed insights rows -- only the 2023/2024 holiday flights' action rows changed (one initiate_checkout row on 2024-11-15 dropped to zero and is no longer emitted)</t>
+          <t>Regenerated 2026-09-29: the 2023 and 2024 holiday flights (38 rows) trimmed to spend exactly their lifetime budget; every other row identical</t>
         </is>
       </c>
       <c r="D260" s="2" t="inlineStr">
@@ -6167,7 +6167,7 @@
     <row r="261">
       <c r="A261" s="2" t="inlineStr">
         <is>
-          <t>data/snap_stats_daily.csv</t>
+          <t>data/meta_ad_actions_daily.csv</t>
         </is>
       </c>
       <c r="B261" s="2" t="inlineStr">
@@ -6177,7 +6177,7 @@
       </c>
       <c r="C261" s="3" t="inlineStr">
         <is>
-          <t>Regenerated 2026-09-29: the 2024 holiday flight (19 rows) trimmed to spend exactly its lifetime budget; every other row identical</t>
+          <t>Regenerated 2026-09-29: re-derived from the trimmed insights rows -- only the 2023/2024 holiday flights' action rows changed (one initiate_checkout row on 2024-11-15 dropped to zero and is no longer emitted)</t>
         </is>
       </c>
       <c r="D261" s="2" t="inlineStr">
@@ -6189,7 +6189,7 @@
     <row r="262">
       <c r="A262" s="2" t="inlineStr">
         <is>
-          <t>data/tiktok_reports_daily.csv</t>
+          <t>data/snap_stats_daily.csv</t>
         </is>
       </c>
       <c r="B262" s="2" t="inlineStr">
@@ -6199,7 +6199,7 @@
       </c>
       <c r="C262" s="3" t="inlineStr">
         <is>
-          <t>Regenerated 2026-09-29: the 2023/2024/2025 holiday flights (56 rows) trimmed to spend exactly their lifetime budgets; every other row identical</t>
+          <t>Regenerated 2026-09-29: the 2024 holiday flight (19 rows) trimmed to spend exactly its lifetime budget; every other row identical</t>
         </is>
       </c>
       <c r="D262" s="2" t="inlineStr">
@@ -6211,51 +6211,51 @@
     <row r="263">
       <c r="A263" s="2" t="inlineStr">
         <is>
-          <t>docs/cross_dataset_alignment_audit.md</t>
+          <t>data/tiktok_reports_daily.csv</t>
         </is>
       </c>
       <c r="B263" s="2" t="inlineStr">
         <is>
-          <t>Docs</t>
+          <t>Shipped table</t>
         </is>
       </c>
       <c r="C263" s="3" t="inlineStr">
         <is>
-          <t>Updated 2026-09-29: added Check 8 (spend vs stored budget) with both fixes and results</t>
+          <t>Regenerated 2026-09-29: the 2023/2024/2025 holiday flights (56 rows) trimmed to spend exactly their lifetime budgets; every other row identical</t>
         </is>
       </c>
       <c r="D263" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 13:54 PDT</t>
+          <t>2026-09-29 13:29 PDT</t>
         </is>
       </c>
     </row>
     <row r="264">
       <c r="A264" s="2" t="inlineStr">
         <is>
-          <t>generator/audit_cross_dataset_alignment.py</t>
+          <t>docs/cross_dataset_alignment_audit.md</t>
         </is>
       </c>
       <c r="B264" s="2" t="inlineStr">
         <is>
-          <t>Code</t>
+          <t>Docs</t>
         </is>
       </c>
       <c r="C264" s="3" t="inlineStr">
         <is>
-          <t>Updated 2026-09-29: Check 8's flight limit tightened from 1.05x to 1.0x now that flights are capped</t>
+          <t>Updated 2026-09-29: added Check 8 (spend vs stored budget) with both fixes and results</t>
         </is>
       </c>
       <c r="D264" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 13:30 PDT</t>
+          <t>2026-09-29 13:54 PDT</t>
         </is>
       </c>
     </row>
     <row r="265">
       <c r="A265" s="2" t="inlineStr">
         <is>
-          <t>dbt/models/staging/kinetic/stg_kinetic__snap_campaigns.sql</t>
+          <t>generator/audit_cross_dataset_alignment.py</t>
         </is>
       </c>
       <c r="B265" s="2" t="inlineStr">
@@ -6265,19 +6265,19 @@
       </c>
       <c r="C265" s="3" t="inlineStr">
         <is>
-          <t>Phase 2 staging (paid media: Snap): campaigns with ad_account_id renamed snap_ad_account_id, current budgets in micros and dollars</t>
+          <t>Updated 2026-09-29: Check 8's flight limit tightened from 1.05x to 1.0x now that flights are capped</t>
         </is>
       </c>
       <c r="D265" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 15:53 PDT</t>
+          <t>2026-09-29 13:30 PDT</t>
         </is>
       </c>
     </row>
     <row r="266">
       <c r="A266" s="2" t="inlineStr">
         <is>
-          <t>dbt/models/staging/kinetic/stg_kinetic__snap_ad_squads.sql</t>
+          <t>dbt/models/staging/kinetic/stg_kinetic__snap_campaigns.sql</t>
         </is>
       </c>
       <c r="B266" s="2" t="inlineStr">
@@ -6287,7 +6287,7 @@
       </c>
       <c r="C266" s="3" t="inlineStr">
         <is>
-          <t>Phase 2 staging (paid media: Snap): 1:1 pass-through of snap_ad_squads (Snap's ad set / ad group level)</t>
+          <t>Phase 2 staging (paid media: Snap): campaigns with ad_account_id renamed snap_ad_account_id, current budgets in micros and dollars</t>
         </is>
       </c>
       <c r="D266" s="2" t="inlineStr">
@@ -6299,7 +6299,7 @@
     <row r="267">
       <c r="A267" s="2" t="inlineStr">
         <is>
-          <t>dbt/models/staging/kinetic/stg_kinetic__snap_ads.sql</t>
+          <t>dbt/models/staging/kinetic/stg_kinetic__snap_ad_squads.sql</t>
         </is>
       </c>
       <c r="B267" s="2" t="inlineStr">
@@ -6309,7 +6309,7 @@
       </c>
       <c r="C267" s="3" t="inlineStr">
         <is>
-          <t>Phase 2 staging (paid media: Snap): 1:1 pass-through of snap_ads</t>
+          <t>Phase 2 staging (paid media: Snap): 1:1 pass-through of snap_ad_squads (Snap's ad set / ad group level)</t>
         </is>
       </c>
       <c r="D267" s="2" t="inlineStr">
@@ -6321,7 +6321,7 @@
     <row r="268">
       <c r="A268" s="2" t="inlineStr">
         <is>
-          <t>dbt/models/staging/kinetic/stg_kinetic__snap_stats_daily.sql</t>
+          <t>dbt/models/staging/kinetic/stg_kinetic__snap_ads.sql</t>
         </is>
       </c>
       <c r="B268" s="2" t="inlineStr">
@@ -6331,7 +6331,7 @@
       </c>
       <c r="C268" s="3" t="inlineStr">
         <is>
-          <t>Phase 2 staging (paid media: Snap): ad-day stats with combined ad_day_id key, spend in micros and dollars; documents swipes as Snap's clicks</t>
+          <t>Phase 2 staging (paid media: Snap): 1:1 pass-through of snap_ads</t>
         </is>
       </c>
       <c r="D268" s="2" t="inlineStr">
@@ -6343,7 +6343,7 @@
     <row r="269">
       <c r="A269" s="2" t="inlineStr">
         <is>
-          <t>dbt/models/staging/kinetic/_kinetic__staging.yml</t>
+          <t>dbt/models/staging/kinetic/stg_kinetic__snap_stats_daily.sql</t>
         </is>
       </c>
       <c r="B269" s="2" t="inlineStr">
@@ -6353,19 +6353,19 @@
       </c>
       <c r="C269" s="3" t="inlineStr">
         <is>
-          <t>Updated: tests for the 4 Snap staging models -- all hand-verified against live data first</t>
+          <t>Phase 2 staging (paid media: Snap): ad-day stats with combined ad_day_id key, spend in micros and dollars; documents swipes as Snap's clicks</t>
         </is>
       </c>
       <c r="D269" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 16:49 PDT</t>
+          <t>2026-09-29 15:53 PDT</t>
         </is>
       </c>
     </row>
     <row r="270">
       <c r="A270" s="2" t="inlineStr">
         <is>
-          <t>dbt/models/staging/kinetic/stg_kinetic__tiktok_campaigns.sql</t>
+          <t>dbt/models/staging/kinetic/_kinetic__staging.yml</t>
         </is>
       </c>
       <c r="B270" s="2" t="inlineStr">
@@ -6375,19 +6375,19 @@
       </c>
       <c r="C270" s="3" t="inlineStr">
         <is>
-          <t>Phase 2 staging (paid media: TikTok): campaigns with the single budget split into daily_budget_usd / lifetime_budget_usd by budget_mode (matching the other platforms), advertiser_id renamed tiktok_advertiser_id</t>
+          <t>Updated: tests for the 4 Snap staging models -- all hand-verified against live data first</t>
         </is>
       </c>
       <c r="D270" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 15:57 PDT</t>
+          <t>2026-09-29 16:49 PDT</t>
         </is>
       </c>
     </row>
     <row r="271">
       <c r="A271" s="2" t="inlineStr">
         <is>
-          <t>dbt/models/staging/kinetic/stg_kinetic__tiktok_adgroups.sql</t>
+          <t>dbt/models/staging/kinetic/stg_kinetic__tiktok_campaigns.sql</t>
         </is>
       </c>
       <c r="B271" s="2" t="inlineStr">
@@ -6397,7 +6397,7 @@
       </c>
       <c r="C271" s="3" t="inlineStr">
         <is>
-          <t>Phase 2 staging (paid media: TikTok): 1:1 pass-through of tiktok_adgroups</t>
+          <t>Phase 2 staging (paid media: TikTok): campaigns with the single budget split into daily_budget_usd / lifetime_budget_usd by budget_mode (matching the other platforms), advertiser_id renamed tiktok_advertiser_id</t>
         </is>
       </c>
       <c r="D271" s="2" t="inlineStr">
@@ -6409,7 +6409,7 @@
     <row r="272">
       <c r="A272" s="2" t="inlineStr">
         <is>
-          <t>dbt/models/staging/kinetic/stg_kinetic__tiktok_ads.sql</t>
+          <t>dbt/models/staging/kinetic/stg_kinetic__tiktok_adgroups.sql</t>
         </is>
       </c>
       <c r="B272" s="2" t="inlineStr">
@@ -6419,7 +6419,7 @@
       </c>
       <c r="C272" s="3" t="inlineStr">
         <is>
-          <t>Phase 2 staging (paid media: TikTok): 1:1 pass-through of tiktok_ads</t>
+          <t>Phase 2 staging (paid media: TikTok): 1:1 pass-through of tiktok_adgroups</t>
         </is>
       </c>
       <c r="D272" s="2" t="inlineStr">
@@ -6431,7 +6431,7 @@
     <row r="273">
       <c r="A273" s="2" t="inlineStr">
         <is>
-          <t>dbt/models/staging/kinetic/stg_kinetic__tiktok_reports_daily.sql</t>
+          <t>dbt/models/staging/kinetic/stg_kinetic__tiktok_ads.sql</t>
         </is>
       </c>
       <c r="B273" s="2" t="inlineStr">
@@ -6441,7 +6441,7 @@
       </c>
       <c r="C273" s="3" t="inlineStr">
         <is>
-          <t>Phase 2 staging (paid media: TikTok): ad-day reports with combined ad_day_id key, spend and CPM in micros and dollars, ctr_fraction</t>
+          <t>Phase 2 staging (paid media: TikTok): 1:1 pass-through of tiktok_ads</t>
         </is>
       </c>
       <c r="D273" s="2" t="inlineStr">
@@ -6453,7 +6453,7 @@
     <row r="274">
       <c r="A274" s="2" t="inlineStr">
         <is>
-          <t>dbt/models/staging/kinetic/stg_kinetic__product_variants.sql</t>
+          <t>dbt/models/staging/kinetic/stg_kinetic__tiktok_reports_daily.sql</t>
         </is>
       </c>
       <c r="B274" s="2" t="inlineStr">
@@ -6463,54 +6463,76 @@
       </c>
       <c r="C274" s="3" t="inlineStr">
         <is>
-          <t>Phase 2 staging (final table, 47 of 47): product variants with variant_option, price_adjustment_usd</t>
+          <t>Phase 2 staging (paid media: TikTok): ad-day reports with combined ad_day_id key, spend and CPM in micros and dollars, ctr_fraction</t>
         </is>
       </c>
       <c r="D274" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 16:08 PDT</t>
+          <t>2026-09-29 15:57 PDT</t>
         </is>
       </c>
     </row>
     <row r="275">
       <c r="A275" s="2" t="inlineStr">
         <is>
-          <t>HANDOFF.md</t>
+          <t>dbt/models/staging/kinetic/stg_kinetic__product_variants.sql</t>
         </is>
       </c>
       <c r="B275" s="2" t="inlineStr">
         <is>
-          <t>Doc</t>
+          <t>Code</t>
         </is>
       </c>
       <c r="C275" s="3" t="inlineStr">
         <is>
-          <t>Handoff note for starting a new chat/project: status, open decisions, prior decisions, pitfalls</t>
+          <t>Phase 2 staging (final table, 47 of 47): product variants with variant_option, price_adjustment_usd</t>
         </is>
       </c>
       <c r="D275" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 17:20 PDT</t>
+          <t>2026-09-29 16:08 PDT</t>
         </is>
       </c>
     </row>
     <row r="276">
       <c r="A276" s="2" t="inlineStr">
         <is>
+          <t>HANDOFF.md</t>
+        </is>
+      </c>
+      <c r="B276" s="2" t="inlineStr">
+        <is>
+          <t>Doc</t>
+        </is>
+      </c>
+      <c r="C276" s="3" t="inlineStr">
+        <is>
+          <t>Handoff note for starting a new chat/project: status, open decisions, prior decisions, pitfalls</t>
+        </is>
+      </c>
+      <c r="D276" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-29 17:25 PDT</t>
+        </is>
+      </c>
+    </row>
+    <row r="277">
+      <c r="A277" s="2" t="inlineStr">
+        <is>
           <t>dbt/models/staging/kinetic/_kinetic__staging.yml</t>
         </is>
       </c>
-      <c r="B276" s="2" t="inlineStr">
-        <is>
-          <t>Code</t>
-        </is>
-      </c>
-      <c r="C276" s="3" t="inlineStr">
+      <c r="B277" s="2" t="inlineStr">
+        <is>
+          <t>Code</t>
+        </is>
+      </c>
+      <c r="C277" s="3" t="inlineStr">
         <is>
           <t>Updated: tests for the 4 TikTok staging models -- all hand-verified against live data first</t>
         </is>
       </c>
-      <c r="D276" s="2" t="inlineStr">
+      <c r="D277" s="2" t="inlineStr">
         <is>
           <t>2026-09-29 16:49 PDT</t>
         </is>

</xml_diff>

<commit_message>
Add Claude Code setup: CLAUDE.md, permissions, overnight plan variant
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012MSGmVw4D6TxU8u8LSeA2e
</commit_message>
<xml_diff>
--- a/File_Manifest.xlsx
+++ b/File_Manifest.xlsx
@@ -435,7 +435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D277"/>
+  <dimension ref="A1:D280"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="48" customWidth="1" min="1" max="1"/>
@@ -506,7 +506,7 @@
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 17:25 PDT</t>
+          <t>2026-09-29 18:25 PDT</t>
         </is>
       </c>
     </row>
@@ -638,7 +638,7 @@
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 18:17 PDT</t>
+          <t>2026-09-29 18:55 PDT</t>
         </is>
       </c>
     </row>
@@ -748,7 +748,7 @@
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 18:17 PDT</t>
+          <t>2026-09-29 18:55 PDT</t>
         </is>
       </c>
     </row>
@@ -5038,80 +5038,80 @@
       </c>
       <c r="D209" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 18:17 PDT</t>
+          <t>2026-09-29 18:25 PDT</t>
         </is>
       </c>
     </row>
     <row r="210">
       <c r="A210" s="2" t="inlineStr">
         <is>
-          <t>dbt/models/marts/mart_storefront_revenue_monthly.sql</t>
+          <t>OVERNIGHT_PLAN_CLAUDE_CODE.md</t>
         </is>
       </c>
       <c r="B210" s="2" t="inlineStr">
         <is>
-          <t>Code</t>
+          <t>Doc</t>
         </is>
       </c>
       <c r="C210" s="3" t="inlineStr">
         <is>
-          <t>Second canonical metric mart: non-subscription (course+merch) gross/net revenue, AOV, guest-checkout share, discount-usage share, refund rate by month -- validated against a hand-run equivalent query on the live database (2026-07: 246 orders, $13,843.71 gross revenue, $56.28 AOV)</t>
+          <t>Overnight runbook variant for Claude Code: dbt builds and branch pushes allowed</t>
         </is>
       </c>
       <c r="D210" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28 14:53 PDT</t>
+          <t>2026-09-29 18:55 PDT</t>
         </is>
       </c>
     </row>
     <row r="211">
       <c r="A211" s="2" t="inlineStr">
         <is>
-          <t>dbt/models/staging/kinetic/stg_kinetic__customer_addresses.sql</t>
+          <t>CLAUDE.md</t>
         </is>
       </c>
       <c r="B211" s="2" t="inlineStr">
         <is>
-          <t>Code</t>
+          <t>Doc</t>
         </is>
       </c>
       <c r="C211" s="3" t="inlineStr">
         <is>
-          <t>Phase 2 staging (Customer 360): 1:1 pass-through of customer_addresses</t>
+          <t>Claude Code project instructions: standing rules, dbt/git/MotherDuck limits, start-of-session reading</t>
         </is>
       </c>
       <c r="D211" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 10:26 PDT</t>
+          <t>2026-09-29 18:55 PDT</t>
         </is>
       </c>
     </row>
     <row r="212">
       <c r="A212" s="2" t="inlineStr">
         <is>
-          <t>dbt/models/staging/kinetic/stg_kinetic__devices.sql</t>
+          <t>.claude/settings.json</t>
         </is>
       </c>
       <c r="B212" s="2" t="inlineStr">
         <is>
-          <t>Code</t>
+          <t>Config</t>
         </is>
       </c>
       <c r="C212" s="3" t="inlineStr">
         <is>
-          <t>Phase 2 staging (Customer 360): 1:1 pass-through of devices, plus is_anonymous_device flag (customer_id null for ~94% of devices by design)</t>
+          <t>Claude Code permissions: allow dbt/git commit/push overnight branch; deny push to master, force push, rm</t>
         </is>
       </c>
       <c r="D212" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 10:26 PDT</t>
+          <t>2026-09-29 18:55 PDT</t>
         </is>
       </c>
     </row>
     <row r="213">
       <c r="A213" s="2" t="inlineStr">
         <is>
-          <t>dbt/models/staging/kinetic/stg_kinetic__identity_map.sql</t>
+          <t>dbt/models/marts/mart_storefront_revenue_monthly.sql</t>
         </is>
       </c>
       <c r="B213" s="2" t="inlineStr">
@@ -5121,19 +5121,19 @@
       </c>
       <c r="C213" s="3" t="inlineStr">
         <is>
-          <t>Phase 2 staging (Customer 360): 1:1 pass-through of identity_map</t>
+          <t>Second canonical metric mart: non-subscription (course+merch) gross/net revenue, AOV, guest-checkout share, discount-usage share, refund rate by month -- validated against a hand-run equivalent query on the live database (2026-07: 246 orders, $13,843.71 gross revenue, $56.28 AOV)</t>
         </is>
       </c>
       <c r="D213" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 10:26 PDT</t>
+          <t>2026-09-28 14:53 PDT</t>
         </is>
       </c>
     </row>
     <row r="214">
       <c r="A214" s="2" t="inlineStr">
         <is>
-          <t>dbt/models/staging/kinetic/stg_kinetic__segments.sql</t>
+          <t>dbt/models/staging/kinetic/stg_kinetic__customer_addresses.sql</t>
         </is>
       </c>
       <c r="B214" s="2" t="inlineStr">
@@ -5143,7 +5143,7 @@
       </c>
       <c r="C214" s="3" t="inlineStr">
         <is>
-          <t>Phase 2 staging (Customer 360): 1:1 pass-through of segments</t>
+          <t>Phase 2 staging (Customer 360): 1:1 pass-through of customer_addresses</t>
         </is>
       </c>
       <c r="D214" s="2" t="inlineStr">
@@ -5155,7 +5155,7 @@
     <row r="215">
       <c r="A215" s="2" t="inlineStr">
         <is>
-          <t>dbt/models/staging/kinetic/stg_kinetic__customer_segment_membership.sql</t>
+          <t>dbt/models/staging/kinetic/stg_kinetic__devices.sql</t>
         </is>
       </c>
       <c r="B215" s="2" t="inlineStr">
@@ -5165,7 +5165,7 @@
       </c>
       <c r="C215" s="3" t="inlineStr">
         <is>
-          <t>Phase 2 staging (Customer 360): 1:1 pass-through of customer_segment_membership, plus is_current_member flag</t>
+          <t>Phase 2 staging (Customer 360): 1:1 pass-through of devices, plus is_anonymous_device flag (customer_id null for ~94% of devices by design)</t>
         </is>
       </c>
       <c r="D215" s="2" t="inlineStr">
@@ -5177,7 +5177,7 @@
     <row r="216">
       <c r="A216" s="2" t="inlineStr">
         <is>
-          <t>dbt/models/staging/kinetic/stg_kinetic__subscription_events.sql</t>
+          <t>dbt/models/staging/kinetic/stg_kinetic__identity_map.sql</t>
         </is>
       </c>
       <c r="B216" s="2" t="inlineStr">
@@ -5187,7 +5187,7 @@
       </c>
       <c r="C216" s="3" t="inlineStr">
         <is>
-          <t>Phase 2 staging (Customer 360): 1:1 pass-through of subscription_events; old_plan/new_plan renamed to old_plan_id/new_plan_id</t>
+          <t>Phase 2 staging (Customer 360): 1:1 pass-through of identity_map</t>
         </is>
       </c>
       <c r="D216" s="2" t="inlineStr">
@@ -5199,7 +5199,7 @@
     <row r="217">
       <c r="A217" s="2" t="inlineStr">
         <is>
-          <t>dbt/models/staging/kinetic/_kinetic__staging.yml</t>
+          <t>dbt/models/staging/kinetic/stg_kinetic__segments.sql</t>
         </is>
       </c>
       <c r="B217" s="2" t="inlineStr">
@@ -5209,19 +5209,19 @@
       </c>
       <c r="C217" s="3" t="inlineStr">
         <is>
-          <t>Updated: tests for the 6 Customer 360 staging models (PK not_null/unique, FK relationships) -- all hand-verified against live data first</t>
+          <t>Phase 2 staging (Customer 360): 1:1 pass-through of segments</t>
         </is>
       </c>
       <c r="D217" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 16:49 PDT</t>
+          <t>2026-09-29 10:26 PDT</t>
         </is>
       </c>
     </row>
     <row r="218">
       <c r="A218" s="2" t="inlineStr">
         <is>
-          <t>dbt/models/staging/kinetic/stg_kinetic__web_sessions.sql</t>
+          <t>dbt/models/staging/kinetic/stg_kinetic__customer_segment_membership.sql</t>
         </is>
       </c>
       <c r="B218" s="2" t="inlineStr">
@@ -5231,19 +5231,19 @@
       </c>
       <c r="C218" s="3" t="inlineStr">
         <is>
-          <t>Phase 2 staging (web/app engagement): 1:1 pass-through of web_sessions, plus is_known_customer flag (customer_id null for ~79% of sessions by design)</t>
+          <t>Phase 2 staging (Customer 360): 1:1 pass-through of customer_segment_membership, plus is_current_member flag</t>
         </is>
       </c>
       <c r="D218" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 12:58 PDT</t>
+          <t>2026-09-29 10:26 PDT</t>
         </is>
       </c>
     </row>
     <row r="219">
       <c r="A219" s="2" t="inlineStr">
         <is>
-          <t>dbt/models/staging/kinetic/stg_kinetic__web_events.sql</t>
+          <t>dbt/models/staging/kinetic/stg_kinetic__subscription_events.sql</t>
         </is>
       </c>
       <c r="B219" s="2" t="inlineStr">
@@ -5253,19 +5253,19 @@
       </c>
       <c r="C219" s="3" t="inlineStr">
         <is>
-          <t>Phase 2 staging (web/app engagement): 1:1 pass-through of web_events</t>
+          <t>Phase 2 staging (Customer 360): 1:1 pass-through of subscription_events; old_plan/new_plan renamed to old_plan_id/new_plan_id</t>
         </is>
       </c>
       <c r="D219" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 12:58 PDT</t>
+          <t>2026-09-29 10:26 PDT</t>
         </is>
       </c>
     </row>
     <row r="220">
       <c r="A220" s="2" t="inlineStr">
         <is>
-          <t>dbt/models/staging/kinetic/stg_kinetic__app_sessions.sql</t>
+          <t>dbt/models/staging/kinetic/_kinetic__staging.yml</t>
         </is>
       </c>
       <c r="B220" s="2" t="inlineStr">
@@ -5275,19 +5275,19 @@
       </c>
       <c r="C220" s="3" t="inlineStr">
         <is>
-          <t>Phase 2 staging (web/app engagement): 1:1 pass-through of app_sessions</t>
+          <t>Updated: tests for the 6 Customer 360 staging models (PK not_null/unique, FK relationships) -- all hand-verified against live data first</t>
         </is>
       </c>
       <c r="D220" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 12:58 PDT</t>
+          <t>2026-09-29 16:49 PDT</t>
         </is>
       </c>
     </row>
     <row r="221">
       <c r="A221" s="2" t="inlineStr">
         <is>
-          <t>dbt/models/staging/kinetic/stg_kinetic__app_events.sql</t>
+          <t>dbt/models/staging/kinetic/stg_kinetic__web_sessions.sql</t>
         </is>
       </c>
       <c r="B221" s="2" t="inlineStr">
@@ -5297,7 +5297,7 @@
       </c>
       <c r="C221" s="3" t="inlineStr">
         <is>
-          <t>Phase 2 staging (web/app engagement): 1:1 pass-through of app_events</t>
+          <t>Phase 2 staging (web/app engagement): 1:1 pass-through of web_sessions, plus is_known_customer flag (customer_id null for ~79% of sessions by design)</t>
         </is>
       </c>
       <c r="D221" s="2" t="inlineStr">
@@ -5309,7 +5309,7 @@
     <row r="222">
       <c r="A222" s="2" t="inlineStr">
         <is>
-          <t>dbt/models/staging/kinetic/_kinetic__staging.yml</t>
+          <t>dbt/models/staging/kinetic/stg_kinetic__web_events.sql</t>
         </is>
       </c>
       <c r="B222" s="2" t="inlineStr">
@@ -5319,19 +5319,19 @@
       </c>
       <c r="C222" s="3" t="inlineStr">
         <is>
-          <t>Updated: tests for the 4 web/app engagement staging models -- all hand-verified against live data first</t>
+          <t>Phase 2 staging (web/app engagement): 1:1 pass-through of web_events</t>
         </is>
       </c>
       <c r="D222" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 16:49 PDT</t>
+          <t>2026-09-29 12:58 PDT</t>
         </is>
       </c>
     </row>
     <row r="223">
       <c r="A223" s="2" t="inlineStr">
         <is>
-          <t>dbt/models/staging/kinetic/stg_kinetic__braze_email_campaigns.sql</t>
+          <t>dbt/models/staging/kinetic/stg_kinetic__app_sessions.sql</t>
         </is>
       </c>
       <c r="B223" s="2" t="inlineStr">
@@ -5341,19 +5341,19 @@
       </c>
       <c r="C223" s="3" t="inlineStr">
         <is>
-          <t>Phase 2 staging (email/push): 1:1 pass-through of braze_email_campaigns</t>
+          <t>Phase 2 staging (web/app engagement): 1:1 pass-through of app_sessions</t>
         </is>
       </c>
       <c r="D223" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 12:59 PDT</t>
+          <t>2026-09-29 12:58 PDT</t>
         </is>
       </c>
     </row>
     <row r="224">
       <c r="A224" s="2" t="inlineStr">
         <is>
-          <t>dbt/models/staging/kinetic/stg_kinetic__braze_push_campaigns.sql</t>
+          <t>dbt/models/staging/kinetic/stg_kinetic__app_events.sql</t>
         </is>
       </c>
       <c r="B224" s="2" t="inlineStr">
@@ -5363,19 +5363,19 @@
       </c>
       <c r="C224" s="3" t="inlineStr">
         <is>
-          <t>Phase 2 staging (email/push): 1:1 pass-through of braze_push_campaigns</t>
+          <t>Phase 2 staging (web/app engagement): 1:1 pass-through of app_events</t>
         </is>
       </c>
       <c r="D224" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 12:59 PDT</t>
+          <t>2026-09-29 12:58 PDT</t>
         </is>
       </c>
     </row>
     <row r="225">
       <c r="A225" s="2" t="inlineStr">
         <is>
-          <t>dbt/models/staging/kinetic/stg_kinetic__braze_email_events.sql</t>
+          <t>dbt/models/staging/kinetic/_kinetic__staging.yml</t>
         </is>
       </c>
       <c r="B225" s="2" t="inlineStr">
@@ -5385,19 +5385,19 @@
       </c>
       <c r="C225" s="3" t="inlineStr">
         <is>
-          <t>Phase 2 staging (email/push): braze_email_events with external_user_id renamed to customer_id and a short event_name (send/open/click/bounce/unsubscribe) alongside Braze's raw event_type</t>
+          <t>Updated: tests for the 4 web/app engagement staging models -- all hand-verified against live data first</t>
         </is>
       </c>
       <c r="D225" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 12:59 PDT</t>
+          <t>2026-09-29 16:49 PDT</t>
         </is>
       </c>
     </row>
     <row r="226">
       <c r="A226" s="2" t="inlineStr">
         <is>
-          <t>dbt/models/staging/kinetic/stg_kinetic__braze_push_events.sql</t>
+          <t>dbt/models/staging/kinetic/stg_kinetic__braze_email_campaigns.sql</t>
         </is>
       </c>
       <c r="B226" s="2" t="inlineStr">
@@ -5407,7 +5407,7 @@
       </c>
       <c r="C226" s="3" t="inlineStr">
         <is>
-          <t>Phase 2 staging (email/push): braze_push_events with external_user_id renamed to customer_id and a short event_name alongside Braze's raw event_type</t>
+          <t>Phase 2 staging (email/push): 1:1 pass-through of braze_email_campaigns</t>
         </is>
       </c>
       <c r="D226" s="2" t="inlineStr">
@@ -5419,7 +5419,7 @@
     <row r="227">
       <c r="A227" s="2" t="inlineStr">
         <is>
-          <t>dbt/models/staging/kinetic/_kinetic__staging.yml</t>
+          <t>dbt/models/staging/kinetic/stg_kinetic__braze_push_campaigns.sql</t>
         </is>
       </c>
       <c r="B227" s="2" t="inlineStr">
@@ -5429,19 +5429,19 @@
       </c>
       <c r="C227" s="3" t="inlineStr">
         <is>
-          <t>Updated: tests for the 4 Braze staging models, incl. accepted_values on event_name -- all hand-verified against live data first</t>
+          <t>Phase 2 staging (email/push): 1:1 pass-through of braze_push_campaigns</t>
         </is>
       </c>
       <c r="D227" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 16:49 PDT</t>
+          <t>2026-09-29 12:59 PDT</t>
         </is>
       </c>
     </row>
     <row r="228">
       <c r="A228" s="2" t="inlineStr">
         <is>
-          <t>dbt/models/staging/kinetic/stg_kinetic__meta_campaigns.sql</t>
+          <t>dbt/models/staging/kinetic/stg_kinetic__braze_email_events.sql</t>
         </is>
       </c>
       <c r="B228" s="2" t="inlineStr">
@@ -5451,19 +5451,19 @@
       </c>
       <c r="C228" s="3" t="inlineStr">
         <is>
-          <t>Phase 2 staging (paid media: Meta): meta_campaigns with budgets in both raw cents and dollars (Meta API stores budgets in cents)</t>
+          <t>Phase 2 staging (email/push): braze_email_events with external_user_id renamed to customer_id and a short event_name (send/open/click/bounce/unsubscribe) alongside Braze's raw event_type</t>
         </is>
       </c>
       <c r="D228" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 13:02 PDT</t>
+          <t>2026-09-29 12:59 PDT</t>
         </is>
       </c>
     </row>
     <row r="229">
       <c r="A229" s="2" t="inlineStr">
         <is>
-          <t>dbt/models/staging/kinetic/stg_kinetic__meta_ads.sql</t>
+          <t>dbt/models/staging/kinetic/stg_kinetic__braze_push_events.sql</t>
         </is>
       </c>
       <c r="B229" s="2" t="inlineStr">
@@ -5473,19 +5473,19 @@
       </c>
       <c r="C229" s="3" t="inlineStr">
         <is>
-          <t>Phase 2 staging (paid media: Meta): 1:1 pass-through of meta_ads</t>
+          <t>Phase 2 staging (email/push): braze_push_events with external_user_id renamed to customer_id and a short event_name alongside Braze's raw event_type</t>
         </is>
       </c>
       <c r="D229" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 13:02 PDT</t>
+          <t>2026-09-29 12:59 PDT</t>
         </is>
       </c>
     </row>
     <row r="230">
       <c r="A230" s="2" t="inlineStr">
         <is>
-          <t>dbt/models/staging/kinetic/stg_kinetic__meta_ad_insights_daily.sql</t>
+          <t>dbt/models/staging/kinetic/_kinetic__staging.yml</t>
         </is>
       </c>
       <c r="B230" s="2" t="inlineStr">
@@ -5495,19 +5495,19 @@
       </c>
       <c r="C230" s="3" t="inlineStr">
         <is>
-          <t>Phase 2 staging (paid media: Meta): meta_ad_insights_daily with a combined ad_day_id key, unit-suffixed columns (spend_usd, cpm_usd, cpc_usd) and ctr renamed ctr_fraction (0.017 = 1.7%)</t>
+          <t>Updated: tests for the 4 Braze staging models, incl. accepted_values on event_name -- all hand-verified against live data first</t>
         </is>
       </c>
       <c r="D230" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 13:02 PDT</t>
+          <t>2026-09-29 16:49 PDT</t>
         </is>
       </c>
     </row>
     <row r="231">
       <c r="A231" s="2" t="inlineStr">
         <is>
-          <t>dbt/models/staging/kinetic/stg_kinetic__meta_ad_actions_daily.sql</t>
+          <t>dbt/models/staging/kinetic/stg_kinetic__meta_campaigns.sql</t>
         </is>
       </c>
       <c r="B231" s="2" t="inlineStr">
@@ -5517,7 +5517,7 @@
       </c>
       <c r="C231" s="3" t="inlineStr">
         <is>
-          <t>Phase 2 staging (paid media: Meta): meta_ad_actions_daily with a combined ad_day_action_id key; value renamed action_count</t>
+          <t>Phase 2 staging (paid media: Meta): meta_campaigns with budgets in both raw cents and dollars (Meta API stores budgets in cents)</t>
         </is>
       </c>
       <c r="D231" s="2" t="inlineStr">
@@ -5529,7 +5529,7 @@
     <row r="232">
       <c r="A232" s="2" t="inlineStr">
         <is>
-          <t>dbt/models/staging/kinetic/_kinetic__staging.yml</t>
+          <t>dbt/models/staging/kinetic/stg_kinetic__meta_ads.sql</t>
         </is>
       </c>
       <c r="B232" s="2" t="inlineStr">
@@ -5539,19 +5539,19 @@
       </c>
       <c r="C232" s="3" t="inlineStr">
         <is>
-          <t>Updated: tests for the 4 Meta staging models, incl. uniqueness of the combined daily keys -- all hand-verified against live data first</t>
+          <t>Phase 2 staging (paid media: Meta): 1:1 pass-through of meta_ads</t>
         </is>
       </c>
       <c r="D232" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 16:49 PDT</t>
+          <t>2026-09-29 13:02 PDT</t>
         </is>
       </c>
     </row>
     <row r="233">
       <c r="A233" s="2" t="inlineStr">
         <is>
-          <t>dbt/models/staging/kinetic/stg_kinetic__google_search_campaigns.sql</t>
+          <t>dbt/models/staging/kinetic/stg_kinetic__meta_ad_insights_daily.sql</t>
         </is>
       </c>
       <c r="B233" s="2" t="inlineStr">
@@ -5561,19 +5561,19 @@
       </c>
       <c r="C233" s="3" t="inlineStr">
         <is>
-          <t>Phase 2 staging (paid media: Google Search): campaigns with the raw customer_id renamed google_ads_account_id (it's the Google Ads account number, not a Kinetic customer), daily budget in micros and dollars, end_date cast back to a date</t>
+          <t>Phase 2 staging (paid media: Meta): meta_ad_insights_daily with a combined ad_day_id key, unit-suffixed columns (spend_usd, cpm_usd, cpc_usd) and ctr renamed ctr_fraction (0.017 = 1.7%)</t>
         </is>
       </c>
       <c r="D233" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 13:13 PDT</t>
+          <t>2026-09-29 13:02 PDT</t>
         </is>
       </c>
     </row>
     <row r="234">
       <c r="A234" s="2" t="inlineStr">
         <is>
-          <t>dbt/models/staging/kinetic/stg_kinetic__google_search_ad_groups.sql</t>
+          <t>dbt/models/staging/kinetic/stg_kinetic__meta_ad_actions_daily.sql</t>
         </is>
       </c>
       <c r="B234" s="2" t="inlineStr">
@@ -5583,19 +5583,19 @@
       </c>
       <c r="C234" s="3" t="inlineStr">
         <is>
-          <t>Phase 2 staging (paid media: Google Search): ad groups; cpc_bid_micros cast back to a number (always empty -- automated bidding)</t>
+          <t>Phase 2 staging (paid media: Meta): meta_ad_actions_daily with a combined ad_day_action_id key; value renamed action_count</t>
         </is>
       </c>
       <c r="D234" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 13:13 PDT</t>
+          <t>2026-09-29 13:02 PDT</t>
         </is>
       </c>
     </row>
     <row r="235">
       <c r="A235" s="2" t="inlineStr">
         <is>
-          <t>dbt/models/staging/kinetic/stg_kinetic__google_search_performance_daily.sql</t>
+          <t>dbt/models/staging/kinetic/_kinetic__staging.yml</t>
         </is>
       </c>
       <c r="B235" s="2" t="inlineStr">
@@ -5605,19 +5605,19 @@
       </c>
       <c r="C235" s="3" t="inlineStr">
         <is>
-          <t>Phase 2 staging (paid media: Google Search): ad-group-day performance with combined ad_group_day_id key, cost converted from micros to dollars, ctr_fraction. The keyword table rolled up -- never add the two together</t>
+          <t>Updated: tests for the 4 Meta staging models, incl. uniqueness of the combined daily keys -- all hand-verified against live data first</t>
         </is>
       </c>
       <c r="D235" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 13:13 PDT</t>
+          <t>2026-09-29 16:49 PDT</t>
         </is>
       </c>
     </row>
     <row r="236">
       <c r="A236" s="2" t="inlineStr">
         <is>
-          <t>dbt/models/staging/kinetic/stg_kinetic__google_search_keyword_performance_daily.sql</t>
+          <t>dbt/models/staging/kinetic/stg_kinetic__google_search_campaigns.sql</t>
         </is>
       </c>
       <c r="B236" s="2" t="inlineStr">
@@ -5627,7 +5627,7 @@
       </c>
       <c r="C236" s="3" t="inlineStr">
         <is>
-          <t>Phase 2 staging (paid media: Google Search): keyword-day performance with combined keyword_day_id key, cost converted from micros to dollars, ctr_fraction</t>
+          <t>Phase 2 staging (paid media: Google Search): campaigns with the raw customer_id renamed google_ads_account_id (it's the Google Ads account number, not a Kinetic customer), daily budget in micros and dollars, end_date cast back to a date</t>
         </is>
       </c>
       <c r="D236" s="2" t="inlineStr">
@@ -5639,7 +5639,7 @@
     <row r="237">
       <c r="A237" s="2" t="inlineStr">
         <is>
-          <t>dbt/models/staging/kinetic/_kinetic__staging.yml</t>
+          <t>dbt/models/staging/kinetic/stg_kinetic__google_search_ad_groups.sql</t>
         </is>
       </c>
       <c r="B237" s="2" t="inlineStr">
@@ -5649,19 +5649,19 @@
       </c>
       <c r="C237" s="3" t="inlineStr">
         <is>
-          <t>Updated: tests for the 4 Google Search staging models -- all hand-verified against live data first</t>
+          <t>Phase 2 staging (paid media: Google Search): ad groups; cpc_bid_micros cast back to a number (always empty -- automated bidding)</t>
         </is>
       </c>
       <c r="D237" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 16:49 PDT</t>
+          <t>2026-09-29 13:13 PDT</t>
         </is>
       </c>
     </row>
     <row r="238">
       <c r="A238" s="2" t="inlineStr">
         <is>
-          <t>dbt/models/staging/kinetic/stg_kinetic__youtube_campaigns.sql</t>
+          <t>dbt/models/staging/kinetic/stg_kinetic__google_search_performance_daily.sql</t>
         </is>
       </c>
       <c r="B238" s="2" t="inlineStr">
@@ -5671,19 +5671,19 @@
       </c>
       <c r="C238" s="3" t="inlineStr">
         <is>
-          <t>Phase 2 staging (paid media: YouTube): campaigns with customer_id renamed google_ads_account_id (the ad account, not a Kinetic customer), budgets in micros and dollars</t>
+          <t>Phase 2 staging (paid media: Google Search): ad-group-day performance with combined ad_group_day_id key, cost converted from micros to dollars, ctr_fraction. The keyword table rolled up -- never add the two together</t>
         </is>
       </c>
       <c r="D238" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 13:14 PDT</t>
+          <t>2026-09-29 13:13 PDT</t>
         </is>
       </c>
     </row>
     <row r="239">
       <c r="A239" s="2" t="inlineStr">
         <is>
-          <t>dbt/models/staging/kinetic/stg_kinetic__youtube_ad_groups.sql</t>
+          <t>dbt/models/staging/kinetic/stg_kinetic__google_search_keyword_performance_daily.sql</t>
         </is>
       </c>
       <c r="B239" s="2" t="inlineStr">
@@ -5693,19 +5693,19 @@
       </c>
       <c r="C239" s="3" t="inlineStr">
         <is>
-          <t>Phase 2 staging (paid media: YouTube): 1:1 pass-through of youtube_ad_groups</t>
+          <t>Phase 2 staging (paid media: Google Search): keyword-day performance with combined keyword_day_id key, cost converted from micros to dollars, ctr_fraction</t>
         </is>
       </c>
       <c r="D239" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 13:14 PDT</t>
+          <t>2026-09-29 13:13 PDT</t>
         </is>
       </c>
     </row>
     <row r="240">
       <c r="A240" s="2" t="inlineStr">
         <is>
-          <t>dbt/models/staging/kinetic/stg_kinetic__youtube_performance_daily.sql</t>
+          <t>dbt/models/staging/kinetic/_kinetic__staging.yml</t>
         </is>
       </c>
       <c r="B240" s="2" t="inlineStr">
@@ -5715,19 +5715,19 @@
       </c>
       <c r="C240" s="3" t="inlineStr">
         <is>
-          <t>Phase 2 staging (paid media: YouTube): ad-group-day performance with combined ad_group_day_id key, cost and cost-per-view converted from micros to dollars, video_view_rate_fraction</t>
+          <t>Updated: tests for the 4 Google Search staging models -- all hand-verified against live data first</t>
         </is>
       </c>
       <c r="D240" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 13:14 PDT</t>
+          <t>2026-09-29 16:49 PDT</t>
         </is>
       </c>
     </row>
     <row r="241">
       <c r="A241" s="2" t="inlineStr">
         <is>
-          <t>dbt/models/staging/kinetic/_kinetic__staging.yml</t>
+          <t>dbt/models/staging/kinetic/stg_kinetic__youtube_campaigns.sql</t>
         </is>
       </c>
       <c r="B241" s="2" t="inlineStr">
@@ -5737,19 +5737,19 @@
       </c>
       <c r="C241" s="3" t="inlineStr">
         <is>
-          <t>Updated: tests for the 3 YouTube staging models -- all hand-verified against live data first</t>
+          <t>Phase 2 staging (paid media: YouTube): campaigns with customer_id renamed google_ads_account_id (the ad account, not a Kinetic customer), budgets in micros and dollars</t>
         </is>
       </c>
       <c r="D241" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 16:49 PDT</t>
+          <t>2026-09-29 13:14 PDT</t>
         </is>
       </c>
     </row>
     <row r="242">
       <c r="A242" s="2" t="inlineStr">
         <is>
-          <t>dbt/models/staging/kinetic/stg_kinetic__dv360_insertion_orders.sql</t>
+          <t>dbt/models/staging/kinetic/stg_kinetic__youtube_ad_groups.sql</t>
         </is>
       </c>
       <c r="B242" s="2" t="inlineStr">
@@ -5759,19 +5759,19 @@
       </c>
       <c r="C242" s="3" t="inlineStr">
         <is>
-          <t>Phase 2 staging (paid media: DV360): insertion orders with budget_micros named monthly_budget_* (it's a monthly budget), end_date cast back to a date; flags the flat-budget-vs-growing-spend known issue</t>
+          <t>Phase 2 staging (paid media: YouTube): 1:1 pass-through of youtube_ad_groups</t>
         </is>
       </c>
       <c r="D242" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 13:27 PDT</t>
+          <t>2026-09-29 13:14 PDT</t>
         </is>
       </c>
     </row>
     <row r="243">
       <c r="A243" s="2" t="inlineStr">
         <is>
-          <t>dbt/models/staging/kinetic/stg_kinetic__dv360_line_items.sql</t>
+          <t>dbt/models/staging/kinetic/stg_kinetic__youtube_performance_daily.sql</t>
         </is>
       </c>
       <c r="B243" s="2" t="inlineStr">
@@ -5781,19 +5781,19 @@
       </c>
       <c r="C243" s="3" t="inlineStr">
         <is>
-          <t>Phase 2 staging (paid media: DV360): 1:1 pass-through of dv360_line_items</t>
+          <t>Phase 2 staging (paid media: YouTube): ad-group-day performance with combined ad_group_day_id key, cost and cost-per-view converted from micros to dollars, video_view_rate_fraction</t>
         </is>
       </c>
       <c r="D243" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 13:19 PDT</t>
+          <t>2026-09-29 13:14 PDT</t>
         </is>
       </c>
     </row>
     <row r="244">
       <c r="A244" s="2" t="inlineStr">
         <is>
-          <t>dbt/models/staging/kinetic/stg_kinetic__dv360_performance_daily.sql</t>
+          <t>dbt/models/staging/kinetic/_kinetic__staging.yml</t>
         </is>
       </c>
       <c r="B244" s="2" t="inlineStr">
@@ -5803,19 +5803,19 @@
       </c>
       <c r="C244" s="3" t="inlineStr">
         <is>
-          <t>Phase 2 staging (paid media: DV360): line-item x day x exchange x environment performance with combined line_item_day_slice_id key, micros converted to dollars, ctr_fraction</t>
+          <t>Updated: tests for the 3 YouTube staging models -- all hand-verified against live data first</t>
         </is>
       </c>
       <c r="D244" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 13:19 PDT</t>
+          <t>2026-09-29 16:49 PDT</t>
         </is>
       </c>
     </row>
     <row r="245">
       <c r="A245" s="2" t="inlineStr">
         <is>
-          <t>dbt/models/staging/kinetic/_kinetic__staging.yml</t>
+          <t>dbt/models/staging/kinetic/stg_kinetic__dv360_insertion_orders.sql</t>
         </is>
       </c>
       <c r="B245" s="2" t="inlineStr">
@@ -5825,19 +5825,19 @@
       </c>
       <c r="C245" s="3" t="inlineStr">
         <is>
-          <t>Updated: tests for the 3 DV360 staging models, incl. accepted_values on exchange and environment -- all hand-verified against live data first</t>
+          <t>Phase 2 staging (paid media: DV360): insertion orders with budget_micros named monthly_budget_* (it's a monthly budget), end_date cast back to a date; flags the flat-budget-vs-growing-spend known issue</t>
         </is>
       </c>
       <c r="D245" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 16:49 PDT</t>
+          <t>2026-09-29 13:27 PDT</t>
         </is>
       </c>
     </row>
     <row r="246">
       <c r="A246" s="2" t="inlineStr">
         <is>
-          <t>generator/params.py</t>
+          <t>dbt/models/staging/kinetic/stg_kinetic__dv360_line_items.sql</t>
         </is>
       </c>
       <c r="B246" s="2" t="inlineStr">
@@ -5847,85 +5847,85 @@
       </c>
       <c r="C246" s="3" t="inlineStr">
         <is>
-          <t>Updated 2026-09-29: every evergreen ad budget on all 6 platforms is now the campaign's CURRENT budget, sized from realized spend (weekly average &lt;= budget, no day &gt; 1.75x; DV360 monthly &gt;= highest month). The old flat 'typical day' budgets let later months spend up to ~20x the stored budget</t>
+          <t>Phase 2 staging (paid media: DV360): 1:1 pass-through of dv360_line_items</t>
         </is>
       </c>
       <c r="D246" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 13:23 PDT</t>
+          <t>2026-09-29 13:19 PDT</t>
         </is>
       </c>
     </row>
     <row r="247">
       <c r="A247" s="2" t="inlineStr">
         <is>
-          <t>data/meta_campaigns.csv</t>
+          <t>dbt/models/staging/kinetic/stg_kinetic__dv360_performance_daily.sql</t>
         </is>
       </c>
       <c r="B247" s="2" t="inlineStr">
         <is>
-          <t>Shipped table</t>
+          <t>Code</t>
         </is>
       </c>
       <c r="C247" s="3" t="inlineStr">
         <is>
-          <t>Regenerated 2026-09-29: evergreen daily_budget values updated to current budgets (only that column, only the 4 evergreen rows changed)</t>
+          <t>Phase 2 staging (paid media: DV360): line-item x day x exchange x environment performance with combined line_item_day_slice_id key, micros converted to dollars, ctr_fraction</t>
         </is>
       </c>
       <c r="D247" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 13:24 PDT</t>
+          <t>2026-09-29 13:19 PDT</t>
         </is>
       </c>
     </row>
     <row r="248">
       <c r="A248" s="2" t="inlineStr">
         <is>
-          <t>data/google_search_campaigns.csv</t>
+          <t>dbt/models/staging/kinetic/_kinetic__staging.yml</t>
         </is>
       </c>
       <c r="B248" s="2" t="inlineStr">
         <is>
-          <t>Shipped table</t>
+          <t>Code</t>
         </is>
       </c>
       <c r="C248" s="3" t="inlineStr">
         <is>
-          <t>Regenerated 2026-09-29: campaign_budget_micros updated to current budgets (only that column changed)</t>
+          <t>Updated: tests for the 3 DV360 staging models, incl. accepted_values on exchange and environment -- all hand-verified against live data first</t>
         </is>
       </c>
       <c r="D248" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 13:24 PDT</t>
+          <t>2026-09-29 16:49 PDT</t>
         </is>
       </c>
     </row>
     <row r="249">
       <c r="A249" s="2" t="inlineStr">
         <is>
-          <t>data/youtube_campaigns.csv</t>
+          <t>generator/params.py</t>
         </is>
       </c>
       <c r="B249" s="2" t="inlineStr">
         <is>
-          <t>Shipped table</t>
+          <t>Code</t>
         </is>
       </c>
       <c r="C249" s="3" t="inlineStr">
         <is>
-          <t>Regenerated 2026-09-29: evergreen campaign_budget_micros updated to current budgets (only that column, only the 4 evergreen rows changed)</t>
+          <t>Updated 2026-09-29: every evergreen ad budget on all 6 platforms is now the campaign's CURRENT budget, sized from realized spend (weekly average &lt;= budget, no day &gt; 1.75x; DV360 monthly &gt;= highest month). The old flat 'typical day' budgets let later months spend up to ~20x the stored budget</t>
         </is>
       </c>
       <c r="D249" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 13:24 PDT</t>
+          <t>2026-09-29 13:23 PDT</t>
         </is>
       </c>
     </row>
     <row r="250">
       <c r="A250" s="2" t="inlineStr">
         <is>
-          <t>data/dv360_insertion_orders.csv</t>
+          <t>data/meta_campaigns.csv</t>
         </is>
       </c>
       <c r="B250" s="2" t="inlineStr">
@@ -5935,7 +5935,7 @@
       </c>
       <c r="C250" s="3" t="inlineStr">
         <is>
-          <t>Regenerated 2026-09-29: monthly budget_micros updated to current budgets (only that column changed)</t>
+          <t>Regenerated 2026-09-29: evergreen daily_budget values updated to current budgets (only that column, only the 4 evergreen rows changed)</t>
         </is>
       </c>
       <c r="D250" s="2" t="inlineStr">
@@ -5947,7 +5947,7 @@
     <row r="251">
       <c r="A251" s="2" t="inlineStr">
         <is>
-          <t>data/snap_campaigns.csv</t>
+          <t>data/google_search_campaigns.csv</t>
         </is>
       </c>
       <c r="B251" s="2" t="inlineStr">
@@ -5957,7 +5957,7 @@
       </c>
       <c r="C251" s="3" t="inlineStr">
         <is>
-          <t>Regenerated 2026-09-29: evergreen daily_budget_micro updated to current budgets (only that column, only the 4 evergreen rows changed)</t>
+          <t>Regenerated 2026-09-29: campaign_budget_micros updated to current budgets (only that column changed)</t>
         </is>
       </c>
       <c r="D251" s="2" t="inlineStr">
@@ -5969,7 +5969,7 @@
     <row r="252">
       <c r="A252" s="2" t="inlineStr">
         <is>
-          <t>data/tiktok_campaigns.csv</t>
+          <t>data/youtube_campaigns.csv</t>
         </is>
       </c>
       <c r="B252" s="2" t="inlineStr">
@@ -5979,7 +5979,7 @@
       </c>
       <c r="C252" s="3" t="inlineStr">
         <is>
-          <t>Regenerated 2026-09-29: BUDGET_MODE_DAY budget_micro updated to current budgets (only that column, only the 4 evergreen rows changed)</t>
+          <t>Regenerated 2026-09-29: evergreen campaign_budget_micros updated to current budgets (only that column, only the 4 evergreen rows changed)</t>
         </is>
       </c>
       <c r="D252" s="2" t="inlineStr">
@@ -5991,73 +5991,73 @@
     <row r="253">
       <c r="A253" s="2" t="inlineStr">
         <is>
-          <t>generator/audit_cross_dataset_alignment.py</t>
+          <t>data/dv360_insertion_orders.csv</t>
         </is>
       </c>
       <c r="B253" s="2" t="inlineStr">
         <is>
-          <t>Code</t>
+          <t>Shipped table</t>
         </is>
       </c>
       <c r="C253" s="3" t="inlineStr">
         <is>
-          <t>Updated 2026-09-29: new Check 8 -- spend vs stored budget for every campaign on all 6 platforms (weekly/daily limits for daily budgets, monthly for DV360, total for holiday flights)</t>
+          <t>Regenerated 2026-09-29: monthly budget_micros updated to current budgets (only that column changed)</t>
         </is>
       </c>
       <c r="D253" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 13:30 PDT</t>
+          <t>2026-09-29 13:24 PDT</t>
         </is>
       </c>
     </row>
     <row r="254">
       <c r="A254" s="2" t="inlineStr">
         <is>
-          <t>dbt/models/staging/kinetic/stg_kinetic__dv360_insertion_orders.sql</t>
+          <t>data/snap_campaigns.csv</t>
         </is>
       </c>
       <c r="B254" s="2" t="inlineStr">
         <is>
-          <t>Code</t>
+          <t>Shipped table</t>
         </is>
       </c>
       <c r="C254" s="3" t="inlineStr">
         <is>
-          <t>Updated: budget known-issue note replaced -- budgets are now current budgets</t>
+          <t>Regenerated 2026-09-29: evergreen daily_budget_micro updated to current budgets (only that column, only the 4 evergreen rows changed)</t>
         </is>
       </c>
       <c r="D254" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 13:27 PDT</t>
+          <t>2026-09-29 13:24 PDT</t>
         </is>
       </c>
     </row>
     <row r="255">
       <c r="A255" s="2" t="inlineStr">
         <is>
-          <t>generator/paid_media_common.py</t>
+          <t>data/tiktok_campaigns.csv</t>
         </is>
       </c>
       <c r="B255" s="2" t="inlineStr">
         <is>
-          <t>Code</t>
+          <t>Shipped table</t>
         </is>
       </c>
       <c r="C255" s="3" t="inlineStr">
         <is>
-          <t>Updated 2026-09-29: new cap_flight_at_budget() -- rescales a holiday flight's days so it never spends past its lifetime budget, replaying the same random rates so every other row is unchanged</t>
+          <t>Regenerated 2026-09-29: BUDGET_MODE_DAY budget_micro updated to current budgets (only that column, only the 4 evergreen rows changed)</t>
         </is>
       </c>
       <c r="D255" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 13:29 PDT</t>
+          <t>2026-09-29 13:24 PDT</t>
         </is>
       </c>
     </row>
     <row r="256">
       <c r="A256" s="2" t="inlineStr">
         <is>
-          <t>generator/build_meta_ad_insights_daily.py</t>
+          <t>generator/audit_cross_dataset_alignment.py</t>
         </is>
       </c>
       <c r="B256" s="2" t="inlineStr">
@@ -6067,19 +6067,19 @@
       </c>
       <c r="C256" s="3" t="inlineStr">
         <is>
-          <t>Updated 2026-09-29: holiday flights capped at their lifetime budget via cap_flight_at_budget()</t>
+          <t>Updated 2026-09-29: new Check 8 -- spend vs stored budget for every campaign on all 6 platforms (weekly/daily limits for daily budgets, monthly for DV360, total for holiday flights)</t>
         </is>
       </c>
       <c r="D256" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 13:29 PDT</t>
+          <t>2026-09-29 13:30 PDT</t>
         </is>
       </c>
     </row>
     <row r="257">
       <c r="A257" s="2" t="inlineStr">
         <is>
-          <t>generator/build_snap_stats_daily.py</t>
+          <t>dbt/models/staging/kinetic/stg_kinetic__dv360_insertion_orders.sql</t>
         </is>
       </c>
       <c r="B257" s="2" t="inlineStr">
@@ -6089,19 +6089,19 @@
       </c>
       <c r="C257" s="3" t="inlineStr">
         <is>
-          <t>Updated 2026-09-29: holiday flights capped at their lifetime budget via cap_flight_at_budget()</t>
+          <t>Updated: budget known-issue note replaced -- budgets are now current budgets</t>
         </is>
       </c>
       <c r="D257" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 13:29 PDT</t>
+          <t>2026-09-29 13:27 PDT</t>
         </is>
       </c>
     </row>
     <row r="258">
       <c r="A258" s="2" t="inlineStr">
         <is>
-          <t>generator/build_tiktok_reports_daily.py</t>
+          <t>generator/paid_media_common.py</t>
         </is>
       </c>
       <c r="B258" s="2" t="inlineStr">
@@ -6111,7 +6111,7 @@
       </c>
       <c r="C258" s="3" t="inlineStr">
         <is>
-          <t>Updated 2026-09-29: holiday flights capped at their lifetime budget via cap_flight_at_budget()</t>
+          <t>Updated 2026-09-29: new cap_flight_at_budget() -- rescales a holiday flight's days so it never spends past its lifetime budget, replaying the same random rates so every other row is unchanged</t>
         </is>
       </c>
       <c r="D258" s="2" t="inlineStr">
@@ -6123,7 +6123,7 @@
     <row r="259">
       <c r="A259" s="2" t="inlineStr">
         <is>
-          <t>generator/build_youtube_performance_daily.py</t>
+          <t>generator/build_meta_ad_insights_daily.py</t>
         </is>
       </c>
       <c r="B259" s="2" t="inlineStr">
@@ -6133,7 +6133,7 @@
       </c>
       <c r="C259" s="3" t="inlineStr">
         <is>
-          <t>Updated 2026-09-29: holiday flights capped at their lifetime budget via cap_flight_at_budget() (no-op today -- all YouTube flights were already under budget)</t>
+          <t>Updated 2026-09-29: holiday flights capped at their lifetime budget via cap_flight_at_budget()</t>
         </is>
       </c>
       <c r="D259" s="2" t="inlineStr">
@@ -6145,17 +6145,17 @@
     <row r="260">
       <c r="A260" s="2" t="inlineStr">
         <is>
-          <t>data/meta_ad_insights_daily.csv</t>
+          <t>generator/build_snap_stats_daily.py</t>
         </is>
       </c>
       <c r="B260" s="2" t="inlineStr">
         <is>
-          <t>Shipped table</t>
+          <t>Code</t>
         </is>
       </c>
       <c r="C260" s="3" t="inlineStr">
         <is>
-          <t>Regenerated 2026-09-29: the 2023 and 2024 holiday flights (38 rows) trimmed to spend exactly their lifetime budget; every other row identical</t>
+          <t>Updated 2026-09-29: holiday flights capped at their lifetime budget via cap_flight_at_budget()</t>
         </is>
       </c>
       <c r="D260" s="2" t="inlineStr">
@@ -6167,17 +6167,17 @@
     <row r="261">
       <c r="A261" s="2" t="inlineStr">
         <is>
-          <t>data/meta_ad_actions_daily.csv</t>
+          <t>generator/build_tiktok_reports_daily.py</t>
         </is>
       </c>
       <c r="B261" s="2" t="inlineStr">
         <is>
-          <t>Shipped table</t>
+          <t>Code</t>
         </is>
       </c>
       <c r="C261" s="3" t="inlineStr">
         <is>
-          <t>Regenerated 2026-09-29: re-derived from the trimmed insights rows -- only the 2023/2024 holiday flights' action rows changed (one initiate_checkout row on 2024-11-15 dropped to zero and is no longer emitted)</t>
+          <t>Updated 2026-09-29: holiday flights capped at their lifetime budget via cap_flight_at_budget()</t>
         </is>
       </c>
       <c r="D261" s="2" t="inlineStr">
@@ -6189,17 +6189,17 @@
     <row r="262">
       <c r="A262" s="2" t="inlineStr">
         <is>
-          <t>data/snap_stats_daily.csv</t>
+          <t>generator/build_youtube_performance_daily.py</t>
         </is>
       </c>
       <c r="B262" s="2" t="inlineStr">
         <is>
-          <t>Shipped table</t>
+          <t>Code</t>
         </is>
       </c>
       <c r="C262" s="3" t="inlineStr">
         <is>
-          <t>Regenerated 2026-09-29: the 2024 holiday flight (19 rows) trimmed to spend exactly its lifetime budget; every other row identical</t>
+          <t>Updated 2026-09-29: holiday flights capped at their lifetime budget via cap_flight_at_budget() (no-op today -- all YouTube flights were already under budget)</t>
         </is>
       </c>
       <c r="D262" s="2" t="inlineStr">
@@ -6211,7 +6211,7 @@
     <row r="263">
       <c r="A263" s="2" t="inlineStr">
         <is>
-          <t>data/tiktok_reports_daily.csv</t>
+          <t>data/meta_ad_insights_daily.csv</t>
         </is>
       </c>
       <c r="B263" s="2" t="inlineStr">
@@ -6221,7 +6221,7 @@
       </c>
       <c r="C263" s="3" t="inlineStr">
         <is>
-          <t>Regenerated 2026-09-29: the 2023/2024/2025 holiday flights (56 rows) trimmed to spend exactly their lifetime budgets; every other row identical</t>
+          <t>Regenerated 2026-09-29: the 2023 and 2024 holiday flights (38 rows) trimmed to spend exactly their lifetime budget; every other row identical</t>
         </is>
       </c>
       <c r="D263" s="2" t="inlineStr">
@@ -6233,95 +6233,95 @@
     <row r="264">
       <c r="A264" s="2" t="inlineStr">
         <is>
-          <t>docs/cross_dataset_alignment_audit.md</t>
+          <t>data/meta_ad_actions_daily.csv</t>
         </is>
       </c>
       <c r="B264" s="2" t="inlineStr">
         <is>
-          <t>Docs</t>
+          <t>Shipped table</t>
         </is>
       </c>
       <c r="C264" s="3" t="inlineStr">
         <is>
-          <t>Updated 2026-09-29: added Check 8 (spend vs stored budget) with both fixes and results</t>
+          <t>Regenerated 2026-09-29: re-derived from the trimmed insights rows -- only the 2023/2024 holiday flights' action rows changed (one initiate_checkout row on 2024-11-15 dropped to zero and is no longer emitted)</t>
         </is>
       </c>
       <c r="D264" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 13:54 PDT</t>
+          <t>2026-09-29 13:29 PDT</t>
         </is>
       </c>
     </row>
     <row r="265">
       <c r="A265" s="2" t="inlineStr">
         <is>
-          <t>generator/audit_cross_dataset_alignment.py</t>
+          <t>data/snap_stats_daily.csv</t>
         </is>
       </c>
       <c r="B265" s="2" t="inlineStr">
         <is>
-          <t>Code</t>
+          <t>Shipped table</t>
         </is>
       </c>
       <c r="C265" s="3" t="inlineStr">
         <is>
-          <t>Updated 2026-09-29: Check 8's flight limit tightened from 1.05x to 1.0x now that flights are capped</t>
+          <t>Regenerated 2026-09-29: the 2024 holiday flight (19 rows) trimmed to spend exactly its lifetime budget; every other row identical</t>
         </is>
       </c>
       <c r="D265" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 13:30 PDT</t>
+          <t>2026-09-29 13:29 PDT</t>
         </is>
       </c>
     </row>
     <row r="266">
       <c r="A266" s="2" t="inlineStr">
         <is>
-          <t>dbt/models/staging/kinetic/stg_kinetic__snap_campaigns.sql</t>
+          <t>data/tiktok_reports_daily.csv</t>
         </is>
       </c>
       <c r="B266" s="2" t="inlineStr">
         <is>
-          <t>Code</t>
+          <t>Shipped table</t>
         </is>
       </c>
       <c r="C266" s="3" t="inlineStr">
         <is>
-          <t>Phase 2 staging (paid media: Snap): campaigns with ad_account_id renamed snap_ad_account_id, current budgets in micros and dollars</t>
+          <t>Regenerated 2026-09-29: the 2023/2024/2025 holiday flights (56 rows) trimmed to spend exactly their lifetime budgets; every other row identical</t>
         </is>
       </c>
       <c r="D266" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 15:53 PDT</t>
+          <t>2026-09-29 13:29 PDT</t>
         </is>
       </c>
     </row>
     <row r="267">
       <c r="A267" s="2" t="inlineStr">
         <is>
-          <t>dbt/models/staging/kinetic/stg_kinetic__snap_ad_squads.sql</t>
+          <t>docs/cross_dataset_alignment_audit.md</t>
         </is>
       </c>
       <c r="B267" s="2" t="inlineStr">
         <is>
-          <t>Code</t>
+          <t>Docs</t>
         </is>
       </c>
       <c r="C267" s="3" t="inlineStr">
         <is>
-          <t>Phase 2 staging (paid media: Snap): 1:1 pass-through of snap_ad_squads (Snap's ad set / ad group level)</t>
+          <t>Updated 2026-09-29: added Check 8 (spend vs stored budget) with both fixes and results</t>
         </is>
       </c>
       <c r="D267" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 15:53 PDT</t>
+          <t>2026-09-29 13:54 PDT</t>
         </is>
       </c>
     </row>
     <row r="268">
       <c r="A268" s="2" t="inlineStr">
         <is>
-          <t>dbt/models/staging/kinetic/stg_kinetic__snap_ads.sql</t>
+          <t>generator/audit_cross_dataset_alignment.py</t>
         </is>
       </c>
       <c r="B268" s="2" t="inlineStr">
@@ -6331,19 +6331,19 @@
       </c>
       <c r="C268" s="3" t="inlineStr">
         <is>
-          <t>Phase 2 staging (paid media: Snap): 1:1 pass-through of snap_ads</t>
+          <t>Updated 2026-09-29: Check 8's flight limit tightened from 1.05x to 1.0x now that flights are capped</t>
         </is>
       </c>
       <c r="D268" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 15:53 PDT</t>
+          <t>2026-09-29 13:30 PDT</t>
         </is>
       </c>
     </row>
     <row r="269">
       <c r="A269" s="2" t="inlineStr">
         <is>
-          <t>dbt/models/staging/kinetic/stg_kinetic__snap_stats_daily.sql</t>
+          <t>dbt/models/staging/kinetic/stg_kinetic__snap_campaigns.sql</t>
         </is>
       </c>
       <c r="B269" s="2" t="inlineStr">
@@ -6353,7 +6353,7 @@
       </c>
       <c r="C269" s="3" t="inlineStr">
         <is>
-          <t>Phase 2 staging (paid media: Snap): ad-day stats with combined ad_day_id key, spend in micros and dollars; documents swipes as Snap's clicks</t>
+          <t>Phase 2 staging (paid media: Snap): campaigns with ad_account_id renamed snap_ad_account_id, current budgets in micros and dollars</t>
         </is>
       </c>
       <c r="D269" s="2" t="inlineStr">
@@ -6365,7 +6365,7 @@
     <row r="270">
       <c r="A270" s="2" t="inlineStr">
         <is>
-          <t>dbt/models/staging/kinetic/_kinetic__staging.yml</t>
+          <t>dbt/models/staging/kinetic/stg_kinetic__snap_ad_squads.sql</t>
         </is>
       </c>
       <c r="B270" s="2" t="inlineStr">
@@ -6375,19 +6375,19 @@
       </c>
       <c r="C270" s="3" t="inlineStr">
         <is>
-          <t>Updated: tests for the 4 Snap staging models -- all hand-verified against live data first</t>
+          <t>Phase 2 staging (paid media: Snap): 1:1 pass-through of snap_ad_squads (Snap's ad set / ad group level)</t>
         </is>
       </c>
       <c r="D270" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 16:49 PDT</t>
+          <t>2026-09-29 15:53 PDT</t>
         </is>
       </c>
     </row>
     <row r="271">
       <c r="A271" s="2" t="inlineStr">
         <is>
-          <t>dbt/models/staging/kinetic/stg_kinetic__tiktok_campaigns.sql</t>
+          <t>dbt/models/staging/kinetic/stg_kinetic__snap_ads.sql</t>
         </is>
       </c>
       <c r="B271" s="2" t="inlineStr">
@@ -6397,19 +6397,19 @@
       </c>
       <c r="C271" s="3" t="inlineStr">
         <is>
-          <t>Phase 2 staging (paid media: TikTok): campaigns with the single budget split into daily_budget_usd / lifetime_budget_usd by budget_mode (matching the other platforms), advertiser_id renamed tiktok_advertiser_id</t>
+          <t>Phase 2 staging (paid media: Snap): 1:1 pass-through of snap_ads</t>
         </is>
       </c>
       <c r="D271" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 15:57 PDT</t>
+          <t>2026-09-29 15:53 PDT</t>
         </is>
       </c>
     </row>
     <row r="272">
       <c r="A272" s="2" t="inlineStr">
         <is>
-          <t>dbt/models/staging/kinetic/stg_kinetic__tiktok_adgroups.sql</t>
+          <t>dbt/models/staging/kinetic/stg_kinetic__snap_stats_daily.sql</t>
         </is>
       </c>
       <c r="B272" s="2" t="inlineStr">
@@ -6419,19 +6419,19 @@
       </c>
       <c r="C272" s="3" t="inlineStr">
         <is>
-          <t>Phase 2 staging (paid media: TikTok): 1:1 pass-through of tiktok_adgroups</t>
+          <t>Phase 2 staging (paid media: Snap): ad-day stats with combined ad_day_id key, spend in micros and dollars; documents swipes as Snap's clicks</t>
         </is>
       </c>
       <c r="D272" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 15:57 PDT</t>
+          <t>2026-09-29 15:53 PDT</t>
         </is>
       </c>
     </row>
     <row r="273">
       <c r="A273" s="2" t="inlineStr">
         <is>
-          <t>dbt/models/staging/kinetic/stg_kinetic__tiktok_ads.sql</t>
+          <t>dbt/models/staging/kinetic/_kinetic__staging.yml</t>
         </is>
       </c>
       <c r="B273" s="2" t="inlineStr">
@@ -6441,19 +6441,19 @@
       </c>
       <c r="C273" s="3" t="inlineStr">
         <is>
-          <t>Phase 2 staging (paid media: TikTok): 1:1 pass-through of tiktok_ads</t>
+          <t>Updated: tests for the 4 Snap staging models -- all hand-verified against live data first</t>
         </is>
       </c>
       <c r="D273" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 15:57 PDT</t>
+          <t>2026-09-29 16:49 PDT</t>
         </is>
       </c>
     </row>
     <row r="274">
       <c r="A274" s="2" t="inlineStr">
         <is>
-          <t>dbt/models/staging/kinetic/stg_kinetic__tiktok_reports_daily.sql</t>
+          <t>dbt/models/staging/kinetic/stg_kinetic__tiktok_campaigns.sql</t>
         </is>
       </c>
       <c r="B274" s="2" t="inlineStr">
@@ -6463,7 +6463,7 @@
       </c>
       <c r="C274" s="3" t="inlineStr">
         <is>
-          <t>Phase 2 staging (paid media: TikTok): ad-day reports with combined ad_day_id key, spend and CPM in micros and dollars, ctr_fraction</t>
+          <t>Phase 2 staging (paid media: TikTok): campaigns with the single budget split into daily_budget_usd / lifetime_budget_usd by budget_mode (matching the other platforms), advertiser_id renamed tiktok_advertiser_id</t>
         </is>
       </c>
       <c r="D274" s="2" t="inlineStr">
@@ -6475,7 +6475,7 @@
     <row r="275">
       <c r="A275" s="2" t="inlineStr">
         <is>
-          <t>dbt/models/staging/kinetic/stg_kinetic__product_variants.sql</t>
+          <t>dbt/models/staging/kinetic/stg_kinetic__tiktok_adgroups.sql</t>
         </is>
       </c>
       <c r="B275" s="2" t="inlineStr">
@@ -6485,54 +6485,120 @@
       </c>
       <c r="C275" s="3" t="inlineStr">
         <is>
-          <t>Phase 2 staging (final table, 47 of 47): product variants with variant_option, price_adjustment_usd</t>
+          <t>Phase 2 staging (paid media: TikTok): 1:1 pass-through of tiktok_adgroups</t>
         </is>
       </c>
       <c r="D275" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 16:08 PDT</t>
+          <t>2026-09-29 15:57 PDT</t>
         </is>
       </c>
     </row>
     <row r="276">
       <c r="A276" s="2" t="inlineStr">
         <is>
-          <t>HANDOFF.md</t>
+          <t>dbt/models/staging/kinetic/stg_kinetic__tiktok_ads.sql</t>
         </is>
       </c>
       <c r="B276" s="2" t="inlineStr">
         <is>
-          <t>Doc</t>
+          <t>Code</t>
         </is>
       </c>
       <c r="C276" s="3" t="inlineStr">
         <is>
-          <t>Handoff note for starting a new chat/project: status, open decisions, prior decisions, pitfalls</t>
+          <t>Phase 2 staging (paid media: TikTok): 1:1 pass-through of tiktok_ads</t>
         </is>
       </c>
       <c r="D276" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 17:25 PDT</t>
+          <t>2026-09-29 15:57 PDT</t>
         </is>
       </c>
     </row>
     <row r="277">
       <c r="A277" s="2" t="inlineStr">
         <is>
+          <t>dbt/models/staging/kinetic/stg_kinetic__tiktok_reports_daily.sql</t>
+        </is>
+      </c>
+      <c r="B277" s="2" t="inlineStr">
+        <is>
+          <t>Code</t>
+        </is>
+      </c>
+      <c r="C277" s="3" t="inlineStr">
+        <is>
+          <t>Phase 2 staging (paid media: TikTok): ad-day reports with combined ad_day_id key, spend and CPM in micros and dollars, ctr_fraction</t>
+        </is>
+      </c>
+      <c r="D277" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-29 15:57 PDT</t>
+        </is>
+      </c>
+    </row>
+    <row r="278">
+      <c r="A278" s="2" t="inlineStr">
+        <is>
+          <t>dbt/models/staging/kinetic/stg_kinetic__product_variants.sql</t>
+        </is>
+      </c>
+      <c r="B278" s="2" t="inlineStr">
+        <is>
+          <t>Code</t>
+        </is>
+      </c>
+      <c r="C278" s="3" t="inlineStr">
+        <is>
+          <t>Phase 2 staging (final table, 47 of 47): product variants with variant_option, price_adjustment_usd</t>
+        </is>
+      </c>
+      <c r="D278" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-29 16:08 PDT</t>
+        </is>
+      </c>
+    </row>
+    <row r="279">
+      <c r="A279" s="2" t="inlineStr">
+        <is>
+          <t>HANDOFF.md</t>
+        </is>
+      </c>
+      <c r="B279" s="2" t="inlineStr">
+        <is>
+          <t>Doc</t>
+        </is>
+      </c>
+      <c r="C279" s="3" t="inlineStr">
+        <is>
+          <t>Handoff note for starting a new chat/project: status, open decisions, prior decisions, pitfalls</t>
+        </is>
+      </c>
+      <c r="D279" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-29 17:25 PDT</t>
+        </is>
+      </c>
+    </row>
+    <row r="280">
+      <c r="A280" s="2" t="inlineStr">
+        <is>
           <t>dbt/models/staging/kinetic/_kinetic__staging.yml</t>
         </is>
       </c>
-      <c r="B277" s="2" t="inlineStr">
-        <is>
-          <t>Code</t>
-        </is>
-      </c>
-      <c r="C277" s="3" t="inlineStr">
+      <c r="B280" s="2" t="inlineStr">
+        <is>
+          <t>Code</t>
+        </is>
+      </c>
+      <c r="C280" s="3" t="inlineStr">
         <is>
           <t>Updated: tests for the 4 TikTok staging models -- all hand-verified against live data first</t>
         </is>
       </c>
-      <c r="D277" s="2" t="inlineStr">
+      <c r="D280" s="2" t="inlineStr">
         <is>
           <t>2026-09-29 16:49 PDT</t>
         </is>

</xml_diff>

<commit_message>
Regenerate File_Manifest for int_messaging_events
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BNXw5rqKjFBrMYnHoaQzEK
</commit_message>
<xml_diff>
--- a/File_Manifest.xlsx
+++ b/File_Manifest.xlsx
@@ -435,7 +435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D280"/>
+  <dimension ref="A1:D284"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="48" customWidth="1" min="1" max="1"/>
@@ -506,7 +506,7 @@
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 18:25 PDT</t>
+          <t>2026-09-29 22:03 PDT</t>
         </is>
       </c>
     </row>
@@ -638,7 +638,7 @@
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 18:55 PDT</t>
+          <t>2026-09-29 22:03 PDT</t>
         </is>
       </c>
     </row>
@@ -748,7 +748,7 @@
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 18:55 PDT</t>
+          <t>2026-09-29 22:04 PDT</t>
         </is>
       </c>
     </row>
@@ -4620,7 +4620,7 @@
       </c>
       <c r="D190" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 17:23 PDT</t>
+          <t>2026-09-29 22:03 PDT</t>
         </is>
       </c>
     </row>
@@ -5038,7 +5038,7 @@
       </c>
       <c r="D209" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 18:25 PDT</t>
+          <t>2026-09-29 22:03 PDT</t>
         </is>
       </c>
     </row>
@@ -5104,7 +5104,7 @@
       </c>
       <c r="D212" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 18:55 PDT</t>
+          <t>2026-09-29 19:22 PDT</t>
         </is>
       </c>
     </row>
@@ -6601,6 +6601,94 @@
       <c r="D280" s="2" t="inlineStr">
         <is>
           <t>2026-09-29 16:49 PDT</t>
+        </is>
+      </c>
+    </row>
+    <row r="281">
+      <c r="A281" s="2" t="inlineStr">
+        <is>
+          <t>dbt/models/intermediate/int_messaging_events.sql</t>
+        </is>
+      </c>
+      <c r="B281" s="2" t="inlineStr">
+        <is>
+          <t>Code</t>
+        </is>
+      </c>
+      <c r="C281" s="3" t="inlineStr">
+        <is>
+          <t>Intermediate model: one row per Braze email or push event in one shape, customer resolved via Braze id or email match (written and hand-verified; needs dbt build)</t>
+        </is>
+      </c>
+      <c r="D281" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-29 22:03 PDT</t>
+        </is>
+      </c>
+    </row>
+    <row r="282">
+      <c r="A282" s="2" t="inlineStr">
+        <is>
+          <t>dbt/tests/assert_int_messaging_events_counts_match_sources.sql</t>
+        </is>
+      </c>
+      <c r="B282" s="2" t="inlineStr">
+        <is>
+          <t>Code</t>
+        </is>
+      </c>
+      <c r="C282" s="3" t="inlineStr">
+        <is>
+          <t>dbt test: unified event count equals email + push event counts</t>
+        </is>
+      </c>
+      <c r="D282" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-29 22:03 PDT</t>
+        </is>
+      </c>
+    </row>
+    <row r="283">
+      <c r="A283" s="2" t="inlineStr">
+        <is>
+          <t>dbt/tests/assert_int_messaging_events_customer_matches_resolution.sql</t>
+        </is>
+      </c>
+      <c r="B283" s="2" t="inlineStr">
+        <is>
+          <t>Code</t>
+        </is>
+      </c>
+      <c r="C283" s="3" t="inlineStr">
+        <is>
+          <t>dbt test: customer_id is null exactly when a messaging event is unresolved</t>
+        </is>
+      </c>
+      <c r="D283" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-29 22:03 PDT</t>
+        </is>
+      </c>
+    </row>
+    <row r="284">
+      <c r="A284" s="2" t="inlineStr">
+        <is>
+          <t>MORNING_LIST.md</t>
+        </is>
+      </c>
+      <c r="B284" s="2" t="inlineStr">
+        <is>
+          <t>Doc</t>
+        </is>
+      </c>
+      <c r="C284" s="3" t="inlineStr">
+        <is>
+          <t>Overnight run report: commands to run first, assumed decisions, done/blocked units, proposed playbook wording</t>
+        </is>
+      </c>
+      <c r="D284" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-29 22:02 PDT</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Phase 3 model 5: int_paid_media_daily (written, hand-verified, needs dbt build)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BNXw5rqKjFBrMYnHoaQzEK
</commit_message>
<xml_diff>
--- a/File_Manifest.xlsx
+++ b/File_Manifest.xlsx
@@ -435,7 +435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D284"/>
+  <dimension ref="A1:D287"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="48" customWidth="1" min="1" max="1"/>
@@ -506,7 +506,7 @@
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 22:03 PDT</t>
+          <t>2026-09-29 22:05 PDT</t>
         </is>
       </c>
     </row>
@@ -638,7 +638,7 @@
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 22:03 PDT</t>
+          <t>2026-09-29 22:05 PDT</t>
         </is>
       </c>
     </row>
@@ -748,7 +748,7 @@
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 22:04 PDT</t>
+          <t>2026-09-29 22:05 PDT</t>
         </is>
       </c>
     </row>
@@ -4620,7 +4620,7 @@
       </c>
       <c r="D190" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 22:03 PDT</t>
+          <t>2026-09-29 22:05 PDT</t>
         </is>
       </c>
     </row>
@@ -6689,6 +6689,72 @@
       <c r="D284" s="2" t="inlineStr">
         <is>
           <t>2026-09-29 22:02 PDT</t>
+        </is>
+      </c>
+    </row>
+    <row r="285">
+      <c r="A285" s="2" t="inlineStr">
+        <is>
+          <t>dbt/models/intermediate/int_paid_media_daily.sql</t>
+        </is>
+      </c>
+      <c r="B285" s="2" t="inlineStr">
+        <is>
+          <t>Code</t>
+        </is>
+      </c>
+      <c r="C285" s="3" t="inlineStr">
+        <is>
+          <t>Intermediate model: one row per ad platform per day, spend/impressions/clicks/conversions in USD (written and hand-verified; needs dbt build)</t>
+        </is>
+      </c>
+      <c r="D285" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-29 22:05 PDT</t>
+        </is>
+      </c>
+    </row>
+    <row r="286">
+      <c r="A286" s="2" t="inlineStr">
+        <is>
+          <t>dbt/tests/assert_int_paid_media_daily_spend_matches_sources.sql</t>
+        </is>
+      </c>
+      <c r="B286" s="2" t="inlineStr">
+        <is>
+          <t>Code</t>
+        </is>
+      </c>
+      <c r="C286" s="3" t="inlineStr">
+        <is>
+          <t>dbt test: platform-day spend total equals the six source spend totals</t>
+        </is>
+      </c>
+      <c r="D286" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-29 22:05 PDT</t>
+        </is>
+      </c>
+    </row>
+    <row r="287">
+      <c r="A287" s="2" t="inlineStr">
+        <is>
+          <t>dbt/tests/assert_int_paid_media_daily_no_missing_days.sql</t>
+        </is>
+      </c>
+      <c r="B287" s="2" t="inlineStr">
+        <is>
+          <t>Code</t>
+        </is>
+      </c>
+      <c r="C287" s="3" t="inlineStr">
+        <is>
+          <t>dbt test: no missing days per platform</t>
+        </is>
+      </c>
+      <c r="D287" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-29 22:05 PDT</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Phase 3 exit: storefront mart reads int_orders_net, paid_revenue_usd rename
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BNXw5rqKjFBrMYnHoaQzEK
</commit_message>
<xml_diff>
--- a/File_Manifest.xlsx
+++ b/File_Manifest.xlsx
@@ -4664,7 +4664,7 @@
       </c>
       <c r="D192" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 17:02 PDT</t>
+          <t>2026-09-29 22:05 PDT</t>
         </is>
       </c>
     </row>
@@ -4862,7 +4862,7 @@
       </c>
       <c r="D201" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 17:18 PDT</t>
+          <t>2026-09-29 22:05 PDT</t>
         </is>
       </c>
     </row>
@@ -5126,7 +5126,7 @@
       </c>
       <c r="D213" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28 14:53 PDT</t>
+          <t>2026-09-29 22:05 PDT</t>
         </is>
       </c>
     </row>
@@ -6688,7 +6688,7 @@
       </c>
       <c r="D284" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 22:02 PDT</t>
+          <t>2026-09-29 22:05 PDT</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Phase 4 mart 1: mart_subscriber_movement_monthly + int_subscription_data_through (written, hand-validated, needs dbt build)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BNXw5rqKjFBrMYnHoaQzEK
</commit_message>
<xml_diff>
--- a/File_Manifest.xlsx
+++ b/File_Manifest.xlsx
@@ -435,7 +435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D287"/>
+  <dimension ref="A1:D291"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="48" customWidth="1" min="1" max="1"/>
@@ -506,7 +506,7 @@
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 22:05 PDT</t>
+          <t>2026-09-29 22:07 PDT</t>
         </is>
       </c>
     </row>
@@ -638,7 +638,7 @@
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 22:05 PDT</t>
+          <t>2026-09-29 22:07 PDT</t>
         </is>
       </c>
     </row>
@@ -748,7 +748,7 @@
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 22:05 PDT</t>
+          <t>2026-09-29 22:07 PDT</t>
         </is>
       </c>
     </row>
@@ -4620,7 +4620,7 @@
       </c>
       <c r="D190" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 22:05 PDT</t>
+          <t>2026-09-29 22:07 PDT</t>
         </is>
       </c>
     </row>
@@ -4642,7 +4642,7 @@
       </c>
       <c r="D191" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 17:02 PDT</t>
+          <t>2026-09-29 22:07 PDT</t>
         </is>
       </c>
     </row>
@@ -4664,7 +4664,7 @@
       </c>
       <c r="D192" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 22:05 PDT</t>
+          <t>2026-09-29 22:07 PDT</t>
         </is>
       </c>
     </row>
@@ -5038,7 +5038,7 @@
       </c>
       <c r="D209" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 22:03 PDT</t>
+          <t>2026-09-29 22:06 PDT</t>
         </is>
       </c>
     </row>
@@ -6755,6 +6755,94 @@
       <c r="D287" s="2" t="inlineStr">
         <is>
           <t>2026-09-29 22:05 PDT</t>
+        </is>
+      </c>
+    </row>
+    <row r="288">
+      <c r="A288" s="2" t="inlineStr">
+        <is>
+          <t>dbt/models/intermediate/int_subscription_data_through.sql</t>
+        </is>
+      </c>
+      <c r="B288" s="2" t="inlineStr">
+        <is>
+          <t>Code</t>
+        </is>
+      </c>
+      <c r="C288" s="3" t="inlineStr">
+        <is>
+          <t>Intermediate model: one row, the last date the subscription/invoice data covers (shared by MRR and subscriber-movement marts) (written; needs dbt build)</t>
+        </is>
+      </c>
+      <c r="D288" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-29 22:07 PDT</t>
+        </is>
+      </c>
+    </row>
+    <row r="289">
+      <c r="A289" s="2" t="inlineStr">
+        <is>
+          <t>dbt/models/marts/mart_subscriber_movement_monthly.sql</t>
+        </is>
+      </c>
+      <c r="B289" s="2" t="inlineStr">
+        <is>
+          <t>Code</t>
+        </is>
+      </c>
+      <c r="C289" s="3" t="inlineStr">
+        <is>
+          <t>Phase 4 mart (CEO): new/returning/churned/net-new/active paying subscribers by month (written and hand-validated; needs dbt build)</t>
+        </is>
+      </c>
+      <c r="D289" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-29 22:07 PDT</t>
+        </is>
+      </c>
+    </row>
+    <row r="290">
+      <c r="A290" s="2" t="inlineStr">
+        <is>
+          <t>dbt/tests/assert_mart_subscriber_movement_monthly_identity.sql</t>
+        </is>
+      </c>
+      <c r="B290" s="2" t="inlineStr">
+        <is>
+          <t>Code</t>
+        </is>
+      </c>
+      <c r="C290" s="3" t="inlineStr">
+        <is>
+          <t>dbt test: end-of-month active = previous + new - churned</t>
+        </is>
+      </c>
+      <c r="D290" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-29 22:07 PDT</t>
+        </is>
+      </c>
+    </row>
+    <row r="291">
+      <c r="A291" s="2" t="inlineStr">
+        <is>
+          <t>dbt/tests/assert_mart_subscriber_movement_monthly_totals_match_source.sql</t>
+        </is>
+      </c>
+      <c r="B291" s="2" t="inlineStr">
+        <is>
+          <t>Code</t>
+        </is>
+      </c>
+      <c r="C291" s="3" t="inlineStr">
+        <is>
+          <t>dbt test: total new and churned match the paid-periods source</t>
+        </is>
+      </c>
+      <c r="D291" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-29 22:07 PDT</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Phase 4 marts 2-3: mart_paid_media_monthly, mart_acquisition_efficiency_monthly (written, hand-validated, need dbt build)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BNXw5rqKjFBrMYnHoaQzEK
</commit_message>
<xml_diff>
--- a/File_Manifest.xlsx
+++ b/File_Manifest.xlsx
@@ -435,7 +435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D291"/>
+  <dimension ref="A1:D295"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="48" customWidth="1" min="1" max="1"/>
@@ -506,7 +506,7 @@
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 22:07 PDT</t>
+          <t>2026-09-29 22:08 PDT</t>
         </is>
       </c>
     </row>
@@ -638,7 +638,7 @@
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 22:07 PDT</t>
+          <t>2026-09-29 22:08 PDT</t>
         </is>
       </c>
     </row>
@@ -748,7 +748,7 @@
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 22:07 PDT</t>
+          <t>2026-09-29 22:08 PDT</t>
         </is>
       </c>
     </row>
@@ -4664,7 +4664,7 @@
       </c>
       <c r="D192" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 22:07 PDT</t>
+          <t>2026-09-29 22:08 PDT</t>
         </is>
       </c>
     </row>
@@ -6688,7 +6688,7 @@
       </c>
       <c r="D284" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 22:05 PDT</t>
+          <t>2026-09-29 22:07 PDT</t>
         </is>
       </c>
     </row>
@@ -6843,6 +6843,94 @@
       <c r="D291" s="2" t="inlineStr">
         <is>
           <t>2026-09-29 22:07 PDT</t>
+        </is>
+      </c>
+    </row>
+    <row r="292">
+      <c r="A292" s="2" t="inlineStr">
+        <is>
+          <t>dbt/models/marts/mart_paid_media_monthly.sql</t>
+        </is>
+      </c>
+      <c r="B292" s="2" t="inlineStr">
+        <is>
+          <t>Code</t>
+        </is>
+      </c>
+      <c r="C292" s="3" t="inlineStr">
+        <is>
+          <t>Phase 4 mart (Performance Marketing/CMO): spend, clicks, platform-reported conversions and ratios by platform by month (written and hand-validated; needs dbt build)</t>
+        </is>
+      </c>
+      <c r="D292" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-29 22:08 PDT</t>
+        </is>
+      </c>
+    </row>
+    <row r="293">
+      <c r="A293" s="2" t="inlineStr">
+        <is>
+          <t>dbt/models/marts/mart_acquisition_efficiency_monthly.sql</t>
+        </is>
+      </c>
+      <c r="B293" s="2" t="inlineStr">
+        <is>
+          <t>Code</t>
+        </is>
+      </c>
+      <c r="C293" s="3" t="inlineStr">
+        <is>
+          <t>Phase 4 mart (CEO/CFO): blended CAC by month = paid spend / first-time paying subscribers (written and hand-validated; needs dbt build)</t>
+        </is>
+      </c>
+      <c r="D293" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-29 22:08 PDT</t>
+        </is>
+      </c>
+    </row>
+    <row r="294">
+      <c r="A294" s="2" t="inlineStr">
+        <is>
+          <t>dbt/tests/assert_mart_paid_media_monthly_spend_matches_daily.sql</t>
+        </is>
+      </c>
+      <c r="B294" s="2" t="inlineStr">
+        <is>
+          <t>Code</t>
+        </is>
+      </c>
+      <c r="C294" s="3" t="inlineStr">
+        <is>
+          <t>dbt test: monthly paid media spend equals daily total</t>
+        </is>
+      </c>
+      <c r="D294" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-29 22:08 PDT</t>
+        </is>
+      </c>
+    </row>
+    <row r="295">
+      <c r="A295" s="2" t="inlineStr">
+        <is>
+          <t>dbt/tests/assert_mart_acquisition_efficiency_monthly_spend_matches_daily.sql</t>
+        </is>
+      </c>
+      <c r="B295" s="2" t="inlineStr">
+        <is>
+          <t>Code</t>
+        </is>
+      </c>
+      <c r="C295" s="3" t="inlineStr">
+        <is>
+          <t>dbt test: CAC mart spend equals total paid media spend</t>
+        </is>
+      </c>
+      <c r="D295" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-29 22:08 PDT</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Phase 5: plain-language descriptions on every model column (staging, intermediate, marts)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BNXw5rqKjFBrMYnHoaQzEK
</commit_message>
<xml_diff>
--- a/File_Manifest.xlsx
+++ b/File_Manifest.xlsx
@@ -506,7 +506,7 @@
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 22:08 PDT</t>
+          <t>2026-09-29 22:12 PDT</t>
         </is>
       </c>
     </row>
@@ -748,7 +748,7 @@
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 22:08 PDT</t>
+          <t>2026-09-29 22:12 PDT</t>
         </is>
       </c>
     </row>
@@ -4422,7 +4422,7 @@
       </c>
       <c r="D181" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 16:43 PDT</t>
+          <t>2026-09-29 22:12 PDT</t>
         </is>
       </c>
     </row>
@@ -4576,7 +4576,7 @@
       </c>
       <c r="D188" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 16:49 PDT</t>
+          <t>2026-09-29 22:11 PDT</t>
         </is>
       </c>
     </row>
@@ -4620,7 +4620,7 @@
       </c>
       <c r="D190" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 22:07 PDT</t>
+          <t>2026-09-29 22:12 PDT</t>
         </is>
       </c>
     </row>
@@ -4664,7 +4664,7 @@
       </c>
       <c r="D192" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 22:08 PDT</t>
+          <t>2026-09-29 22:12 PDT</t>
         </is>
       </c>
     </row>
@@ -4686,7 +4686,7 @@
       </c>
       <c r="D193" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 16:43 PDT</t>
+          <t>2026-09-29 22:12 PDT</t>
         </is>
       </c>
     </row>
@@ -5280,7 +5280,7 @@
       </c>
       <c r="D220" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 16:49 PDT</t>
+          <t>2026-09-29 22:11 PDT</t>
         </is>
       </c>
     </row>
@@ -5390,7 +5390,7 @@
       </c>
       <c r="D225" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 16:49 PDT</t>
+          <t>2026-09-29 22:11 PDT</t>
         </is>
       </c>
     </row>
@@ -5500,7 +5500,7 @@
       </c>
       <c r="D230" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 16:49 PDT</t>
+          <t>2026-09-29 22:11 PDT</t>
         </is>
       </c>
     </row>
@@ -5610,7 +5610,7 @@
       </c>
       <c r="D235" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 16:49 PDT</t>
+          <t>2026-09-29 22:11 PDT</t>
         </is>
       </c>
     </row>
@@ -5720,7 +5720,7 @@
       </c>
       <c r="D240" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 16:49 PDT</t>
+          <t>2026-09-29 22:11 PDT</t>
         </is>
       </c>
     </row>
@@ -5808,7 +5808,7 @@
       </c>
       <c r="D244" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 16:49 PDT</t>
+          <t>2026-09-29 22:11 PDT</t>
         </is>
       </c>
     </row>
@@ -5896,7 +5896,7 @@
       </c>
       <c r="D248" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 16:49 PDT</t>
+          <t>2026-09-29 22:11 PDT</t>
         </is>
       </c>
     </row>
@@ -6446,7 +6446,7 @@
       </c>
       <c r="D273" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 16:49 PDT</t>
+          <t>2026-09-29 22:11 PDT</t>
         </is>
       </c>
     </row>
@@ -6600,7 +6600,7 @@
       </c>
       <c r="D280" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 16:49 PDT</t>
+          <t>2026-09-29 22:11 PDT</t>
         </is>
       </c>
     </row>
@@ -6688,7 +6688,7 @@
       </c>
       <c r="D284" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 22:07 PDT</t>
+          <t>2026-09-29 22:08 PDT</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Phase 6 DRAFT: semantic layer definitions and validation set (unvalidated)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BNXw5rqKjFBrMYnHoaQzEK
</commit_message>
<xml_diff>
--- a/File_Manifest.xlsx
+++ b/File_Manifest.xlsx
@@ -435,7 +435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D295"/>
+  <dimension ref="A1:D297"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="48" customWidth="1" min="1" max="1"/>
@@ -506,7 +506,7 @@
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 22:12 PDT</t>
+          <t>2026-09-29 22:13 PDT</t>
         </is>
       </c>
     </row>
@@ -638,7 +638,7 @@
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 22:08 PDT</t>
+          <t>2026-09-29 22:13 PDT</t>
         </is>
       </c>
     </row>
@@ -748,7 +748,7 @@
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 22:12 PDT</t>
+          <t>2026-09-29 22:13 PDT</t>
         </is>
       </c>
     </row>
@@ -5038,7 +5038,7 @@
       </c>
       <c r="D209" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 22:06 PDT</t>
+          <t>2026-09-29 22:12 PDT</t>
         </is>
       </c>
     </row>
@@ -6688,7 +6688,7 @@
       </c>
       <c r="D284" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 22:08 PDT</t>
+          <t>2026-09-29 22:12 PDT</t>
         </is>
       </c>
     </row>
@@ -6931,6 +6931,50 @@
       <c r="D295" s="2" t="inlineStr">
         <is>
           <t>2026-09-29 22:08 PDT</t>
+        </is>
+      </c>
+    </row>
+    <row r="296">
+      <c r="A296" s="2" t="inlineStr">
+        <is>
+          <t>dbt/drafts/semantic_layer_DRAFT.yml</t>
+        </is>
+      </c>
+      <c r="B296" s="2" t="inlineStr">
+        <is>
+          <t>Config</t>
+        </is>
+      </c>
+      <c r="C296" s="3" t="inlineStr">
+        <is>
+          <t>DRAFT Phase 6 semantic layer (MetricFlow semantic models + metrics) for the marts built so far; unvalidated, outside model-paths</t>
+        </is>
+      </c>
+      <c r="D296" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-29 22:13 PDT</t>
+        </is>
+      </c>
+    </row>
+    <row r="297">
+      <c r="A297" s="2" t="inlineStr">
+        <is>
+          <t>docs/semantic_layer_validation_DRAFT.md</t>
+        </is>
+      </c>
+      <c r="B297" s="2" t="inlineStr">
+        <is>
+          <t>Doc</t>
+        </is>
+      </c>
+      <c r="C297" s="3" t="inlineStr">
+        <is>
+          <t>DRAFT Phase 6 validation set: mf query commands with expected values from hand SQL (not yet run)</t>
+        </is>
+      </c>
+      <c r="D297" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-29 22:13 PDT</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Phase 7 DRAFT Skill; MORNING_LIST and HANDOFF final for overnight run 1
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BNXw5rqKjFBrMYnHoaQzEK
</commit_message>
<xml_diff>
--- a/File_Manifest.xlsx
+++ b/File_Manifest.xlsx
@@ -435,7 +435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D297"/>
+  <dimension ref="A1:D298"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="48" customWidth="1" min="1" max="1"/>
@@ -638,7 +638,7 @@
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 22:13 PDT</t>
+          <t>2026-09-29 22:14 PDT</t>
         </is>
       </c>
     </row>
@@ -748,7 +748,7 @@
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 22:13 PDT</t>
+          <t>2026-09-29 22:14 PDT</t>
         </is>
       </c>
     </row>
@@ -6578,7 +6578,7 @@
       </c>
       <c r="D279" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 17:25 PDT</t>
+          <t>2026-09-29 22:14 PDT</t>
         </is>
       </c>
     </row>
@@ -6688,7 +6688,7 @@
       </c>
       <c r="D284" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 22:12 PDT</t>
+          <t>2026-09-29 22:14 PDT</t>
         </is>
       </c>
     </row>
@@ -6973,6 +6973,28 @@
         </is>
       </c>
       <c r="D297" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-29 22:13 PDT</t>
+        </is>
+      </c>
+    </row>
+    <row r="298">
+      <c r="A298" s="2" t="inlineStr">
+        <is>
+          <t>docs/kinetic_skill_DRAFT.md</t>
+        </is>
+      </c>
+      <c r="B298" s="2" t="inlineStr">
+        <is>
+          <t>Doc</t>
+        </is>
+      </c>
+      <c r="C298" s="3" t="inlineStr">
+        <is>
+          <t>DRAFT Phase 7 Skill: which mart answers which question, Phase 5 caveats as instructions, 'I don't have this data' rules (not reviewed by data owner)</t>
+        </is>
+      </c>
+      <c r="D298" s="2" t="inlineStr">
         <is>
           <t>2026-09-29 22:13 PDT</t>
         </is>

</xml_diff>

<commit_message>
Phase 5: metrics glossary; changelog for docs site branch
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BNXw5rqKjFBrMYnHoaQzEK
</commit_message>
<xml_diff>
--- a/File_Manifest.xlsx
+++ b/File_Manifest.xlsx
@@ -435,7 +435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D298"/>
+  <dimension ref="A1:D299"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="48" customWidth="1" min="1" max="1"/>
@@ -506,7 +506,7 @@
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 22:13 PDT</t>
+          <t>2026-09-30 08:17 PDT</t>
         </is>
       </c>
     </row>
@@ -638,7 +638,7 @@
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 22:14 PDT</t>
+          <t>2026-09-30 08:17 PDT</t>
         </is>
       </c>
     </row>
@@ -748,7 +748,7 @@
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 22:14 PDT</t>
+          <t>2026-09-30 08:17 PDT</t>
         </is>
       </c>
     </row>
@@ -6578,7 +6578,7 @@
       </c>
       <c r="D279" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 22:14 PDT</t>
+          <t>2026-09-30 08:10 PDT</t>
         </is>
       </c>
     </row>
@@ -6688,7 +6688,7 @@
       </c>
       <c r="D284" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 22:14 PDT</t>
+          <t>2026-09-30 06:53 PDT</t>
         </is>
       </c>
     </row>
@@ -6997,6 +6997,28 @@
       <c r="D298" s="2" t="inlineStr">
         <is>
           <t>2026-09-29 22:13 PDT</t>
+        </is>
+      </c>
+    </row>
+    <row r="299">
+      <c r="A299" s="2" t="inlineStr">
+        <is>
+          <t>docs/metrics_glossary.md</t>
+        </is>
+      </c>
+      <c r="B299" s="2" t="inlineStr">
+        <is>
+          <t>Doc</t>
+        </is>
+      </c>
+      <c r="C299" s="3" t="inlineStr">
+        <is>
+          <t>Phase 5 metrics glossary: plain-language definition of every mart metric, its grain, source and what it does NOT mean</t>
+        </is>
+      </c>
+      <c r="D299" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-30 08:17 PDT</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Claude Code setup: playbook editing from Code, unit fix, docs-site script, teaching rules
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BNXw5rqKjFBrMYnHoaQzEK
</commit_message>
<xml_diff>
--- a/File_Manifest.xlsx
+++ b/File_Manifest.xlsx
@@ -435,7 +435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D299"/>
+  <dimension ref="A1:D300"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="48" customWidth="1" min="1" max="1"/>
@@ -506,7 +506,7 @@
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30 08:17 PDT</t>
+          <t>2026-09-30 08:34 PDT</t>
         </is>
       </c>
     </row>
@@ -638,7 +638,7 @@
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30 08:17 PDT</t>
+          <t>2026-09-30 08:34 PDT</t>
         </is>
       </c>
     </row>
@@ -748,7 +748,7 @@
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30 08:17 PDT</t>
+          <t>2026-09-30 08:34 PDT</t>
         </is>
       </c>
     </row>
@@ -5082,7 +5082,7 @@
       </c>
       <c r="D211" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 18:55 PDT</t>
+          <t>2026-09-30 08:34 PDT</t>
         </is>
       </c>
     </row>
@@ -5104,7 +5104,7 @@
       </c>
       <c r="D212" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 19:22 PDT</t>
+          <t>2026-09-30 08:34 PDT</t>
         </is>
       </c>
     </row>
@@ -6578,7 +6578,7 @@
       </c>
       <c r="D279" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30 08:10 PDT</t>
+          <t>2026-09-30 08:29 PDT</t>
         </is>
       </c>
     </row>
@@ -7019,6 +7019,28 @@
       <c r="D299" s="2" t="inlineStr">
         <is>
           <t>2026-09-30 08:17 PDT</t>
+        </is>
+      </c>
+    </row>
+    <row r="300">
+      <c r="A300" s="2" t="inlineStr">
+        <is>
+          <t>scripts/rebuild_docs_branch.sh</t>
+        </is>
+      </c>
+      <c r="B300" s="2" t="inlineStr">
+        <is>
+          <t>Code</t>
+        </is>
+      </c>
+      <c r="C300" s="3" t="inlineStr">
+        <is>
+          <t>Script: rebuild the gh-pages branch (published dbt docs site) from dbt/target as one fast-forward commit; refuses local paths/tokens</t>
+        </is>
+      </c>
+      <c r="D300" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-30 08:34 PDT</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Manifest script runs from the dbt venv (openpyxl); CLAUDE.md, settings, HANDOFF updated
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/File_Manifest.xlsx
+++ b/File_Manifest.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="File Manifest" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="File Manifest" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -482,11 +482,7 @@
           <t>Project overview and folder structure guide</t>
         </is>
       </c>
-      <c r="D2" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-28 14:47 PDT</t>
-        </is>
-      </c>
+      <c r="D2" s="2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -504,11 +500,7 @@
           <t>Plain-English log of every decision and build step</t>
         </is>
       </c>
-      <c r="D3" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-30 08:34 PDT</t>
-        </is>
-      </c>
+      <c r="D3" s="2" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -526,11 +518,7 @@
           <t>Kinetic business model: subscriptions, courses, merch, seasonality</t>
         </is>
       </c>
-      <c r="D4" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-28 14:09 PDT</t>
-        </is>
-      </c>
+      <c r="D4" s="2" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -548,11 +536,7 @@
           <t>Full 47-table schema reference across all domains</t>
         </is>
       </c>
-      <c r="D5" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-28 14:09 PDT</t>
-        </is>
-      </c>
+      <c r="D5" s="2" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -570,11 +554,7 @@
           <t>Build sequence, validation approach, canonical metrics, locked conventions</t>
         </is>
       </c>
-      <c r="D6" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-28 14:09 PDT</t>
-        </is>
-      </c>
+      <c r="D6" s="2" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -592,11 +572,7 @@
           <t>Phase 0 Step 1: global constants (scale, dates, pricing, rates)</t>
         </is>
       </c>
-      <c r="D7" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-29 13:23 PDT</t>
-        </is>
-      </c>
+      <c r="D7" s="2" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -614,11 +590,7 @@
           <t>Phase 0 Steps 2-3: builds seasonality calendar + channel mix schedule</t>
         </is>
       </c>
-      <c r="D8" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-28 14:09 PDT</t>
-        </is>
-      </c>
+      <c r="D8" s="2" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -636,11 +608,7 @@
           <t>Builds/refreshes this file manifest spreadsheet</t>
         </is>
       </c>
-      <c r="D9" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-30 08:34 PDT</t>
-        </is>
-      </c>
+      <c r="D9" s="2" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -658,11 +626,7 @@
           <t>Weekly demand multiplier driving signups/spend/traffic</t>
         </is>
       </c>
-      <c r="D10" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-28 14:09 PDT</t>
-        </is>
-      </c>
+      <c r="D10" s="2" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -680,11 +644,7 @@
           <t>Acquisition channel share over time (Meta/Google/YouTube/DV360/Snap/TikTok/organic)</t>
         </is>
       </c>
-      <c r="D11" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-28 14:09 PDT</t>
-        </is>
-      </c>
+      <c r="D11" s="2" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -702,11 +662,7 @@
           <t>Visual sanity-check of the seasonality calendar</t>
         </is>
       </c>
-      <c r="D12" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-28 14:09 PDT</t>
-        </is>
-      </c>
+      <c r="D12" s="2" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -724,11 +680,7 @@
           <t>Excludes Python __pycache__ from git/sync</t>
         </is>
       </c>
-      <c r="D13" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-29 16:43 PDT</t>
-        </is>
-      </c>
+      <c r="D13" s="2" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -748,7 +700,7 @@
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30 08:34 PDT</t>
+          <t>2026-09-30 08:55 PDT</t>
         </is>
       </c>
     </row>
@@ -768,11 +720,7 @@
           <t>Shared weighted date/channel sampling helpers</t>
         </is>
       </c>
-      <c r="D15" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-28 14:09 PDT</t>
-        </is>
-      </c>
+      <c r="D15" s="2" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -790,11 +738,7 @@
           <t>Phase 0 Step 4: builds the ~2,000-person anonymous ghost population (anon_id now hash-derived, not uuid4 -- reproducibility fix)</t>
         </is>
       </c>
-      <c r="D16" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-28 14:09 PDT</t>
-        </is>
-      </c>
+      <c r="D16" s="2" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -812,11 +756,7 @@
           <t>Phase 0 Steps 5-6: per-customer master timeline + attribution ground truth (fixed: course_merch_only orders now reconciled against the eventual subscription window; pre_signup_anon_id now hash-derived, not uuid4)</t>
         </is>
       </c>
-      <c r="D17" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-28 14:09 PDT</t>
-        </is>
-      </c>
+      <c r="D17" s="2" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -834,11 +774,7 @@
           <t>Anonymous visitors who never become tracked customers; source of guest merch orders</t>
         </is>
       </c>
-      <c r="D18" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-28 14:09 PDT</t>
-        </is>
-      </c>
+      <c r="D18" s="2" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -856,11 +792,7 @@
           <t>Full nested ground-truth simulation for all 100 customers (signup, trial, subscriptions, orders, churn)</t>
         </is>
       </c>
-      <c r="D19" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-28 14:09 PDT</t>
-        </is>
-      </c>
+      <c r="D19" s="2" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -878,11 +810,7 @@
           <t>Flattened, spreadsheet-readable summary of the customer timeline</t>
         </is>
       </c>
-      <c r="D20" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-28 14:09 PDT</t>
-        </is>
-      </c>
+      <c r="D20" s="2" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
@@ -900,11 +828,7 @@
           <t>True acquisition/reactivation channel per customer, kept separate from intentionally messy shipped UTM data</t>
         </is>
       </c>
-      <c r="D21" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-28 14:09 PDT</t>
-        </is>
-      </c>
+      <c r="D21" s="2" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
@@ -922,11 +846,7 @@
           <t>Builds the funnel + segment breakdown charts for the simulation analysis</t>
         </is>
       </c>
-      <c r="D22" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-28 14:09 PDT</t>
-        </is>
-      </c>
+      <c r="D22" s="2" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
@@ -944,11 +864,7 @@
           <t>Customer funnel: total -&gt; trial started -&gt; converted -&gt; active today</t>
         </is>
       </c>
-      <c r="D23" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-28 14:09 PDT</t>
-        </is>
-      </c>
+      <c r="D23" s="2" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
@@ -966,11 +882,7 @@
           <t>Part-to-whole breakdown of all customers' current status</t>
         </is>
       </c>
-      <c r="D24" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-28 14:09 PDT</t>
-        </is>
-      </c>
+      <c r="D24" s="2" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
@@ -988,11 +900,7 @@
           <t>Summary analysis of the recalibrated Phase 0 simulation results</t>
         </is>
       </c>
-      <c r="D25" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-28 14:09 PDT</t>
-        </is>
-      </c>
+      <c r="D25" s="2" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
@@ -1010,11 +918,7 @@
           <t>Phase 1: builds the products table (~12-item course/merch catalog)</t>
         </is>
       </c>
-      <c r="D26" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-28 14:09 PDT</t>
-        </is>
-      </c>
+      <c r="D26" s="2" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
@@ -1032,11 +936,7 @@
           <t>Phase 1: 5-layer validation for products (structural/referential/temporal/business-rule/distributional)</t>
         </is>
       </c>
-      <c r="D27" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-28 14:09 PDT</t>
-        </is>
-      </c>
+      <c r="D27" s="2" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
@@ -1054,11 +954,7 @@
           <t>Phase 1: products table (course + merch catalog)</t>
         </is>
       </c>
-      <c r="D28" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-28 14:09 PDT</t>
-        </is>
-      </c>
+      <c r="D28" s="2" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
@@ -1076,11 +972,7 @@
           <t>Phase 1: builds product_variants (sizes for apparel, single variant elsewhere)</t>
         </is>
       </c>
-      <c r="D29" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-28 14:09 PDT</t>
-        </is>
-      </c>
+      <c r="D29" s="2" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
@@ -1098,11 +990,7 @@
           <t>Phase 1: 5-layer validation for product_variants, including FK to products</t>
         </is>
       </c>
-      <c r="D30" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-28 14:09 PDT</t>
-        </is>
-      </c>
+      <c r="D30" s="2" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
@@ -1120,11 +1008,7 @@
           <t>Phase 1: product_variants table (21 variants across 12 products)</t>
         </is>
       </c>
-      <c r="D31" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-28 14:09 PDT</t>
-        </is>
-      </c>
+      <c r="D31" s="2" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
@@ -1142,11 +1026,7 @@
           <t>Phase 1: builds subscription_plans (Basic/Plus x monthly/annual)</t>
         </is>
       </c>
-      <c r="D32" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-28 14:09 PDT</t>
-        </is>
-      </c>
+      <c r="D32" s="2" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
@@ -1164,11 +1044,7 @@
           <t>Phase 1: 5-layer validation for subscription_plans</t>
         </is>
       </c>
-      <c r="D33" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-28 14:09 PDT</t>
-        </is>
-      </c>
+      <c r="D33" s="2" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
@@ -1186,11 +1062,7 @@
           <t>Phase 1: subscription_plans table (4 plans)</t>
         </is>
       </c>
-      <c r="D34" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-28 14:09 PDT</t>
-        </is>
-      </c>
+      <c r="D34" s="2" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
@@ -1208,11 +1080,7 @@
           <t>Phase 1: builds customers table from the master timeline; defines customer_id mapping</t>
         </is>
       </c>
-      <c r="D35" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-28 14:09 PDT</t>
-        </is>
-      </c>
+      <c r="D35" s="2" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
@@ -1230,11 +1098,7 @@
           <t>Phase 1: 5-layer validation for customers, incl. 1:1 reconciliation vs. the timeline</t>
         </is>
       </c>
-      <c r="D36" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-28 14:09 PDT</t>
-        </is>
-      </c>
+      <c r="D36" s="2" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
@@ -1252,11 +1116,7 @@
           <t>Phase 1: customers table (860 rows, one per simulated customer)</t>
         </is>
       </c>
-      <c r="D37" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-28 14:09 PDT</t>
-        </is>
-      </c>
+      <c r="D37" s="2" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
@@ -1274,11 +1134,7 @@
           <t>Phase 1: builds customer_addresses (billing/shipping, obviously-fake streets)</t>
         </is>
       </c>
-      <c r="D38" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-28 14:09 PDT</t>
-        </is>
-      </c>
+      <c r="D38" s="2" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
@@ -1296,11 +1152,7 @@
           <t>Phase 1: 5-layer validation for customer_addresses</t>
         </is>
       </c>
-      <c r="D39" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-28 14:09 PDT</t>
-        </is>
-      </c>
+      <c r="D39" s="2" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
@@ -1318,11 +1170,7 @@
           <t>Phase 1: customer_addresses table (1,431 rows)</t>
         </is>
       </c>
-      <c r="D40" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-28 14:09 PDT</t>
-        </is>
-      </c>
+      <c r="D40" s="2" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
@@ -1340,11 +1188,7 @@
           <t>Phase 1: builds devices (customer + anonymous-ghost devices; 2nd-device anon_id now hash-derived, not uuid4)</t>
         </is>
       </c>
-      <c r="D41" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-28 14:09 PDT</t>
-        </is>
-      </c>
+      <c r="D41" s="2" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
@@ -1362,11 +1206,7 @@
           <t>Phase 1: 5-layer validation for devices</t>
         </is>
       </c>
-      <c r="D42" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-28 14:09 PDT</t>
-        </is>
-      </c>
+      <c r="D42" s="2" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
@@ -1384,11 +1224,7 @@
           <t>Phase 1: devices table (18,042 rows: known-customer + ghost devices)</t>
         </is>
       </c>
-      <c r="D43" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-28 14:09 PDT</t>
-        </is>
-      </c>
+      <c r="D43" s="2" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
@@ -1406,11 +1242,7 @@
           <t>Phase 1: builds identity_map (anonymous_id -&gt; customer_id resolution events)</t>
         </is>
       </c>
-      <c r="D44" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-28 14:09 PDT</t>
-        </is>
-      </c>
+      <c r="D44" s="2" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
@@ -1428,11 +1260,7 @@
           <t>Phase 1: 5-layer validation for identity_map</t>
         </is>
       </c>
-      <c r="D45" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-28 14:09 PDT</t>
-        </is>
-      </c>
+      <c r="D45" s="2" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
@@ -1450,11 +1278,7 @@
           <t>Phase 1: identity_map table (992 rows)</t>
         </is>
       </c>
-      <c r="D46" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-28 14:09 PDT</t>
-        </is>
-      </c>
+      <c r="D46" s="2" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
@@ -1472,11 +1296,7 @@
           <t>Phase 1: builds segments (27 definitions: 9 customer-grain, 18 anonymous -- 3 audience concepts x 6 ad platforms)</t>
         </is>
       </c>
-      <c r="D47" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-28 14:09 PDT</t>
-        </is>
-      </c>
+      <c r="D47" s="2" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
@@ -1494,11 +1314,7 @@
           <t>Phase 1: 5-layer validation for segments</t>
         </is>
       </c>
-      <c r="D48" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-28 14:09 PDT</t>
-        </is>
-      </c>
+      <c r="D48" s="2" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
@@ -1516,11 +1332,7 @@
           <t>Phase 1: segments table (27 rows) -- completes Phase 1 (all 8 tables)</t>
         </is>
       </c>
-      <c r="D49" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-28 14:09 PDT</t>
-        </is>
-      </c>
+      <c r="D49" s="2" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
@@ -1538,11 +1350,7 @@
           <t>Phase 2: builds subscriptions (Stripe-shaped subscription objects; assigns billing_interval + next-renewal date, resolving the long-flagged Phase 2 gap)</t>
         </is>
       </c>
-      <c r="D50" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-28 14:09 PDT</t>
-        </is>
-      </c>
+      <c r="D50" s="2" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
@@ -1560,11 +1368,7 @@
           <t>Phase 2: 5-layer validation for subscriptions</t>
         </is>
       </c>
-      <c r="D51" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-28 14:09 PDT</t>
-        </is>
-      </c>
+      <c r="D51" s="2" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
@@ -1582,11 +1386,7 @@
           <t>Phase 2: subscriptions table (576 rows: one Stripe-shaped subscription object per trial-or-interval)</t>
         </is>
       </c>
-      <c r="D52" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-28 14:09 PDT</t>
-        </is>
-      </c>
+      <c r="D52" s="2" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
@@ -1604,11 +1404,7 @@
           <t>Phase 2: builds subscription_events (event log behind every subscription: trial_started/converted/expired, renewed, upgraded/downgraded, payment_failed, canceled, resumed)</t>
         </is>
       </c>
-      <c r="D53" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-28 14:09 PDT</t>
-        </is>
-      </c>
+      <c r="D53" s="2" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
@@ -1626,11 +1422,7 @@
           <t>Phase 2: 5-layer validation for subscription_events</t>
         </is>
       </c>
-      <c r="D54" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-28 14:09 PDT</t>
-        </is>
-      </c>
+      <c r="D54" s="2" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
@@ -1648,11 +1440,7 @@
           <t>Phase 2: subscription_events table (2,423 rows, incl. ~3% deliberate duplicate webhook-style rows)</t>
         </is>
       </c>
-      <c r="D55" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-28 14:09 PDT</t>
-        </is>
-      </c>
+      <c r="D55" s="2" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
@@ -1670,11 +1458,7 @@
           <t>Phase 2: builds invoices (one per initial charge + renewal, plus uncollectible/open for failed payments) -- completes Phase 2 (all 3 tables)</t>
         </is>
       </c>
-      <c r="D56" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-28 14:09 PDT</t>
-        </is>
-      </c>
+      <c r="D56" s="2" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
@@ -1692,11 +1476,7 @@
           <t>Phase 2: 5-layer validation for invoices</t>
         </is>
       </c>
-      <c r="D57" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-28 14:09 PDT</t>
-        </is>
-      </c>
+      <c r="D57" s="2" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
@@ -1714,11 +1494,7 @@
           <t>Phase 2: invoices table (1,229 rows) -- completes Phase 2</t>
         </is>
       </c>
-      <c r="D58" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-28 14:09 PDT</t>
-        </is>
-      </c>
+      <c r="D58" s="2" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
@@ -1736,11 +1512,7 @@
           <t>Phase 3: builds discount_codes (hand-curated list: evergreen + seasonal promo codes) -- built first in Phase 3 since orders needs it</t>
         </is>
       </c>
-      <c r="D59" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-28 14:09 PDT</t>
-        </is>
-      </c>
+      <c r="D59" s="2" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
@@ -1758,11 +1530,7 @@
           <t>Phase 3: 5-layer validation for discount_codes</t>
         </is>
       </c>
-      <c r="D60" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-28 14:09 PDT</t>
-        </is>
-      </c>
+      <c r="D60" s="2" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
@@ -1780,11 +1548,7 @@
           <t>Phase 3: discount_codes table (7 rows)</t>
         </is>
       </c>
-      <c r="D61" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-28 14:09 PDT</t>
-        </is>
-      </c>
+      <c r="D61" s="2" t="inlineStr"/>
     </row>
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
@@ -1802,11 +1566,7 @@
           <t>Phase 3: builds orders (customer course/merch + guest merch), cross-validated against subscriptions.csv</t>
         </is>
       </c>
-      <c r="D62" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-28 14:09 PDT</t>
-        </is>
-      </c>
+      <c r="D62" s="2" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
@@ -1824,11 +1584,7 @@
           <t>Phase 3: 5-layer validation for orders, incl. the no-course-during-subscription cross-check</t>
         </is>
       </c>
-      <c r="D63" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-28 14:09 PDT</t>
-        </is>
-      </c>
+      <c r="D63" s="2" t="inlineStr"/>
     </row>
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
@@ -1846,11 +1602,7 @@
           <t>Phase 3: orders table (3,650 rows: 1,061 course + 1,332 customer-merch + 1,257 guest-merch)</t>
         </is>
       </c>
-      <c r="D64" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-28 14:09 PDT</t>
-        </is>
-      </c>
+      <c r="D64" s="2" t="inlineStr"/>
     </row>
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
@@ -1868,11 +1620,7 @@
           <t>Phase 3: builds order_line_items (one row per order -- resolves each order's price tier down to a specific product + variant)</t>
         </is>
       </c>
-      <c r="D65" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-28 14:09 PDT</t>
-        </is>
-      </c>
+      <c r="D65" s="2" t="inlineStr"/>
     </row>
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
@@ -1890,11 +1638,7 @@
           <t>Phase 3: 5-layer validation for order_line_items</t>
         </is>
       </c>
-      <c r="D66" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-28 14:09 PDT</t>
-        </is>
-      </c>
+      <c r="D66" s="2" t="inlineStr"/>
     </row>
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
@@ -1912,11 +1656,7 @@
           <t>Phase 3: order_line_items table (3,650 rows, one per order)</t>
         </is>
       </c>
-      <c r="D67" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-28 14:09 PDT</t>
-        </is>
-      </c>
+      <c r="D67" s="2" t="inlineStr"/>
     </row>
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
@@ -1934,11 +1674,7 @@
           <t>Phase 3: builds payments (one Stripe-shaped Charge attempt per row; models realistic declined-then-retried charge attempts)</t>
         </is>
       </c>
-      <c r="D68" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-28 14:09 PDT</t>
-        </is>
-      </c>
+      <c r="D68" s="2" t="inlineStr"/>
     </row>
     <row r="69">
       <c r="A69" s="2" t="inlineStr">
@@ -1956,11 +1692,7 @@
           <t>Phase 3: 5-layer validation for payments</t>
         </is>
       </c>
-      <c r="D69" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-28 14:09 PDT</t>
-        </is>
-      </c>
+      <c r="D69" s="2" t="inlineStr"/>
     </row>
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
@@ -1978,11 +1710,7 @@
           <t>Phase 3: payments table (3,964 rows: 3,650 succeeded + 314 failed retry attempts)</t>
         </is>
       </c>
-      <c r="D70" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-28 14:09 PDT</t>
-        </is>
-      </c>
+      <c r="D70" s="2" t="inlineStr"/>
     </row>
     <row r="71">
       <c r="A71" s="2" t="inlineStr">
@@ -2000,11 +1728,7 @@
           <t>Phase 3: builds refunds (against a small share of orders' succeeded payments) -- completes Phase 3 (all 5 tables)</t>
         </is>
       </c>
-      <c r="D71" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-28 14:09 PDT</t>
-        </is>
-      </c>
+      <c r="D71" s="2" t="inlineStr"/>
     </row>
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
@@ -2022,11 +1746,7 @@
           <t>Phase 3: 5-layer validation for refunds</t>
         </is>
       </c>
-      <c r="D72" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-28 14:09 PDT</t>
-        </is>
-      </c>
+      <c r="D72" s="2" t="inlineStr"/>
     </row>
     <row r="73">
       <c r="A73" s="2" t="inlineStr">
@@ -2044,11 +1764,7 @@
           <t>Phase 3: refunds table (159 rows, 4.4% of orders) -- completes Phase 3</t>
         </is>
       </c>
-      <c r="D73" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-28 14:09 PDT</t>
-        </is>
-      </c>
+      <c r="D73" s="2" t="inlineStr"/>
     </row>
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
@@ -2066,11 +1782,7 @@
           <t>Phase 4: builds customer_segment_membership (effective-dated, derived entirely from subscriptions/orders/invoices -- seg_009 skipped, needs Phase 5) -- completes Phase 4</t>
         </is>
       </c>
-      <c r="D74" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-28 14:09 PDT</t>
-        </is>
-      </c>
+      <c r="D74" s="2" t="inlineStr"/>
     </row>
     <row r="75">
       <c r="A75" s="2" t="inlineStr">
@@ -2088,11 +1800,7 @@
           <t>Phase 4: 5-layer validation for customer_segment_membership</t>
         </is>
       </c>
-      <c r="D75" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-28 14:09 PDT</t>
-        </is>
-      </c>
+      <c r="D75" s="2" t="inlineStr"/>
     </row>
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
@@ -2110,11 +1818,7 @@
           <t>Phase 4: customer_segment_membership table (2,234 rows across 8 of 9 customer-grain segments) -- completes Phase 4</t>
         </is>
       </c>
-      <c r="D76" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-28 14:09 PDT</t>
-        </is>
-      </c>
+      <c r="D76" s="2" t="inlineStr"/>
     </row>
     <row r="77">
       <c r="A77" s="2" t="inlineStr">
@@ -2132,11 +1836,7 @@
           <t>Phase 5: builds web_sessions (marketing-site browsing; known customers + anonymous ghosts, engagement_tier-driven volume)</t>
         </is>
       </c>
-      <c r="D77" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-28 14:09 PDT</t>
-        </is>
-      </c>
+      <c r="D77" s="2" t="inlineStr"/>
     </row>
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
@@ -2154,11 +1854,7 @@
           <t>Phase 5: 5-layer validation for web_sessions</t>
         </is>
       </c>
-      <c r="D78" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-28 14:09 PDT</t>
-        </is>
-      </c>
+      <c r="D78" s="2" t="inlineStr"/>
     </row>
     <row r="79">
       <c r="A79" s="2" t="inlineStr">
@@ -2176,11 +1872,7 @@
           <t>Phase 5: web_sessions table (30,285 rows: 6,476 identity-resolved + 23,809 anonymous)</t>
         </is>
       </c>
-      <c r="D79" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-28 14:09 PDT</t>
-        </is>
-      </c>
+      <c r="D79" s="2" t="inlineStr"/>
     </row>
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
@@ -2198,11 +1890,7 @@
           <t>Phase 5: builds web_events (page_view/product_view/add_to_cart/begin_checkout/purchase/search; every order gets exactly one purchase event)</t>
         </is>
       </c>
-      <c r="D80" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-28 14:09 PDT</t>
-        </is>
-      </c>
+      <c r="D80" s="2" t="inlineStr"/>
     </row>
     <row r="81">
       <c r="A81" s="2" t="inlineStr">
@@ -2220,11 +1908,7 @@
           <t>Phase 5: 5-layer validation for web_events</t>
         </is>
       </c>
-      <c r="D81" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-28 14:09 PDT</t>
-        </is>
-      </c>
+      <c r="D81" s="2" t="inlineStr"/>
     </row>
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
@@ -2242,11 +1926,7 @@
           <t>Phase 5: web_events table (117,706 rows)</t>
         </is>
       </c>
-      <c r="D82" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-28 14:09 PDT</t>
-        </is>
-      </c>
+      <c r="D82" s="2" t="inlineStr"/>
     </row>
     <row r="83">
       <c r="A83" s="2" t="inlineStr">
@@ -2264,11 +1944,7 @@
           <t>Phase 5: builds app_sessions (in-app fitness usage, driven by real subscription intervals + course orders, keyed off engagement_tier)</t>
         </is>
       </c>
-      <c r="D83" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-28 14:09 PDT</t>
-        </is>
-      </c>
+      <c r="D83" s="2" t="inlineStr"/>
     </row>
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
@@ -2286,11 +1962,7 @@
           <t>Phase 5: 5-layer validation for app_sessions</t>
         </is>
       </c>
-      <c r="D84" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-28 14:09 PDT</t>
-        </is>
-      </c>
+      <c r="D84" s="2" t="inlineStr"/>
     </row>
     <row r="85">
       <c r="A85" s="2" t="inlineStr">
@@ -2308,11 +1980,7 @@
           <t>Phase 5: app_sessions table (19,610 rows across 496 customers)</t>
         </is>
       </c>
-      <c r="D85" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-28 14:09 PDT</t>
-        </is>
-      </c>
+      <c r="D85" s="2" t="inlineStr"/>
     </row>
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
@@ -2330,11 +1998,7 @@
           <t>Phase 5: builds app_events (class_started/workout_completed/workout_abandoned/streak_achieved -- streaks derived from real consecutive session dates) -- completes Phase 5</t>
         </is>
       </c>
-      <c r="D86" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-28 14:09 PDT</t>
-        </is>
-      </c>
+      <c r="D86" s="2" t="inlineStr"/>
     </row>
     <row r="87">
       <c r="A87" s="2" t="inlineStr">
@@ -2352,11 +2016,7 @@
           <t>Phase 5: 5-layer validation for app_events</t>
         </is>
       </c>
-      <c r="D87" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-28 14:09 PDT</t>
-        </is>
-      </c>
+      <c r="D87" s="2" t="inlineStr"/>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
@@ -2374,11 +2034,7 @@
           <t>Phase 5: app_events table (39,370 rows) -- completes Phase 5</t>
         </is>
       </c>
-      <c r="D88" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-28 14:09 PDT</t>
-        </is>
-      </c>
+      <c r="D88" s="2" t="inlineStr"/>
     </row>
     <row r="89">
       <c r="A89" s="2" t="inlineStr">
@@ -2396,11 +2052,7 @@
           <t>Phase 6: builds braze_email_campaigns (hand-curated: 7 triggered + 2 broadcast) -- built first, events table needs it</t>
         </is>
       </c>
-      <c r="D89" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-28 14:09 PDT</t>
-        </is>
-      </c>
+      <c r="D89" s="2" t="inlineStr"/>
     </row>
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
@@ -2418,11 +2070,7 @@
           <t>Phase 6: 5-layer validation for braze_email_campaigns</t>
         </is>
       </c>
-      <c r="D90" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-28 14:09 PDT</t>
-        </is>
-      </c>
+      <c r="D90" s="2" t="inlineStr"/>
     </row>
     <row r="91">
       <c r="A91" s="2" t="inlineStr">
@@ -2440,11 +2088,7 @@
           <t>Phase 6: braze_email_campaigns table (9 rows)</t>
         </is>
       </c>
-      <c r="D91" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-28 14:09 PDT</t>
-        </is>
-      </c>
+      <c r="D91" s="2" t="inlineStr"/>
     </row>
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
@@ -2462,11 +2106,7 @@
           <t>Phase 5: builds web_events (retroactive fix: timestamp offsets now rounded to whole seconds, fixing a latent fractional-second formatting bug across all 117,706 rows)</t>
         </is>
       </c>
-      <c r="D92" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-28 14:09 PDT</t>
-        </is>
-      </c>
+      <c r="D92" s="2" t="inlineStr"/>
     </row>
     <row r="93">
       <c r="A93" s="2" t="inlineStr">
@@ -2484,11 +2124,7 @@
           <t>Phase 5: web_events table (117,706 rows; retroactively rebuilt for the whole-second timestamp fix, same counts/logic)</t>
         </is>
       </c>
-      <c r="D93" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-28 14:09 PDT</t>
-        </is>
-      </c>
+      <c r="D93" s="2" t="inlineStr"/>
     </row>
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
@@ -2506,11 +2142,7 @@
           <t>Phase 6: builds braze_email_events (Send/Open/Click/Bounce/Unsubscribe funnel, derived from real trial/payment-failure/order/cart/reactivation sources)</t>
         </is>
       </c>
-      <c r="D94" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-28 14:09 PDT</t>
-        </is>
-      </c>
+      <c r="D94" s="2" t="inlineStr"/>
     </row>
     <row r="95">
       <c r="A95" s="2" t="inlineStr">
@@ -2528,11 +2160,7 @@
           <t>Phase 6: 5-layer validation for braze_email_events</t>
         </is>
       </c>
-      <c r="D95" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-28 14:09 PDT</t>
-        </is>
-      </c>
+      <c r="D95" s="2" t="inlineStr"/>
     </row>
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
@@ -2550,11 +2178,7 @@
           <t>Phase 6: braze_email_events table (26,335 rows, 18,187 sends) -- updated 2026-08-13 by the cross-dataset audit's Check 6 fix (merch_to_sub_trigger send time-of-day)</t>
         </is>
       </c>
-      <c r="D96" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-28 14:09 PDT</t>
-        </is>
-      </c>
+      <c r="D96" s="2" t="inlineStr"/>
     </row>
     <row r="97">
       <c r="A97" s="2" t="inlineStr">
@@ -2572,11 +2196,7 @@
           <t>Phase 6: builds braze_push_campaigns (hand-curated: 5 triggered + 2 broadcast, push-appropriate subset) -- built before events table needs it</t>
         </is>
       </c>
-      <c r="D97" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-28 14:09 PDT</t>
-        </is>
-      </c>
+      <c r="D97" s="2" t="inlineStr"/>
     </row>
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
@@ -2594,11 +2214,7 @@
           <t>Phase 6: 5-layer validation for braze_push_campaigns</t>
         </is>
       </c>
-      <c r="D98" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-28 14:09 PDT</t>
-        </is>
-      </c>
+      <c r="D98" s="2" t="inlineStr"/>
     </row>
     <row r="99">
       <c r="A99" s="2" t="inlineStr">
@@ -2616,11 +2232,7 @@
           <t>Phase 6: braze_push_campaigns table (7 rows)</t>
         </is>
       </c>
-      <c r="D99" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-28 14:09 PDT</t>
-        </is>
-      </c>
+      <c r="D99" s="2" t="inlineStr"/>
     </row>
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
@@ -2638,11 +2250,7 @@
           <t>Phase 6: builds braze_push_events (Send/Open/Click/Bounce/Unsubscribe funnel, gated on push_opt_in as a hard delivery precondition) -- completes Phase 6 (all 4 tables)</t>
         </is>
       </c>
-      <c r="D100" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-28 14:09 PDT</t>
-        </is>
-      </c>
+      <c r="D100" s="2" t="inlineStr"/>
     </row>
     <row r="101">
       <c r="A101" s="2" t="inlineStr">
@@ -2660,11 +2268,7 @@
           <t>Phase 6: 5-layer validation for braze_push_events</t>
         </is>
       </c>
-      <c r="D101" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-28 14:09 PDT</t>
-        </is>
-      </c>
+      <c r="D101" s="2" t="inlineStr"/>
     </row>
     <row r="102">
       <c r="A102" s="2" t="inlineStr">
@@ -2682,11 +2286,7 @@
           <t>Phase 6: braze_push_events table (9,897 rows, 7,851 sends) -- completes Phase 6 (25 of 47 tables shipped; Phase 7 paid media remains)</t>
         </is>
       </c>
-      <c r="D102" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-28 14:09 PDT</t>
-        </is>
-      </c>
+      <c r="D102" s="2" t="inlineStr"/>
     </row>
     <row r="103">
       <c r="A103" s="2" t="inlineStr">
@@ -2704,11 +2304,7 @@
           <t>Phase 7: shared helpers used by all 6 platforms' daily performance tables -- maps any date to the seasonality calendar/channel-mix week and draws each day's per-channel spend baseline</t>
         </is>
       </c>
-      <c r="D103" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-29 13:29 PDT</t>
-        </is>
-      </c>
+      <c r="D103" s="2" t="inlineStr"/>
     </row>
     <row r="104">
       <c r="A104" s="2" t="inlineStr">
@@ -2726,11 +2322,7 @@
           <t>Phase 7 (Meta 1/4): builds meta_campaigns (4 evergreen objective campaigns + 3 flighted brand_lift campaigns timed near BFCM)</t>
         </is>
       </c>
-      <c r="D104" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-28 14:09 PDT</t>
-        </is>
-      </c>
+      <c r="D104" s="2" t="inlineStr"/>
     </row>
     <row r="105">
       <c r="A105" s="2" t="inlineStr">
@@ -2748,11 +2340,7 @@
           <t>Phase 7: 5-layer validation for meta_campaigns</t>
         </is>
       </c>
-      <c r="D105" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-28 14:09 PDT</t>
-        </is>
-      </c>
+      <c r="D105" s="2" t="inlineStr"/>
     </row>
     <row r="106">
       <c r="A106" s="2" t="inlineStr">
@@ -2770,11 +2358,7 @@
           <t>Phase 7 (Meta 1/4): meta_campaigns table (7 rows)</t>
         </is>
       </c>
-      <c r="D106" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-29 13:24 PDT</t>
-        </is>
-      </c>
+      <c r="D106" s="2" t="inlineStr"/>
     </row>
     <row r="107">
       <c r="A107" s="2" t="inlineStr">
@@ -2792,11 +2376,7 @@
           <t>Phase 7 (Meta 2/4): builds meta_ads (functions as the ad-set-level entity -- targeting_segment_id for retargeting/lookalike only)</t>
         </is>
       </c>
-      <c r="D107" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-28 14:09 PDT</t>
-        </is>
-      </c>
+      <c r="D107" s="2" t="inlineStr"/>
     </row>
     <row r="108">
       <c r="A108" s="2" t="inlineStr">
@@ -2814,11 +2394,7 @@
           <t>Phase 7: 5-layer validation for meta_ads</t>
         </is>
       </c>
-      <c r="D108" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-28 14:09 PDT</t>
-        </is>
-      </c>
+      <c r="D108" s="2" t="inlineStr"/>
     </row>
     <row r="109">
       <c r="A109" s="2" t="inlineStr">
@@ -2836,11 +2412,7 @@
           <t>Phase 7 (Meta 2/4): meta_ads table (10 rows)</t>
         </is>
       </c>
-      <c r="D109" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-28 14:09 PDT</t>
-        </is>
-      </c>
+      <c r="D109" s="2" t="inlineStr"/>
     </row>
     <row r="110">
       <c r="A110" s="2" t="inlineStr">
@@ -2858,11 +2430,7 @@
           <t>Phase 7 (Meta 3/4): builds meta_ad_insights_daily (spend/impressions/clicks driven by the shared seasonality calendar + channel-mix schedule)</t>
         </is>
       </c>
-      <c r="D110" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-29 13:29 PDT</t>
-        </is>
-      </c>
+      <c r="D110" s="2" t="inlineStr"/>
     </row>
     <row r="111">
       <c r="A111" s="2" t="inlineStr">
@@ -2880,11 +2448,7 @@
           <t>Phase 7: 5-layer validation for meta_ad_insights_daily, incl. weekly-spend-vs-web_sessions correlation check</t>
         </is>
       </c>
-      <c r="D111" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-28 14:09 PDT</t>
-        </is>
-      </c>
+      <c r="D111" s="2" t="inlineStr"/>
     </row>
     <row r="112">
       <c r="A112" s="2" t="inlineStr">
@@ -2902,11 +2466,7 @@
           <t>Phase 7 (Meta 3/4): meta_ad_insights_daily table (7,396 rows)</t>
         </is>
       </c>
-      <c r="D112" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-29 13:29 PDT</t>
-        </is>
-      </c>
+      <c r="D112" s="2" t="inlineStr"/>
     </row>
     <row r="113">
       <c r="A113" s="2" t="inlineStr">
@@ -2924,11 +2484,7 @@
           <t>Phase 7 (Meta 4/4): builds meta_ad_actions_daily (normalized actions array, derived directly from meta_ad_insights_daily.csv's own clicks) -- completes Meta (1 of 6 platforms)</t>
         </is>
       </c>
-      <c r="D113" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-28 14:09 PDT</t>
-        </is>
-      </c>
+      <c r="D113" s="2" t="inlineStr"/>
     </row>
     <row r="114">
       <c r="A114" s="2" t="inlineStr">
@@ -2946,11 +2502,7 @@
           <t>Phase 7: 5-layer validation for meta_ad_actions_daily</t>
         </is>
       </c>
-      <c r="D114" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-28 14:09 PDT</t>
-        </is>
-      </c>
+      <c r="D114" s="2" t="inlineStr"/>
     </row>
     <row r="115">
       <c r="A115" s="2" t="inlineStr">
@@ -2968,11 +2520,7 @@
           <t>Phase 7 (Meta 4/4): meta_ad_actions_daily table (35,504 rows) -- completes Meta</t>
         </is>
       </c>
-      <c r="D115" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-29 13:29 PDT</t>
-        </is>
-      </c>
+      <c r="D115" s="2" t="inlineStr"/>
     </row>
     <row r="116">
       <c r="A116" s="2" t="inlineStr">
@@ -2990,11 +2538,7 @@
           <t>Phase 7 (Google Search 1/4): builds google_search_campaigns (5 evergreen objective campaigns, incl. an always-on brand-term defense campaign)</t>
         </is>
       </c>
-      <c r="D116" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-28 14:09 PDT</t>
-        </is>
-      </c>
+      <c r="D116" s="2" t="inlineStr"/>
     </row>
     <row r="117">
       <c r="A117" s="2" t="inlineStr">
@@ -3012,11 +2556,7 @@
           <t>Phase 7: 5-layer validation for google_search_campaigns</t>
         </is>
       </c>
-      <c r="D117" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-28 14:09 PDT</t>
-        </is>
-      </c>
+      <c r="D117" s="2" t="inlineStr"/>
     </row>
     <row r="118">
       <c r="A118" s="2" t="inlineStr">
@@ -3034,11 +2574,7 @@
           <t>Phase 7 (Google Search 1/4): google_search_campaigns table (5 rows)</t>
         </is>
       </c>
-      <c r="D118" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-29 13:24 PDT</t>
-        </is>
-      </c>
+      <c r="D118" s="2" t="inlineStr"/>
     </row>
     <row r="119">
       <c r="A119" s="2" t="inlineStr">
@@ -3056,11 +2592,7 @@
           <t>Phase 7 (Google Search 2/4): builds google_search_ad_groups (targeting_segment_id for RLSA retargeting/similar-audience lookalike only)</t>
         </is>
       </c>
-      <c r="D119" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-28 14:09 PDT</t>
-        </is>
-      </c>
+      <c r="D119" s="2" t="inlineStr"/>
     </row>
     <row r="120">
       <c r="A120" s="2" t="inlineStr">
@@ -3078,11 +2610,7 @@
           <t>Phase 7: 5-layer validation for google_search_ad_groups</t>
         </is>
       </c>
-      <c r="D120" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-28 14:09 PDT</t>
-        </is>
-      </c>
+      <c r="D120" s="2" t="inlineStr"/>
     </row>
     <row r="121">
       <c r="A121" s="2" t="inlineStr">
@@ -3100,11 +2628,7 @@
           <t>Phase 7 (Google Search 2/4): google_search_ad_groups table (8 rows)</t>
         </is>
       </c>
-      <c r="D121" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-28 14:09 PDT</t>
-        </is>
-      </c>
+      <c r="D121" s="2" t="inlineStr"/>
     </row>
     <row r="122">
       <c r="A122" s="2" t="inlineStr">
@@ -3122,11 +2646,7 @@
           <t>Phase 7 (Google Search 4/4 by build order): builds google_search_keyword_performance_daily -- the granular ground truth google_search_performance_daily aggregates from</t>
         </is>
       </c>
-      <c r="D122" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-28 14:09 PDT</t>
-        </is>
-      </c>
+      <c r="D122" s="2" t="inlineStr"/>
     </row>
     <row r="123">
       <c r="A123" s="2" t="inlineStr">
@@ -3144,11 +2664,7 @@
           <t>Phase 7: 5-layer validation for google_search_keyword_performance_daily, incl. weekly-spend-vs-web_sessions correlation check</t>
         </is>
       </c>
-      <c r="D123" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-28 14:09 PDT</t>
-        </is>
-      </c>
+      <c r="D123" s="2" t="inlineStr"/>
     </row>
     <row r="124">
       <c r="A124" s="2" t="inlineStr">
@@ -3166,11 +2682,7 @@
           <t>Phase 7 (Google Search 4/4 by build order): google_search_keyword_performance_daily table (19,932 rows)</t>
         </is>
       </c>
-      <c r="D124" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-28 14:09 PDT</t>
-        </is>
-      </c>
+      <c r="D124" s="2" t="inlineStr"/>
     </row>
     <row r="125">
       <c r="A125" s="2" t="inlineStr">
@@ -3188,11 +2700,7 @@
           <t>Phase 7 (Google Search 3/4 by schema order): builds google_search_performance_daily, aggregated exactly from keyword_performance_daily.csv up to ad_group/day grain -- completes Google Search (2 of 6 platforms)</t>
         </is>
       </c>
-      <c r="D125" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-28 14:09 PDT</t>
-        </is>
-      </c>
+      <c r="D125" s="2" t="inlineStr"/>
     </row>
     <row r="126">
       <c r="A126" s="2" t="inlineStr">
@@ -3210,11 +2718,7 @@
           <t>Phase 7: 5-layer validation for google_search_performance_daily, incl. exact-sum reconciliation against keyword_performance_daily.csv</t>
         </is>
       </c>
-      <c r="D126" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-28 14:09 PDT</t>
-        </is>
-      </c>
+      <c r="D126" s="2" t="inlineStr"/>
     </row>
     <row r="127">
       <c r="A127" s="2" t="inlineStr">
@@ -3232,11 +2736,7 @@
           <t>Phase 7 (Google Search 3/4 by schema order): google_search_performance_daily table (8,751 rows) -- completes Google Search</t>
         </is>
       </c>
-      <c r="D127" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-28 14:09 PDT</t>
-        </is>
-      </c>
+      <c r="D127" s="2" t="inlineStr"/>
     </row>
     <row r="128">
       <c r="A128" s="2" t="inlineStr">
@@ -3254,11 +2754,7 @@
           <t>Phase 7 (YouTube 1/3): builds youtube_campaigns (4 evergreen objective campaigns + 3 flighted brand_lift campaigns, mirroring Meta's structure since YouTube Brand Lift is a real flighted measurement product)</t>
         </is>
       </c>
-      <c r="D128" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-28 14:09 PDT</t>
-        </is>
-      </c>
+      <c r="D128" s="2" t="inlineStr"/>
     </row>
     <row r="129">
       <c r="A129" s="2" t="inlineStr">
@@ -3276,11 +2772,7 @@
           <t>Phase 7: 5-layer validation for youtube_campaigns</t>
         </is>
       </c>
-      <c r="D129" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-28 14:09 PDT</t>
-        </is>
-      </c>
+      <c r="D129" s="2" t="inlineStr"/>
     </row>
     <row r="130">
       <c r="A130" s="2" t="inlineStr">
@@ -3298,11 +2790,7 @@
           <t>Phase 7 (YouTube 1/3): youtube_campaigns table (7 rows)</t>
         </is>
       </c>
-      <c r="D130" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-29 13:24 PDT</t>
-        </is>
-      </c>
+      <c r="D130" s="2" t="inlineStr"/>
     </row>
     <row r="131">
       <c r="A131" s="2" t="inlineStr">
@@ -3320,11 +2808,7 @@
           <t>Phase 7 (YouTube 2/3): builds youtube_ad_groups (targeting_segment_id for retargeting/lookalike only)</t>
         </is>
       </c>
-      <c r="D131" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-28 14:09 PDT</t>
-        </is>
-      </c>
+      <c r="D131" s="2" t="inlineStr"/>
     </row>
     <row r="132">
       <c r="A132" s="2" t="inlineStr">
@@ -3342,11 +2826,7 @@
           <t>Phase 7: 5-layer validation for youtube_ad_groups</t>
         </is>
       </c>
-      <c r="D132" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-28 14:09 PDT</t>
-        </is>
-      </c>
+      <c r="D132" s="2" t="inlineStr"/>
     </row>
     <row r="133">
       <c r="A133" s="2" t="inlineStr">
@@ -3364,11 +2844,7 @@
           <t>Phase 7 (YouTube 2/3): youtube_ad_groups table (9 rows)</t>
         </is>
       </c>
-      <c r="D133" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-28 14:09 PDT</t>
-        </is>
-      </c>
+      <c r="D133" s="2" t="inlineStr"/>
     </row>
     <row r="134">
       <c r="A134" s="2" t="inlineStr">
@@ -3386,11 +2862,7 @@
           <t>Phase 7 (YouTube 3/3): builds youtube_performance_daily (video_views/video_view_rate/average_cpv, spend-driven by the shared seasonality calendar + channel-mix schedule) -- completes YouTube (3 of 6 platforms)</t>
         </is>
       </c>
-      <c r="D134" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-29 13:29 PDT</t>
-        </is>
-      </c>
+      <c r="D134" s="2" t="inlineStr"/>
     </row>
     <row r="135">
       <c r="A135" s="2" t="inlineStr">
@@ -3408,11 +2880,7 @@
           <t>Phase 7: 5-layer validation for youtube_performance_daily, incl. weekly-spend-vs-web_sessions correlation check</t>
         </is>
       </c>
-      <c r="D135" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-28 14:09 PDT</t>
-        </is>
-      </c>
+      <c r="D135" s="2" t="inlineStr"/>
     </row>
     <row r="136">
       <c r="A136" s="2" t="inlineStr">
@@ -3430,11 +2898,7 @@
           <t>Phase 7 (YouTube 3/3): youtube_performance_daily table (6,394 rows) -- completes YouTube</t>
         </is>
       </c>
-      <c r="D136" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-29 13:29 PDT</t>
-        </is>
-      </c>
+      <c r="D136" s="2" t="inlineStr"/>
     </row>
     <row r="137">
       <c r="A137" s="2" t="inlineStr">
@@ -3452,11 +2916,7 @@
           <t>Phase 7 (DV360 1/3): builds dv360_insertion_orders (5 evergreen objective IOs, incl. a VIEWABLE_CPM awareness IO)</t>
         </is>
       </c>
-      <c r="D137" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-28 14:09 PDT</t>
-        </is>
-      </c>
+      <c r="D137" s="2" t="inlineStr"/>
     </row>
     <row r="138">
       <c r="A138" s="2" t="inlineStr">
@@ -3474,11 +2934,7 @@
           <t>Phase 7: 5-layer validation for dv360_insertion_orders</t>
         </is>
       </c>
-      <c r="D138" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-28 14:09 PDT</t>
-        </is>
-      </c>
+      <c r="D138" s="2" t="inlineStr"/>
     </row>
     <row r="139">
       <c r="A139" s="2" t="inlineStr">
@@ -3496,11 +2952,7 @@
           <t>Phase 7 (DV360 1/3): dv360_insertion_orders table (5 rows)</t>
         </is>
       </c>
-      <c r="D139" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-29 13:24 PDT</t>
-        </is>
-      </c>
+      <c r="D139" s="2" t="inlineStr"/>
     </row>
     <row r="140">
       <c r="A140" s="2" t="inlineStr">
@@ -3518,11 +2970,7 @@
           <t>Phase 7 (DV360 2/3): builds dv360_line_items (targeting_segment_id for retargeting/lookalike only; brand_lift IO's line item is VIDEO type)</t>
         </is>
       </c>
-      <c r="D140" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-28 14:09 PDT</t>
-        </is>
-      </c>
+      <c r="D140" s="2" t="inlineStr"/>
     </row>
     <row r="141">
       <c r="A141" s="2" t="inlineStr">
@@ -3540,11 +2988,7 @@
           <t>Phase 7: 5-layer validation for dv360_line_items</t>
         </is>
       </c>
-      <c r="D141" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-28 14:09 PDT</t>
-        </is>
-      </c>
+      <c r="D141" s="2" t="inlineStr"/>
     </row>
     <row r="142">
       <c r="A142" s="2" t="inlineStr">
@@ -3562,11 +3006,7 @@
           <t>Phase 7 (DV360 2/3): dv360_line_items table (6 rows)</t>
         </is>
       </c>
-      <c r="D142" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-28 14:09 PDT</t>
-        </is>
-      </c>
+      <c r="D142" s="2" t="inlineStr"/>
     </row>
     <row r="143">
       <c r="A143" s="2" t="inlineStr">
@@ -3584,11 +3024,7 @@
           <t>Phase 7 (DV360 3/3): builds dv360_performance_daily -- fragments each line_item/day into several (exchange, environment) rows, DV360's genuinely different real-time-bidding schema shape -- completes DV360 (4 of 6 platforms)</t>
         </is>
       </c>
-      <c r="D143" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-28 14:09 PDT</t>
-        </is>
-      </c>
+      <c r="D143" s="2" t="inlineStr"/>
     </row>
     <row r="144">
       <c r="A144" s="2" t="inlineStr">
@@ -3606,11 +3042,7 @@
           <t>Phase 7: 5-layer validation for dv360_performance_daily, incl. weekly-spend-vs-web_sessions correlation check and CONNECTED_TV-only-on-video-line-item check</t>
         </is>
       </c>
-      <c r="D144" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-28 14:09 PDT</t>
-        </is>
-      </c>
+      <c r="D144" s="2" t="inlineStr"/>
     </row>
     <row r="145">
       <c r="A145" s="2" t="inlineStr">
@@ -3628,11 +3060,7 @@
           <t>Phase 7 (DV360 3/3): dv360_performance_daily table (25,776 rows) -- completes DV360</t>
         </is>
       </c>
-      <c r="D145" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-28 14:09 PDT</t>
-        </is>
-      </c>
+      <c r="D145" s="2" t="inlineStr"/>
     </row>
     <row r="146">
       <c r="A146" s="2" t="inlineStr">
@@ -3650,11 +3078,7 @@
           <t>Phase 7 (Snap 1/4): builds snap_campaigns (4 evergreen objective campaigns + 3 flighted brand_lift campaigns, flight budgets calibrated to avoid YouTube's earlier scale bug)</t>
         </is>
       </c>
-      <c r="D146" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-28 14:09 PDT</t>
-        </is>
-      </c>
+      <c r="D146" s="2" t="inlineStr"/>
     </row>
     <row r="147">
       <c r="A147" s="2" t="inlineStr">
@@ -3672,11 +3096,7 @@
           <t>Phase 7: 5-layer validation for snap_campaigns</t>
         </is>
       </c>
-      <c r="D147" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-28 14:09 PDT</t>
-        </is>
-      </c>
+      <c r="D147" s="2" t="inlineStr"/>
     </row>
     <row r="148">
       <c r="A148" s="2" t="inlineStr">
@@ -3694,11 +3114,7 @@
           <t>Phase 7 (Snap 1/4): snap_campaigns table (7 rows)</t>
         </is>
       </c>
-      <c r="D148" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-29 13:24 PDT</t>
-        </is>
-      </c>
+      <c r="D148" s="2" t="inlineStr"/>
     </row>
     <row r="149">
       <c r="A149" s="2" t="inlineStr">
@@ -3716,11 +3132,7 @@
           <t>Phase 7 (Snap 2/4): builds snap_ad_squads (Snap's own real ad-set-level targeting entity, unlike Meta -- targeting_segment_id for retargeting/lookalike only)</t>
         </is>
       </c>
-      <c r="D149" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-28 14:09 PDT</t>
-        </is>
-      </c>
+      <c r="D149" s="2" t="inlineStr"/>
     </row>
     <row r="150">
       <c r="A150" s="2" t="inlineStr">
@@ -3738,11 +3150,7 @@
           <t>Phase 7: 5-layer validation for snap_ad_squads</t>
         </is>
       </c>
-      <c r="D150" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-28 14:09 PDT</t>
-        </is>
-      </c>
+      <c r="D150" s="2" t="inlineStr"/>
     </row>
     <row r="151">
       <c r="A151" s="2" t="inlineStr">
@@ -3760,11 +3168,7 @@
           <t>Phase 7 (Snap 2/4): snap_ad_squads table (8 rows)</t>
         </is>
       </c>
-      <c r="D151" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-28 14:09 PDT</t>
-        </is>
-      </c>
+      <c r="D151" s="2" t="inlineStr"/>
     </row>
     <row r="152">
       <c r="A152" s="2" t="inlineStr">
@@ -3782,11 +3186,7 @@
           <t>Phase 7 (Snap 3/4): builds snap_ads (creative-level entity, no targeting -- that lives on the ad squad)</t>
         </is>
       </c>
-      <c r="D152" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-28 14:09 PDT</t>
-        </is>
-      </c>
+      <c r="D152" s="2" t="inlineStr"/>
     </row>
     <row r="153">
       <c r="A153" s="2" t="inlineStr">
@@ -3804,11 +3204,7 @@
           <t>Phase 7: 5-layer validation for snap_ads</t>
         </is>
       </c>
-      <c r="D153" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-28 14:09 PDT</t>
-        </is>
-      </c>
+      <c r="D153" s="2" t="inlineStr"/>
     </row>
     <row r="154">
       <c r="A154" s="2" t="inlineStr">
@@ -3826,11 +3222,7 @@
           <t>Phase 7 (Snap 3/4): snap_ads table (10 rows)</t>
         </is>
       </c>
-      <c r="D154" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-28 14:09 PDT</t>
-        </is>
-      </c>
+      <c r="D154" s="2" t="inlineStr"/>
     </row>
     <row r="155">
       <c r="A155" s="2" t="inlineStr">
@@ -3848,11 +3240,7 @@
           <t>Phase 7 (Snap 4/4): builds snap_stats_daily (spend in Snap's own micro-currency unit, swipes as the click-equivalent) -- completes Snap (5 of 6 platforms)</t>
         </is>
       </c>
-      <c r="D155" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-29 13:29 PDT</t>
-        </is>
-      </c>
+      <c r="D155" s="2" t="inlineStr"/>
     </row>
     <row r="156">
       <c r="A156" s="2" t="inlineStr">
@@ -3870,11 +3258,7 @@
           <t>Phase 7: 5-layer validation for snap_stats_daily, incl. weekly-spend-vs-web_sessions correlation check</t>
         </is>
       </c>
-      <c r="D156" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-28 14:09 PDT</t>
-        </is>
-      </c>
+      <c r="D156" s="2" t="inlineStr"/>
     </row>
     <row r="157">
       <c r="A157" s="2" t="inlineStr">
@@ -3892,11 +3276,7 @@
           <t>Phase 7 (Snap 4/4): snap_stats_daily table (7,407 rows) -- completes Snap</t>
         </is>
       </c>
-      <c r="D157" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-29 13:29 PDT</t>
-        </is>
-      </c>
+      <c r="D157" s="2" t="inlineStr"/>
     </row>
     <row r="158">
       <c r="A158" s="2" t="inlineStr">
@@ -3914,11 +3294,7 @@
           <t>Phase 7 (TikTok 1/4): builds tiktok_campaigns (4 evergreen objective campaigns + 3 flighted brand_lift campaigns)</t>
         </is>
       </c>
-      <c r="D158" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-28 14:09 PDT</t>
-        </is>
-      </c>
+      <c r="D158" s="2" t="inlineStr"/>
     </row>
     <row r="159">
       <c r="A159" s="2" t="inlineStr">
@@ -3936,11 +3312,7 @@
           <t>Phase 7: 5-layer validation for tiktok_campaigns</t>
         </is>
       </c>
-      <c r="D159" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-28 14:09 PDT</t>
-        </is>
-      </c>
+      <c r="D159" s="2" t="inlineStr"/>
     </row>
     <row r="160">
       <c r="A160" s="2" t="inlineStr">
@@ -3958,11 +3330,7 @@
           <t>Phase 7 (TikTok 1/4): tiktok_campaigns table (7 rows)</t>
         </is>
       </c>
-      <c r="D160" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-29 13:24 PDT</t>
-        </is>
-      </c>
+      <c r="D160" s="2" t="inlineStr"/>
     </row>
     <row r="161">
       <c r="A161" s="2" t="inlineStr">
@@ -3980,11 +3348,7 @@
           <t>Phase 7 (TikTok 2/4): builds tiktok_adgroups (TikTok's own real ad-set-level targeting entity -- targeting_segment_id for retargeting/lookalike only)</t>
         </is>
       </c>
-      <c r="D161" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-28 14:09 PDT</t>
-        </is>
-      </c>
+      <c r="D161" s="2" t="inlineStr"/>
     </row>
     <row r="162">
       <c r="A162" s="2" t="inlineStr">
@@ -4002,11 +3366,7 @@
           <t>Phase 7: 5-layer validation for tiktok_adgroups</t>
         </is>
       </c>
-      <c r="D162" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-28 14:09 PDT</t>
-        </is>
-      </c>
+      <c r="D162" s="2" t="inlineStr"/>
     </row>
     <row r="163">
       <c r="A163" s="2" t="inlineStr">
@@ -4024,11 +3384,7 @@
           <t>Phase 7 (TikTok 2/4): tiktok_adgroups table (8 rows)</t>
         </is>
       </c>
-      <c r="D163" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-28 14:09 PDT</t>
-        </is>
-      </c>
+      <c r="D163" s="2" t="inlineStr"/>
     </row>
     <row r="164">
       <c r="A164" s="2" t="inlineStr">
@@ -4046,11 +3402,7 @@
           <t>Phase 7 (TikTok 3/4): builds tiktok_ads (creative-level entity, no targeting -- that lives on the ad group)</t>
         </is>
       </c>
-      <c r="D164" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-28 14:09 PDT</t>
-        </is>
-      </c>
+      <c r="D164" s="2" t="inlineStr"/>
     </row>
     <row r="165">
       <c r="A165" s="2" t="inlineStr">
@@ -4068,11 +3420,7 @@
           <t>Phase 7: 5-layer validation for tiktok_ads</t>
         </is>
       </c>
-      <c r="D165" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-28 14:09 PDT</t>
-        </is>
-      </c>
+      <c r="D165" s="2" t="inlineStr"/>
     </row>
     <row r="166">
       <c r="A166" s="2" t="inlineStr">
@@ -4090,11 +3438,7 @@
           <t>Phase 7 (TikTok 3/4): tiktok_ads table (10 rows)</t>
         </is>
       </c>
-      <c r="D166" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-28 14:09 PDT</t>
-        </is>
-      </c>
+      <c r="D166" s="2" t="inlineStr"/>
     </row>
     <row r="167">
       <c r="A167" s="2" t="inlineStr">
@@ -4112,11 +3456,7 @@
           <t>Phase 7 (TikTok 4/4): builds tiktok_reports_daily (spend/impressions/video_views, TikTok's always-video ad format) -- completes TikTok (6 of 6 platforms) AND all 47 tables</t>
         </is>
       </c>
-      <c r="D167" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-29 13:29 PDT</t>
-        </is>
-      </c>
+      <c r="D167" s="2" t="inlineStr"/>
     </row>
     <row r="168">
       <c r="A168" s="2" t="inlineStr">
@@ -4134,11 +3474,7 @@
           <t>Phase 7: 5-layer validation for tiktok_reports_daily, incl. weekly-spend-vs-web_sessions correlation check</t>
         </is>
       </c>
-      <c r="D168" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-28 14:09 PDT</t>
-        </is>
-      </c>
+      <c r="D168" s="2" t="inlineStr"/>
     </row>
     <row r="169">
       <c r="A169" s="2" t="inlineStr">
@@ -4156,11 +3492,7 @@
           <t>Phase 7 (TikTok 4/4): tiktok_reports_daily table (7,416 rows) -- completes TikTok, Phase 7, and the full 47-table dataset</t>
         </is>
       </c>
-      <c r="D169" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-29 13:29 PDT</t>
-        </is>
-      </c>
+      <c r="D169" s="2" t="inlineStr"/>
     </row>
     <row r="170">
       <c r="A170" s="2" t="inlineStr">
@@ -4178,11 +3510,7 @@
           <t>Post-completion cross-dataset alignment audit -- NOT a shipped-table script. 7 checks: aggregate spend vs. demand, channel mix vs. schedule, calendar-event alignment, long-run growth trend, renewal/lag structure, day-of-week/hour-of-day, timezone/precision sweep. Found and fixed a real bug (Check 6 -- merch_to_sub_trigger Braze sends all landing at exactly midnight); Checks 3 and 5 surfaced genuine, documented (non-bug) characteristics.</t>
         </is>
       </c>
-      <c r="D170" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-29 13:30 PDT</t>
-        </is>
-      </c>
+      <c r="D170" s="2" t="inlineStr"/>
     </row>
     <row r="171">
       <c r="A171" s="2" t="inlineStr">
@@ -4200,11 +3528,7 @@
           <t>Write-up of the 7-check cross-dataset alignment audit's results, including the merch_to_sub_trigger bug fix and the two documented (non-bug) findings from Checks 3 and 5</t>
         </is>
       </c>
-      <c r="D171" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-29 13:54 PDT</t>
-        </is>
-      </c>
+      <c r="D171" s="2" t="inlineStr"/>
     </row>
     <row r="172">
       <c r="A172" s="2" t="inlineStr">
@@ -4222,11 +3546,7 @@
           <t>Post-dataset-completion tooling -- loads all 47 CSVs into a free MotherDuck (hosted DuckDB) database, one table per CSV, with a row-count verification per table. Run on the user's own machine, not inside the Cowork cloud sandbox (MotherDuck needs outbound internet the sandbox doesn't have). Reads its motherduck_token from either a shell env var or an optional warehouse/.env file (gitignored -- NOT tracked or synced by this manifest, since it holds a live credential). Confirmed working end-to-end against the user's own MotherDuck account (47/47 tables, exact row-count match).</t>
         </is>
       </c>
-      <c r="D172" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-28 14:09 PDT</t>
-        </is>
-      </c>
+      <c r="D172" s="2" t="inlineStr"/>
     </row>
     <row r="173">
       <c r="A173" s="2" t="inlineStr">
@@ -4244,11 +3564,7 @@
           <t>6 starter SQL queries against the kinetic MotherDuck database: monthly paid media spend by partner, directly attributed revenue by paid/owned channel, active subscribers by month, non-subscription revenue by month, monthly churn rate, top 5 grossing products per year. Heavily commented to explain modeling choices (e.g. the paid/owned attribution methodology split between storefront orders and subscription invoices).</t>
         </is>
       </c>
-      <c r="D173" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-28 14:09 PDT</t>
-        </is>
-      </c>
+      <c r="D173" s="2" t="inlineStr"/>
     </row>
     <row r="174">
       <c r="A174" s="2" t="inlineStr">
@@ -4266,11 +3582,7 @@
           <t>One-off interactive chart visualizing Query 1's actual output (pasted by the user from their own MotherDuck run): monthly paid media spend by partner, Aug 2023-Jul 2026. Multi-line chart with hover tooltip, legend isolate-toggle, dark mode, and a table view -- built per the dataviz skill (validated categorical palette, accessible contrast handling).</t>
         </is>
       </c>
-      <c r="D174" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-28 14:09 PDT</t>
-        </is>
-      </c>
+      <c r="D174" s="2" t="inlineStr"/>
     </row>
     <row r="175">
       <c r="A175" s="2" t="inlineStr">
@@ -4288,11 +3600,7 @@
           <t>Source for the 'Kinetic -- Marketing &amp; Revenue Overview' MotherDuck Dive -- a live, hosted interactive dashboard (React/Recharts), now organized as 5 tabs. Overview tab: the original 6 starter queries + KPI row. CEO tab: revenue growth/net-new-vs-churned subscribers/CAC payback, revenue mix (subscription vs. course vs. merch). CMO tab: acquisition funnel by channel (sessions -&gt; trial starts -&gt; conversions), retention/app engagement by acquisition channel. CFO tab: CAC and LTV:CAC by acquisition cohort, discount code cost + failed-payment recovery rate + a documented net-margin proxy (no COGS data exists for a true gross margin). Performance Marketing tab: campaign-level spend and platform-self-reported efficiency across all 38 real campaigns (sorted worst-CAC-first), CTR/CVR by platform and ad format. Each new section documents its modeling limits explicitly (e.g. platform-reported vs. site-attributed conversions have no shared join key in this dataset). Re-runs live SQL against the kinetic database on every open. Saved to MotherDuck via the MCP tools; this file is the local source-of-truth copy for sync/history. Live at https://app.motherduck.com/dives/kinetic-marketing-revenue-overview-58909b4e-d301-4794-bb59-ce46f9dc73a6 (dive_id 58909b4e-d301-4794-bb59-ce46f9dc73a6, version 2).</t>
         </is>
       </c>
-      <c r="D175" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-28 14:09 PDT</t>
-        </is>
-      </c>
+      <c r="D175" s="2" t="inlineStr"/>
     </row>
     <row r="176">
       <c r="A176" s="2" t="inlineStr">
@@ -4310,11 +3618,7 @@
           <t>Updated 2026-09-28: real project status (47/47 tables built+validated, live in MotherDuck) + direct link to the live Dive dashboard, replacing the stale 'planning complete, next step Phase 0' placeholder text</t>
         </is>
       </c>
-      <c r="D176" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-28 14:47 PDT</t>
-        </is>
-      </c>
+      <c r="D176" s="2" t="inlineStr"/>
     </row>
     <row r="177">
       <c r="A177" s="2" t="inlineStr">
@@ -4332,11 +3636,7 @@
           <t>Updated 2026-09-28: closed the one open item (brand_lift/holiday-discount-code asymmetry across the 3 Novembers) -- reviewed and confirmed intentional, no data changed</t>
         </is>
       </c>
-      <c r="D177" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-29 13:54 PDT</t>
-        </is>
-      </c>
+      <c r="D177" s="2" t="inlineStr"/>
     </row>
     <row r="178">
       <c r="A178" s="2" t="inlineStr">
@@ -4354,11 +3654,7 @@
           <t>dbt project config for the new semantic layer -- staging views, intermediate views, mart tables</t>
         </is>
       </c>
-      <c r="D178" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-28 14:48 PDT</t>
-        </is>
-      </c>
+      <c r="D178" s="2" t="inlineStr"/>
     </row>
     <row r="179">
       <c r="A179" s="2" t="inlineStr">
@@ -4376,11 +3672,7 @@
           <t>dbt connection profile (MotherDuck md:kinetic, schema dbt_dev); no secrets</t>
         </is>
       </c>
-      <c r="D179" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-29 16:43 PDT</t>
-        </is>
-      </c>
+      <c r="D179" s="2" t="inlineStr"/>
     </row>
     <row r="180">
       <c r="A180" s="2" t="inlineStr">
@@ -4398,11 +3690,7 @@
           <t>Excludes dbt's target/, dbt_packages/, logs/ from git</t>
         </is>
       </c>
-      <c r="D180" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-28 14:48 PDT</t>
-        </is>
-      </c>
+      <c r="D180" s="2" t="inlineStr"/>
     </row>
     <row r="181">
       <c r="A181" s="2" t="inlineStr">
@@ -4420,11 +3708,7 @@
           <t>How to install dbt-core + dbt-duckdb and run this project locally against MotherDuck (neither of Claude's environments can reach motherduck.com directly, so dbt run/test must be executed on the user's own machine)</t>
         </is>
       </c>
-      <c r="D181" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-29 22:12 PDT</t>
-        </is>
-      </c>
+      <c r="D181" s="2" t="inlineStr"/>
     </row>
     <row r="182">
       <c r="A182" s="2" t="inlineStr">
@@ -4442,11 +3726,7 @@
           <t>Declares all 47 raw kinetic tables as dbt sources, so every staging model references source() rather than a hardcoded table name</t>
         </is>
       </c>
-      <c r="D182" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-28 14:48 PDT</t>
-        </is>
-      </c>
+      <c r="D182" s="2" t="inlineStr"/>
     </row>
     <row r="183">
       <c r="A183" s="2" t="inlineStr">
@@ -4464,11 +3744,7 @@
           <t>Staging model: 1:1 pass-through of customers with light renaming</t>
         </is>
       </c>
-      <c r="D183" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-28 14:48 PDT</t>
-        </is>
-      </c>
+      <c r="D183" s="2" t="inlineStr"/>
     </row>
     <row r="184">
       <c r="A184" s="2" t="inlineStr">
@@ -4486,11 +3762,7 @@
           <t>Staging model: 1:1 pass-through of subscription_plans</t>
         </is>
       </c>
-      <c r="D184" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-28 14:48 PDT</t>
-        </is>
-      </c>
+      <c r="D184" s="2" t="inlineStr"/>
     </row>
     <row r="185">
       <c r="A185" s="2" t="inlineStr">
@@ -4508,11 +3780,7 @@
           <t>Staging model: 1:1 pass-through of subscriptions</t>
         </is>
       </c>
-      <c r="D185" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-28 14:48 PDT</t>
-        </is>
-      </c>
+      <c r="D185" s="2" t="inlineStr"/>
     </row>
     <row r="186">
       <c r="A186" s="2" t="inlineStr">
@@ -4530,11 +3798,7 @@
           <t>Staging model: 1:1 pass-through of invoices</t>
         </is>
       </c>
-      <c r="D186" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-28 14:48 PDT</t>
-        </is>
-      </c>
+      <c r="D186" s="2" t="inlineStr"/>
     </row>
     <row r="187">
       <c r="A187" s="2" t="inlineStr">
@@ -4552,11 +3816,7 @@
           <t>Staging model: 1:1 pass-through of products</t>
         </is>
       </c>
-      <c r="D187" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-28 14:48 PDT</t>
-        </is>
-      </c>
+      <c r="D187" s="2" t="inlineStr"/>
     </row>
     <row r="188">
       <c r="A188" s="2" t="inlineStr">
@@ -4574,11 +3834,7 @@
           <t>not_null/unique/relationships tests for the Phase 1/2 staging models</t>
         </is>
       </c>
-      <c r="D188" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-29 22:11 PDT</t>
-        </is>
-      </c>
+      <c r="D188" s="2" t="inlineStr"/>
     </row>
     <row r="189">
       <c r="A189" s="2" t="inlineStr">
@@ -4596,11 +3852,7 @@
           <t>Intermediate model: resolves each subscription's true paid-start date (trial-vs-paid logic), defined once so every downstream mart agrees</t>
         </is>
       </c>
-      <c r="D189" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-28 14:48 PDT</t>
-        </is>
-      </c>
+      <c r="D189" s="2" t="inlineStr"/>
     </row>
     <row r="190">
       <c r="A190" s="2" t="inlineStr">
@@ -4618,11 +3870,7 @@
           <t>Descriptions and tests for all intermediate models</t>
         </is>
       </c>
-      <c r="D190" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-29 22:12 PDT</t>
-        </is>
-      </c>
+      <c r="D190" s="2" t="inlineStr"/>
     </row>
     <row r="191">
       <c r="A191" s="2" t="inlineStr">
@@ -4640,11 +3888,7 @@
           <t>First canonical metric mart: active subscribers + MRR/ARR by month, validated against a hand-run equivalent query on the live database (2026-07: 90 active subscribers, ~$2,133 MRR)</t>
         </is>
       </c>
-      <c r="D191" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-29 22:07 PDT</t>
-        </is>
-      </c>
+      <c r="D191" s="2" t="inlineStr"/>
     </row>
     <row r="192">
       <c r="A192" s="2" t="inlineStr">
@@ -4662,11 +3906,7 @@
           <t>Tests for mart_mrr_monthly</t>
         </is>
       </c>
-      <c r="D192" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-29 22:12 PDT</t>
-        </is>
-      </c>
+      <c r="D192" s="2" t="inlineStr"/>
     </row>
     <row r="193">
       <c r="A193" s="2" t="inlineStr">
@@ -4684,11 +3924,7 @@
           <t>Updated: what's built so far now includes the Phase 3 storefront staging models + mart_storefront_revenue_monthly</t>
         </is>
       </c>
-      <c r="D193" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-29 22:12 PDT</t>
-        </is>
-      </c>
+      <c r="D193" s="2" t="inlineStr"/>
     </row>
     <row r="194">
       <c r="A194" s="2" t="inlineStr">
@@ -4706,11 +3942,7 @@
           <t>Staging model: 1:1 pass-through of orders, plus is_guest_order/has_discount convenience booleans</t>
         </is>
       </c>
-      <c r="D194" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-28 14:53 PDT</t>
-        </is>
-      </c>
+      <c r="D194" s="2" t="inlineStr"/>
     </row>
     <row r="195">
       <c r="A195" s="2" t="inlineStr">
@@ -4728,11 +3960,7 @@
           <t>Staging model: 1:1 pass-through of order_line_items</t>
         </is>
       </c>
-      <c r="D195" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-28 14:53 PDT</t>
-        </is>
-      </c>
+      <c r="D195" s="2" t="inlineStr"/>
     </row>
     <row r="196">
       <c r="A196" s="2" t="inlineStr">
@@ -4750,11 +3978,7 @@
           <t>Staging model: 1:1 pass-through of payments</t>
         </is>
       </c>
-      <c r="D196" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-28 14:53 PDT</t>
-        </is>
-      </c>
+      <c r="D196" s="2" t="inlineStr"/>
     </row>
     <row r="197">
       <c r="A197" s="2" t="inlineStr">
@@ -4772,11 +3996,7 @@
           <t>Staging model: 1:1 pass-through of refunds</t>
         </is>
       </c>
-      <c r="D197" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-28 14:53 PDT</t>
-        </is>
-      </c>
+      <c r="D197" s="2" t="inlineStr"/>
     </row>
     <row r="198">
       <c r="A198" s="2" t="inlineStr">
@@ -4794,11 +4014,7 @@
           <t>Staging model: 1:1 pass-through of discount_codes</t>
         </is>
       </c>
-      <c r="D198" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-28 14:53 PDT</t>
-        </is>
-      </c>
+      <c r="D198" s="2" t="inlineStr"/>
     </row>
     <row r="199">
       <c r="A199" s="2" t="inlineStr">
@@ -4816,11 +4032,7 @@
           <t>Intermediate model: per-order total of succeeded refunds only (failed/pending refunds don't reduce reported revenue)</t>
         </is>
       </c>
-      <c r="D199" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-28 14:53 PDT</t>
-        </is>
-      </c>
+      <c r="D199" s="2" t="inlineStr"/>
     </row>
     <row r="200">
       <c r="A200" s="2" t="inlineStr">
@@ -4838,11 +4050,7 @@
           <t>Intermediate model: lookup from every web anonymous_id and account email to its customer (guest emails matched by email; anonymous sessions back-filled; deleted accounts excluded)</t>
         </is>
       </c>
-      <c r="D200" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-29 16:39 PDT</t>
-        </is>
-      </c>
+      <c r="D200" s="2" t="inlineStr"/>
     </row>
     <row r="201">
       <c r="A201" s="2" t="inlineStr">
@@ -4860,11 +4068,7 @@
           <t>Intermediate model: one row per order with gross (pre-discount), discount, paid, succeeded-refund and net amounts, plus customer_id resolved for guest orders via email match</t>
         </is>
       </c>
-      <c r="D201" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-29 22:05 PDT</t>
-        </is>
-      </c>
+      <c r="D201" s="2" t="inlineStr"/>
     </row>
     <row r="202">
       <c r="A202" s="2" t="inlineStr">
@@ -4882,11 +4086,7 @@
           <t>dbt test: fails if any order's net is below zero (net is deliberately not floored)</t>
         </is>
       </c>
-      <c r="D202" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-29 17:18 PDT</t>
-        </is>
-      </c>
+      <c r="D202" s="2" t="inlineStr"/>
     </row>
     <row r="203">
       <c r="A203" s="2" t="inlineStr">
@@ -4904,11 +4104,7 @@
           <t>dbt test: gross - discount = paid and paid - refund = net on every order</t>
         </is>
       </c>
-      <c r="D203" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-29 17:18 PDT</t>
-        </is>
-      </c>
+      <c r="D203" s="2" t="inlineStr"/>
     </row>
     <row r="204">
       <c r="A204" s="2" t="inlineStr">
@@ -4926,11 +4122,7 @@
           <t>dbt test: total refunds in int_orders_net equal total succeeded refunds in int_orders_refunded</t>
         </is>
       </c>
-      <c r="D204" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-29 17:18 PDT</t>
-        </is>
-      </c>
+      <c r="D204" s="2" t="inlineStr"/>
     </row>
     <row r="205">
       <c r="A205" s="2" t="inlineStr">
@@ -4948,11 +4140,7 @@
           <t>Intermediate model: one row per web or app session, with customer_id resolved (known at the time, or back-filled from the visitor's anonymous_id via int_customer_identity)</t>
         </is>
       </c>
-      <c r="D205" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-29 17:23 PDT</t>
-        </is>
-      </c>
+      <c r="D205" s="2" t="inlineStr"/>
     </row>
     <row r="206">
       <c r="A206" s="2" t="inlineStr">
@@ -4970,11 +4158,7 @@
           <t>dbt test: customer_id is null exactly when a session is anonymous</t>
         </is>
       </c>
-      <c r="D206" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-29 17:23 PDT</t>
-        </is>
-      </c>
+      <c r="D206" s="2" t="inlineStr"/>
     </row>
     <row r="207">
       <c r="A207" s="2" t="inlineStr">
@@ -4992,11 +4176,7 @@
           <t>dbt test: unified session count equals web + app session counts</t>
         </is>
       </c>
-      <c r="D207" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-29 17:23 PDT</t>
-        </is>
-      </c>
+      <c r="D207" s="2" t="inlineStr"/>
     </row>
     <row r="208">
       <c r="A208" s="2" t="inlineStr">
@@ -5014,11 +4194,7 @@
           <t>dbt test: no session ends before it starts</t>
         </is>
       </c>
-      <c r="D208" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-29 17:23 PDT</t>
-        </is>
-      </c>
+      <c r="D208" s="2" t="inlineStr"/>
     </row>
     <row r="209">
       <c r="A209" s="2" t="inlineStr">
@@ -5036,11 +4212,7 @@
           <t>Runbook for the unattended overnight run: queue, rules, stop rules, morning list format</t>
         </is>
       </c>
-      <c r="D209" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-29 22:12 PDT</t>
-        </is>
-      </c>
+      <c r="D209" s="2" t="inlineStr"/>
     </row>
     <row r="210">
       <c r="A210" s="2" t="inlineStr">
@@ -5058,11 +4230,7 @@
           <t>Overnight runbook variant for Claude Code: dbt builds and branch pushes allowed</t>
         </is>
       </c>
-      <c r="D210" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-29 18:55 PDT</t>
-        </is>
-      </c>
+      <c r="D210" s="2" t="inlineStr"/>
     </row>
     <row r="211">
       <c r="A211" s="2" t="inlineStr">
@@ -5080,11 +4248,7 @@
           <t>Claude Code project instructions: standing rules, dbt/git/MotherDuck limits, start-of-session reading</t>
         </is>
       </c>
-      <c r="D211" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-30 08:34 PDT</t>
-        </is>
-      </c>
+      <c r="D211" s="2" t="inlineStr"/>
     </row>
     <row r="212">
       <c r="A212" s="2" t="inlineStr">
@@ -5102,11 +4266,7 @@
           <t>Claude Code permissions: allow dbt/git commit/push overnight branch; deny push to master, force push, rm</t>
         </is>
       </c>
-      <c r="D212" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-30 08:34 PDT</t>
-        </is>
-      </c>
+      <c r="D212" s="2" t="inlineStr"/>
     </row>
     <row r="213">
       <c r="A213" s="2" t="inlineStr">
@@ -5124,11 +4284,7 @@
           <t>Second canonical metric mart: non-subscription (course+merch) gross/net revenue, AOV, guest-checkout share, discount-usage share, refund rate by month -- validated against a hand-run equivalent query on the live database (2026-07: 246 orders, $13,843.71 gross revenue, $56.28 AOV)</t>
         </is>
       </c>
-      <c r="D213" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-29 22:05 PDT</t>
-        </is>
-      </c>
+      <c r="D213" s="2" t="inlineStr"/>
     </row>
     <row r="214">
       <c r="A214" s="2" t="inlineStr">
@@ -5146,11 +4302,7 @@
           <t>Phase 2 staging (Customer 360): 1:1 pass-through of customer_addresses</t>
         </is>
       </c>
-      <c r="D214" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-29 10:26 PDT</t>
-        </is>
-      </c>
+      <c r="D214" s="2" t="inlineStr"/>
     </row>
     <row r="215">
       <c r="A215" s="2" t="inlineStr">
@@ -5168,11 +4320,7 @@
           <t>Phase 2 staging (Customer 360): 1:1 pass-through of devices, plus is_anonymous_device flag (customer_id null for ~94% of devices by design)</t>
         </is>
       </c>
-      <c r="D215" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-29 10:26 PDT</t>
-        </is>
-      </c>
+      <c r="D215" s="2" t="inlineStr"/>
     </row>
     <row r="216">
       <c r="A216" s="2" t="inlineStr">
@@ -5190,11 +4338,7 @@
           <t>Phase 2 staging (Customer 360): 1:1 pass-through of identity_map</t>
         </is>
       </c>
-      <c r="D216" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-29 10:26 PDT</t>
-        </is>
-      </c>
+      <c r="D216" s="2" t="inlineStr"/>
     </row>
     <row r="217">
       <c r="A217" s="2" t="inlineStr">
@@ -5212,11 +4356,7 @@
           <t>Phase 2 staging (Customer 360): 1:1 pass-through of segments</t>
         </is>
       </c>
-      <c r="D217" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-29 10:26 PDT</t>
-        </is>
-      </c>
+      <c r="D217" s="2" t="inlineStr"/>
     </row>
     <row r="218">
       <c r="A218" s="2" t="inlineStr">
@@ -5234,11 +4374,7 @@
           <t>Phase 2 staging (Customer 360): 1:1 pass-through of customer_segment_membership, plus is_current_member flag</t>
         </is>
       </c>
-      <c r="D218" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-29 10:26 PDT</t>
-        </is>
-      </c>
+      <c r="D218" s="2" t="inlineStr"/>
     </row>
     <row r="219">
       <c r="A219" s="2" t="inlineStr">
@@ -5256,11 +4392,7 @@
           <t>Phase 2 staging (Customer 360): 1:1 pass-through of subscription_events; old_plan/new_plan renamed to old_plan_id/new_plan_id</t>
         </is>
       </c>
-      <c r="D219" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-29 10:26 PDT</t>
-        </is>
-      </c>
+      <c r="D219" s="2" t="inlineStr"/>
     </row>
     <row r="220">
       <c r="A220" s="2" t="inlineStr">
@@ -5278,11 +4410,7 @@
           <t>Updated: tests for the 6 Customer 360 staging models (PK not_null/unique, FK relationships) -- all hand-verified against live data first</t>
         </is>
       </c>
-      <c r="D220" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-29 22:11 PDT</t>
-        </is>
-      </c>
+      <c r="D220" s="2" t="inlineStr"/>
     </row>
     <row r="221">
       <c r="A221" s="2" t="inlineStr">
@@ -5300,11 +4428,7 @@
           <t>Phase 2 staging (web/app engagement): 1:1 pass-through of web_sessions, plus is_known_customer flag (customer_id null for ~79% of sessions by design)</t>
         </is>
       </c>
-      <c r="D221" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-29 12:58 PDT</t>
-        </is>
-      </c>
+      <c r="D221" s="2" t="inlineStr"/>
     </row>
     <row r="222">
       <c r="A222" s="2" t="inlineStr">
@@ -5322,11 +4446,7 @@
           <t>Phase 2 staging (web/app engagement): 1:1 pass-through of web_events</t>
         </is>
       </c>
-      <c r="D222" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-29 12:58 PDT</t>
-        </is>
-      </c>
+      <c r="D222" s="2" t="inlineStr"/>
     </row>
     <row r="223">
       <c r="A223" s="2" t="inlineStr">
@@ -5344,11 +4464,7 @@
           <t>Phase 2 staging (web/app engagement): 1:1 pass-through of app_sessions</t>
         </is>
       </c>
-      <c r="D223" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-29 12:58 PDT</t>
-        </is>
-      </c>
+      <c r="D223" s="2" t="inlineStr"/>
     </row>
     <row r="224">
       <c r="A224" s="2" t="inlineStr">
@@ -5366,11 +4482,7 @@
           <t>Phase 2 staging (web/app engagement): 1:1 pass-through of app_events</t>
         </is>
       </c>
-      <c r="D224" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-29 12:58 PDT</t>
-        </is>
-      </c>
+      <c r="D224" s="2" t="inlineStr"/>
     </row>
     <row r="225">
       <c r="A225" s="2" t="inlineStr">
@@ -5388,11 +4500,7 @@
           <t>Updated: tests for the 4 web/app engagement staging models -- all hand-verified against live data first</t>
         </is>
       </c>
-      <c r="D225" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-29 22:11 PDT</t>
-        </is>
-      </c>
+      <c r="D225" s="2" t="inlineStr"/>
     </row>
     <row r="226">
       <c r="A226" s="2" t="inlineStr">
@@ -5410,11 +4518,7 @@
           <t>Phase 2 staging (email/push): 1:1 pass-through of braze_email_campaigns</t>
         </is>
       </c>
-      <c r="D226" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-29 12:59 PDT</t>
-        </is>
-      </c>
+      <c r="D226" s="2" t="inlineStr"/>
     </row>
     <row r="227">
       <c r="A227" s="2" t="inlineStr">
@@ -5432,11 +4536,7 @@
           <t>Phase 2 staging (email/push): 1:1 pass-through of braze_push_campaigns</t>
         </is>
       </c>
-      <c r="D227" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-29 12:59 PDT</t>
-        </is>
-      </c>
+      <c r="D227" s="2" t="inlineStr"/>
     </row>
     <row r="228">
       <c r="A228" s="2" t="inlineStr">
@@ -5454,11 +4554,7 @@
           <t>Phase 2 staging (email/push): braze_email_events with external_user_id renamed to customer_id and a short event_name (send/open/click/bounce/unsubscribe) alongside Braze's raw event_type</t>
         </is>
       </c>
-      <c r="D228" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-29 12:59 PDT</t>
-        </is>
-      </c>
+      <c r="D228" s="2" t="inlineStr"/>
     </row>
     <row r="229">
       <c r="A229" s="2" t="inlineStr">
@@ -5476,11 +4572,7 @@
           <t>Phase 2 staging (email/push): braze_push_events with external_user_id renamed to customer_id and a short event_name alongside Braze's raw event_type</t>
         </is>
       </c>
-      <c r="D229" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-29 12:59 PDT</t>
-        </is>
-      </c>
+      <c r="D229" s="2" t="inlineStr"/>
     </row>
     <row r="230">
       <c r="A230" s="2" t="inlineStr">
@@ -5498,11 +4590,7 @@
           <t>Updated: tests for the 4 Braze staging models, incl. accepted_values on event_name -- all hand-verified against live data first</t>
         </is>
       </c>
-      <c r="D230" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-29 22:11 PDT</t>
-        </is>
-      </c>
+      <c r="D230" s="2" t="inlineStr"/>
     </row>
     <row r="231">
       <c r="A231" s="2" t="inlineStr">
@@ -5520,11 +4608,7 @@
           <t>Phase 2 staging (paid media: Meta): meta_campaigns with budgets in both raw cents and dollars (Meta API stores budgets in cents)</t>
         </is>
       </c>
-      <c r="D231" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-29 13:02 PDT</t>
-        </is>
-      </c>
+      <c r="D231" s="2" t="inlineStr"/>
     </row>
     <row r="232">
       <c r="A232" s="2" t="inlineStr">
@@ -5542,11 +4626,7 @@
           <t>Phase 2 staging (paid media: Meta): 1:1 pass-through of meta_ads</t>
         </is>
       </c>
-      <c r="D232" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-29 13:02 PDT</t>
-        </is>
-      </c>
+      <c r="D232" s="2" t="inlineStr"/>
     </row>
     <row r="233">
       <c r="A233" s="2" t="inlineStr">
@@ -5564,11 +4644,7 @@
           <t>Phase 2 staging (paid media: Meta): meta_ad_insights_daily with a combined ad_day_id key, unit-suffixed columns (spend_usd, cpm_usd, cpc_usd) and ctr renamed ctr_fraction (0.017 = 1.7%)</t>
         </is>
       </c>
-      <c r="D233" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-29 13:02 PDT</t>
-        </is>
-      </c>
+      <c r="D233" s="2" t="inlineStr"/>
     </row>
     <row r="234">
       <c r="A234" s="2" t="inlineStr">
@@ -5586,11 +4662,7 @@
           <t>Phase 2 staging (paid media: Meta): meta_ad_actions_daily with a combined ad_day_action_id key; value renamed action_count</t>
         </is>
       </c>
-      <c r="D234" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-29 13:02 PDT</t>
-        </is>
-      </c>
+      <c r="D234" s="2" t="inlineStr"/>
     </row>
     <row r="235">
       <c r="A235" s="2" t="inlineStr">
@@ -5608,11 +4680,7 @@
           <t>Updated: tests for the 4 Meta staging models, incl. uniqueness of the combined daily keys -- all hand-verified against live data first</t>
         </is>
       </c>
-      <c r="D235" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-29 22:11 PDT</t>
-        </is>
-      </c>
+      <c r="D235" s="2" t="inlineStr"/>
     </row>
     <row r="236">
       <c r="A236" s="2" t="inlineStr">
@@ -5630,11 +4698,7 @@
           <t>Phase 2 staging (paid media: Google Search): campaigns with the raw customer_id renamed google_ads_account_id (it's the Google Ads account number, not a Kinetic customer), daily budget in micros and dollars, end_date cast back to a date</t>
         </is>
       </c>
-      <c r="D236" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-29 13:13 PDT</t>
-        </is>
-      </c>
+      <c r="D236" s="2" t="inlineStr"/>
     </row>
     <row r="237">
       <c r="A237" s="2" t="inlineStr">
@@ -5652,11 +4716,7 @@
           <t>Phase 2 staging (paid media: Google Search): ad groups; cpc_bid_micros cast back to a number (always empty -- automated bidding)</t>
         </is>
       </c>
-      <c r="D237" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-29 13:13 PDT</t>
-        </is>
-      </c>
+      <c r="D237" s="2" t="inlineStr"/>
     </row>
     <row r="238">
       <c r="A238" s="2" t="inlineStr">
@@ -5674,11 +4734,7 @@
           <t>Phase 2 staging (paid media: Google Search): ad-group-day performance with combined ad_group_day_id key, cost converted from micros to dollars, ctr_fraction. The keyword table rolled up -- never add the two together</t>
         </is>
       </c>
-      <c r="D238" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-29 13:13 PDT</t>
-        </is>
-      </c>
+      <c r="D238" s="2" t="inlineStr"/>
     </row>
     <row r="239">
       <c r="A239" s="2" t="inlineStr">
@@ -5696,11 +4752,7 @@
           <t>Phase 2 staging (paid media: Google Search): keyword-day performance with combined keyword_day_id key, cost converted from micros to dollars, ctr_fraction</t>
         </is>
       </c>
-      <c r="D239" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-29 13:13 PDT</t>
-        </is>
-      </c>
+      <c r="D239" s="2" t="inlineStr"/>
     </row>
     <row r="240">
       <c r="A240" s="2" t="inlineStr">
@@ -5718,11 +4770,7 @@
           <t>Updated: tests for the 4 Google Search staging models -- all hand-verified against live data first</t>
         </is>
       </c>
-      <c r="D240" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-29 22:11 PDT</t>
-        </is>
-      </c>
+      <c r="D240" s="2" t="inlineStr"/>
     </row>
     <row r="241">
       <c r="A241" s="2" t="inlineStr">
@@ -5740,11 +4788,7 @@
           <t>Phase 2 staging (paid media: YouTube): campaigns with customer_id renamed google_ads_account_id (the ad account, not a Kinetic customer), budgets in micros and dollars</t>
         </is>
       </c>
-      <c r="D241" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-29 13:14 PDT</t>
-        </is>
-      </c>
+      <c r="D241" s="2" t="inlineStr"/>
     </row>
     <row r="242">
       <c r="A242" s="2" t="inlineStr">
@@ -5762,11 +4806,7 @@
           <t>Phase 2 staging (paid media: YouTube): 1:1 pass-through of youtube_ad_groups</t>
         </is>
       </c>
-      <c r="D242" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-29 13:14 PDT</t>
-        </is>
-      </c>
+      <c r="D242" s="2" t="inlineStr"/>
     </row>
     <row r="243">
       <c r="A243" s="2" t="inlineStr">
@@ -5784,11 +4824,7 @@
           <t>Phase 2 staging (paid media: YouTube): ad-group-day performance with combined ad_group_day_id key, cost and cost-per-view converted from micros to dollars, video_view_rate_fraction</t>
         </is>
       </c>
-      <c r="D243" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-29 13:14 PDT</t>
-        </is>
-      </c>
+      <c r="D243" s="2" t="inlineStr"/>
     </row>
     <row r="244">
       <c r="A244" s="2" t="inlineStr">
@@ -5806,11 +4842,7 @@
           <t>Updated: tests for the 3 YouTube staging models -- all hand-verified against live data first</t>
         </is>
       </c>
-      <c r="D244" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-29 22:11 PDT</t>
-        </is>
-      </c>
+      <c r="D244" s="2" t="inlineStr"/>
     </row>
     <row r="245">
       <c r="A245" s="2" t="inlineStr">
@@ -5828,11 +4860,7 @@
           <t>Phase 2 staging (paid media: DV360): insertion orders with budget_micros named monthly_budget_* (it's a monthly budget), end_date cast back to a date; flags the flat-budget-vs-growing-spend known issue</t>
         </is>
       </c>
-      <c r="D245" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-29 13:27 PDT</t>
-        </is>
-      </c>
+      <c r="D245" s="2" t="inlineStr"/>
     </row>
     <row r="246">
       <c r="A246" s="2" t="inlineStr">
@@ -5850,11 +4878,7 @@
           <t>Phase 2 staging (paid media: DV360): 1:1 pass-through of dv360_line_items</t>
         </is>
       </c>
-      <c r="D246" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-29 13:19 PDT</t>
-        </is>
-      </c>
+      <c r="D246" s="2" t="inlineStr"/>
     </row>
     <row r="247">
       <c r="A247" s="2" t="inlineStr">
@@ -5872,11 +4896,7 @@
           <t>Phase 2 staging (paid media: DV360): line-item x day x exchange x environment performance with combined line_item_day_slice_id key, micros converted to dollars, ctr_fraction</t>
         </is>
       </c>
-      <c r="D247" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-29 13:19 PDT</t>
-        </is>
-      </c>
+      <c r="D247" s="2" t="inlineStr"/>
     </row>
     <row r="248">
       <c r="A248" s="2" t="inlineStr">
@@ -5894,11 +4914,7 @@
           <t>Updated: tests for the 3 DV360 staging models, incl. accepted_values on exchange and environment -- all hand-verified against live data first</t>
         </is>
       </c>
-      <c r="D248" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-29 22:11 PDT</t>
-        </is>
-      </c>
+      <c r="D248" s="2" t="inlineStr"/>
     </row>
     <row r="249">
       <c r="A249" s="2" t="inlineStr">
@@ -5916,11 +4932,7 @@
           <t>Updated 2026-09-29: every evergreen ad budget on all 6 platforms is now the campaign's CURRENT budget, sized from realized spend (weekly average &lt;= budget, no day &gt; 1.75x; DV360 monthly &gt;= highest month). The old flat 'typical day' budgets let later months spend up to ~20x the stored budget</t>
         </is>
       </c>
-      <c r="D249" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-29 13:23 PDT</t>
-        </is>
-      </c>
+      <c r="D249" s="2" t="inlineStr"/>
     </row>
     <row r="250">
       <c r="A250" s="2" t="inlineStr">
@@ -5938,11 +4950,7 @@
           <t>Regenerated 2026-09-29: evergreen daily_budget values updated to current budgets (only that column, only the 4 evergreen rows changed)</t>
         </is>
       </c>
-      <c r="D250" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-29 13:24 PDT</t>
-        </is>
-      </c>
+      <c r="D250" s="2" t="inlineStr"/>
     </row>
     <row r="251">
       <c r="A251" s="2" t="inlineStr">
@@ -5960,11 +4968,7 @@
           <t>Regenerated 2026-09-29: campaign_budget_micros updated to current budgets (only that column changed)</t>
         </is>
       </c>
-      <c r="D251" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-29 13:24 PDT</t>
-        </is>
-      </c>
+      <c r="D251" s="2" t="inlineStr"/>
     </row>
     <row r="252">
       <c r="A252" s="2" t="inlineStr">
@@ -5982,11 +4986,7 @@
           <t>Regenerated 2026-09-29: evergreen campaign_budget_micros updated to current budgets (only that column, only the 4 evergreen rows changed)</t>
         </is>
       </c>
-      <c r="D252" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-29 13:24 PDT</t>
-        </is>
-      </c>
+      <c r="D252" s="2" t="inlineStr"/>
     </row>
     <row r="253">
       <c r="A253" s="2" t="inlineStr">
@@ -6004,11 +5004,7 @@
           <t>Regenerated 2026-09-29: monthly budget_micros updated to current budgets (only that column changed)</t>
         </is>
       </c>
-      <c r="D253" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-29 13:24 PDT</t>
-        </is>
-      </c>
+      <c r="D253" s="2" t="inlineStr"/>
     </row>
     <row r="254">
       <c r="A254" s="2" t="inlineStr">
@@ -6026,11 +5022,7 @@
           <t>Regenerated 2026-09-29: evergreen daily_budget_micro updated to current budgets (only that column, only the 4 evergreen rows changed)</t>
         </is>
       </c>
-      <c r="D254" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-29 13:24 PDT</t>
-        </is>
-      </c>
+      <c r="D254" s="2" t="inlineStr"/>
     </row>
     <row r="255">
       <c r="A255" s="2" t="inlineStr">
@@ -6048,11 +5040,7 @@
           <t>Regenerated 2026-09-29: BUDGET_MODE_DAY budget_micro updated to current budgets (only that column, only the 4 evergreen rows changed)</t>
         </is>
       </c>
-      <c r="D255" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-29 13:24 PDT</t>
-        </is>
-      </c>
+      <c r="D255" s="2" t="inlineStr"/>
     </row>
     <row r="256">
       <c r="A256" s="2" t="inlineStr">
@@ -6070,11 +5058,7 @@
           <t>Updated 2026-09-29: new Check 8 -- spend vs stored budget for every campaign on all 6 platforms (weekly/daily limits for daily budgets, monthly for DV360, total for holiday flights)</t>
         </is>
       </c>
-      <c r="D256" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-29 13:30 PDT</t>
-        </is>
-      </c>
+      <c r="D256" s="2" t="inlineStr"/>
     </row>
     <row r="257">
       <c r="A257" s="2" t="inlineStr">
@@ -6092,11 +5076,7 @@
           <t>Updated: budget known-issue note replaced -- budgets are now current budgets</t>
         </is>
       </c>
-      <c r="D257" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-29 13:27 PDT</t>
-        </is>
-      </c>
+      <c r="D257" s="2" t="inlineStr"/>
     </row>
     <row r="258">
       <c r="A258" s="2" t="inlineStr">
@@ -6114,11 +5094,7 @@
           <t>Updated 2026-09-29: new cap_flight_at_budget() -- rescales a holiday flight's days so it never spends past its lifetime budget, replaying the same random rates so every other row is unchanged</t>
         </is>
       </c>
-      <c r="D258" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-29 13:29 PDT</t>
-        </is>
-      </c>
+      <c r="D258" s="2" t="inlineStr"/>
     </row>
     <row r="259">
       <c r="A259" s="2" t="inlineStr">
@@ -6136,11 +5112,7 @@
           <t>Updated 2026-09-29: holiday flights capped at their lifetime budget via cap_flight_at_budget()</t>
         </is>
       </c>
-      <c r="D259" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-29 13:29 PDT</t>
-        </is>
-      </c>
+      <c r="D259" s="2" t="inlineStr"/>
     </row>
     <row r="260">
       <c r="A260" s="2" t="inlineStr">
@@ -6158,11 +5130,7 @@
           <t>Updated 2026-09-29: holiday flights capped at their lifetime budget via cap_flight_at_budget()</t>
         </is>
       </c>
-      <c r="D260" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-29 13:29 PDT</t>
-        </is>
-      </c>
+      <c r="D260" s="2" t="inlineStr"/>
     </row>
     <row r="261">
       <c r="A261" s="2" t="inlineStr">
@@ -6180,11 +5148,7 @@
           <t>Updated 2026-09-29: holiday flights capped at their lifetime budget via cap_flight_at_budget()</t>
         </is>
       </c>
-      <c r="D261" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-29 13:29 PDT</t>
-        </is>
-      </c>
+      <c r="D261" s="2" t="inlineStr"/>
     </row>
     <row r="262">
       <c r="A262" s="2" t="inlineStr">
@@ -6202,11 +5166,7 @@
           <t>Updated 2026-09-29: holiday flights capped at their lifetime budget via cap_flight_at_budget() (no-op today -- all YouTube flights were already under budget)</t>
         </is>
       </c>
-      <c r="D262" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-29 13:29 PDT</t>
-        </is>
-      </c>
+      <c r="D262" s="2" t="inlineStr"/>
     </row>
     <row r="263">
       <c r="A263" s="2" t="inlineStr">
@@ -6224,11 +5184,7 @@
           <t>Regenerated 2026-09-29: the 2023 and 2024 holiday flights (38 rows) trimmed to spend exactly their lifetime budget; every other row identical</t>
         </is>
       </c>
-      <c r="D263" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-29 13:29 PDT</t>
-        </is>
-      </c>
+      <c r="D263" s="2" t="inlineStr"/>
     </row>
     <row r="264">
       <c r="A264" s="2" t="inlineStr">
@@ -6246,11 +5202,7 @@
           <t>Regenerated 2026-09-29: re-derived from the trimmed insights rows -- only the 2023/2024 holiday flights' action rows changed (one initiate_checkout row on 2024-11-15 dropped to zero and is no longer emitted)</t>
         </is>
       </c>
-      <c r="D264" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-29 13:29 PDT</t>
-        </is>
-      </c>
+      <c r="D264" s="2" t="inlineStr"/>
     </row>
     <row r="265">
       <c r="A265" s="2" t="inlineStr">
@@ -6268,11 +5220,7 @@
           <t>Regenerated 2026-09-29: the 2024 holiday flight (19 rows) trimmed to spend exactly its lifetime budget; every other row identical</t>
         </is>
       </c>
-      <c r="D265" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-29 13:29 PDT</t>
-        </is>
-      </c>
+      <c r="D265" s="2" t="inlineStr"/>
     </row>
     <row r="266">
       <c r="A266" s="2" t="inlineStr">
@@ -6290,11 +5238,7 @@
           <t>Regenerated 2026-09-29: the 2023/2024/2025 holiday flights (56 rows) trimmed to spend exactly their lifetime budgets; every other row identical</t>
         </is>
       </c>
-      <c r="D266" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-29 13:29 PDT</t>
-        </is>
-      </c>
+      <c r="D266" s="2" t="inlineStr"/>
     </row>
     <row r="267">
       <c r="A267" s="2" t="inlineStr">
@@ -6312,11 +5256,7 @@
           <t>Updated 2026-09-29: added Check 8 (spend vs stored budget) with both fixes and results</t>
         </is>
       </c>
-      <c r="D267" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-29 13:54 PDT</t>
-        </is>
-      </c>
+      <c r="D267" s="2" t="inlineStr"/>
     </row>
     <row r="268">
       <c r="A268" s="2" t="inlineStr">
@@ -6334,11 +5274,7 @@
           <t>Updated 2026-09-29: Check 8's flight limit tightened from 1.05x to 1.0x now that flights are capped</t>
         </is>
       </c>
-      <c r="D268" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-29 13:30 PDT</t>
-        </is>
-      </c>
+      <c r="D268" s="2" t="inlineStr"/>
     </row>
     <row r="269">
       <c r="A269" s="2" t="inlineStr">
@@ -6356,11 +5292,7 @@
           <t>Phase 2 staging (paid media: Snap): campaigns with ad_account_id renamed snap_ad_account_id, current budgets in micros and dollars</t>
         </is>
       </c>
-      <c r="D269" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-29 15:53 PDT</t>
-        </is>
-      </c>
+      <c r="D269" s="2" t="inlineStr"/>
     </row>
     <row r="270">
       <c r="A270" s="2" t="inlineStr">
@@ -6378,11 +5310,7 @@
           <t>Phase 2 staging (paid media: Snap): 1:1 pass-through of snap_ad_squads (Snap's ad set / ad group level)</t>
         </is>
       </c>
-      <c r="D270" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-29 15:53 PDT</t>
-        </is>
-      </c>
+      <c r="D270" s="2" t="inlineStr"/>
     </row>
     <row r="271">
       <c r="A271" s="2" t="inlineStr">
@@ -6400,11 +5328,7 @@
           <t>Phase 2 staging (paid media: Snap): 1:1 pass-through of snap_ads</t>
         </is>
       </c>
-      <c r="D271" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-29 15:53 PDT</t>
-        </is>
-      </c>
+      <c r="D271" s="2" t="inlineStr"/>
     </row>
     <row r="272">
       <c r="A272" s="2" t="inlineStr">
@@ -6422,11 +5346,7 @@
           <t>Phase 2 staging (paid media: Snap): ad-day stats with combined ad_day_id key, spend in micros and dollars; documents swipes as Snap's clicks</t>
         </is>
       </c>
-      <c r="D272" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-29 15:53 PDT</t>
-        </is>
-      </c>
+      <c r="D272" s="2" t="inlineStr"/>
     </row>
     <row r="273">
       <c r="A273" s="2" t="inlineStr">
@@ -6444,11 +5364,7 @@
           <t>Updated: tests for the 4 Snap staging models -- all hand-verified against live data first</t>
         </is>
       </c>
-      <c r="D273" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-29 22:11 PDT</t>
-        </is>
-      </c>
+      <c r="D273" s="2" t="inlineStr"/>
     </row>
     <row r="274">
       <c r="A274" s="2" t="inlineStr">
@@ -6466,11 +5382,7 @@
           <t>Phase 2 staging (paid media: TikTok): campaigns with the single budget split into daily_budget_usd / lifetime_budget_usd by budget_mode (matching the other platforms), advertiser_id renamed tiktok_advertiser_id</t>
         </is>
       </c>
-      <c r="D274" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-29 15:57 PDT</t>
-        </is>
-      </c>
+      <c r="D274" s="2" t="inlineStr"/>
     </row>
     <row r="275">
       <c r="A275" s="2" t="inlineStr">
@@ -6488,11 +5400,7 @@
           <t>Phase 2 staging (paid media: TikTok): 1:1 pass-through of tiktok_adgroups</t>
         </is>
       </c>
-      <c r="D275" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-29 15:57 PDT</t>
-        </is>
-      </c>
+      <c r="D275" s="2" t="inlineStr"/>
     </row>
     <row r="276">
       <c r="A276" s="2" t="inlineStr">
@@ -6510,11 +5418,7 @@
           <t>Phase 2 staging (paid media: TikTok): 1:1 pass-through of tiktok_ads</t>
         </is>
       </c>
-      <c r="D276" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-29 15:57 PDT</t>
-        </is>
-      </c>
+      <c r="D276" s="2" t="inlineStr"/>
     </row>
     <row r="277">
       <c r="A277" s="2" t="inlineStr">
@@ -6532,11 +5436,7 @@
           <t>Phase 2 staging (paid media: TikTok): ad-day reports with combined ad_day_id key, spend and CPM in micros and dollars, ctr_fraction</t>
         </is>
       </c>
-      <c r="D277" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-29 15:57 PDT</t>
-        </is>
-      </c>
+      <c r="D277" s="2" t="inlineStr"/>
     </row>
     <row r="278">
       <c r="A278" s="2" t="inlineStr">
@@ -6554,11 +5454,7 @@
           <t>Phase 2 staging (final table, 47 of 47): product variants with variant_option, price_adjustment_usd</t>
         </is>
       </c>
-      <c r="D278" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-29 16:08 PDT</t>
-        </is>
-      </c>
+      <c r="D278" s="2" t="inlineStr"/>
     </row>
     <row r="279">
       <c r="A279" s="2" t="inlineStr">
@@ -6576,11 +5472,7 @@
           <t>Handoff note for starting a new chat/project: status, open decisions, prior decisions, pitfalls</t>
         </is>
       </c>
-      <c r="D279" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-30 08:29 PDT</t>
-        </is>
-      </c>
+      <c r="D279" s="2" t="inlineStr"/>
     </row>
     <row r="280">
       <c r="A280" s="2" t="inlineStr">
@@ -6598,11 +5490,7 @@
           <t>Updated: tests for the 4 TikTok staging models -- all hand-verified against live data first</t>
         </is>
       </c>
-      <c r="D280" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-29 22:11 PDT</t>
-        </is>
-      </c>
+      <c r="D280" s="2" t="inlineStr"/>
     </row>
     <row r="281">
       <c r="A281" s="2" t="inlineStr">
@@ -6620,11 +5508,7 @@
           <t>Intermediate model: one row per Braze email or push event in one shape, customer resolved via Braze id or email match (written and hand-verified; needs dbt build)</t>
         </is>
       </c>
-      <c r="D281" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-29 22:03 PDT</t>
-        </is>
-      </c>
+      <c r="D281" s="2" t="inlineStr"/>
     </row>
     <row r="282">
       <c r="A282" s="2" t="inlineStr">
@@ -6642,11 +5526,7 @@
           <t>dbt test: unified event count equals email + push event counts</t>
         </is>
       </c>
-      <c r="D282" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-29 22:03 PDT</t>
-        </is>
-      </c>
+      <c r="D282" s="2" t="inlineStr"/>
     </row>
     <row r="283">
       <c r="A283" s="2" t="inlineStr">
@@ -6664,11 +5544,7 @@
           <t>dbt test: customer_id is null exactly when a messaging event is unresolved</t>
         </is>
       </c>
-      <c r="D283" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-29 22:03 PDT</t>
-        </is>
-      </c>
+      <c r="D283" s="2" t="inlineStr"/>
     </row>
     <row r="284">
       <c r="A284" s="2" t="inlineStr">
@@ -6686,11 +5562,7 @@
           <t>Overnight run report: commands to run first, assumed decisions, done/blocked units, proposed playbook wording</t>
         </is>
       </c>
-      <c r="D284" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-30 06:53 PDT</t>
-        </is>
-      </c>
+      <c r="D284" s="2" t="inlineStr"/>
     </row>
     <row r="285">
       <c r="A285" s="2" t="inlineStr">
@@ -6708,11 +5580,7 @@
           <t>Intermediate model: one row per ad platform per day, spend/impressions/clicks/conversions in USD (written and hand-verified; needs dbt build)</t>
         </is>
       </c>
-      <c r="D285" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-29 22:05 PDT</t>
-        </is>
-      </c>
+      <c r="D285" s="2" t="inlineStr"/>
     </row>
     <row r="286">
       <c r="A286" s="2" t="inlineStr">
@@ -6730,11 +5598,7 @@
           <t>dbt test: platform-day spend total equals the six source spend totals</t>
         </is>
       </c>
-      <c r="D286" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-29 22:05 PDT</t>
-        </is>
-      </c>
+      <c r="D286" s="2" t="inlineStr"/>
     </row>
     <row r="287">
       <c r="A287" s="2" t="inlineStr">
@@ -6752,11 +5616,7 @@
           <t>dbt test: no missing days per platform</t>
         </is>
       </c>
-      <c r="D287" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-29 22:05 PDT</t>
-        </is>
-      </c>
+      <c r="D287" s="2" t="inlineStr"/>
     </row>
     <row r="288">
       <c r="A288" s="2" t="inlineStr">
@@ -6774,11 +5634,7 @@
           <t>Intermediate model: one row, the last date the subscription/invoice data covers (shared by MRR and subscriber-movement marts) (written; needs dbt build)</t>
         </is>
       </c>
-      <c r="D288" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-29 22:07 PDT</t>
-        </is>
-      </c>
+      <c r="D288" s="2" t="inlineStr"/>
     </row>
     <row r="289">
       <c r="A289" s="2" t="inlineStr">
@@ -6796,11 +5652,7 @@
           <t>Phase 4 mart (CEO): new/returning/churned/net-new/active paying subscribers by month (written and hand-validated; needs dbt build)</t>
         </is>
       </c>
-      <c r="D289" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-29 22:07 PDT</t>
-        </is>
-      </c>
+      <c r="D289" s="2" t="inlineStr"/>
     </row>
     <row r="290">
       <c r="A290" s="2" t="inlineStr">
@@ -6818,11 +5670,7 @@
           <t>dbt test: end-of-month active = previous + new - churned</t>
         </is>
       </c>
-      <c r="D290" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-29 22:07 PDT</t>
-        </is>
-      </c>
+      <c r="D290" s="2" t="inlineStr"/>
     </row>
     <row r="291">
       <c r="A291" s="2" t="inlineStr">
@@ -6840,11 +5688,7 @@
           <t>dbt test: total new and churned match the paid-periods source</t>
         </is>
       </c>
-      <c r="D291" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-29 22:07 PDT</t>
-        </is>
-      </c>
+      <c r="D291" s="2" t="inlineStr"/>
     </row>
     <row r="292">
       <c r="A292" s="2" t="inlineStr">
@@ -6862,11 +5706,7 @@
           <t>Phase 4 mart (Performance Marketing/CMO): spend, clicks, platform-reported conversions and ratios by platform by month (written and hand-validated; needs dbt build)</t>
         </is>
       </c>
-      <c r="D292" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-29 22:08 PDT</t>
-        </is>
-      </c>
+      <c r="D292" s="2" t="inlineStr"/>
     </row>
     <row r="293">
       <c r="A293" s="2" t="inlineStr">
@@ -6884,11 +5724,7 @@
           <t>Phase 4 mart (CEO/CFO): blended CAC by month = paid spend / first-time paying subscribers (written and hand-validated; needs dbt build)</t>
         </is>
       </c>
-      <c r="D293" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-29 22:08 PDT</t>
-        </is>
-      </c>
+      <c r="D293" s="2" t="inlineStr"/>
     </row>
     <row r="294">
       <c r="A294" s="2" t="inlineStr">
@@ -6906,11 +5742,7 @@
           <t>dbt test: monthly paid media spend equals daily total</t>
         </is>
       </c>
-      <c r="D294" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-29 22:08 PDT</t>
-        </is>
-      </c>
+      <c r="D294" s="2" t="inlineStr"/>
     </row>
     <row r="295">
       <c r="A295" s="2" t="inlineStr">
@@ -6928,11 +5760,7 @@
           <t>dbt test: CAC mart spend equals total paid media spend</t>
         </is>
       </c>
-      <c r="D295" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-29 22:08 PDT</t>
-        </is>
-      </c>
+      <c r="D295" s="2" t="inlineStr"/>
     </row>
     <row r="296">
       <c r="A296" s="2" t="inlineStr">
@@ -6950,11 +5778,7 @@
           <t>DRAFT Phase 6 semantic layer (MetricFlow semantic models + metrics) for the marts built so far; unvalidated, outside model-paths</t>
         </is>
       </c>
-      <c r="D296" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-29 22:13 PDT</t>
-        </is>
-      </c>
+      <c r="D296" s="2" t="inlineStr"/>
     </row>
     <row r="297">
       <c r="A297" s="2" t="inlineStr">
@@ -6972,11 +5796,7 @@
           <t>DRAFT Phase 6 validation set: mf query commands with expected values from hand SQL (not yet run)</t>
         </is>
       </c>
-      <c r="D297" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-29 22:13 PDT</t>
-        </is>
-      </c>
+      <c r="D297" s="2" t="inlineStr"/>
     </row>
     <row r="298">
       <c r="A298" s="2" t="inlineStr">
@@ -6994,11 +5814,7 @@
           <t>DRAFT Phase 7 Skill: which mart answers which question, Phase 5 caveats as instructions, 'I don't have this data' rules (not reviewed by data owner)</t>
         </is>
       </c>
-      <c r="D298" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-29 22:13 PDT</t>
-        </is>
-      </c>
+      <c r="D298" s="2" t="inlineStr"/>
     </row>
     <row r="299">
       <c r="A299" s="2" t="inlineStr">
@@ -7016,11 +5832,7 @@
           <t>Phase 5 metrics glossary: plain-language definition of every mart metric, its grain, source and what it does NOT mean</t>
         </is>
       </c>
-      <c r="D299" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-30 08:17 PDT</t>
-        </is>
-      </c>
+      <c r="D299" s="2" t="inlineStr"/>
     </row>
     <row r="300">
       <c r="A300" s="2" t="inlineStr">
@@ -7038,11 +5850,7 @@
           <t>Script: rebuild the gh-pages branch (published dbt docs site) from dbt/target as one fast-forward commit; refuses local paths/tokens</t>
         </is>
       </c>
-      <c r="D300" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-30 08:34 PDT</t>
-        </is>
-      </c>
+      <c r="D300" s="2" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Phase 6: semantic layer validated with MetricFlow (time spine, 10/10 queries match)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/File_Manifest.xlsx
+++ b/File_Manifest.xlsx
@@ -435,7 +435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D300"/>
+  <dimension ref="A1:D301"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="48" customWidth="1" min="1" max="1"/>
@@ -700,7 +700,7 @@
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30 08:57 PDT</t>
+          <t>2026-09-30 09:56 PDT</t>
         </is>
       </c>
     </row>
@@ -5765,7 +5765,7 @@
     <row r="296">
       <c r="A296" s="2" t="inlineStr">
         <is>
-          <t>dbt/drafts/semantic_layer_DRAFT.yml</t>
+          <t>dbt/models/marts/_semantic_layer.yml</t>
         </is>
       </c>
       <c r="B296" s="2" t="inlineStr">
@@ -5775,7 +5775,7 @@
       </c>
       <c r="C296" s="3" t="inlineStr">
         <is>
-          <t>DRAFT Phase 6 semantic layer (MetricFlow semantic models + metrics) for the marts built so far; unvalidated, outside model-paths</t>
+          <t>Phase 6 semantic layer (MetricFlow): 5 semantic models, 25 metrics on the marts; validated 2026-09-30</t>
         </is>
       </c>
       <c r="D296" s="2" t="inlineStr"/>
@@ -5783,17 +5783,17 @@
     <row r="297">
       <c r="A297" s="2" t="inlineStr">
         <is>
-          <t>docs/semantic_layer_validation_DRAFT.md</t>
+          <t>dbt/models/marts/metricflow_time_spine.sql</t>
         </is>
       </c>
       <c r="B297" s="2" t="inlineStr">
         <is>
-          <t>Doc</t>
+          <t>Code</t>
         </is>
       </c>
       <c r="C297" s="3" t="inlineStr">
         <is>
-          <t>DRAFT Phase 6 validation set: mf query commands with expected values from hand SQL (not yet run)</t>
+          <t>Phase 6 calendar table (one row per day, ends at the data's last day) required by MetricFlow</t>
         </is>
       </c>
       <c r="D297" s="2" t="inlineStr"/>
@@ -5801,7 +5801,7 @@
     <row r="298">
       <c r="A298" s="2" t="inlineStr">
         <is>
-          <t>docs/kinetic_skill_DRAFT.md</t>
+          <t>docs/semantic_layer_validation.md</t>
         </is>
       </c>
       <c r="B298" s="2" t="inlineStr">
@@ -5811,7 +5811,7 @@
       </c>
       <c r="C298" s="3" t="inlineStr">
         <is>
-          <t>DRAFT Phase 7 Skill: which mart answers which question, Phase 5 caveats as instructions, 'I don't have this data' rules (not reviewed by data owner)</t>
+          <t>Phase 6 validation set: 10 mf query commands with expected and returned values (all match, run 2026-09-30)</t>
         </is>
       </c>
       <c r="D298" s="2" t="inlineStr"/>
@@ -5819,7 +5819,7 @@
     <row r="299">
       <c r="A299" s="2" t="inlineStr">
         <is>
-          <t>docs/metrics_glossary.md</t>
+          <t>docs/kinetic_skill_DRAFT.md</t>
         </is>
       </c>
       <c r="B299" s="2" t="inlineStr">
@@ -5829,7 +5829,7 @@
       </c>
       <c r="C299" s="3" t="inlineStr">
         <is>
-          <t>Phase 5 metrics glossary: plain-language definition of every mart metric, its grain, source and what it does NOT mean</t>
+          <t>DRAFT Phase 7 Skill: which mart answers which question, Phase 5 caveats as instructions, 'I don't have this data' rules (not reviewed by data owner)</t>
         </is>
       </c>
       <c r="D299" s="2" t="inlineStr"/>
@@ -5837,20 +5837,38 @@
     <row r="300">
       <c r="A300" s="2" t="inlineStr">
         <is>
+          <t>docs/metrics_glossary.md</t>
+        </is>
+      </c>
+      <c r="B300" s="2" t="inlineStr">
+        <is>
+          <t>Doc</t>
+        </is>
+      </c>
+      <c r="C300" s="3" t="inlineStr">
+        <is>
+          <t>Phase 5 metrics glossary: plain-language definition of every mart metric, its grain, source and what it does NOT mean</t>
+        </is>
+      </c>
+      <c r="D300" s="2" t="inlineStr"/>
+    </row>
+    <row r="301">
+      <c r="A301" s="2" t="inlineStr">
+        <is>
           <t>scripts/rebuild_docs_branch.sh</t>
         </is>
       </c>
-      <c r="B300" s="2" t="inlineStr">
-        <is>
-          <t>Code</t>
-        </is>
-      </c>
-      <c r="C300" s="3" t="inlineStr">
+      <c r="B301" s="2" t="inlineStr">
+        <is>
+          <t>Code</t>
+        </is>
+      </c>
+      <c r="C301" s="3" t="inlineStr">
         <is>
           <t>Script: rebuild the gh-pages branch (published dbt docs site) from dbt/target as one fast-forward commit; refuses local paths/tokens</t>
         </is>
       </c>
-      <c r="D300" s="2" t="inlineStr"/>
+      <c r="D301" s="2" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Close Phase 6; add read-only SQL helper md_select.py; allow rules
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/File_Manifest.xlsx
+++ b/File_Manifest.xlsx
@@ -435,7 +435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D301"/>
+  <dimension ref="A1:D302"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="48" customWidth="1" min="1" max="1"/>
@@ -700,7 +700,7 @@
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30 09:56 PDT</t>
+          <t>2026-09-30 10:19 PDT</t>
         </is>
       </c>
     </row>
@@ -5855,20 +5855,38 @@
     <row r="301">
       <c r="A301" s="2" t="inlineStr">
         <is>
+          <t>scripts/md_select.py</t>
+        </is>
+      </c>
+      <c r="B301" s="2" t="inlineStr">
+        <is>
+          <t>Code</t>
+        </is>
+      </c>
+      <c r="C301" s="3" t="inlineStr">
+        <is>
+          <t>Script: run ONE read-only SQL statement (SELECT/WITH/DESCRIBE...) on MotherDuck kinetic; refuses writes/DDL; loads the token itself, never prints it</t>
+        </is>
+      </c>
+      <c r="D301" s="2" t="inlineStr"/>
+    </row>
+    <row r="302">
+      <c r="A302" s="2" t="inlineStr">
+        <is>
           <t>scripts/rebuild_docs_branch.sh</t>
         </is>
       </c>
-      <c r="B301" s="2" t="inlineStr">
-        <is>
-          <t>Code</t>
-        </is>
-      </c>
-      <c r="C301" s="3" t="inlineStr">
+      <c r="B302" s="2" t="inlineStr">
+        <is>
+          <t>Code</t>
+        </is>
+      </c>
+      <c r="C302" s="3" t="inlineStr">
         <is>
           <t>Script: rebuild the gh-pages branch (published dbt docs site) from dbt/target as one fast-forward commit; refuses local paths/tokens</t>
         </is>
       </c>
-      <c r="D301" s="2" t="inlineStr"/>
+      <c r="D302" s="2" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Phase 7: Skill v2 checked against live data, adds query routes (marts SQL + MetricFlow)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/File_Manifest.xlsx
+++ b/File_Manifest.xlsx
@@ -700,7 +700,7 @@
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30 10:19 PDT</t>
+          <t>2026-09-30 10:23 PDT</t>
         </is>
       </c>
     </row>
@@ -5829,7 +5829,7 @@
       </c>
       <c r="C299" s="3" t="inlineStr">
         <is>
-          <t>DRAFT Phase 7 Skill: which mart answers which question, Phase 5 caveats as instructions, 'I don't have this data' rules (not reviewed by data owner)</t>
+          <t>DRAFT Phase 7 Skill: which mart answers which question, Phase 5 caveats as instructions, 'I don't have this data' rules; v2 adds how to get the numbers (SQL on marts, or MetricFlow metrics); in Ben's review</t>
         </is>
       </c>
       <c r="D299" s="2" t="inlineStr"/>

</xml_diff>

<commit_message>
Sign off Phase 7: Kinetic Skill v1 (renamed from DRAFT), HANDOFF and CHANGELOG
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/File_Manifest.xlsx
+++ b/File_Manifest.xlsx
@@ -700,7 +700,7 @@
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30 10:23 PDT</t>
+          <t>2026-09-30 10:30 PDT</t>
         </is>
       </c>
     </row>
@@ -5819,7 +5819,7 @@
     <row r="299">
       <c r="A299" s="2" t="inlineStr">
         <is>
-          <t>docs/kinetic_skill_DRAFT.md</t>
+          <t>docs/kinetic_skill.md</t>
         </is>
       </c>
       <c r="B299" s="2" t="inlineStr">
@@ -5829,7 +5829,7 @@
       </c>
       <c r="C299" s="3" t="inlineStr">
         <is>
-          <t>DRAFT Phase 7 Skill: which mart answers which question, Phase 5 caveats as instructions, 'I don't have this data' rules; v2 adds how to get the numbers (SQL on marts, or MetricFlow metrics); in Ben's review</t>
+          <t>Phase 7 Skill (signed off 2026-09-30): which mart answers which question, Phase 5 caveats as instructions, 'I don't have this data' rules; v2 adds how to get the numbers (SQL on marts, or MetricFlow metrics); in Ben's review</t>
         </is>
       </c>
       <c r="D299" s="2" t="inlineStr"/>

</xml_diff>

<commit_message>
Phase 8: scope pilot use case (CMO paid-media check), draft
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/File_Manifest.xlsx
+++ b/File_Manifest.xlsx
@@ -435,7 +435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D302"/>
+  <dimension ref="A1:D303"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="48" customWidth="1" min="1" max="1"/>
@@ -700,7 +700,7 @@
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30 10:30 PDT</t>
+          <t>2026-09-30 10:36 PDT</t>
         </is>
       </c>
     </row>
@@ -5837,7 +5837,7 @@
     <row r="300">
       <c r="A300" s="2" t="inlineStr">
         <is>
-          <t>docs/metrics_glossary.md</t>
+          <t>docs/phase8_pilot_scope.md</t>
         </is>
       </c>
       <c r="B300" s="2" t="inlineStr">
@@ -5847,7 +5847,7 @@
       </c>
       <c r="C300" s="3" t="inlineStr">
         <is>
-          <t>Phase 5 metrics glossary: plain-language definition of every mart metric, its grain, source and what it does NOT mean</t>
+          <t>Phase 8 pilot scope (DRAFT, Ben reviewing): CMO paid-media check, 6 test questions with live-checked answers, guardrails, pass criteria, open setup decisions</t>
         </is>
       </c>
       <c r="D300" s="2" t="inlineStr"/>
@@ -5855,17 +5855,17 @@
     <row r="301">
       <c r="A301" s="2" t="inlineStr">
         <is>
-          <t>scripts/md_select.py</t>
+          <t>docs/metrics_glossary.md</t>
         </is>
       </c>
       <c r="B301" s="2" t="inlineStr">
         <is>
-          <t>Code</t>
+          <t>Doc</t>
         </is>
       </c>
       <c r="C301" s="3" t="inlineStr">
         <is>
-          <t>Script: run ONE read-only SQL statement (SELECT/WITH/DESCRIBE...) on MotherDuck kinetic; refuses writes/DDL; loads the token itself, never prints it</t>
+          <t>Phase 5 metrics glossary: plain-language definition of every mart metric, its grain, source and what it does NOT mean</t>
         </is>
       </c>
       <c r="D301" s="2" t="inlineStr"/>
@@ -5873,20 +5873,38 @@
     <row r="302">
       <c r="A302" s="2" t="inlineStr">
         <is>
+          <t>scripts/md_select.py</t>
+        </is>
+      </c>
+      <c r="B302" s="2" t="inlineStr">
+        <is>
+          <t>Code</t>
+        </is>
+      </c>
+      <c r="C302" s="3" t="inlineStr">
+        <is>
+          <t>Script: run ONE read-only SQL statement (SELECT/WITH/DESCRIBE...) on MotherDuck kinetic; refuses writes/DDL; loads the token itself, never prints it</t>
+        </is>
+      </c>
+      <c r="D302" s="2" t="inlineStr"/>
+    </row>
+    <row r="303">
+      <c r="A303" s="2" t="inlineStr">
+        <is>
           <t>scripts/rebuild_docs_branch.sh</t>
         </is>
       </c>
-      <c r="B302" s="2" t="inlineStr">
-        <is>
-          <t>Code</t>
-        </is>
-      </c>
-      <c r="C302" s="3" t="inlineStr">
+      <c r="B303" s="2" t="inlineStr">
+        <is>
+          <t>Code</t>
+        </is>
+      </c>
+      <c r="C303" s="3" t="inlineStr">
         <is>
           <t>Script: rebuild the gh-pages branch (published dbt docs site) from dbt/target as one fast-forward commit; refuses local paths/tokens</t>
         </is>
       </c>
-      <c r="D302" s="2" t="inlineStr"/>
+      <c r="D303" s="2" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Phase 8: scope approved, pilot setup decisions, Skill v1.1 read-only rule, pilot log
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/File_Manifest.xlsx
+++ b/File_Manifest.xlsx
@@ -435,7 +435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D303"/>
+  <dimension ref="A1:D304"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="48" customWidth="1" min="1" max="1"/>
@@ -700,7 +700,7 @@
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30 10:36 PDT</t>
+          <t>2026-09-30 10:42 PDT</t>
         </is>
       </c>
     </row>
@@ -5829,7 +5829,7 @@
       </c>
       <c r="C299" s="3" t="inlineStr">
         <is>
-          <t>Phase 7 Skill (signed off 2026-09-30): which mart answers which question, Phase 5 caveats as instructions, 'I don't have this data' rules; v2 adds how to get the numbers (SQL on marts, or MetricFlow metrics); in Ben's review</t>
+          <t>Phase 7 Skill (signed off 2026-09-30): which mart answers which question, Phase 5 caveats as instructions, 'I don't have this data' rules; v2 adds how to get the numbers (SQL on marts, or MetricFlow metrics); v1.1 adds a read-only (SELECT only) rule for the Phase 8 pilot</t>
         </is>
       </c>
       <c r="D299" s="2" t="inlineStr"/>
@@ -5847,7 +5847,7 @@
       </c>
       <c r="C300" s="3" t="inlineStr">
         <is>
-          <t>Phase 8 pilot scope (DRAFT, Ben reviewing): CMO paid-media check, 6 test questions with live-checked answers, guardrails, pass criteria, open setup decisions</t>
+          <t>Phase 8 pilot scope (approved 2026-09-30): CMO paid-media check, 6 test questions with live-checked answers, pass criteria, Ben's setup decisions (dev schema, claude.ai, write tool off, pilot log)</t>
         </is>
       </c>
       <c r="D300" s="2" t="inlineStr"/>
@@ -5855,7 +5855,7 @@
     <row r="301">
       <c r="A301" s="2" t="inlineStr">
         <is>
-          <t>docs/metrics_glossary.md</t>
+          <t>docs/phase8_pilot_log.md</t>
         </is>
       </c>
       <c r="B301" s="2" t="inlineStr">
@@ -5865,7 +5865,7 @@
       </c>
       <c r="C301" s="3" t="inlineStr">
         <is>
-          <t>Phase 5 metrics glossary: plain-language definition of every mart metric, its grain, source and what it does NOT mean</t>
+          <t>Phase 8 pilot log: one graded row per question asked to the pilot agent (verdict, cited or not, notes)</t>
         </is>
       </c>
       <c r="D301" s="2" t="inlineStr"/>
@@ -5873,17 +5873,17 @@
     <row r="302">
       <c r="A302" s="2" t="inlineStr">
         <is>
-          <t>scripts/md_select.py</t>
+          <t>docs/metrics_glossary.md</t>
         </is>
       </c>
       <c r="B302" s="2" t="inlineStr">
         <is>
-          <t>Code</t>
+          <t>Doc</t>
         </is>
       </c>
       <c r="C302" s="3" t="inlineStr">
         <is>
-          <t>Script: run ONE read-only SQL statement (SELECT/WITH/DESCRIBE...) on MotherDuck kinetic; refuses writes/DDL; loads the token itself, never prints it</t>
+          <t>Phase 5 metrics glossary: plain-language definition of every mart metric, its grain, source and what it does NOT mean</t>
         </is>
       </c>
       <c r="D302" s="2" t="inlineStr"/>
@@ -5891,20 +5891,38 @@
     <row r="303">
       <c r="A303" s="2" t="inlineStr">
         <is>
+          <t>scripts/md_select.py</t>
+        </is>
+      </c>
+      <c r="B303" s="2" t="inlineStr">
+        <is>
+          <t>Code</t>
+        </is>
+      </c>
+      <c r="C303" s="3" t="inlineStr">
+        <is>
+          <t>Script: run ONE read-only SQL statement (SELECT/WITH/DESCRIBE...) on MotherDuck kinetic; refuses writes/DDL; loads the token itself, never prints it</t>
+        </is>
+      </c>
+      <c r="D303" s="2" t="inlineStr"/>
+    </row>
+    <row r="304">
+      <c r="A304" s="2" t="inlineStr">
+        <is>
           <t>scripts/rebuild_docs_branch.sh</t>
         </is>
       </c>
-      <c r="B303" s="2" t="inlineStr">
-        <is>
-          <t>Code</t>
-        </is>
-      </c>
-      <c r="C303" s="3" t="inlineStr">
+      <c r="B304" s="2" t="inlineStr">
+        <is>
+          <t>Code</t>
+        </is>
+      </c>
+      <c r="C304" s="3" t="inlineStr">
         <is>
           <t>Script: rebuild the gh-pages branch (published dbt docs site) from dbt/target as one fast-forward commit; refuses local paths/tokens</t>
         </is>
       </c>
-      <c r="D303" s="2" t="inlineStr"/>
+      <c r="D304" s="2" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Add mart_messaging_monthly (email + push), tests, md_env.sh wrapper
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/File_Manifest.xlsx
+++ b/File_Manifest.xlsx
@@ -435,7 +435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D304"/>
+  <dimension ref="A1:D308"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="48" customWidth="1" min="1" max="1"/>
@@ -700,7 +700,7 @@
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30 10:42 PDT</t>
+          <t>2026-09-30 11:28 PDT</t>
         </is>
       </c>
     </row>
@@ -5693,7 +5693,7 @@
     <row r="292">
       <c r="A292" s="2" t="inlineStr">
         <is>
-          <t>dbt/models/marts/mart_paid_media_monthly.sql</t>
+          <t>dbt/models/marts/mart_messaging_monthly.sql</t>
         </is>
       </c>
       <c r="B292" s="2" t="inlineStr">
@@ -5703,7 +5703,7 @@
       </c>
       <c r="C292" s="3" t="inlineStr">
         <is>
-          <t>Phase 4 mart (Performance Marketing/CMO): spend, clicks, platform-reported conversions and ratios by platform by month (written and hand-validated; needs dbt build)</t>
+          <t>dbt mart: email and push by channel x campaign type x month (sends, bounces, delivered, opens, clicks, unsubscribes and rates); hand-validated, built 12/12</t>
         </is>
       </c>
       <c r="D292" s="2" t="inlineStr"/>
@@ -5711,7 +5711,7 @@
     <row r="293">
       <c r="A293" s="2" t="inlineStr">
         <is>
-          <t>dbt/models/marts/mart_acquisition_efficiency_monthly.sql</t>
+          <t>dbt/tests/assert_mart_messaging_monthly_totals_match_events.sql</t>
         </is>
       </c>
       <c r="B293" s="2" t="inlineStr">
@@ -5721,7 +5721,7 @@
       </c>
       <c r="C293" s="3" t="inlineStr">
         <is>
-          <t>Phase 4 mart (CEO/CFO): blended CAC by month = paid spend / first-time paying subscribers (written and hand-validated; needs dbt build)</t>
+          <t>dbt test: messaging mart totals per channel equal the events in int_messaging_events</t>
         </is>
       </c>
       <c r="D293" s="2" t="inlineStr"/>
@@ -5729,7 +5729,7 @@
     <row r="294">
       <c r="A294" s="2" t="inlineStr">
         <is>
-          <t>dbt/tests/assert_mart_paid_media_monthly_spend_matches_daily.sql</t>
+          <t>dbt/tests/assert_mart_messaging_monthly_identity.sql</t>
         </is>
       </c>
       <c r="B294" s="2" t="inlineStr">
@@ -5739,7 +5739,7 @@
       </c>
       <c r="C294" s="3" t="inlineStr">
         <is>
-          <t>dbt test: monthly paid media spend equals daily total</t>
+          <t>dbt test: messaging funnel logic (delivered = sends - bounces, opens &lt;= delivered, clicks &lt;= opens, rates in 0-1)</t>
         </is>
       </c>
       <c r="D294" s="2" t="inlineStr"/>
@@ -5747,7 +5747,7 @@
     <row r="295">
       <c r="A295" s="2" t="inlineStr">
         <is>
-          <t>dbt/tests/assert_mart_acquisition_efficiency_monthly_spend_matches_daily.sql</t>
+          <t>dbt/models/marts/mart_paid_media_monthly.sql</t>
         </is>
       </c>
       <c r="B295" s="2" t="inlineStr">
@@ -5757,7 +5757,7 @@
       </c>
       <c r="C295" s="3" t="inlineStr">
         <is>
-          <t>dbt test: CAC mart spend equals total paid media spend</t>
+          <t>Phase 4 mart (Performance Marketing/CMO): spend, clicks, platform-reported conversions and ratios by platform by month (written and hand-validated; needs dbt build)</t>
         </is>
       </c>
       <c r="D295" s="2" t="inlineStr"/>
@@ -5765,17 +5765,17 @@
     <row r="296">
       <c r="A296" s="2" t="inlineStr">
         <is>
-          <t>dbt/models/marts/_semantic_layer.yml</t>
+          <t>dbt/models/marts/mart_acquisition_efficiency_monthly.sql</t>
         </is>
       </c>
       <c r="B296" s="2" t="inlineStr">
         <is>
-          <t>Config</t>
+          <t>Code</t>
         </is>
       </c>
       <c r="C296" s="3" t="inlineStr">
         <is>
-          <t>Phase 6 semantic layer (MetricFlow): 5 semantic models, 25 metrics on the marts; validated 2026-09-30</t>
+          <t>Phase 4 mart (CEO/CFO): blended CAC by month = paid spend / first-time paying subscribers (written and hand-validated; needs dbt build)</t>
         </is>
       </c>
       <c r="D296" s="2" t="inlineStr"/>
@@ -5783,7 +5783,7 @@
     <row r="297">
       <c r="A297" s="2" t="inlineStr">
         <is>
-          <t>dbt/models/marts/metricflow_time_spine.sql</t>
+          <t>dbt/tests/assert_mart_paid_media_monthly_spend_matches_daily.sql</t>
         </is>
       </c>
       <c r="B297" s="2" t="inlineStr">
@@ -5793,7 +5793,7 @@
       </c>
       <c r="C297" s="3" t="inlineStr">
         <is>
-          <t>Phase 6 calendar table (one row per day, ends at the data's last day) required by MetricFlow</t>
+          <t>dbt test: monthly paid media spend equals daily total</t>
         </is>
       </c>
       <c r="D297" s="2" t="inlineStr"/>
@@ -5801,17 +5801,17 @@
     <row r="298">
       <c r="A298" s="2" t="inlineStr">
         <is>
-          <t>docs/semantic_layer_validation.md</t>
+          <t>dbt/tests/assert_mart_acquisition_efficiency_monthly_spend_matches_daily.sql</t>
         </is>
       </c>
       <c r="B298" s="2" t="inlineStr">
         <is>
-          <t>Doc</t>
+          <t>Code</t>
         </is>
       </c>
       <c r="C298" s="3" t="inlineStr">
         <is>
-          <t>Phase 6 validation set: 10 mf query commands with expected and returned values (all match, run 2026-09-30)</t>
+          <t>dbt test: CAC mart spend equals total paid media spend</t>
         </is>
       </c>
       <c r="D298" s="2" t="inlineStr"/>
@@ -5819,17 +5819,17 @@
     <row r="299">
       <c r="A299" s="2" t="inlineStr">
         <is>
-          <t>docs/kinetic_skill.md</t>
+          <t>dbt/models/marts/_semantic_layer.yml</t>
         </is>
       </c>
       <c r="B299" s="2" t="inlineStr">
         <is>
-          <t>Doc</t>
+          <t>Config</t>
         </is>
       </c>
       <c r="C299" s="3" t="inlineStr">
         <is>
-          <t>Phase 7 Skill (signed off 2026-09-30): which mart answers which question, Phase 5 caveats as instructions, 'I don't have this data' rules; v2 adds how to get the numbers (SQL on marts, or MetricFlow metrics); v1.1 adds a read-only (SELECT only) rule for the Phase 8 pilot</t>
+          <t>Phase 6 semantic layer (MetricFlow): 5 semantic models, 25 metrics on the marts; validated 2026-09-30</t>
         </is>
       </c>
       <c r="D299" s="2" t="inlineStr"/>
@@ -5837,17 +5837,17 @@
     <row r="300">
       <c r="A300" s="2" t="inlineStr">
         <is>
-          <t>docs/phase8_pilot_scope.md</t>
+          <t>dbt/models/marts/metricflow_time_spine.sql</t>
         </is>
       </c>
       <c r="B300" s="2" t="inlineStr">
         <is>
-          <t>Doc</t>
+          <t>Code</t>
         </is>
       </c>
       <c r="C300" s="3" t="inlineStr">
         <is>
-          <t>Phase 8 pilot scope (approved 2026-09-30): CMO paid-media check, 6 test questions with live-checked answers, pass criteria, Ben's setup decisions (dev schema, claude.ai, write tool off, pilot log)</t>
+          <t>Phase 6 calendar table (one row per day, ends at the data's last day) required by MetricFlow</t>
         </is>
       </c>
       <c r="D300" s="2" t="inlineStr"/>
@@ -5855,7 +5855,7 @@
     <row r="301">
       <c r="A301" s="2" t="inlineStr">
         <is>
-          <t>docs/phase8_pilot_log.md</t>
+          <t>docs/semantic_layer_validation.md</t>
         </is>
       </c>
       <c r="B301" s="2" t="inlineStr">
@@ -5865,7 +5865,7 @@
       </c>
       <c r="C301" s="3" t="inlineStr">
         <is>
-          <t>Phase 8 pilot log: one graded row per question asked to the pilot agent (verdict, cited or not, notes)</t>
+          <t>Phase 6 validation set: 10 mf query commands with expected and returned values (all match, run 2026-09-30)</t>
         </is>
       </c>
       <c r="D301" s="2" t="inlineStr"/>
@@ -5873,7 +5873,7 @@
     <row r="302">
       <c r="A302" s="2" t="inlineStr">
         <is>
-          <t>docs/metrics_glossary.md</t>
+          <t>docs/kinetic_skill.md</t>
         </is>
       </c>
       <c r="B302" s="2" t="inlineStr">
@@ -5883,7 +5883,7 @@
       </c>
       <c r="C302" s="3" t="inlineStr">
         <is>
-          <t>Phase 5 metrics glossary: plain-language definition of every mart metric, its grain, source and what it does NOT mean</t>
+          <t>Phase 7 Skill (signed off 2026-09-30): which mart answers which question, Phase 5 caveats as instructions, 'I don't have this data' rules; v2 adds how to get the numbers (SQL on marts, or MetricFlow metrics); v1.1 adds a read-only (SELECT only) rule for the Phase 8 pilot</t>
         </is>
       </c>
       <c r="D302" s="2" t="inlineStr"/>
@@ -5891,17 +5891,17 @@
     <row r="303">
       <c r="A303" s="2" t="inlineStr">
         <is>
-          <t>scripts/md_select.py</t>
+          <t>docs/phase8_pilot_scope.md</t>
         </is>
       </c>
       <c r="B303" s="2" t="inlineStr">
         <is>
-          <t>Code</t>
+          <t>Doc</t>
         </is>
       </c>
       <c r="C303" s="3" t="inlineStr">
         <is>
-          <t>Script: run ONE read-only SQL statement (SELECT/WITH/DESCRIBE...) on MotherDuck kinetic; refuses writes/DDL; loads the token itself, never prints it</t>
+          <t>Phase 8 pilot scope (approved 2026-09-30): CMO paid-media check, 6 test questions with live-checked answers, pass criteria, Ben's setup decisions (dev schema, claude.ai, write tool off, pilot log)</t>
         </is>
       </c>
       <c r="D303" s="2" t="inlineStr"/>
@@ -5909,20 +5909,92 @@
     <row r="304">
       <c r="A304" s="2" t="inlineStr">
         <is>
+          <t>docs/phase8_pilot_log.md</t>
+        </is>
+      </c>
+      <c r="B304" s="2" t="inlineStr">
+        <is>
+          <t>Doc</t>
+        </is>
+      </c>
+      <c r="C304" s="3" t="inlineStr">
+        <is>
+          <t>Phase 8 pilot log: one graded row per question asked to the pilot agent (verdict, cited or not, notes)</t>
+        </is>
+      </c>
+      <c r="D304" s="2" t="inlineStr"/>
+    </row>
+    <row r="305">
+      <c r="A305" s="2" t="inlineStr">
+        <is>
+          <t>docs/metrics_glossary.md</t>
+        </is>
+      </c>
+      <c r="B305" s="2" t="inlineStr">
+        <is>
+          <t>Doc</t>
+        </is>
+      </c>
+      <c r="C305" s="3" t="inlineStr">
+        <is>
+          <t>Phase 5 metrics glossary: plain-language definition of every mart metric, its grain, source and what it does NOT mean</t>
+        </is>
+      </c>
+      <c r="D305" s="2" t="inlineStr"/>
+    </row>
+    <row r="306">
+      <c r="A306" s="2" t="inlineStr">
+        <is>
+          <t>scripts/md_env.sh</t>
+        </is>
+      </c>
+      <c r="B306" s="2" t="inlineStr">
+        <is>
+          <t>Code</t>
+        </is>
+      </c>
+      <c r="C306" s="3" t="inlineStr">
+        <is>
+          <t>Script: run ONLY dbt or mf (MetricFlow) from dbt/ with the MotherDuck token loaded from ~/.zshrc (never printed), so no browser sign-in</t>
+        </is>
+      </c>
+      <c r="D306" s="2" t="inlineStr"/>
+    </row>
+    <row r="307">
+      <c r="A307" s="2" t="inlineStr">
+        <is>
+          <t>scripts/md_select.py</t>
+        </is>
+      </c>
+      <c r="B307" s="2" t="inlineStr">
+        <is>
+          <t>Code</t>
+        </is>
+      </c>
+      <c r="C307" s="3" t="inlineStr">
+        <is>
+          <t>Script: run ONE read-only SQL statement (SELECT/WITH/DESCRIBE...) on MotherDuck kinetic; refuses writes/DDL; loads the token itself, never prints it</t>
+        </is>
+      </c>
+      <c r="D307" s="2" t="inlineStr"/>
+    </row>
+    <row r="308">
+      <c r="A308" s="2" t="inlineStr">
+        <is>
           <t>scripts/rebuild_docs_branch.sh</t>
         </is>
       </c>
-      <c r="B304" s="2" t="inlineStr">
-        <is>
-          <t>Code</t>
-        </is>
-      </c>
-      <c r="C304" s="3" t="inlineStr">
+      <c r="B308" s="2" t="inlineStr">
+        <is>
+          <t>Code</t>
+        </is>
+      </c>
+      <c r="C308" s="3" t="inlineStr">
         <is>
           <t>Script: rebuild the gh-pages branch (published dbt docs site) from dbt/target as one fast-forward commit; refuses local paths/tokens</t>
         </is>
       </c>
-      <c r="D304" s="2" t="inlineStr"/>
+      <c r="D308" s="2" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Add mart_traffic_monthly (web + app sessions), tests
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/File_Manifest.xlsx
+++ b/File_Manifest.xlsx
@@ -435,7 +435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D308"/>
+  <dimension ref="A1:D311"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="48" customWidth="1" min="1" max="1"/>
@@ -700,7 +700,7 @@
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30 11:28 PDT</t>
+          <t>2026-09-30 11:29 PDT</t>
         </is>
       </c>
     </row>
@@ -5693,7 +5693,7 @@
     <row r="292">
       <c r="A292" s="2" t="inlineStr">
         <is>
-          <t>dbt/models/marts/mart_messaging_monthly.sql</t>
+          <t>dbt/models/marts/mart_traffic_monthly.sql</t>
         </is>
       </c>
       <c r="B292" s="2" t="inlineStr">
@@ -5703,7 +5703,7 @@
       </c>
       <c r="C292" s="3" t="inlineStr">
         <is>
-          <t>dbt mart: email and push by channel x campaign type x month (sends, bounces, delivered, opens, clicks, unsubscribes and rates); hand-validated, built 12/12</t>
+          <t>dbt mart: web and app sessions by month x traffic source x landing page (sessions, known/anonymous, duration); hand-validated, built 11/11</t>
         </is>
       </c>
       <c r="D292" s="2" t="inlineStr"/>
@@ -5711,7 +5711,7 @@
     <row r="293">
       <c r="A293" s="2" t="inlineStr">
         <is>
-          <t>dbt/tests/assert_mart_messaging_monthly_totals_match_events.sql</t>
+          <t>dbt/tests/assert_mart_traffic_monthly_totals_match_sessions.sql</t>
         </is>
       </c>
       <c r="B293" s="2" t="inlineStr">
@@ -5721,7 +5721,7 @@
       </c>
       <c r="C293" s="3" t="inlineStr">
         <is>
-          <t>dbt test: messaging mart totals per channel equal the events in int_messaging_events</t>
+          <t>dbt test: traffic mart sessions and seconds equal int_sessions_unified</t>
         </is>
       </c>
       <c r="D293" s="2" t="inlineStr"/>
@@ -5729,7 +5729,7 @@
     <row r="294">
       <c r="A294" s="2" t="inlineStr">
         <is>
-          <t>dbt/tests/assert_mart_messaging_monthly_identity.sql</t>
+          <t>dbt/tests/assert_mart_traffic_monthly_identity.sql</t>
         </is>
       </c>
       <c r="B294" s="2" t="inlineStr">
@@ -5739,7 +5739,7 @@
       </c>
       <c r="C294" s="3" t="inlineStr">
         <is>
-          <t>dbt test: messaging funnel logic (delivered = sends - bounces, opens &lt;= delivered, clicks &lt;= opens, rates in 0-1)</t>
+          <t>dbt test: traffic mart known + anonymous = sessions, rates in 0-1</t>
         </is>
       </c>
       <c r="D294" s="2" t="inlineStr"/>
@@ -5747,7 +5747,7 @@
     <row r="295">
       <c r="A295" s="2" t="inlineStr">
         <is>
-          <t>dbt/models/marts/mart_paid_media_monthly.sql</t>
+          <t>dbt/models/marts/mart_messaging_monthly.sql</t>
         </is>
       </c>
       <c r="B295" s="2" t="inlineStr">
@@ -5757,7 +5757,7 @@
       </c>
       <c r="C295" s="3" t="inlineStr">
         <is>
-          <t>Phase 4 mart (Performance Marketing/CMO): spend, clicks, platform-reported conversions and ratios by platform by month (written and hand-validated; needs dbt build)</t>
+          <t>dbt mart: email and push by channel x campaign type x month (sends, bounces, delivered, opens, clicks, unsubscribes and rates); hand-validated, built 12/12</t>
         </is>
       </c>
       <c r="D295" s="2" t="inlineStr"/>
@@ -5765,7 +5765,7 @@
     <row r="296">
       <c r="A296" s="2" t="inlineStr">
         <is>
-          <t>dbt/models/marts/mart_acquisition_efficiency_monthly.sql</t>
+          <t>dbt/tests/assert_mart_messaging_monthly_totals_match_events.sql</t>
         </is>
       </c>
       <c r="B296" s="2" t="inlineStr">
@@ -5775,7 +5775,7 @@
       </c>
       <c r="C296" s="3" t="inlineStr">
         <is>
-          <t>Phase 4 mart (CEO/CFO): blended CAC by month = paid spend / first-time paying subscribers (written and hand-validated; needs dbt build)</t>
+          <t>dbt test: messaging mart totals per channel equal the events in int_messaging_events</t>
         </is>
       </c>
       <c r="D296" s="2" t="inlineStr"/>
@@ -5783,7 +5783,7 @@
     <row r="297">
       <c r="A297" s="2" t="inlineStr">
         <is>
-          <t>dbt/tests/assert_mart_paid_media_monthly_spend_matches_daily.sql</t>
+          <t>dbt/tests/assert_mart_messaging_monthly_identity.sql</t>
         </is>
       </c>
       <c r="B297" s="2" t="inlineStr">
@@ -5793,7 +5793,7 @@
       </c>
       <c r="C297" s="3" t="inlineStr">
         <is>
-          <t>dbt test: monthly paid media spend equals daily total</t>
+          <t>dbt test: messaging funnel logic (delivered = sends - bounces, opens &lt;= delivered, clicks &lt;= opens, rates in 0-1)</t>
         </is>
       </c>
       <c r="D297" s="2" t="inlineStr"/>
@@ -5801,7 +5801,7 @@
     <row r="298">
       <c r="A298" s="2" t="inlineStr">
         <is>
-          <t>dbt/tests/assert_mart_acquisition_efficiency_monthly_spend_matches_daily.sql</t>
+          <t>dbt/models/marts/mart_paid_media_monthly.sql</t>
         </is>
       </c>
       <c r="B298" s="2" t="inlineStr">
@@ -5811,7 +5811,7 @@
       </c>
       <c r="C298" s="3" t="inlineStr">
         <is>
-          <t>dbt test: CAC mart spend equals total paid media spend</t>
+          <t>Phase 4 mart (Performance Marketing/CMO): spend, clicks, platform-reported conversions and ratios by platform by month (written and hand-validated; needs dbt build)</t>
         </is>
       </c>
       <c r="D298" s="2" t="inlineStr"/>
@@ -5819,17 +5819,17 @@
     <row r="299">
       <c r="A299" s="2" t="inlineStr">
         <is>
-          <t>dbt/models/marts/_semantic_layer.yml</t>
+          <t>dbt/models/marts/mart_acquisition_efficiency_monthly.sql</t>
         </is>
       </c>
       <c r="B299" s="2" t="inlineStr">
         <is>
-          <t>Config</t>
+          <t>Code</t>
         </is>
       </c>
       <c r="C299" s="3" t="inlineStr">
         <is>
-          <t>Phase 6 semantic layer (MetricFlow): 5 semantic models, 25 metrics on the marts; validated 2026-09-30</t>
+          <t>Phase 4 mart (CEO/CFO): blended CAC by month = paid spend / first-time paying subscribers (written and hand-validated; needs dbt build)</t>
         </is>
       </c>
       <c r="D299" s="2" t="inlineStr"/>
@@ -5837,7 +5837,7 @@
     <row r="300">
       <c r="A300" s="2" t="inlineStr">
         <is>
-          <t>dbt/models/marts/metricflow_time_spine.sql</t>
+          <t>dbt/tests/assert_mart_paid_media_monthly_spend_matches_daily.sql</t>
         </is>
       </c>
       <c r="B300" s="2" t="inlineStr">
@@ -5847,7 +5847,7 @@
       </c>
       <c r="C300" s="3" t="inlineStr">
         <is>
-          <t>Phase 6 calendar table (one row per day, ends at the data's last day) required by MetricFlow</t>
+          <t>dbt test: monthly paid media spend equals daily total</t>
         </is>
       </c>
       <c r="D300" s="2" t="inlineStr"/>
@@ -5855,17 +5855,17 @@
     <row r="301">
       <c r="A301" s="2" t="inlineStr">
         <is>
-          <t>docs/semantic_layer_validation.md</t>
+          <t>dbt/tests/assert_mart_acquisition_efficiency_monthly_spend_matches_daily.sql</t>
         </is>
       </c>
       <c r="B301" s="2" t="inlineStr">
         <is>
-          <t>Doc</t>
+          <t>Code</t>
         </is>
       </c>
       <c r="C301" s="3" t="inlineStr">
         <is>
-          <t>Phase 6 validation set: 10 mf query commands with expected and returned values (all match, run 2026-09-30)</t>
+          <t>dbt test: CAC mart spend equals total paid media spend</t>
         </is>
       </c>
       <c r="D301" s="2" t="inlineStr"/>
@@ -5873,17 +5873,17 @@
     <row r="302">
       <c r="A302" s="2" t="inlineStr">
         <is>
-          <t>docs/kinetic_skill.md</t>
+          <t>dbt/models/marts/_semantic_layer.yml</t>
         </is>
       </c>
       <c r="B302" s="2" t="inlineStr">
         <is>
-          <t>Doc</t>
+          <t>Config</t>
         </is>
       </c>
       <c r="C302" s="3" t="inlineStr">
         <is>
-          <t>Phase 7 Skill (signed off 2026-09-30): which mart answers which question, Phase 5 caveats as instructions, 'I don't have this data' rules; v2 adds how to get the numbers (SQL on marts, or MetricFlow metrics); v1.1 adds a read-only (SELECT only) rule for the Phase 8 pilot</t>
+          <t>Phase 6 semantic layer (MetricFlow): 5 semantic models, 25 metrics on the marts; validated 2026-09-30</t>
         </is>
       </c>
       <c r="D302" s="2" t="inlineStr"/>
@@ -5891,17 +5891,17 @@
     <row r="303">
       <c r="A303" s="2" t="inlineStr">
         <is>
-          <t>docs/phase8_pilot_scope.md</t>
+          <t>dbt/models/marts/metricflow_time_spine.sql</t>
         </is>
       </c>
       <c r="B303" s="2" t="inlineStr">
         <is>
-          <t>Doc</t>
+          <t>Code</t>
         </is>
       </c>
       <c r="C303" s="3" t="inlineStr">
         <is>
-          <t>Phase 8 pilot scope (approved 2026-09-30): CMO paid-media check, 6 test questions with live-checked answers, pass criteria, Ben's setup decisions (dev schema, claude.ai, write tool off, pilot log)</t>
+          <t>Phase 6 calendar table (one row per day, ends at the data's last day) required by MetricFlow</t>
         </is>
       </c>
       <c r="D303" s="2" t="inlineStr"/>
@@ -5909,7 +5909,7 @@
     <row r="304">
       <c r="A304" s="2" t="inlineStr">
         <is>
-          <t>docs/phase8_pilot_log.md</t>
+          <t>docs/semantic_layer_validation.md</t>
         </is>
       </c>
       <c r="B304" s="2" t="inlineStr">
@@ -5919,7 +5919,7 @@
       </c>
       <c r="C304" s="3" t="inlineStr">
         <is>
-          <t>Phase 8 pilot log: one graded row per question asked to the pilot agent (verdict, cited or not, notes)</t>
+          <t>Phase 6 validation set: 10 mf query commands with expected and returned values (all match, run 2026-09-30)</t>
         </is>
       </c>
       <c r="D304" s="2" t="inlineStr"/>
@@ -5927,7 +5927,7 @@
     <row r="305">
       <c r="A305" s="2" t="inlineStr">
         <is>
-          <t>docs/metrics_glossary.md</t>
+          <t>docs/kinetic_skill.md</t>
         </is>
       </c>
       <c r="B305" s="2" t="inlineStr">
@@ -5937,7 +5937,7 @@
       </c>
       <c r="C305" s="3" t="inlineStr">
         <is>
-          <t>Phase 5 metrics glossary: plain-language definition of every mart metric, its grain, source and what it does NOT mean</t>
+          <t>Phase 7 Skill (signed off 2026-09-30): which mart answers which question, Phase 5 caveats as instructions, 'I don't have this data' rules; v2 adds how to get the numbers (SQL on marts, or MetricFlow metrics); v1.1 adds a read-only (SELECT only) rule for the Phase 8 pilot</t>
         </is>
       </c>
       <c r="D305" s="2" t="inlineStr"/>
@@ -5945,17 +5945,17 @@
     <row r="306">
       <c r="A306" s="2" t="inlineStr">
         <is>
-          <t>scripts/md_env.sh</t>
+          <t>docs/phase8_pilot_scope.md</t>
         </is>
       </c>
       <c r="B306" s="2" t="inlineStr">
         <is>
-          <t>Code</t>
+          <t>Doc</t>
         </is>
       </c>
       <c r="C306" s="3" t="inlineStr">
         <is>
-          <t>Script: run ONLY dbt or mf (MetricFlow) from dbt/ with the MotherDuck token loaded from ~/.zshrc (never printed), so no browser sign-in</t>
+          <t>Phase 8 pilot scope (approved 2026-09-30): CMO paid-media check, 6 test questions with live-checked answers, pass criteria, Ben's setup decisions (dev schema, claude.ai, write tool off, pilot log)</t>
         </is>
       </c>
       <c r="D306" s="2" t="inlineStr"/>
@@ -5963,17 +5963,17 @@
     <row r="307">
       <c r="A307" s="2" t="inlineStr">
         <is>
-          <t>scripts/md_select.py</t>
+          <t>docs/phase8_pilot_log.md</t>
         </is>
       </c>
       <c r="B307" s="2" t="inlineStr">
         <is>
-          <t>Code</t>
+          <t>Doc</t>
         </is>
       </c>
       <c r="C307" s="3" t="inlineStr">
         <is>
-          <t>Script: run ONE read-only SQL statement (SELECT/WITH/DESCRIBE...) on MotherDuck kinetic; refuses writes/DDL; loads the token itself, never prints it</t>
+          <t>Phase 8 pilot log: one graded row per question asked to the pilot agent (verdict, cited or not, notes)</t>
         </is>
       </c>
       <c r="D307" s="2" t="inlineStr"/>
@@ -5981,20 +5981,74 @@
     <row r="308">
       <c r="A308" s="2" t="inlineStr">
         <is>
+          <t>docs/metrics_glossary.md</t>
+        </is>
+      </c>
+      <c r="B308" s="2" t="inlineStr">
+        <is>
+          <t>Doc</t>
+        </is>
+      </c>
+      <c r="C308" s="3" t="inlineStr">
+        <is>
+          <t>Phase 5 metrics glossary: plain-language definition of every mart metric, its grain, source and what it does NOT mean</t>
+        </is>
+      </c>
+      <c r="D308" s="2" t="inlineStr"/>
+    </row>
+    <row r="309">
+      <c r="A309" s="2" t="inlineStr">
+        <is>
+          <t>scripts/md_env.sh</t>
+        </is>
+      </c>
+      <c r="B309" s="2" t="inlineStr">
+        <is>
+          <t>Code</t>
+        </is>
+      </c>
+      <c r="C309" s="3" t="inlineStr">
+        <is>
+          <t>Script: run ONLY dbt or mf (MetricFlow) from dbt/ with the MotherDuck token loaded from ~/.zshrc (never printed), so no browser sign-in</t>
+        </is>
+      </c>
+      <c r="D309" s="2" t="inlineStr"/>
+    </row>
+    <row r="310">
+      <c r="A310" s="2" t="inlineStr">
+        <is>
+          <t>scripts/md_select.py</t>
+        </is>
+      </c>
+      <c r="B310" s="2" t="inlineStr">
+        <is>
+          <t>Code</t>
+        </is>
+      </c>
+      <c r="C310" s="3" t="inlineStr">
+        <is>
+          <t>Script: run ONE read-only SQL statement (SELECT/WITH/DESCRIBE...) on MotherDuck kinetic; refuses writes/DDL; loads the token itself, never prints it</t>
+        </is>
+      </c>
+      <c r="D310" s="2" t="inlineStr"/>
+    </row>
+    <row r="311">
+      <c r="A311" s="2" t="inlineStr">
+        <is>
           <t>scripts/rebuild_docs_branch.sh</t>
         </is>
       </c>
-      <c r="B308" s="2" t="inlineStr">
-        <is>
-          <t>Code</t>
-        </is>
-      </c>
-      <c r="C308" s="3" t="inlineStr">
+      <c r="B311" s="2" t="inlineStr">
+        <is>
+          <t>Code</t>
+        </is>
+      </c>
+      <c r="C311" s="3" t="inlineStr">
         <is>
           <t>Script: rebuild the gh-pages branch (published dbt docs site) from dbt/target as one fast-forward commit; refuses local paths/tokens</t>
         </is>
       </c>
-      <c r="D308" s="2" t="inlineStr"/>
+      <c r="D311" s="2" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>